<commit_message>
Add Household section in Demo_Generator
Test the household section with 1 and 2 persons.
</commit_message>
<xml_diff>
--- a/example/demo_generator/references/Household_Travel_Generate_Survey.xlsx
+++ b/example/demo_generator/references/Household_Travel_Generate_Survey.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28922"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="567" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C5483AD5-6D98-4611-80B2-E389FD18E1E7}"/>
+  <xr:revisionPtr revIDLastSave="681" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AB5A37E8-8767-4056-91CD-F7CE27EF0031}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="188">
   <si>
     <t>questionName</t>
   </si>
@@ -355,10 +355,89 @@
     <t>Save and continue</t>
   </si>
   <si>
+    <t>householdMembers</t>
+  </si>
+  <si>
+    <t>household</t>
+  </si>
+  <si>
+    <t>personNickname</t>
+  </si>
+  <si>
+    <t>nickname</t>
+  </si>
+  <si>
+    <t>**Nom ou surnom** pour identifier cette personne pour la suite de l'entrevue.
+__Peut être un surnom, des initiales, ou encore ce que cette personne est pour vous (ex: 'Moi', 'Toto', 'Maman', 'PN').
+Ce nom est seulement utilisé pour faciliter l'enquête et sera ensuite supprimé.__</t>
+  </si>
+  <si>
+    <t>**Name or nickname** that will allow you to identify this person for the remainder of the interview.
+__Can be a nickname, initials, or who this person represents to you (ex: 'Me','Kiddo','Mum','JT').
+The name is only used to simplify the response process and will be removed from the final dataset.__</t>
+  </si>
+  <si>
+    <t>personAge</t>
+  </si>
+  <si>
+    <t>personGender</t>
+  </si>
+  <si>
+    <t>personWorkerType</t>
+  </si>
+  <si>
+    <t>personSchoolType</t>
+  </si>
+  <si>
+    <t>personStudentType</t>
+  </si>
+  <si>
+    <t>personOccupation</t>
+  </si>
+  <si>
+    <t>personDrivingLicenseOwner</t>
+  </si>
+  <si>
+    <t>personCarSharingMember</t>
+  </si>
+  <si>
+    <t>personTransitFares</t>
+  </si>
+  <si>
+    <t>personHasDisability</t>
+  </si>
+  <si>
+    <t>personWorkLocationType</t>
+  </si>
+  <si>
+    <t>personSchoolLocationType</t>
+  </si>
+  <si>
+    <t>personUsualWorkPlaceName</t>
+  </si>
+  <si>
+    <t>personUsualWorkPlaceGeography</t>
+  </si>
+  <si>
+    <t>personUsualSchoolPlaceName</t>
+  </si>
+  <si>
+    <t>personUsualSchoolPlaceGeography</t>
+  </si>
+  <si>
+    <t>personTravelToWorkDays</t>
+  </si>
+  <si>
+    <t>personRemoteWorkDays</t>
+  </si>
+  <si>
+    <t>personTravelToStudyDays</t>
+  </si>
+  <si>
+    <t xml:space="preserve">personRemoteStudyDays   </t>
+  </si>
+  <si>
     <t>household_save</t>
-  </si>
-  <si>
-    <t>household</t>
   </si>
   <si>
     <t>completedText</t>
@@ -553,7 +632,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -618,6 +697,17 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -645,7 +735,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -677,11 +767,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -752,6 +851,48 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1158,14 +1299,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V20"/>
+  <dimension ref="A1:V42"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="19.85546875" style="9" customWidth="1"/>
     <col min="2" max="2" width="12.85546875" style="9" customWidth="1"/>
     <col min="3" max="3" width="6.42578125" style="9" customWidth="1"/>
     <col min="4" max="4" width="10.5703125" style="9" customWidth="1"/>
-    <col min="5" max="5" width="5.7109375" style="9" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.5703125" style="9" customWidth="1"/>
     <col min="6" max="6" width="17" style="9" customWidth="1"/>
     <col min="7" max="7" width="31.28515625" style="9" customWidth="1"/>
     <col min="8" max="8" width="31.5703125" style="9" bestFit="1" customWidth="1"/>
@@ -1478,7 +1619,7 @@
       </c>
       <c r="E7" s="10"/>
       <c r="F7" s="10" t="str">
-        <f t="shared" ref="F7:F19" si="0">REPLACE(A7, FIND("_", A7), 1, ".")</f>
+        <f t="shared" ref="F7:F41" si="0">REPLACE(A7, FIND("_", A7), 1, ".")</f>
         <v>home.address</v>
       </c>
       <c r="G7" s="10" t="s">
@@ -1949,147 +2090,905 @@
       <c r="V17" s="10"/>
     </row>
     <row r="18" spans="1:22">
-      <c r="A18" s="11" t="s">
+      <c r="A18" s="26" t="s">
         <v>95</v>
       </c>
-      <c r="B18" s="11" t="s">
+      <c r="B18" s="26" t="s">
         <v>96</v>
       </c>
-      <c r="C18" s="11" t="b">
+      <c r="C18" s="26" t="b">
         <v>1</v>
       </c>
       <c r="D18" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="E18" s="12"/>
-      <c r="F18" s="20" t="str">
+      <c r="E18" s="27"/>
+      <c r="F18" s="28" t="str">
         <f t="shared" si="0"/>
         <v>home.save</v>
       </c>
-      <c r="G18" s="11" t="s">
+      <c r="G18" s="26" t="s">
         <v>97</v>
       </c>
-      <c r="H18" s="11" t="s">
+      <c r="H18" s="26" t="s">
         <v>98</v>
       </c>
-      <c r="I18" s="11"/>
-      <c r="J18" s="12"/>
-      <c r="K18" s="12"/>
-      <c r="L18" s="12"/>
-      <c r="M18" s="12"/>
-      <c r="N18" s="12"/>
-      <c r="O18" s="12"/>
-      <c r="P18" s="12"/>
-      <c r="Q18" s="12"/>
+      <c r="I18" s="26"/>
+      <c r="J18" s="27"/>
+      <c r="K18" s="27"/>
+      <c r="L18" s="27"/>
+      <c r="M18" s="27"/>
+      <c r="N18" s="27"/>
+      <c r="O18" s="27"/>
+      <c r="P18" s="27"/>
+      <c r="Q18" s="27"/>
       <c r="R18" s="11" t="b">
         <v>1</v>
       </c>
-      <c r="S18" s="12"/>
-      <c r="T18" s="12"/>
-      <c r="U18" s="12"/>
-      <c r="V18" s="12"/>
-    </row>
-    <row r="19" spans="1:22">
-      <c r="A19" s="11" t="s">
+      <c r="S18" s="27"/>
+      <c r="T18" s="27"/>
+      <c r="U18" s="27"/>
+      <c r="V18" s="27"/>
+    </row>
+    <row r="19" spans="1:22" s="25" customFormat="1">
+      <c r="A19" s="33" t="s">
         <v>99</v>
       </c>
-      <c r="B19" s="11" t="s">
+      <c r="B19" s="30" t="s">
+        <v>67</v>
+      </c>
+      <c r="C19" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="D19" s="34" t="s">
+        <v>100</v>
+      </c>
+      <c r="E19" s="31"/>
+      <c r="F19" s="32"/>
+      <c r="G19" s="30"/>
+      <c r="H19" s="30"/>
+      <c r="I19" s="30"/>
+      <c r="J19" s="31"/>
+      <c r="K19" s="31"/>
+      <c r="L19" s="31"/>
+      <c r="M19" s="31"/>
+      <c r="N19" s="31"/>
+      <c r="O19" s="31"/>
+      <c r="P19" s="31"/>
+      <c r="Q19" s="31"/>
+      <c r="R19" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="S19" s="31"/>
+      <c r="T19" s="31"/>
+      <c r="U19" s="31"/>
+      <c r="V19" s="31"/>
+    </row>
+    <row r="20" spans="1:22" s="29" customFormat="1" ht="144" customHeight="1">
+      <c r="A20" s="37" t="s">
+        <v>101</v>
+      </c>
+      <c r="B20" s="34" t="s">
+        <v>23</v>
+      </c>
+      <c r="C20" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="D20" s="34" t="s">
+        <v>100</v>
+      </c>
+      <c r="E20" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="F20" s="28" t="s">
+        <v>102</v>
+      </c>
+      <c r="G20" s="34" t="s">
+        <v>103</v>
+      </c>
+      <c r="H20" s="38" t="s">
+        <v>104</v>
+      </c>
+      <c r="I20" s="26"/>
+      <c r="J20" s="27"/>
+      <c r="K20" s="27" t="s">
+        <v>93</v>
+      </c>
+      <c r="L20" s="35"/>
+      <c r="M20" s="27"/>
+      <c r="N20" s="27"/>
+      <c r="O20" s="27"/>
+      <c r="P20" s="27"/>
+      <c r="Q20" s="27"/>
+      <c r="R20" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="S20" s="27"/>
+      <c r="T20" s="27"/>
+      <c r="U20" s="27"/>
+      <c r="V20" s="27"/>
+    </row>
+    <row r="21" spans="1:22" s="29" customFormat="1" ht="27">
+      <c r="A21" s="36" t="s">
+        <v>105</v>
+      </c>
+      <c r="B21" s="26"/>
+      <c r="C21" s="34" t="b">
+        <v>0</v>
+      </c>
+      <c r="D21" s="34" t="s">
+        <v>100</v>
+      </c>
+      <c r="E21" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="F21" s="28"/>
+      <c r="G21" s="26"/>
+      <c r="H21" s="26"/>
+      <c r="I21" s="26"/>
+      <c r="J21" s="27"/>
+      <c r="K21" s="27"/>
+      <c r="L21" s="27"/>
+      <c r="M21" s="27"/>
+      <c r="N21" s="27"/>
+      <c r="O21" s="27"/>
+      <c r="P21" s="27"/>
+      <c r="Q21" s="27"/>
+      <c r="R21" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="S21" s="27"/>
+      <c r="T21" s="27"/>
+      <c r="U21" s="27"/>
+      <c r="V21" s="27"/>
+    </row>
+    <row r="22" spans="1:22" s="29" customFormat="1" ht="27">
+      <c r="A22" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="B22" s="26"/>
+      <c r="C22" s="34" t="b">
+        <v>0</v>
+      </c>
+      <c r="D22" s="34" t="s">
+        <v>100</v>
+      </c>
+      <c r="E22" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="F22" s="28"/>
+      <c r="G22" s="26"/>
+      <c r="H22" s="26"/>
+      <c r="I22" s="26"/>
+      <c r="J22" s="27"/>
+      <c r="K22" s="27"/>
+      <c r="L22" s="27"/>
+      <c r="M22" s="27"/>
+      <c r="N22" s="27"/>
+      <c r="O22" s="27"/>
+      <c r="P22" s="27"/>
+      <c r="Q22" s="27"/>
+      <c r="R22" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="S22" s="27"/>
+      <c r="T22" s="27"/>
+      <c r="U22" s="27"/>
+      <c r="V22" s="27"/>
+    </row>
+    <row r="23" spans="1:22" s="29" customFormat="1" ht="27">
+      <c r="A23" s="36" t="s">
+        <v>107</v>
+      </c>
+      <c r="B23" s="26"/>
+      <c r="C23" s="34" t="b">
+        <v>0</v>
+      </c>
+      <c r="D23" s="34" t="s">
+        <v>100</v>
+      </c>
+      <c r="E23" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="F23" s="28"/>
+      <c r="G23" s="26"/>
+      <c r="H23" s="26"/>
+      <c r="I23" s="26"/>
+      <c r="J23" s="27"/>
+      <c r="K23" s="27"/>
+      <c r="L23" s="27"/>
+      <c r="M23" s="27"/>
+      <c r="N23" s="27"/>
+      <c r="O23" s="27"/>
+      <c r="P23" s="27"/>
+      <c r="Q23" s="27"/>
+      <c r="R23" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="S23" s="27"/>
+      <c r="T23" s="27"/>
+      <c r="U23" s="27"/>
+      <c r="V23" s="27"/>
+    </row>
+    <row r="24" spans="1:22" s="29" customFormat="1" ht="27">
+      <c r="A24" s="36" t="s">
+        <v>108</v>
+      </c>
+      <c r="B24" s="26"/>
+      <c r="C24" s="34" t="b">
+        <v>0</v>
+      </c>
+      <c r="D24" s="34" t="s">
+        <v>100</v>
+      </c>
+      <c r="E24" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="F24" s="28"/>
+      <c r="G24" s="26"/>
+      <c r="H24" s="26"/>
+      <c r="I24" s="26"/>
+      <c r="J24" s="27"/>
+      <c r="K24" s="27"/>
+      <c r="L24" s="27"/>
+      <c r="M24" s="27"/>
+      <c r="N24" s="27"/>
+      <c r="O24" s="27"/>
+      <c r="P24" s="27"/>
+      <c r="Q24" s="27"/>
+      <c r="R24" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="S24" s="27"/>
+      <c r="T24" s="27"/>
+      <c r="U24" s="27"/>
+      <c r="V24" s="27"/>
+    </row>
+    <row r="25" spans="1:22" s="29" customFormat="1" ht="27">
+      <c r="A25" s="36" t="s">
+        <v>109</v>
+      </c>
+      <c r="B25" s="26"/>
+      <c r="C25" s="34" t="b">
+        <v>0</v>
+      </c>
+      <c r="D25" s="34" t="s">
+        <v>100</v>
+      </c>
+      <c r="E25" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="F25" s="28"/>
+      <c r="G25" s="26"/>
+      <c r="H25" s="26"/>
+      <c r="I25" s="26"/>
+      <c r="J25" s="27"/>
+      <c r="K25" s="27"/>
+      <c r="L25" s="27"/>
+      <c r="M25" s="27"/>
+      <c r="N25" s="27"/>
+      <c r="O25" s="27"/>
+      <c r="P25" s="27"/>
+      <c r="Q25" s="27"/>
+      <c r="R25" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="S25" s="27"/>
+      <c r="T25" s="27"/>
+      <c r="U25" s="27"/>
+      <c r="V25" s="27"/>
+    </row>
+    <row r="26" spans="1:22" s="29" customFormat="1" ht="27">
+      <c r="A26" s="36" t="s">
+        <v>110</v>
+      </c>
+      <c r="B26" s="26"/>
+      <c r="C26" s="34" t="b">
+        <v>0</v>
+      </c>
+      <c r="D26" s="34" t="s">
+        <v>100</v>
+      </c>
+      <c r="E26" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="F26" s="28"/>
+      <c r="G26" s="26"/>
+      <c r="H26" s="26"/>
+      <c r="I26" s="26"/>
+      <c r="J26" s="27"/>
+      <c r="K26" s="27"/>
+      <c r="L26" s="27"/>
+      <c r="M26" s="27"/>
+      <c r="N26" s="27"/>
+      <c r="O26" s="27"/>
+      <c r="P26" s="27"/>
+      <c r="Q26" s="27"/>
+      <c r="R26" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="S26" s="27"/>
+      <c r="T26" s="27"/>
+      <c r="U26" s="27"/>
+      <c r="V26" s="27"/>
+    </row>
+    <row r="27" spans="1:22" s="29" customFormat="1" ht="27">
+      <c r="A27" s="36" t="s">
+        <v>111</v>
+      </c>
+      <c r="B27" s="26"/>
+      <c r="C27" s="34" t="b">
+        <v>0</v>
+      </c>
+      <c r="D27" s="34" t="s">
+        <v>100</v>
+      </c>
+      <c r="E27" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="F27" s="28"/>
+      <c r="G27" s="26"/>
+      <c r="H27" s="26"/>
+      <c r="I27" s="26"/>
+      <c r="J27" s="27"/>
+      <c r="K27" s="27"/>
+      <c r="L27" s="27"/>
+      <c r="M27" s="27"/>
+      <c r="N27" s="27"/>
+      <c r="O27" s="27"/>
+      <c r="P27" s="27"/>
+      <c r="Q27" s="27"/>
+      <c r="R27" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="S27" s="27"/>
+      <c r="T27" s="27"/>
+      <c r="U27" s="27"/>
+      <c r="V27" s="27"/>
+    </row>
+    <row r="28" spans="1:22" s="29" customFormat="1" ht="27">
+      <c r="A28" s="36" t="s">
+        <v>112</v>
+      </c>
+      <c r="B28" s="26"/>
+      <c r="C28" s="34" t="b">
+        <v>0</v>
+      </c>
+      <c r="D28" s="34" t="s">
+        <v>100</v>
+      </c>
+      <c r="E28" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="F28" s="28"/>
+      <c r="G28" s="26"/>
+      <c r="H28" s="26"/>
+      <c r="I28" s="26"/>
+      <c r="J28" s="27"/>
+      <c r="K28" s="27"/>
+      <c r="L28" s="27"/>
+      <c r="M28" s="27"/>
+      <c r="N28" s="27"/>
+      <c r="O28" s="27"/>
+      <c r="P28" s="27"/>
+      <c r="Q28" s="27"/>
+      <c r="R28" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="S28" s="27"/>
+      <c r="T28" s="27"/>
+      <c r="U28" s="27"/>
+      <c r="V28" s="27"/>
+    </row>
+    <row r="29" spans="1:22" s="29" customFormat="1" ht="27">
+      <c r="A29" s="36" t="s">
+        <v>113</v>
+      </c>
+      <c r="B29" s="26"/>
+      <c r="C29" s="34" t="b">
+        <v>0</v>
+      </c>
+      <c r="D29" s="34" t="s">
+        <v>100</v>
+      </c>
+      <c r="E29" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="F29" s="28"/>
+      <c r="G29" s="26"/>
+      <c r="H29" s="26"/>
+      <c r="I29" s="26"/>
+      <c r="J29" s="27"/>
+      <c r="K29" s="27"/>
+      <c r="L29" s="27"/>
+      <c r="M29" s="27"/>
+      <c r="N29" s="27"/>
+      <c r="O29" s="27"/>
+      <c r="P29" s="27"/>
+      <c r="Q29" s="27"/>
+      <c r="R29" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="S29" s="27"/>
+      <c r="T29" s="27"/>
+      <c r="U29" s="27"/>
+      <c r="V29" s="27"/>
+    </row>
+    <row r="30" spans="1:22" s="29" customFormat="1" ht="27">
+      <c r="A30" s="36" t="s">
+        <v>114</v>
+      </c>
+      <c r="B30" s="26"/>
+      <c r="C30" s="34" t="b">
+        <v>0</v>
+      </c>
+      <c r="D30" s="34" t="s">
+        <v>100</v>
+      </c>
+      <c r="E30" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="F30" s="28"/>
+      <c r="G30" s="26"/>
+      <c r="H30" s="26"/>
+      <c r="I30" s="26"/>
+      <c r="J30" s="27"/>
+      <c r="K30" s="27"/>
+      <c r="L30" s="27"/>
+      <c r="M30" s="27"/>
+      <c r="N30" s="27"/>
+      <c r="O30" s="27"/>
+      <c r="P30" s="27"/>
+      <c r="Q30" s="27"/>
+      <c r="R30" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="S30" s="27"/>
+      <c r="T30" s="27"/>
+      <c r="U30" s="27"/>
+      <c r="V30" s="27"/>
+    </row>
+    <row r="31" spans="1:22" s="29" customFormat="1" ht="27">
+      <c r="A31" s="36" t="s">
+        <v>115</v>
+      </c>
+      <c r="B31" s="26"/>
+      <c r="C31" s="34" t="b">
+        <v>0</v>
+      </c>
+      <c r="D31" s="34" t="s">
+        <v>100</v>
+      </c>
+      <c r="E31" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="F31" s="28"/>
+      <c r="G31" s="26"/>
+      <c r="H31" s="26"/>
+      <c r="I31" s="26"/>
+      <c r="J31" s="27"/>
+      <c r="K31" s="27"/>
+      <c r="L31" s="27"/>
+      <c r="M31" s="27"/>
+      <c r="N31" s="27"/>
+      <c r="O31" s="27"/>
+      <c r="P31" s="27"/>
+      <c r="Q31" s="27"/>
+      <c r="R31" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="S31" s="27"/>
+      <c r="T31" s="27"/>
+      <c r="U31" s="27"/>
+      <c r="V31" s="27"/>
+    </row>
+    <row r="32" spans="1:22" s="29" customFormat="1" ht="27">
+      <c r="A32" s="36" t="s">
+        <v>116</v>
+      </c>
+      <c r="B32" s="26"/>
+      <c r="C32" s="34" t="b">
+        <v>0</v>
+      </c>
+      <c r="D32" s="34" t="s">
+        <v>100</v>
+      </c>
+      <c r="E32" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="F32" s="28"/>
+      <c r="G32" s="26"/>
+      <c r="H32" s="26"/>
+      <c r="I32" s="26"/>
+      <c r="J32" s="27"/>
+      <c r="K32" s="27"/>
+      <c r="L32" s="27"/>
+      <c r="M32" s="27"/>
+      <c r="N32" s="27"/>
+      <c r="O32" s="27"/>
+      <c r="P32" s="27"/>
+      <c r="Q32" s="27"/>
+      <c r="R32" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="S32" s="27"/>
+      <c r="T32" s="27"/>
+      <c r="U32" s="27"/>
+      <c r="V32" s="27"/>
+    </row>
+    <row r="33" spans="1:22" s="29" customFormat="1" ht="27">
+      <c r="A33" s="36" t="s">
+        <v>117</v>
+      </c>
+      <c r="B33" s="26"/>
+      <c r="C33" s="34" t="b">
+        <v>0</v>
+      </c>
+      <c r="D33" s="34" t="s">
+        <v>100</v>
+      </c>
+      <c r="E33" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="F33" s="28"/>
+      <c r="G33" s="26"/>
+      <c r="H33" s="26"/>
+      <c r="I33" s="26"/>
+      <c r="J33" s="27"/>
+      <c r="K33" s="27"/>
+      <c r="L33" s="27"/>
+      <c r="M33" s="27"/>
+      <c r="N33" s="27"/>
+      <c r="O33" s="27"/>
+      <c r="P33" s="27"/>
+      <c r="Q33" s="27"/>
+      <c r="R33" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="S33" s="27"/>
+      <c r="T33" s="27"/>
+      <c r="U33" s="27"/>
+      <c r="V33" s="27"/>
+    </row>
+    <row r="34" spans="1:22" s="29" customFormat="1" ht="27">
+      <c r="A34" s="36" t="s">
+        <v>118</v>
+      </c>
+      <c r="B34" s="26"/>
+      <c r="C34" s="34" t="b">
+        <v>0</v>
+      </c>
+      <c r="D34" s="34" t="s">
+        <v>100</v>
+      </c>
+      <c r="E34" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="F34" s="28"/>
+      <c r="G34" s="26"/>
+      <c r="H34" s="26"/>
+      <c r="I34" s="26"/>
+      <c r="J34" s="27"/>
+      <c r="K34" s="27"/>
+      <c r="L34" s="27"/>
+      <c r="M34" s="27"/>
+      <c r="N34" s="27"/>
+      <c r="O34" s="27"/>
+      <c r="P34" s="27"/>
+      <c r="Q34" s="27"/>
+      <c r="R34" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="S34" s="27"/>
+      <c r="T34" s="27"/>
+      <c r="U34" s="27"/>
+      <c r="V34" s="27"/>
+    </row>
+    <row r="35" spans="1:22" s="29" customFormat="1" ht="27">
+      <c r="A35" s="36" t="s">
+        <v>119</v>
+      </c>
+      <c r="B35" s="26"/>
+      <c r="C35" s="34" t="b">
+        <v>0</v>
+      </c>
+      <c r="D35" s="34" t="s">
+        <v>100</v>
+      </c>
+      <c r="E35" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="F35" s="28"/>
+      <c r="G35" s="26"/>
+      <c r="H35" s="26"/>
+      <c r="I35" s="26"/>
+      <c r="J35" s="27"/>
+      <c r="K35" s="27"/>
+      <c r="L35" s="27"/>
+      <c r="M35" s="27"/>
+      <c r="N35" s="27"/>
+      <c r="O35" s="27"/>
+      <c r="P35" s="27"/>
+      <c r="Q35" s="27"/>
+      <c r="R35" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="S35" s="27"/>
+      <c r="T35" s="27"/>
+      <c r="U35" s="27"/>
+      <c r="V35" s="27"/>
+    </row>
+    <row r="36" spans="1:22" s="29" customFormat="1" ht="27">
+      <c r="A36" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="B36" s="26"/>
+      <c r="C36" s="34" t="b">
+        <v>0</v>
+      </c>
+      <c r="D36" s="34" t="s">
+        <v>100</v>
+      </c>
+      <c r="E36" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="F36" s="28"/>
+      <c r="G36" s="26"/>
+      <c r="H36" s="26"/>
+      <c r="I36" s="26"/>
+      <c r="J36" s="27"/>
+      <c r="K36" s="27"/>
+      <c r="L36" s="27"/>
+      <c r="M36" s="27"/>
+      <c r="N36" s="27"/>
+      <c r="O36" s="27"/>
+      <c r="P36" s="27"/>
+      <c r="Q36" s="27"/>
+      <c r="R36" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="S36" s="27"/>
+      <c r="T36" s="27"/>
+      <c r="U36" s="27"/>
+      <c r="V36" s="27"/>
+    </row>
+    <row r="37" spans="1:22" s="29" customFormat="1" ht="27">
+      <c r="A37" s="36" t="s">
+        <v>121</v>
+      </c>
+      <c r="B37" s="26"/>
+      <c r="C37" s="34" t="b">
+        <v>0</v>
+      </c>
+      <c r="D37" s="34" t="s">
+        <v>100</v>
+      </c>
+      <c r="E37" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="F37" s="28"/>
+      <c r="G37" s="26"/>
+      <c r="H37" s="26"/>
+      <c r="I37" s="26"/>
+      <c r="J37" s="27"/>
+      <c r="K37" s="27"/>
+      <c r="L37" s="27"/>
+      <c r="M37" s="27"/>
+      <c r="N37" s="27"/>
+      <c r="O37" s="27"/>
+      <c r="P37" s="27"/>
+      <c r="Q37" s="27"/>
+      <c r="R37" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="S37" s="27"/>
+      <c r="T37" s="27"/>
+      <c r="U37" s="27"/>
+      <c r="V37" s="27"/>
+    </row>
+    <row r="38" spans="1:22" s="29" customFormat="1" ht="27">
+      <c r="A38" s="36" t="s">
+        <v>122</v>
+      </c>
+      <c r="B38" s="26"/>
+      <c r="C38" s="34" t="b">
+        <v>0</v>
+      </c>
+      <c r="D38" s="34" t="s">
+        <v>100</v>
+      </c>
+      <c r="E38" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="F38" s="28"/>
+      <c r="G38" s="26"/>
+      <c r="H38" s="26"/>
+      <c r="I38" s="26"/>
+      <c r="J38" s="27"/>
+      <c r="K38" s="27"/>
+      <c r="L38" s="27"/>
+      <c r="M38" s="27"/>
+      <c r="N38" s="27"/>
+      <c r="O38" s="27"/>
+      <c r="P38" s="27"/>
+      <c r="Q38" s="27"/>
+      <c r="R38" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="S38" s="27"/>
+      <c r="T38" s="27"/>
+      <c r="U38" s="27"/>
+      <c r="V38" s="27"/>
+    </row>
+    <row r="39" spans="1:22" s="29" customFormat="1" ht="27">
+      <c r="A39" s="36" t="s">
+        <v>123</v>
+      </c>
+      <c r="B39" s="26"/>
+      <c r="C39" s="34" t="b">
+        <v>0</v>
+      </c>
+      <c r="D39" s="34" t="s">
+        <v>100</v>
+      </c>
+      <c r="E39" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="F39" s="28"/>
+      <c r="G39" s="26"/>
+      <c r="H39" s="26"/>
+      <c r="I39" s="26"/>
+      <c r="J39" s="27"/>
+      <c r="K39" s="27"/>
+      <c r="L39" s="27"/>
+      <c r="M39" s="27"/>
+      <c r="N39" s="27"/>
+      <c r="O39" s="27"/>
+      <c r="P39" s="27"/>
+      <c r="Q39" s="27"/>
+      <c r="R39" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="S39" s="27"/>
+      <c r="T39" s="27"/>
+      <c r="U39" s="27"/>
+      <c r="V39" s="27"/>
+    </row>
+    <row r="40" spans="1:22" s="29" customFormat="1" ht="27">
+      <c r="A40" s="36" t="s">
+        <v>124</v>
+      </c>
+      <c r="B40" s="26"/>
+      <c r="C40" s="34" t="b">
+        <v>0</v>
+      </c>
+      <c r="D40" s="34" t="s">
+        <v>100</v>
+      </c>
+      <c r="E40" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="F40" s="28"/>
+      <c r="G40" s="26"/>
+      <c r="H40" s="26"/>
+      <c r="I40" s="26"/>
+      <c r="J40" s="27"/>
+      <c r="K40" s="27"/>
+      <c r="L40" s="27"/>
+      <c r="M40" s="27"/>
+      <c r="N40" s="27"/>
+      <c r="O40" s="27"/>
+      <c r="P40" s="27"/>
+      <c r="Q40" s="27"/>
+      <c r="R40" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="S40" s="27"/>
+      <c r="T40" s="27"/>
+      <c r="U40" s="27"/>
+      <c r="V40" s="27"/>
+    </row>
+    <row r="41" spans="1:22">
+      <c r="A41" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="B41" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="C19" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="D19" s="11" t="s">
+      <c r="C41" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="D41" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="E19" s="12"/>
-      <c r="F19" s="20" t="str">
+      <c r="E41" s="12"/>
+      <c r="F41" s="20" t="str">
         <f t="shared" si="0"/>
         <v>household.save</v>
       </c>
-      <c r="G19" s="11" t="s">
+      <c r="G41" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="H19" s="11" t="s">
+      <c r="H41" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="I19" s="11"/>
-      <c r="J19" s="12"/>
-      <c r="K19" s="12"/>
-      <c r="L19" s="12"/>
-      <c r="M19" s="12"/>
-      <c r="N19" s="12"/>
-      <c r="O19" s="12"/>
-      <c r="P19" s="12"/>
-      <c r="Q19" s="12"/>
-      <c r="R19" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="S19" s="12"/>
-      <c r="T19" s="12"/>
-      <c r="U19" s="12"/>
-      <c r="V19" s="12"/>
-    </row>
-    <row r="20" spans="1:22" ht="130.5">
-      <c r="A20" s="9" t="s">
-        <v>101</v>
-      </c>
-      <c r="B20" s="9" t="s">
+      <c r="I41" s="11"/>
+      <c r="J41" s="12"/>
+      <c r="K41" s="12"/>
+      <c r="L41" s="12"/>
+      <c r="M41" s="12"/>
+      <c r="N41" s="12"/>
+      <c r="O41" s="12"/>
+      <c r="P41" s="12"/>
+      <c r="Q41" s="12"/>
+      <c r="R41" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="S41" s="12"/>
+      <c r="T41" s="12"/>
+      <c r="U41" s="12"/>
+      <c r="V41" s="12"/>
+    </row>
+    <row r="42" spans="1:22" ht="130.5">
+      <c r="A42" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="B42" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="C20" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="D20" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="F20" s="9" t="s">
-        <v>101</v>
-      </c>
-      <c r="G20" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="H20" s="9" t="s">
-        <v>104</v>
-      </c>
-      <c r="J20" s="24"/>
-      <c r="K20" s="22"/>
-      <c r="R20" s="9" t="b">
+      <c r="C42" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="D42" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="F42" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="G42" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="H42" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="J42" s="24"/>
+      <c r="K42" s="22"/>
+      <c r="R42" s="9" t="b">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="C21:C1048576 C1:C19">
+  <conditionalFormatting sqref="C43:C1048576 C1:C41">
     <cfRule type="cellIs" dxfId="6" priority="7" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C21:C1048576 C1:C19">
+  <conditionalFormatting sqref="C43:C1048576 C1:C41">
     <cfRule type="containsText" dxfId="5" priority="6" operator="containsText" text="FALSE">
       <formula>NOT(ISERROR(SEARCH("FALSE",C1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C20">
+  <conditionalFormatting sqref="C42">
     <cfRule type="containsText" dxfId="4" priority="3" operator="containsText" text="FALSE">
-      <formula>NOT(ISERROR(SEARCH("FALSE",C20)))</formula>
+      <formula>NOT(ISERROR(SEARCH("FALSE",C42)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="TRUE">
-      <formula>NOT(ISERROR(SEARCH("TRUE",C20)))</formula>
+      <formula>NOT(ISERROR(SEARCH("TRUE",C42)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L20:O20">
+  <conditionalFormatting sqref="L42:O42">
     <cfRule type="expression" dxfId="2" priority="1">
-      <formula>AND($B1048348="Custom",  $B1048348&lt;&gt;"", ROW(L1048348)&lt;&gt;1)</formula>
+      <formula>AND($B1048370="Custom",  $B1048370&lt;&gt;"", ROW(L1048370)&lt;&gt;1)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M20:N20">
+  <conditionalFormatting sqref="M42:N42">
     <cfRule type="expression" dxfId="1" priority="5">
-      <formula>AND($B20&lt;&gt;"Select", $B20&lt;&gt;"Checkbox", $B20&lt;&gt;"Radio",  $B20&lt;&gt;"", ROW(M20)&lt;&gt;1)</formula>
+      <formula>AND($B42&lt;&gt;"Select", $B42&lt;&gt;"Checkbox", $B42&lt;&gt;"Radio",  $B42&lt;&gt;"", ROW(M42)&lt;&gt;1)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O20">
+  <conditionalFormatting sqref="O42">
     <cfRule type="expression" dxfId="0" priority="2">
-      <formula>AND($B20&lt;&gt;"Range", $B20&lt;&gt;"", ROW(O20)&lt;&gt;1)</formula>
+      <formula>AND($B42&lt;&gt;"Range", $B42&lt;&gt;"", ROW(O42)&lt;&gt;1)</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2111,34 +3010,34 @@
   <sheetData>
     <row r="1" spans="1:6" s="6" customFormat="1">
       <c r="A1" s="16" t="s">
-        <v>105</v>
+        <v>130</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>106</v>
+        <v>131</v>
       </c>
       <c r="C1" s="16" t="s">
         <v>5</v>
       </c>
       <c r="D1" s="18" t="s">
-        <v>107</v>
+        <v>132</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>108</v>
+        <v>133</v>
       </c>
       <c r="F1" s="16" t="s">
-        <v>109</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="29.25">
       <c r="A2" s="14" t="s">
-        <v>110</v>
+        <v>135</v>
       </c>
       <c r="B2" s="14"/>
       <c r="C2" s="14" t="s">
-        <v>111</v>
+        <v>136</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>112</v>
+        <v>137</v>
       </c>
       <c r="E2" s="14">
         <v>1</v>
@@ -2151,10 +3050,10 @@
       </c>
       <c r="B3" s="14"/>
       <c r="C3" s="14" t="s">
-        <v>111</v>
+        <v>136</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>113</v>
+        <v>138</v>
       </c>
       <c r="E3" s="14">
         <v>2</v>
@@ -2186,25 +3085,25 @@
         <v>3</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>114</v>
+        <v>139</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>115</v>
+        <v>140</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>116</v>
+        <v>141</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>117</v>
+        <v>142</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>118</v>
+        <v>143</v>
       </c>
       <c r="G1" s="21" t="s">
-        <v>119</v>
+        <v>144</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>120</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -2212,13 +3111,13 @@
         <v>24</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>121</v>
+        <v>146</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>122</v>
+        <v>147</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>123</v>
+        <v>148</v>
       </c>
       <c r="E2" s="14" t="b">
         <v>1</v>
@@ -2235,13 +3134,13 @@
         <v>100</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>124</v>
+        <v>149</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>125</v>
+        <v>150</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>126</v>
+        <v>151</v>
       </c>
       <c r="E3" s="14" t="b">
         <v>1</v>
@@ -2255,16 +3154,16 @@
     </row>
     <row r="4" spans="1:8" ht="29.25">
       <c r="A4" s="14" t="s">
-        <v>102</v>
+        <v>127</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>127</v>
+        <v>152</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>128</v>
+        <v>153</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>129</v>
+        <v>154</v>
       </c>
       <c r="E4" s="14" t="b">
         <v>0</v>
@@ -2296,10 +3195,10 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="3" t="s">
-        <v>130</v>
+        <v>155</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>108</v>
+        <v>133</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>6</v>
@@ -2308,7 +3207,7 @@
         <v>7</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>131</v>
+        <v>156</v>
       </c>
       <c r="F1" s="3" t="s">
         <v>10</v>
@@ -2316,72 +3215,72 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>132</v>
+        <v>157</v>
       </c>
       <c r="B2" t="s">
-        <v>132</v>
+        <v>157</v>
       </c>
       <c r="C2" t="s">
-        <v>133</v>
+        <v>158</v>
       </c>
       <c r="D2" t="s">
-        <v>134</v>
+        <v>159</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>135</v>
+        <v>160</v>
       </c>
       <c r="B3" t="s">
-        <v>135</v>
+        <v>160</v>
       </c>
       <c r="C3" t="s">
-        <v>136</v>
+        <v>161</v>
       </c>
       <c r="D3" t="s">
-        <v>137</v>
+        <v>162</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>138</v>
+        <v>163</v>
       </c>
       <c r="B4" t="s">
-        <v>138</v>
+        <v>163</v>
       </c>
       <c r="C4" t="s">
-        <v>139</v>
+        <v>164</v>
       </c>
       <c r="D4" t="s">
-        <v>140</v>
+        <v>165</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>141</v>
+        <v>166</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>141</v>
+        <v>166</v>
       </c>
       <c r="C5" t="s">
-        <v>142</v>
+        <v>167</v>
       </c>
       <c r="D5" t="s">
-        <v>143</v>
+        <v>168</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>144</v>
+        <v>169</v>
       </c>
       <c r="B6" t="s">
-        <v>144</v>
+        <v>169</v>
       </c>
       <c r="C6" t="s">
-        <v>145</v>
+        <v>170</v>
       </c>
       <c r="D6" t="s">
-        <v>146</v>
+        <v>171</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -2389,7 +3288,7 @@
         <v>31</v>
       </c>
       <c r="E7" t="s">
-        <v>132</v>
+        <v>157</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -2397,12 +3296,12 @@
         <v>31</v>
       </c>
       <c r="E8" t="s">
-        <v>135</v>
+        <v>160</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>147</v>
+        <v>172</v>
       </c>
       <c r="E9" t="s">
         <v>31</v>
@@ -2410,10 +3309,10 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>147</v>
+        <v>172</v>
       </c>
       <c r="E10" t="s">
-        <v>141</v>
+        <v>166</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -2421,7 +3320,7 @@
         <v>94</v>
       </c>
       <c r="E11" t="s">
-        <v>132</v>
+        <v>157</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -2429,7 +3328,7 @@
         <v>94</v>
       </c>
       <c r="E12" t="s">
-        <v>135</v>
+        <v>160</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -2437,7 +3336,7 @@
         <v>94</v>
       </c>
       <c r="E13" t="s">
-        <v>144</v>
+        <v>169</v>
       </c>
     </row>
   </sheetData>
@@ -2464,40 +3363,40 @@
   <sheetData>
     <row r="1" spans="1:12" s="5" customFormat="1">
       <c r="A1" s="4" t="s">
-        <v>148</v>
+        <v>173</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>149</v>
+        <v>174</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>150</v>
+        <v>175</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>151</v>
+        <v>176</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>152</v>
+        <v>177</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>153</v>
+        <v>178</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>154</v>
+        <v>179</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>155</v>
+        <v>180</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>156</v>
+        <v>181</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>157</v>
+        <v>182</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>158</v>
+        <v>183</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>159</v>
+        <v>184</v>
       </c>
     </row>
   </sheetData>
@@ -2512,19 +3411,19 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>160</v>
+        <v>185</v>
       </c>
       <c r="B1" t="s">
         <v>6</v>
       </c>
       <c r="C1" t="s">
-        <v>161</v>
+        <v>186</v>
       </c>
       <c r="D1" t="s">
         <v>7</v>
       </c>
       <c r="E1" t="s">
-        <v>162</v>
+        <v>187</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
BREAKING POINT: Rename preload to customPreload
Add some customPreload to the Demo_Generator.
Add the function countAdults and some tests in the helper.
Add preload for each section, because we need to call the customPreloadBase in each section.
BREAKING POINT: You need to rename each preload to customPreload in each survey.
</commit_message>
<xml_diff>
--- a/example/demo_generator/references/Household_Travel_Generate_Survey.xlsx
+++ b/example/demo_generator/references/Household_Travel_Generate_Survey.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28922"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28926"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="681" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AB5A37E8-8767-4056-91CD-F7CE27EF0031}"/>
+  <xr:revisionPtr revIDLastSave="684" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AD6D3077-663E-4E58-A164-1387DA22EFF7}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Widgets" sheetId="1" r:id="rId1"/>
@@ -780,7 +780,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -855,16 +855,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -879,19 +870,13 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2102,8 +2087,8 @@
       <c r="D18" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="E18" s="27"/>
-      <c r="F18" s="28" t="str">
+      <c r="E18" s="10"/>
+      <c r="F18" s="7" t="str">
         <f t="shared" si="0"/>
         <v>home.save</v>
       </c>
@@ -2114,779 +2099,779 @@
         <v>98</v>
       </c>
       <c r="I18" s="26"/>
-      <c r="J18" s="27"/>
-      <c r="K18" s="27"/>
-      <c r="L18" s="27"/>
-      <c r="M18" s="27"/>
-      <c r="N18" s="27"/>
-      <c r="O18" s="27"/>
-      <c r="P18" s="27"/>
-      <c r="Q18" s="27"/>
+      <c r="J18" s="10"/>
+      <c r="K18" s="10"/>
+      <c r="L18" s="10"/>
+      <c r="M18" s="10"/>
+      <c r="N18" s="10"/>
+      <c r="O18" s="10"/>
+      <c r="P18" s="10"/>
+      <c r="Q18" s="10"/>
       <c r="R18" s="11" t="b">
         <v>1</v>
       </c>
-      <c r="S18" s="27"/>
-      <c r="T18" s="27"/>
-      <c r="U18" s="27"/>
-      <c r="V18" s="27"/>
+      <c r="S18" s="10"/>
+      <c r="T18" s="10"/>
+      <c r="U18" s="10"/>
+      <c r="V18" s="10"/>
     </row>
     <row r="19" spans="1:22" s="25" customFormat="1">
-      <c r="A19" s="33" t="s">
+      <c r="A19" s="30" t="s">
         <v>99</v>
       </c>
-      <c r="B19" s="30" t="s">
+      <c r="B19" s="27" t="s">
         <v>67</v>
       </c>
-      <c r="C19" s="33" t="b">
-        <v>1</v>
-      </c>
-      <c r="D19" s="34" t="s">
+      <c r="C19" s="30" t="b">
+        <v>1</v>
+      </c>
+      <c r="D19" s="31" t="s">
         <v>100</v>
       </c>
-      <c r="E19" s="31"/>
-      <c r="F19" s="32"/>
-      <c r="G19" s="30"/>
-      <c r="H19" s="30"/>
-      <c r="I19" s="30"/>
-      <c r="J19" s="31"/>
-      <c r="K19" s="31"/>
-      <c r="L19" s="31"/>
-      <c r="M19" s="31"/>
-      <c r="N19" s="31"/>
-      <c r="O19" s="31"/>
-      <c r="P19" s="31"/>
-      <c r="Q19" s="31"/>
-      <c r="R19" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="S19" s="31"/>
-      <c r="T19" s="31"/>
-      <c r="U19" s="31"/>
-      <c r="V19" s="31"/>
-    </row>
-    <row r="20" spans="1:22" s="29" customFormat="1" ht="144" customHeight="1">
-      <c r="A20" s="37" t="s">
+      <c r="E19" s="28"/>
+      <c r="F19" s="29"/>
+      <c r="G19" s="27"/>
+      <c r="H19" s="27"/>
+      <c r="I19" s="27"/>
+      <c r="J19" s="28"/>
+      <c r="K19" s="28"/>
+      <c r="L19" s="28"/>
+      <c r="M19" s="28"/>
+      <c r="N19" s="28"/>
+      <c r="O19" s="28"/>
+      <c r="P19" s="28"/>
+      <c r="Q19" s="28"/>
+      <c r="R19" s="31" t="b">
+        <v>1</v>
+      </c>
+      <c r="S19" s="28"/>
+      <c r="T19" s="28"/>
+      <c r="U19" s="28"/>
+      <c r="V19" s="28"/>
+    </row>
+    <row r="20" spans="1:22" ht="144" customHeight="1">
+      <c r="A20" s="31" t="s">
         <v>101</v>
       </c>
-      <c r="B20" s="34" t="s">
+      <c r="B20" s="31" t="s">
         <v>23</v>
       </c>
-      <c r="C20" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="D20" s="34" t="s">
+      <c r="C20" s="31" t="b">
+        <v>1</v>
+      </c>
+      <c r="D20" s="31" t="s">
         <v>100</v>
       </c>
-      <c r="E20" s="27" t="s">
+      <c r="E20" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="F20" s="28" t="s">
+      <c r="F20" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="G20" s="34" t="s">
+      <c r="G20" s="31" t="s">
         <v>103</v>
       </c>
-      <c r="H20" s="38" t="s">
+      <c r="H20" s="33" t="s">
         <v>104</v>
       </c>
       <c r="I20" s="26"/>
-      <c r="J20" s="27"/>
-      <c r="K20" s="27" t="s">
+      <c r="J20" s="10"/>
+      <c r="K20" s="10" t="s">
         <v>93</v>
       </c>
-      <c r="L20" s="35"/>
-      <c r="M20" s="27"/>
-      <c r="N20" s="27"/>
-      <c r="O20" s="27"/>
-      <c r="P20" s="27"/>
-      <c r="Q20" s="27"/>
-      <c r="R20" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="S20" s="27"/>
-      <c r="T20" s="27"/>
-      <c r="U20" s="27"/>
-      <c r="V20" s="27"/>
-    </row>
-    <row r="21" spans="1:22" s="29" customFormat="1" ht="27">
-      <c r="A21" s="36" t="s">
+      <c r="L20" s="13"/>
+      <c r="M20" s="10"/>
+      <c r="N20" s="10"/>
+      <c r="O20" s="10"/>
+      <c r="P20" s="10"/>
+      <c r="Q20" s="10"/>
+      <c r="R20" s="31" t="b">
+        <v>1</v>
+      </c>
+      <c r="S20" s="10"/>
+      <c r="T20" s="10"/>
+      <c r="U20" s="10"/>
+      <c r="V20" s="10"/>
+    </row>
+    <row r="21" spans="1:22" ht="27">
+      <c r="A21" s="32" t="s">
         <v>105</v>
       </c>
       <c r="B21" s="26"/>
-      <c r="C21" s="34" t="b">
+      <c r="C21" s="31" t="b">
         <v>0</v>
       </c>
-      <c r="D21" s="34" t="s">
+      <c r="D21" s="31" t="s">
         <v>100</v>
       </c>
-      <c r="E21" s="27" t="s">
+      <c r="E21" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="F21" s="28"/>
+      <c r="F21" s="7"/>
       <c r="G21" s="26"/>
       <c r="H21" s="26"/>
       <c r="I21" s="26"/>
-      <c r="J21" s="27"/>
-      <c r="K21" s="27"/>
-      <c r="L21" s="27"/>
-      <c r="M21" s="27"/>
-      <c r="N21" s="27"/>
-      <c r="O21" s="27"/>
-      <c r="P21" s="27"/>
-      <c r="Q21" s="27"/>
-      <c r="R21" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="S21" s="27"/>
-      <c r="T21" s="27"/>
-      <c r="U21" s="27"/>
-      <c r="V21" s="27"/>
-    </row>
-    <row r="22" spans="1:22" s="29" customFormat="1" ht="27">
-      <c r="A22" s="36" t="s">
+      <c r="J21" s="10"/>
+      <c r="K21" s="10"/>
+      <c r="L21" s="10"/>
+      <c r="M21" s="10"/>
+      <c r="N21" s="10"/>
+      <c r="O21" s="10"/>
+      <c r="P21" s="10"/>
+      <c r="Q21" s="10"/>
+      <c r="R21" s="31" t="b">
+        <v>1</v>
+      </c>
+      <c r="S21" s="10"/>
+      <c r="T21" s="10"/>
+      <c r="U21" s="10"/>
+      <c r="V21" s="10"/>
+    </row>
+    <row r="22" spans="1:22" ht="27">
+      <c r="A22" s="32" t="s">
         <v>106</v>
       </c>
       <c r="B22" s="26"/>
-      <c r="C22" s="34" t="b">
+      <c r="C22" s="31" t="b">
         <v>0</v>
       </c>
-      <c r="D22" s="34" t="s">
+      <c r="D22" s="31" t="s">
         <v>100</v>
       </c>
-      <c r="E22" s="27" t="s">
+      <c r="E22" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="F22" s="28"/>
+      <c r="F22" s="7"/>
       <c r="G22" s="26"/>
       <c r="H22" s="26"/>
       <c r="I22" s="26"/>
-      <c r="J22" s="27"/>
-      <c r="K22" s="27"/>
-      <c r="L22" s="27"/>
-      <c r="M22" s="27"/>
-      <c r="N22" s="27"/>
-      <c r="O22" s="27"/>
-      <c r="P22" s="27"/>
-      <c r="Q22" s="27"/>
-      <c r="R22" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="S22" s="27"/>
-      <c r="T22" s="27"/>
-      <c r="U22" s="27"/>
-      <c r="V22" s="27"/>
-    </row>
-    <row r="23" spans="1:22" s="29" customFormat="1" ht="27">
-      <c r="A23" s="36" t="s">
+      <c r="J22" s="10"/>
+      <c r="K22" s="10"/>
+      <c r="L22" s="10"/>
+      <c r="M22" s="10"/>
+      <c r="N22" s="10"/>
+      <c r="O22" s="10"/>
+      <c r="P22" s="10"/>
+      <c r="Q22" s="10"/>
+      <c r="R22" s="31" t="b">
+        <v>1</v>
+      </c>
+      <c r="S22" s="10"/>
+      <c r="T22" s="10"/>
+      <c r="U22" s="10"/>
+      <c r="V22" s="10"/>
+    </row>
+    <row r="23" spans="1:22" ht="27">
+      <c r="A23" s="32" t="s">
         <v>107</v>
       </c>
       <c r="B23" s="26"/>
-      <c r="C23" s="34" t="b">
+      <c r="C23" s="31" t="b">
         <v>0</v>
       </c>
-      <c r="D23" s="34" t="s">
+      <c r="D23" s="31" t="s">
         <v>100</v>
       </c>
-      <c r="E23" s="27" t="s">
+      <c r="E23" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="F23" s="28"/>
+      <c r="F23" s="7"/>
       <c r="G23" s="26"/>
       <c r="H23" s="26"/>
       <c r="I23" s="26"/>
-      <c r="J23" s="27"/>
-      <c r="K23" s="27"/>
-      <c r="L23" s="27"/>
-      <c r="M23" s="27"/>
-      <c r="N23" s="27"/>
-      <c r="O23" s="27"/>
-      <c r="P23" s="27"/>
-      <c r="Q23" s="27"/>
-      <c r="R23" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="S23" s="27"/>
-      <c r="T23" s="27"/>
-      <c r="U23" s="27"/>
-      <c r="V23" s="27"/>
-    </row>
-    <row r="24" spans="1:22" s="29" customFormat="1" ht="27">
-      <c r="A24" s="36" t="s">
+      <c r="J23" s="10"/>
+      <c r="K23" s="10"/>
+      <c r="L23" s="10"/>
+      <c r="M23" s="10"/>
+      <c r="N23" s="10"/>
+      <c r="O23" s="10"/>
+      <c r="P23" s="10"/>
+      <c r="Q23" s="10"/>
+      <c r="R23" s="31" t="b">
+        <v>1</v>
+      </c>
+      <c r="S23" s="10"/>
+      <c r="T23" s="10"/>
+      <c r="U23" s="10"/>
+      <c r="V23" s="10"/>
+    </row>
+    <row r="24" spans="1:22" ht="27">
+      <c r="A24" s="32" t="s">
         <v>108</v>
       </c>
       <c r="B24" s="26"/>
-      <c r="C24" s="34" t="b">
+      <c r="C24" s="31" t="b">
         <v>0</v>
       </c>
-      <c r="D24" s="34" t="s">
+      <c r="D24" s="31" t="s">
         <v>100</v>
       </c>
-      <c r="E24" s="27" t="s">
+      <c r="E24" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="F24" s="28"/>
+      <c r="F24" s="7"/>
       <c r="G24" s="26"/>
       <c r="H24" s="26"/>
       <c r="I24" s="26"/>
-      <c r="J24" s="27"/>
-      <c r="K24" s="27"/>
-      <c r="L24" s="27"/>
-      <c r="M24" s="27"/>
-      <c r="N24" s="27"/>
-      <c r="O24" s="27"/>
-      <c r="P24" s="27"/>
-      <c r="Q24" s="27"/>
-      <c r="R24" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="S24" s="27"/>
-      <c r="T24" s="27"/>
-      <c r="U24" s="27"/>
-      <c r="V24" s="27"/>
-    </row>
-    <row r="25" spans="1:22" s="29" customFormat="1" ht="27">
-      <c r="A25" s="36" t="s">
+      <c r="J24" s="10"/>
+      <c r="K24" s="10"/>
+      <c r="L24" s="10"/>
+      <c r="M24" s="10"/>
+      <c r="N24" s="10"/>
+      <c r="O24" s="10"/>
+      <c r="P24" s="10"/>
+      <c r="Q24" s="10"/>
+      <c r="R24" s="31" t="b">
+        <v>1</v>
+      </c>
+      <c r="S24" s="10"/>
+      <c r="T24" s="10"/>
+      <c r="U24" s="10"/>
+      <c r="V24" s="10"/>
+    </row>
+    <row r="25" spans="1:22" ht="27">
+      <c r="A25" s="32" t="s">
         <v>109</v>
       </c>
       <c r="B25" s="26"/>
-      <c r="C25" s="34" t="b">
+      <c r="C25" s="31" t="b">
         <v>0</v>
       </c>
-      <c r="D25" s="34" t="s">
+      <c r="D25" s="31" t="s">
         <v>100</v>
       </c>
-      <c r="E25" s="27" t="s">
+      <c r="E25" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="F25" s="28"/>
+      <c r="F25" s="7"/>
       <c r="G25" s="26"/>
       <c r="H25" s="26"/>
       <c r="I25" s="26"/>
-      <c r="J25" s="27"/>
-      <c r="K25" s="27"/>
-      <c r="L25" s="27"/>
-      <c r="M25" s="27"/>
-      <c r="N25" s="27"/>
-      <c r="O25" s="27"/>
-      <c r="P25" s="27"/>
-      <c r="Q25" s="27"/>
-      <c r="R25" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="S25" s="27"/>
-      <c r="T25" s="27"/>
-      <c r="U25" s="27"/>
-      <c r="V25" s="27"/>
-    </row>
-    <row r="26" spans="1:22" s="29" customFormat="1" ht="27">
-      <c r="A26" s="36" t="s">
+      <c r="J25" s="10"/>
+      <c r="K25" s="10"/>
+      <c r="L25" s="10"/>
+      <c r="M25" s="10"/>
+      <c r="N25" s="10"/>
+      <c r="O25" s="10"/>
+      <c r="P25" s="10"/>
+      <c r="Q25" s="10"/>
+      <c r="R25" s="31" t="b">
+        <v>1</v>
+      </c>
+      <c r="S25" s="10"/>
+      <c r="T25" s="10"/>
+      <c r="U25" s="10"/>
+      <c r="V25" s="10"/>
+    </row>
+    <row r="26" spans="1:22" ht="27">
+      <c r="A26" s="32" t="s">
         <v>110</v>
       </c>
       <c r="B26" s="26"/>
-      <c r="C26" s="34" t="b">
+      <c r="C26" s="31" t="b">
         <v>0</v>
       </c>
-      <c r="D26" s="34" t="s">
+      <c r="D26" s="31" t="s">
         <v>100</v>
       </c>
-      <c r="E26" s="27" t="s">
+      <c r="E26" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="F26" s="28"/>
+      <c r="F26" s="7"/>
       <c r="G26" s="26"/>
       <c r="H26" s="26"/>
       <c r="I26" s="26"/>
-      <c r="J26" s="27"/>
-      <c r="K26" s="27"/>
-      <c r="L26" s="27"/>
-      <c r="M26" s="27"/>
-      <c r="N26" s="27"/>
-      <c r="O26" s="27"/>
-      <c r="P26" s="27"/>
-      <c r="Q26" s="27"/>
-      <c r="R26" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="S26" s="27"/>
-      <c r="T26" s="27"/>
-      <c r="U26" s="27"/>
-      <c r="V26" s="27"/>
-    </row>
-    <row r="27" spans="1:22" s="29" customFormat="1" ht="27">
-      <c r="A27" s="36" t="s">
+      <c r="J26" s="10"/>
+      <c r="K26" s="10"/>
+      <c r="L26" s="10"/>
+      <c r="M26" s="10"/>
+      <c r="N26" s="10"/>
+      <c r="O26" s="10"/>
+      <c r="P26" s="10"/>
+      <c r="Q26" s="10"/>
+      <c r="R26" s="31" t="b">
+        <v>1</v>
+      </c>
+      <c r="S26" s="10"/>
+      <c r="T26" s="10"/>
+      <c r="U26" s="10"/>
+      <c r="V26" s="10"/>
+    </row>
+    <row r="27" spans="1:22" ht="27">
+      <c r="A27" s="32" t="s">
         <v>111</v>
       </c>
       <c r="B27" s="26"/>
-      <c r="C27" s="34" t="b">
+      <c r="C27" s="31" t="b">
         <v>0</v>
       </c>
-      <c r="D27" s="34" t="s">
+      <c r="D27" s="31" t="s">
         <v>100</v>
       </c>
-      <c r="E27" s="27" t="s">
+      <c r="E27" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="F27" s="28"/>
+      <c r="F27" s="7"/>
       <c r="G27" s="26"/>
       <c r="H27" s="26"/>
       <c r="I27" s="26"/>
-      <c r="J27" s="27"/>
-      <c r="K27" s="27"/>
-      <c r="L27" s="27"/>
-      <c r="M27" s="27"/>
-      <c r="N27" s="27"/>
-      <c r="O27" s="27"/>
-      <c r="P27" s="27"/>
-      <c r="Q27" s="27"/>
-      <c r="R27" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="S27" s="27"/>
-      <c r="T27" s="27"/>
-      <c r="U27" s="27"/>
-      <c r="V27" s="27"/>
-    </row>
-    <row r="28" spans="1:22" s="29" customFormat="1" ht="27">
-      <c r="A28" s="36" t="s">
+      <c r="J27" s="10"/>
+      <c r="K27" s="10"/>
+      <c r="L27" s="10"/>
+      <c r="M27" s="10"/>
+      <c r="N27" s="10"/>
+      <c r="O27" s="10"/>
+      <c r="P27" s="10"/>
+      <c r="Q27" s="10"/>
+      <c r="R27" s="31" t="b">
+        <v>1</v>
+      </c>
+      <c r="S27" s="10"/>
+      <c r="T27" s="10"/>
+      <c r="U27" s="10"/>
+      <c r="V27" s="10"/>
+    </row>
+    <row r="28" spans="1:22" ht="27">
+      <c r="A28" s="32" t="s">
         <v>112</v>
       </c>
       <c r="B28" s="26"/>
-      <c r="C28" s="34" t="b">
+      <c r="C28" s="31" t="b">
         <v>0</v>
       </c>
-      <c r="D28" s="34" t="s">
+      <c r="D28" s="31" t="s">
         <v>100</v>
       </c>
-      <c r="E28" s="27" t="s">
+      <c r="E28" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="F28" s="28"/>
+      <c r="F28" s="7"/>
       <c r="G28" s="26"/>
       <c r="H28" s="26"/>
       <c r="I28" s="26"/>
-      <c r="J28" s="27"/>
-      <c r="K28" s="27"/>
-      <c r="L28" s="27"/>
-      <c r="M28" s="27"/>
-      <c r="N28" s="27"/>
-      <c r="O28" s="27"/>
-      <c r="P28" s="27"/>
-      <c r="Q28" s="27"/>
-      <c r="R28" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="S28" s="27"/>
-      <c r="T28" s="27"/>
-      <c r="U28" s="27"/>
-      <c r="V28" s="27"/>
-    </row>
-    <row r="29" spans="1:22" s="29" customFormat="1" ht="27">
-      <c r="A29" s="36" t="s">
+      <c r="J28" s="10"/>
+      <c r="K28" s="10"/>
+      <c r="L28" s="10"/>
+      <c r="M28" s="10"/>
+      <c r="N28" s="10"/>
+      <c r="O28" s="10"/>
+      <c r="P28" s="10"/>
+      <c r="Q28" s="10"/>
+      <c r="R28" s="31" t="b">
+        <v>1</v>
+      </c>
+      <c r="S28" s="10"/>
+      <c r="T28" s="10"/>
+      <c r="U28" s="10"/>
+      <c r="V28" s="10"/>
+    </row>
+    <row r="29" spans="1:22" ht="27">
+      <c r="A29" s="32" t="s">
         <v>113</v>
       </c>
       <c r="B29" s="26"/>
-      <c r="C29" s="34" t="b">
+      <c r="C29" s="31" t="b">
         <v>0</v>
       </c>
-      <c r="D29" s="34" t="s">
+      <c r="D29" s="31" t="s">
         <v>100</v>
       </c>
-      <c r="E29" s="27" t="s">
+      <c r="E29" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="F29" s="28"/>
+      <c r="F29" s="7"/>
       <c r="G29" s="26"/>
       <c r="H29" s="26"/>
       <c r="I29" s="26"/>
-      <c r="J29" s="27"/>
-      <c r="K29" s="27"/>
-      <c r="L29" s="27"/>
-      <c r="M29" s="27"/>
-      <c r="N29" s="27"/>
-      <c r="O29" s="27"/>
-      <c r="P29" s="27"/>
-      <c r="Q29" s="27"/>
-      <c r="R29" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="S29" s="27"/>
-      <c r="T29" s="27"/>
-      <c r="U29" s="27"/>
-      <c r="V29" s="27"/>
-    </row>
-    <row r="30" spans="1:22" s="29" customFormat="1" ht="27">
-      <c r="A30" s="36" t="s">
+      <c r="J29" s="10"/>
+      <c r="K29" s="10"/>
+      <c r="L29" s="10"/>
+      <c r="M29" s="10"/>
+      <c r="N29" s="10"/>
+      <c r="O29" s="10"/>
+      <c r="P29" s="10"/>
+      <c r="Q29" s="10"/>
+      <c r="R29" s="31" t="b">
+        <v>1</v>
+      </c>
+      <c r="S29" s="10"/>
+      <c r="T29" s="10"/>
+      <c r="U29" s="10"/>
+      <c r="V29" s="10"/>
+    </row>
+    <row r="30" spans="1:22" ht="27">
+      <c r="A30" s="32" t="s">
         <v>114</v>
       </c>
       <c r="B30" s="26"/>
-      <c r="C30" s="34" t="b">
+      <c r="C30" s="31" t="b">
         <v>0</v>
       </c>
-      <c r="D30" s="34" t="s">
+      <c r="D30" s="31" t="s">
         <v>100</v>
       </c>
-      <c r="E30" s="27" t="s">
+      <c r="E30" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="F30" s="28"/>
+      <c r="F30" s="7"/>
       <c r="G30" s="26"/>
       <c r="H30" s="26"/>
       <c r="I30" s="26"/>
-      <c r="J30" s="27"/>
-      <c r="K30" s="27"/>
-      <c r="L30" s="27"/>
-      <c r="M30" s="27"/>
-      <c r="N30" s="27"/>
-      <c r="O30" s="27"/>
-      <c r="P30" s="27"/>
-      <c r="Q30" s="27"/>
-      <c r="R30" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="S30" s="27"/>
-      <c r="T30" s="27"/>
-      <c r="U30" s="27"/>
-      <c r="V30" s="27"/>
-    </row>
-    <row r="31" spans="1:22" s="29" customFormat="1" ht="27">
-      <c r="A31" s="36" t="s">
+      <c r="J30" s="10"/>
+      <c r="K30" s="10"/>
+      <c r="L30" s="10"/>
+      <c r="M30" s="10"/>
+      <c r="N30" s="10"/>
+      <c r="O30" s="10"/>
+      <c r="P30" s="10"/>
+      <c r="Q30" s="10"/>
+      <c r="R30" s="31" t="b">
+        <v>1</v>
+      </c>
+      <c r="S30" s="10"/>
+      <c r="T30" s="10"/>
+      <c r="U30" s="10"/>
+      <c r="V30" s="10"/>
+    </row>
+    <row r="31" spans="1:22" ht="27">
+      <c r="A31" s="32" t="s">
         <v>115</v>
       </c>
       <c r="B31" s="26"/>
-      <c r="C31" s="34" t="b">
+      <c r="C31" s="31" t="b">
         <v>0</v>
       </c>
-      <c r="D31" s="34" t="s">
+      <c r="D31" s="31" t="s">
         <v>100</v>
       </c>
-      <c r="E31" s="27" t="s">
+      <c r="E31" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="F31" s="28"/>
+      <c r="F31" s="7"/>
       <c r="G31" s="26"/>
       <c r="H31" s="26"/>
       <c r="I31" s="26"/>
-      <c r="J31" s="27"/>
-      <c r="K31" s="27"/>
-      <c r="L31" s="27"/>
-      <c r="M31" s="27"/>
-      <c r="N31" s="27"/>
-      <c r="O31" s="27"/>
-      <c r="P31" s="27"/>
-      <c r="Q31" s="27"/>
-      <c r="R31" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="S31" s="27"/>
-      <c r="T31" s="27"/>
-      <c r="U31" s="27"/>
-      <c r="V31" s="27"/>
-    </row>
-    <row r="32" spans="1:22" s="29" customFormat="1" ht="27">
-      <c r="A32" s="36" t="s">
+      <c r="J31" s="10"/>
+      <c r="K31" s="10"/>
+      <c r="L31" s="10"/>
+      <c r="M31" s="10"/>
+      <c r="N31" s="10"/>
+      <c r="O31" s="10"/>
+      <c r="P31" s="10"/>
+      <c r="Q31" s="10"/>
+      <c r="R31" s="31" t="b">
+        <v>1</v>
+      </c>
+      <c r="S31" s="10"/>
+      <c r="T31" s="10"/>
+      <c r="U31" s="10"/>
+      <c r="V31" s="10"/>
+    </row>
+    <row r="32" spans="1:22" ht="27">
+      <c r="A32" s="32" t="s">
         <v>116</v>
       </c>
       <c r="B32" s="26"/>
-      <c r="C32" s="34" t="b">
+      <c r="C32" s="31" t="b">
         <v>0</v>
       </c>
-      <c r="D32" s="34" t="s">
+      <c r="D32" s="31" t="s">
         <v>100</v>
       </c>
-      <c r="E32" s="27" t="s">
+      <c r="E32" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="F32" s="28"/>
+      <c r="F32" s="7"/>
       <c r="G32" s="26"/>
       <c r="H32" s="26"/>
       <c r="I32" s="26"/>
-      <c r="J32" s="27"/>
-      <c r="K32" s="27"/>
-      <c r="L32" s="27"/>
-      <c r="M32" s="27"/>
-      <c r="N32" s="27"/>
-      <c r="O32" s="27"/>
-      <c r="P32" s="27"/>
-      <c r="Q32" s="27"/>
-      <c r="R32" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="S32" s="27"/>
-      <c r="T32" s="27"/>
-      <c r="U32" s="27"/>
-      <c r="V32" s="27"/>
-    </row>
-    <row r="33" spans="1:22" s="29" customFormat="1" ht="27">
-      <c r="A33" s="36" t="s">
+      <c r="J32" s="10"/>
+      <c r="K32" s="10"/>
+      <c r="L32" s="10"/>
+      <c r="M32" s="10"/>
+      <c r="N32" s="10"/>
+      <c r="O32" s="10"/>
+      <c r="P32" s="10"/>
+      <c r="Q32" s="10"/>
+      <c r="R32" s="31" t="b">
+        <v>1</v>
+      </c>
+      <c r="S32" s="10"/>
+      <c r="T32" s="10"/>
+      <c r="U32" s="10"/>
+      <c r="V32" s="10"/>
+    </row>
+    <row r="33" spans="1:22" ht="27">
+      <c r="A33" s="32" t="s">
         <v>117</v>
       </c>
       <c r="B33" s="26"/>
-      <c r="C33" s="34" t="b">
+      <c r="C33" s="31" t="b">
         <v>0</v>
       </c>
-      <c r="D33" s="34" t="s">
+      <c r="D33" s="31" t="s">
         <v>100</v>
       </c>
-      <c r="E33" s="27" t="s">
+      <c r="E33" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="F33" s="28"/>
+      <c r="F33" s="7"/>
       <c r="G33" s="26"/>
       <c r="H33" s="26"/>
       <c r="I33" s="26"/>
-      <c r="J33" s="27"/>
-      <c r="K33" s="27"/>
-      <c r="L33" s="27"/>
-      <c r="M33" s="27"/>
-      <c r="N33" s="27"/>
-      <c r="O33" s="27"/>
-      <c r="P33" s="27"/>
-      <c r="Q33" s="27"/>
-      <c r="R33" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="S33" s="27"/>
-      <c r="T33" s="27"/>
-      <c r="U33" s="27"/>
-      <c r="V33" s="27"/>
-    </row>
-    <row r="34" spans="1:22" s="29" customFormat="1" ht="27">
-      <c r="A34" s="36" t="s">
+      <c r="J33" s="10"/>
+      <c r="K33" s="10"/>
+      <c r="L33" s="10"/>
+      <c r="M33" s="10"/>
+      <c r="N33" s="10"/>
+      <c r="O33" s="10"/>
+      <c r="P33" s="10"/>
+      <c r="Q33" s="10"/>
+      <c r="R33" s="31" t="b">
+        <v>1</v>
+      </c>
+      <c r="S33" s="10"/>
+      <c r="T33" s="10"/>
+      <c r="U33" s="10"/>
+      <c r="V33" s="10"/>
+    </row>
+    <row r="34" spans="1:22" ht="27">
+      <c r="A34" s="32" t="s">
         <v>118</v>
       </c>
       <c r="B34" s="26"/>
-      <c r="C34" s="34" t="b">
+      <c r="C34" s="31" t="b">
         <v>0</v>
       </c>
-      <c r="D34" s="34" t="s">
+      <c r="D34" s="31" t="s">
         <v>100</v>
       </c>
-      <c r="E34" s="27" t="s">
+      <c r="E34" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="F34" s="28"/>
+      <c r="F34" s="7"/>
       <c r="G34" s="26"/>
       <c r="H34" s="26"/>
       <c r="I34" s="26"/>
-      <c r="J34" s="27"/>
-      <c r="K34" s="27"/>
-      <c r="L34" s="27"/>
-      <c r="M34" s="27"/>
-      <c r="N34" s="27"/>
-      <c r="O34" s="27"/>
-      <c r="P34" s="27"/>
-      <c r="Q34" s="27"/>
-      <c r="R34" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="S34" s="27"/>
-      <c r="T34" s="27"/>
-      <c r="U34" s="27"/>
-      <c r="V34" s="27"/>
-    </row>
-    <row r="35" spans="1:22" s="29" customFormat="1" ht="27">
-      <c r="A35" s="36" t="s">
+      <c r="J34" s="10"/>
+      <c r="K34" s="10"/>
+      <c r="L34" s="10"/>
+      <c r="M34" s="10"/>
+      <c r="N34" s="10"/>
+      <c r="O34" s="10"/>
+      <c r="P34" s="10"/>
+      <c r="Q34" s="10"/>
+      <c r="R34" s="31" t="b">
+        <v>1</v>
+      </c>
+      <c r="S34" s="10"/>
+      <c r="T34" s="10"/>
+      <c r="U34" s="10"/>
+      <c r="V34" s="10"/>
+    </row>
+    <row r="35" spans="1:22" ht="27">
+      <c r="A35" s="32" t="s">
         <v>119</v>
       </c>
       <c r="B35" s="26"/>
-      <c r="C35" s="34" t="b">
+      <c r="C35" s="31" t="b">
         <v>0</v>
       </c>
-      <c r="D35" s="34" t="s">
+      <c r="D35" s="31" t="s">
         <v>100</v>
       </c>
-      <c r="E35" s="27" t="s">
+      <c r="E35" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="F35" s="28"/>
+      <c r="F35" s="7"/>
       <c r="G35" s="26"/>
       <c r="H35" s="26"/>
       <c r="I35" s="26"/>
-      <c r="J35" s="27"/>
-      <c r="K35" s="27"/>
-      <c r="L35" s="27"/>
-      <c r="M35" s="27"/>
-      <c r="N35" s="27"/>
-      <c r="O35" s="27"/>
-      <c r="P35" s="27"/>
-      <c r="Q35" s="27"/>
-      <c r="R35" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="S35" s="27"/>
-      <c r="T35" s="27"/>
-      <c r="U35" s="27"/>
-      <c r="V35" s="27"/>
-    </row>
-    <row r="36" spans="1:22" s="29" customFormat="1" ht="27">
-      <c r="A36" s="36" t="s">
+      <c r="J35" s="10"/>
+      <c r="K35" s="10"/>
+      <c r="L35" s="10"/>
+      <c r="M35" s="10"/>
+      <c r="N35" s="10"/>
+      <c r="O35" s="10"/>
+      <c r="P35" s="10"/>
+      <c r="Q35" s="10"/>
+      <c r="R35" s="31" t="b">
+        <v>1</v>
+      </c>
+      <c r="S35" s="10"/>
+      <c r="T35" s="10"/>
+      <c r="U35" s="10"/>
+      <c r="V35" s="10"/>
+    </row>
+    <row r="36" spans="1:22" ht="27">
+      <c r="A36" s="32" t="s">
         <v>120</v>
       </c>
       <c r="B36" s="26"/>
-      <c r="C36" s="34" t="b">
+      <c r="C36" s="31" t="b">
         <v>0</v>
       </c>
-      <c r="D36" s="34" t="s">
+      <c r="D36" s="31" t="s">
         <v>100</v>
       </c>
-      <c r="E36" s="27" t="s">
+      <c r="E36" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="F36" s="28"/>
+      <c r="F36" s="7"/>
       <c r="G36" s="26"/>
       <c r="H36" s="26"/>
       <c r="I36" s="26"/>
-      <c r="J36" s="27"/>
-      <c r="K36" s="27"/>
-      <c r="L36" s="27"/>
-      <c r="M36" s="27"/>
-      <c r="N36" s="27"/>
-      <c r="O36" s="27"/>
-      <c r="P36" s="27"/>
-      <c r="Q36" s="27"/>
-      <c r="R36" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="S36" s="27"/>
-      <c r="T36" s="27"/>
-      <c r="U36" s="27"/>
-      <c r="V36" s="27"/>
-    </row>
-    <row r="37" spans="1:22" s="29" customFormat="1" ht="27">
-      <c r="A37" s="36" t="s">
+      <c r="J36" s="10"/>
+      <c r="K36" s="10"/>
+      <c r="L36" s="10"/>
+      <c r="M36" s="10"/>
+      <c r="N36" s="10"/>
+      <c r="O36" s="10"/>
+      <c r="P36" s="10"/>
+      <c r="Q36" s="10"/>
+      <c r="R36" s="31" t="b">
+        <v>1</v>
+      </c>
+      <c r="S36" s="10"/>
+      <c r="T36" s="10"/>
+      <c r="U36" s="10"/>
+      <c r="V36" s="10"/>
+    </row>
+    <row r="37" spans="1:22" ht="27">
+      <c r="A37" s="32" t="s">
         <v>121</v>
       </c>
       <c r="B37" s="26"/>
-      <c r="C37" s="34" t="b">
+      <c r="C37" s="31" t="b">
         <v>0</v>
       </c>
-      <c r="D37" s="34" t="s">
+      <c r="D37" s="31" t="s">
         <v>100</v>
       </c>
-      <c r="E37" s="27" t="s">
+      <c r="E37" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="F37" s="28"/>
+      <c r="F37" s="7"/>
       <c r="G37" s="26"/>
       <c r="H37" s="26"/>
       <c r="I37" s="26"/>
-      <c r="J37" s="27"/>
-      <c r="K37" s="27"/>
-      <c r="L37" s="27"/>
-      <c r="M37" s="27"/>
-      <c r="N37" s="27"/>
-      <c r="O37" s="27"/>
-      <c r="P37" s="27"/>
-      <c r="Q37" s="27"/>
-      <c r="R37" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="S37" s="27"/>
-      <c r="T37" s="27"/>
-      <c r="U37" s="27"/>
-      <c r="V37" s="27"/>
-    </row>
-    <row r="38" spans="1:22" s="29" customFormat="1" ht="27">
-      <c r="A38" s="36" t="s">
+      <c r="J37" s="10"/>
+      <c r="K37" s="10"/>
+      <c r="L37" s="10"/>
+      <c r="M37" s="10"/>
+      <c r="N37" s="10"/>
+      <c r="O37" s="10"/>
+      <c r="P37" s="10"/>
+      <c r="Q37" s="10"/>
+      <c r="R37" s="31" t="b">
+        <v>1</v>
+      </c>
+      <c r="S37" s="10"/>
+      <c r="T37" s="10"/>
+      <c r="U37" s="10"/>
+      <c r="V37" s="10"/>
+    </row>
+    <row r="38" spans="1:22" ht="27">
+      <c r="A38" s="32" t="s">
         <v>122</v>
       </c>
       <c r="B38" s="26"/>
-      <c r="C38" s="34" t="b">
+      <c r="C38" s="31" t="b">
         <v>0</v>
       </c>
-      <c r="D38" s="34" t="s">
+      <c r="D38" s="31" t="s">
         <v>100</v>
       </c>
-      <c r="E38" s="27" t="s">
+      <c r="E38" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="F38" s="28"/>
+      <c r="F38" s="7"/>
       <c r="G38" s="26"/>
       <c r="H38" s="26"/>
       <c r="I38" s="26"/>
-      <c r="J38" s="27"/>
-      <c r="K38" s="27"/>
-      <c r="L38" s="27"/>
-      <c r="M38" s="27"/>
-      <c r="N38" s="27"/>
-      <c r="O38" s="27"/>
-      <c r="P38" s="27"/>
-      <c r="Q38" s="27"/>
-      <c r="R38" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="S38" s="27"/>
-      <c r="T38" s="27"/>
-      <c r="U38" s="27"/>
-      <c r="V38" s="27"/>
-    </row>
-    <row r="39" spans="1:22" s="29" customFormat="1" ht="27">
-      <c r="A39" s="36" t="s">
+      <c r="J38" s="10"/>
+      <c r="K38" s="10"/>
+      <c r="L38" s="10"/>
+      <c r="M38" s="10"/>
+      <c r="N38" s="10"/>
+      <c r="O38" s="10"/>
+      <c r="P38" s="10"/>
+      <c r="Q38" s="10"/>
+      <c r="R38" s="31" t="b">
+        <v>1</v>
+      </c>
+      <c r="S38" s="10"/>
+      <c r="T38" s="10"/>
+      <c r="U38" s="10"/>
+      <c r="V38" s="10"/>
+    </row>
+    <row r="39" spans="1:22" ht="27">
+      <c r="A39" s="32" t="s">
         <v>123</v>
       </c>
       <c r="B39" s="26"/>
-      <c r="C39" s="34" t="b">
+      <c r="C39" s="31" t="b">
         <v>0</v>
       </c>
-      <c r="D39" s="34" t="s">
+      <c r="D39" s="31" t="s">
         <v>100</v>
       </c>
-      <c r="E39" s="27" t="s">
+      <c r="E39" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="F39" s="28"/>
+      <c r="F39" s="7"/>
       <c r="G39" s="26"/>
       <c r="H39" s="26"/>
       <c r="I39" s="26"/>
-      <c r="J39" s="27"/>
-      <c r="K39" s="27"/>
-      <c r="L39" s="27"/>
-      <c r="M39" s="27"/>
-      <c r="N39" s="27"/>
-      <c r="O39" s="27"/>
-      <c r="P39" s="27"/>
-      <c r="Q39" s="27"/>
-      <c r="R39" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="S39" s="27"/>
-      <c r="T39" s="27"/>
-      <c r="U39" s="27"/>
-      <c r="V39" s="27"/>
-    </row>
-    <row r="40" spans="1:22" s="29" customFormat="1" ht="27">
-      <c r="A40" s="36" t="s">
+      <c r="J39" s="10"/>
+      <c r="K39" s="10"/>
+      <c r="L39" s="10"/>
+      <c r="M39" s="10"/>
+      <c r="N39" s="10"/>
+      <c r="O39" s="10"/>
+      <c r="P39" s="10"/>
+      <c r="Q39" s="10"/>
+      <c r="R39" s="31" t="b">
+        <v>1</v>
+      </c>
+      <c r="S39" s="10"/>
+      <c r="T39" s="10"/>
+      <c r="U39" s="10"/>
+      <c r="V39" s="10"/>
+    </row>
+    <row r="40" spans="1:22" ht="27">
+      <c r="A40" s="32" t="s">
         <v>124</v>
       </c>
       <c r="B40" s="26"/>
-      <c r="C40" s="34" t="b">
+      <c r="C40" s="31" t="b">
         <v>0</v>
       </c>
-      <c r="D40" s="34" t="s">
+      <c r="D40" s="31" t="s">
         <v>100</v>
       </c>
-      <c r="E40" s="27" t="s">
+      <c r="E40" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="F40" s="28"/>
+      <c r="F40" s="7"/>
       <c r="G40" s="26"/>
       <c r="H40" s="26"/>
       <c r="I40" s="26"/>
-      <c r="J40" s="27"/>
-      <c r="K40" s="27"/>
-      <c r="L40" s="27"/>
-      <c r="M40" s="27"/>
-      <c r="N40" s="27"/>
-      <c r="O40" s="27"/>
-      <c r="P40" s="27"/>
-      <c r="Q40" s="27"/>
-      <c r="R40" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="S40" s="27"/>
-      <c r="T40" s="27"/>
-      <c r="U40" s="27"/>
-      <c r="V40" s="27"/>
+      <c r="J40" s="10"/>
+      <c r="K40" s="10"/>
+      <c r="L40" s="10"/>
+      <c r="M40" s="10"/>
+      <c r="N40" s="10"/>
+      <c r="O40" s="10"/>
+      <c r="P40" s="10"/>
+      <c r="Q40" s="10"/>
+      <c r="R40" s="31" t="b">
+        <v>1</v>
+      </c>
+      <c r="S40" s="10"/>
+      <c r="T40" s="10"/>
+      <c r="U40" s="10"/>
+      <c r="V40" s="10"/>
     </row>
     <row r="41" spans="1:22">
       <c r="A41" s="11" t="s">
@@ -3126,7 +3111,7 @@
         <v>0</v>
       </c>
       <c r="G2" s="14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -3149,7 +3134,7 @@
         <v>0</v>
       </c>
       <c r="G3" s="14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="29.25">
@@ -3172,7 +3157,7 @@
         <v>0</v>
       </c>
       <c r="G4" s="14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add count context for translation with the Generator
We can now add translations for one-person interview.
Fix generate_label tests with different contexts.
</commit_message>
<xml_diff>
--- a/example/demo_generator/references/Household_Travel_Generate_Survey.xlsx
+++ b/example/demo_generator/references/Household_Travel_Generate_Survey.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28928"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="964" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FD3B125B-8CC8-42DD-AD5E-7C91AD056CF1}"/>
+  <xr:revisionPtr revIDLastSave="978" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C0AF4DD7-5803-4D81-ABD0-4FE84017DD06}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Labels" sheetId="6" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Widgets!$A$1:$V$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Widgets!$A$1:$X$1</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="254">
   <si>
     <t>questionName</t>
   </si>
@@ -63,6 +63,12 @@
   </si>
   <si>
     <t>label::en</t>
+  </si>
+  <si>
+    <t>label_one::fr</t>
+  </si>
+  <si>
+    <t>label_one::en</t>
   </si>
   <si>
     <t>parameters</t>
@@ -395,6 +401,12 @@
   <si>
     <t>**Age**
 __For babies under the age of 1, write "0"__</t>
+  </si>
+  <si>
+    <t>**Votre âge**</t>
+  </si>
+  <si>
+    <t>**Your age**</t>
   </si>
   <si>
     <t>ageValidation</t>
@@ -1010,7 +1022,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -1113,6 +1125,12 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1521,7 +1539,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:V42"/>
+  <dimension ref="A1:X42"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="19.85546875" style="8" customWidth="1"/>
@@ -1532,24 +1550,25 @@
     <col min="6" max="6" width="17" style="8" customWidth="1"/>
     <col min="7" max="7" width="31.28515625" style="8" customWidth="1"/>
     <col min="8" max="8" width="31.5703125" style="8" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.5703125" style="8" customWidth="1"/>
-    <col min="10" max="10" width="22.7109375" style="8" customWidth="1"/>
-    <col min="11" max="11" width="19.7109375" style="8" customWidth="1"/>
-    <col min="12" max="12" width="13.5703125" style="8" customWidth="1"/>
-    <col min="13" max="13" width="13" style="8" customWidth="1"/>
-    <col min="14" max="14" width="13.42578125" style="8" customWidth="1"/>
-    <col min="15" max="15" width="10" style="8" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="9.28515625" style="8" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="14.42578125" style="8" customWidth="1"/>
-    <col min="18" max="18" width="14.140625" style="8" customWidth="1"/>
-    <col min="19" max="19" width="10.28515625" style="8" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="15.42578125" style="8" customWidth="1"/>
-    <col min="21" max="21" width="11.140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="19.5703125" style="8" customWidth="1"/>
-    <col min="23" max="16384" width="9.140625" style="8"/>
+    <col min="9" max="10" width="31.5703125" style="8" customWidth="1"/>
+    <col min="11" max="11" width="20.5703125" style="8" customWidth="1"/>
+    <col min="12" max="12" width="22.7109375" style="8" customWidth="1"/>
+    <col min="13" max="13" width="19.7109375" style="8" customWidth="1"/>
+    <col min="14" max="14" width="13.5703125" style="8" customWidth="1"/>
+    <col min="15" max="15" width="13" style="8" customWidth="1"/>
+    <col min="16" max="16" width="13.42578125" style="8" customWidth="1"/>
+    <col min="17" max="17" width="10" style="8" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="14.42578125" style="8" customWidth="1"/>
+    <col min="20" max="20" width="14.140625" style="8" customWidth="1"/>
+    <col min="21" max="21" width="10.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="15.42578125" style="8" customWidth="1"/>
+    <col min="23" max="23" width="11.140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="19.5703125" style="8" customWidth="1"/>
+    <col min="25" max="16384" width="9.140625" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" s="18" customFormat="1" ht="17.25" customHeight="1">
+    <row r="1" spans="1:24" s="18" customFormat="1" ht="17.25" customHeight="1">
       <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
@@ -1574,16 +1593,16 @@
       <c r="H1" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="23" t="s">
+      <c r="I1" s="36" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="25" t="s">
+      <c r="J1" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="24" t="s">
+      <c r="K1" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="24" t="s">
+      <c r="L1" s="25" t="s">
         <v>11</v>
       </c>
       <c r="M1" s="24" t="s">
@@ -1598,10 +1617,10 @@
       <c r="P1" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="23" t="s">
+      <c r="Q1" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="23" t="s">
+      <c r="R1" s="24" t="s">
         <v>17</v>
       </c>
       <c r="S1" s="23" t="s">
@@ -1616,228 +1635,244 @@
       <c r="V1" s="23" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="2" spans="1:22" ht="27" hidden="1">
+      <c r="W1" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="23" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:24" ht="27" hidden="1">
       <c r="A2" s="9" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C2" s="9" t="b">
         <v>1</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E2" s="9"/>
       <c r="F2" s="9" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="H2" s="9" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="I2" s="9"/>
       <c r="J2" s="9"/>
       <c r="K2" s="9"/>
-      <c r="L2" s="11"/>
+      <c r="L2" s="9"/>
       <c r="M2" s="9"/>
-      <c r="N2" s="9"/>
+      <c r="N2" s="11"/>
       <c r="O2" s="9"/>
       <c r="P2" s="9"/>
       <c r="Q2" s="9"/>
-      <c r="R2" s="9" t="b">
-        <v>1</v>
-      </c>
+      <c r="R2" s="9"/>
       <c r="S2" s="9"/>
-      <c r="T2" s="9"/>
+      <c r="T2" s="9" t="b">
+        <v>1</v>
+      </c>
       <c r="U2" s="9"/>
       <c r="V2" s="9"/>
-    </row>
-    <row r="3" spans="1:22" ht="81" hidden="1">
+      <c r="W2" s="9"/>
+      <c r="X2" s="9"/>
+    </row>
+    <row r="3" spans="1:24" ht="81" hidden="1">
       <c r="A3" s="9" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C3" s="9" t="b">
         <v>1</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E3" s="9"/>
       <c r="F3" s="9" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="I3" s="9"/>
-      <c r="K3" s="11"/>
-      <c r="L3" s="11"/>
-      <c r="M3" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="N3" s="9"/>
-      <c r="O3" s="9"/>
+      <c r="J3" s="9"/>
+      <c r="K3" s="9"/>
+      <c r="M3" s="11"/>
+      <c r="N3" s="11"/>
+      <c r="O3" s="9" t="s">
+        <v>33</v>
+      </c>
       <c r="P3" s="9"/>
       <c r="Q3" s="9"/>
-      <c r="R3" s="9" t="b">
-        <v>1</v>
-      </c>
+      <c r="R3" s="9"/>
       <c r="S3" s="9"/>
-      <c r="T3" s="9"/>
+      <c r="T3" s="9" t="b">
+        <v>1</v>
+      </c>
       <c r="U3" s="9"/>
       <c r="V3" s="9"/>
-    </row>
-    <row r="4" spans="1:22" ht="40.5" hidden="1">
+      <c r="W3" s="9"/>
+      <c r="X3" s="9"/>
+    </row>
+    <row r="4" spans="1:24" ht="40.5" hidden="1">
       <c r="A4" s="9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C4" s="9" t="b">
         <v>1</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E4" s="9"/>
       <c r="F4" s="9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="I4" s="9"/>
       <c r="J4" s="9"/>
-      <c r="K4" s="11"/>
+      <c r="K4" s="9"/>
       <c r="L4" s="9"/>
-      <c r="M4" s="9" t="s">
-        <v>36</v>
-      </c>
+      <c r="M4" s="11"/>
       <c r="N4" s="9"/>
-      <c r="O4" s="9"/>
+      <c r="O4" s="9" t="s">
+        <v>38</v>
+      </c>
       <c r="P4" s="9"/>
       <c r="Q4" s="9"/>
-      <c r="R4" s="9" t="b">
-        <v>1</v>
-      </c>
+      <c r="R4" s="9"/>
       <c r="S4" s="9"/>
-      <c r="T4" s="9"/>
+      <c r="T4" s="9" t="b">
+        <v>1</v>
+      </c>
       <c r="U4" s="9"/>
       <c r="V4" s="9"/>
-    </row>
-    <row r="5" spans="1:22" hidden="1">
+      <c r="W4" s="9"/>
+      <c r="X4" s="9"/>
+    </row>
+    <row r="5" spans="1:24" hidden="1">
       <c r="A5" s="9" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C5" s="9" t="b">
         <v>1</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E5" s="9"/>
       <c r="F5" s="9" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="I5" s="9"/>
       <c r="J5" s="9"/>
-      <c r="K5" s="11"/>
-      <c r="L5" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="M5" s="9"/>
-      <c r="N5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="11"/>
+      <c r="N5" s="9" t="s">
+        <v>42</v>
+      </c>
       <c r="O5" s="9"/>
       <c r="P5" s="9"/>
       <c r="Q5" s="9"/>
-      <c r="R5" s="9" t="b">
-        <v>1</v>
-      </c>
+      <c r="R5" s="9"/>
       <c r="S5" s="9"/>
-      <c r="T5" s="9"/>
+      <c r="T5" s="9" t="b">
+        <v>1</v>
+      </c>
       <c r="U5" s="9"/>
       <c r="V5" s="9"/>
-    </row>
-    <row r="6" spans="1:22" ht="27" hidden="1">
+      <c r="W5" s="9"/>
+      <c r="X5" s="9"/>
+    </row>
+    <row r="6" spans="1:24" ht="27" hidden="1">
       <c r="A6" s="9" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C6" s="9" t="b">
         <v>1</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E6" s="9"/>
       <c r="F6" s="9" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="I6" s="9"/>
-      <c r="J6" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="K6" s="11"/>
+      <c r="J6" s="9"/>
+      <c r="K6" s="9"/>
       <c r="L6" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="M6" s="9"/>
-      <c r="N6" s="9"/>
+        <v>46</v>
+      </c>
+      <c r="M6" s="11"/>
+      <c r="N6" s="9" t="s">
+        <v>47</v>
+      </c>
       <c r="O6" s="9"/>
       <c r="P6" s="9"/>
       <c r="Q6" s="9"/>
-      <c r="R6" s="9" t="b">
-        <v>1</v>
-      </c>
+      <c r="R6" s="9"/>
       <c r="S6" s="9"/>
-      <c r="T6" s="9"/>
+      <c r="T6" s="9" t="b">
+        <v>1</v>
+      </c>
       <c r="U6" s="9"/>
       <c r="V6" s="9"/>
-    </row>
-    <row r="7" spans="1:22" hidden="1">
+      <c r="W6" s="9"/>
+      <c r="X6" s="9"/>
+    </row>
+    <row r="7" spans="1:24" hidden="1">
       <c r="A7" s="9" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C7" s="9" t="b">
         <v>1</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E7" s="9"/>
       <c r="F7" s="9" t="str">
@@ -1845,10 +1880,10 @@
         <v>home.address</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="H7" s="9" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="I7" s="9"/>
       <c r="J7" s="9"/>
@@ -1859,26 +1894,28 @@
       <c r="O7" s="9"/>
       <c r="P7" s="9"/>
       <c r="Q7" s="9"/>
-      <c r="R7" s="9" t="b">
-        <v>1</v>
-      </c>
+      <c r="R7" s="9"/>
       <c r="S7" s="9"/>
-      <c r="T7" s="9"/>
+      <c r="T7" s="9" t="b">
+        <v>1</v>
+      </c>
       <c r="U7" s="9"/>
       <c r="V7" s="9"/>
-    </row>
-    <row r="8" spans="1:22" hidden="1">
+      <c r="W7" s="9"/>
+      <c r="X7" s="9"/>
+    </row>
+    <row r="8" spans="1:24" hidden="1">
       <c r="A8" s="9" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C8" s="9" t="b">
         <v>1</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E8" s="9"/>
       <c r="F8" s="9" t="str">
@@ -1886,42 +1923,44 @@
         <v>home.city</v>
       </c>
       <c r="G8" s="9" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="I8" s="9"/>
       <c r="J8" s="9"/>
       <c r="K8" s="9"/>
       <c r="L8" s="9"/>
       <c r="M8" s="9"/>
-      <c r="N8" s="9" t="s">
-        <v>52</v>
-      </c>
+      <c r="N8" s="9"/>
       <c r="O8" s="9"/>
-      <c r="P8" s="9"/>
+      <c r="P8" s="9" t="s">
+        <v>54</v>
+      </c>
       <c r="Q8" s="9"/>
-      <c r="R8" s="9" t="b">
-        <v>1</v>
-      </c>
+      <c r="R8" s="9"/>
       <c r="S8" s="9"/>
-      <c r="T8" s="9"/>
+      <c r="T8" s="9" t="b">
+        <v>1</v>
+      </c>
       <c r="U8" s="9"/>
       <c r="V8" s="9"/>
-    </row>
-    <row r="9" spans="1:22" ht="40.5" hidden="1">
+      <c r="W8" s="9"/>
+      <c r="X8" s="9"/>
+    </row>
+    <row r="9" spans="1:24" ht="40.5" hidden="1">
       <c r="A9" s="9" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C9" s="9" t="b">
         <v>1</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E9" s="9"/>
       <c r="F9" s="9" t="str">
@@ -1929,44 +1968,46 @@
         <v>home.region</v>
       </c>
       <c r="G9" s="9" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="H9" s="9" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I9" s="9"/>
       <c r="J9" s="9"/>
-      <c r="K9" s="9" t="s">
-        <v>55</v>
-      </c>
+      <c r="K9" s="9"/>
       <c r="L9" s="9"/>
-      <c r="M9" s="9"/>
+      <c r="M9" s="9" t="s">
+        <v>57</v>
+      </c>
       <c r="N9" s="9"/>
       <c r="O9" s="9"/>
       <c r="P9" s="9"/>
       <c r="Q9" s="9"/>
-      <c r="R9" s="9" t="b">
-        <v>1</v>
-      </c>
+      <c r="R9" s="9"/>
       <c r="S9" s="9"/>
-      <c r="T9" s="9"/>
-      <c r="U9" s="9" t="s">
-        <v>56</v>
-      </c>
+      <c r="T9" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="U9" s="9"/>
       <c r="V9" s="9"/>
-    </row>
-    <row r="10" spans="1:22" ht="40.5" hidden="1">
+      <c r="W9" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="X9" s="9"/>
+    </row>
+    <row r="10" spans="1:24" ht="40.5" hidden="1">
       <c r="A10" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C10" s="9" t="b">
         <v>1</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E10" s="9"/>
       <c r="F10" s="9" t="str">
@@ -1974,44 +2015,46 @@
         <v>home.country</v>
       </c>
       <c r="G10" s="9" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="I10" s="9"/>
       <c r="J10" s="9"/>
-      <c r="K10" s="9" t="s">
-        <v>60</v>
-      </c>
+      <c r="K10" s="9"/>
       <c r="L10" s="9"/>
-      <c r="M10" s="9"/>
+      <c r="M10" s="9" t="s">
+        <v>62</v>
+      </c>
       <c r="N10" s="9"/>
       <c r="O10" s="9"/>
       <c r="P10" s="9"/>
       <c r="Q10" s="9"/>
-      <c r="R10" s="9" t="b">
-        <v>1</v>
-      </c>
+      <c r="R10" s="9"/>
       <c r="S10" s="9"/>
-      <c r="T10" s="9"/>
-      <c r="U10" s="9" t="s">
-        <v>61</v>
-      </c>
+      <c r="T10" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="U10" s="9"/>
       <c r="V10" s="9"/>
-    </row>
-    <row r="11" spans="1:22" ht="27" hidden="1">
+      <c r="W10" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="X10" s="9"/>
+    </row>
+    <row r="11" spans="1:24" ht="27" hidden="1">
       <c r="A11" s="9" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C11" s="9" t="b">
         <v>1</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E11" s="9"/>
       <c r="F11" s="9" t="str">
@@ -2019,42 +2062,44 @@
         <v>home.postalCode</v>
       </c>
       <c r="G11" s="9" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="H11" s="9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I11" s="9"/>
       <c r="J11" s="9"/>
       <c r="K11" s="9"/>
-      <c r="L11" s="9" t="s">
-        <v>65</v>
-      </c>
+      <c r="L11" s="9"/>
       <c r="M11" s="9"/>
-      <c r="N11" s="9"/>
+      <c r="N11" s="9" t="s">
+        <v>67</v>
+      </c>
       <c r="O11" s="9"/>
       <c r="P11" s="9"/>
       <c r="Q11" s="9"/>
-      <c r="R11" s="9" t="b">
-        <v>1</v>
-      </c>
+      <c r="R11" s="9"/>
       <c r="S11" s="9"/>
-      <c r="T11" s="9"/>
+      <c r="T11" s="9" t="b">
+        <v>1</v>
+      </c>
       <c r="U11" s="9"/>
       <c r="V11" s="9"/>
-    </row>
-    <row r="12" spans="1:22" ht="117.75" hidden="1" customHeight="1">
+      <c r="W11" s="9"/>
+      <c r="X11" s="9"/>
+    </row>
+    <row r="12" spans="1:24" ht="117.75" hidden="1" customHeight="1">
       <c r="A12" s="13" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C12" s="9" t="b">
         <v>1</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E12" s="9"/>
       <c r="F12" s="9" t="str">
@@ -2062,40 +2107,42 @@
         <v>home.geography</v>
       </c>
       <c r="G12" s="9" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="I12" s="9"/>
       <c r="J12" s="9"/>
-      <c r="K12" s="13"/>
+      <c r="K12" s="9"/>
       <c r="L12" s="9"/>
-      <c r="M12" s="9"/>
+      <c r="M12" s="13"/>
       <c r="N12" s="9"/>
       <c r="O12" s="9"/>
       <c r="P12" s="9"/>
       <c r="Q12" s="9"/>
-      <c r="R12" s="9" t="b">
-        <v>1</v>
-      </c>
+      <c r="R12" s="9"/>
       <c r="S12" s="9"/>
-      <c r="T12" s="9"/>
+      <c r="T12" s="9" t="b">
+        <v>1</v>
+      </c>
       <c r="U12" s="9"/>
       <c r="V12" s="9"/>
-    </row>
-    <row r="13" spans="1:22" ht="48" hidden="1" customHeight="1">
+      <c r="W12" s="9"/>
+      <c r="X12" s="9"/>
+    </row>
+    <row r="13" spans="1:24" ht="48" hidden="1" customHeight="1">
       <c r="A13" s="9" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C13" s="9" t="b">
         <v>1</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E13" s="9"/>
       <c r="F13" s="9" t="str">
@@ -2103,46 +2150,48 @@
         <v>household.size</v>
       </c>
       <c r="G13" s="9" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="H13" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="I13" s="9" t="s">
-        <v>74</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="I13" s="9"/>
       <c r="J13" s="9"/>
-      <c r="K13" s="9"/>
-      <c r="L13" s="9" t="s">
-        <v>75</v>
-      </c>
+      <c r="K13" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="L13" s="9"/>
       <c r="M13" s="9"/>
       <c r="N13" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O13" s="9"/>
-      <c r="P13" s="9"/>
+      <c r="P13" s="9" t="s">
+        <v>78</v>
+      </c>
       <c r="Q13" s="9"/>
-      <c r="R13" s="9" t="b">
-        <v>1</v>
-      </c>
+      <c r="R13" s="9"/>
       <c r="S13" s="9"/>
-      <c r="T13" s="9"/>
+      <c r="T13" s="9" t="b">
+        <v>1</v>
+      </c>
       <c r="U13" s="9"/>
       <c r="V13" s="9"/>
-    </row>
-    <row r="14" spans="1:22" ht="56.25" hidden="1" customHeight="1">
+      <c r="W13" s="9"/>
+      <c r="X13" s="9"/>
+    </row>
+    <row r="14" spans="1:24" ht="56.25" hidden="1" customHeight="1">
       <c r="A14" s="9" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C14" s="9" t="b">
         <v>1</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E14" s="9"/>
       <c r="F14" s="9" t="str">
@@ -2150,46 +2199,48 @@
         <v>household.carNumber</v>
       </c>
       <c r="G14" s="9" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="I14" s="9" t="s">
-        <v>80</v>
-      </c>
+        <v>81</v>
+      </c>
+      <c r="I14" s="9"/>
       <c r="J14" s="9"/>
-      <c r="K14" s="9"/>
-      <c r="L14" s="9" t="s">
-        <v>81</v>
-      </c>
+      <c r="K14" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="L14" s="9"/>
       <c r="M14" s="9"/>
       <c r="N14" s="9" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="O14" s="9"/>
-      <c r="P14" s="9"/>
+      <c r="P14" s="9" t="s">
+        <v>84</v>
+      </c>
       <c r="Q14" s="9"/>
-      <c r="R14" s="9" t="b">
-        <v>1</v>
-      </c>
+      <c r="R14" s="9"/>
       <c r="S14" s="9"/>
-      <c r="T14" s="9"/>
+      <c r="T14" s="9" t="b">
+        <v>1</v>
+      </c>
       <c r="U14" s="9"/>
       <c r="V14" s="9"/>
-    </row>
-    <row r="15" spans="1:22" ht="76.5" hidden="1" customHeight="1">
+      <c r="W14" s="9"/>
+      <c r="X14" s="9"/>
+    </row>
+    <row r="15" spans="1:24" ht="76.5" hidden="1" customHeight="1">
       <c r="A15" s="9" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C15" s="9" t="b">
         <v>1</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E15" s="9"/>
       <c r="F15" s="9" t="str">
@@ -2197,44 +2248,46 @@
         <v>household.bicycleNumber</v>
       </c>
       <c r="G15" s="9" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="H15" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="I15" s="9" t="s">
-        <v>80</v>
-      </c>
+        <v>87</v>
+      </c>
+      <c r="I15" s="9"/>
       <c r="J15" s="9"/>
-      <c r="K15" s="9"/>
-      <c r="L15" s="9" t="s">
-        <v>86</v>
-      </c>
+      <c r="K15" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="L15" s="9"/>
       <c r="M15" s="9"/>
-      <c r="N15" s="9"/>
+      <c r="N15" s="9" t="s">
+        <v>88</v>
+      </c>
       <c r="O15" s="9"/>
       <c r="P15" s="9"/>
       <c r="Q15" s="9"/>
-      <c r="R15" s="9" t="b">
-        <v>1</v>
-      </c>
+      <c r="R15" s="9"/>
       <c r="S15" s="9"/>
-      <c r="T15" s="9"/>
+      <c r="T15" s="9" t="b">
+        <v>1</v>
+      </c>
       <c r="U15" s="9"/>
       <c r="V15" s="9"/>
-    </row>
-    <row r="16" spans="1:22" ht="40.5" hidden="1">
+      <c r="W15" s="9"/>
+      <c r="X15" s="9"/>
+    </row>
+    <row r="16" spans="1:24" ht="40.5" hidden="1">
       <c r="A16" s="9" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C16" s="9" t="b">
         <v>1</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E16" s="9"/>
       <c r="F16" s="9" t="str">
@@ -2242,42 +2295,44 @@
         <v>household.electricBicycleNumber</v>
       </c>
       <c r="G16" s="9" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="I16" s="9" t="s">
-        <v>80</v>
-      </c>
+        <v>91</v>
+      </c>
+      <c r="I16" s="9"/>
       <c r="J16" s="9"/>
-      <c r="K16" s="11"/>
-      <c r="L16" s="11"/>
-      <c r="M16" s="9"/>
-      <c r="N16" s="9"/>
+      <c r="K16" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="L16" s="9"/>
+      <c r="M16" s="11"/>
+      <c r="N16" s="11"/>
       <c r="O16" s="9"/>
       <c r="P16" s="9"/>
       <c r="Q16" s="9"/>
-      <c r="R16" s="9" t="b">
-        <v>1</v>
-      </c>
+      <c r="R16" s="9"/>
       <c r="S16" s="9"/>
-      <c r="T16" s="9"/>
+      <c r="T16" s="9" t="b">
+        <v>1</v>
+      </c>
       <c r="U16" s="9"/>
       <c r="V16" s="9"/>
-    </row>
-    <row r="17" spans="1:22" ht="76.5" hidden="1" customHeight="1">
+      <c r="W16" s="9"/>
+      <c r="X16" s="9"/>
+    </row>
+    <row r="17" spans="1:24" ht="76.5" hidden="1" customHeight="1">
       <c r="A17" s="9" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C17" s="9" t="b">
         <v>1</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E17" s="9"/>
       <c r="F17" s="9" t="str">
@@ -2285,44 +2340,46 @@
         <v>household.atLeastOnePersonWithDisability</v>
       </c>
       <c r="G17" s="9" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="H17" s="9" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="I17" s="9"/>
       <c r="J17" s="9"/>
-      <c r="K17" s="9" t="s">
-        <v>93</v>
-      </c>
+      <c r="K17" s="9"/>
       <c r="L17" s="9"/>
       <c r="M17" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="N17" s="9"/>
-      <c r="O17" s="9"/>
+      <c r="O17" s="9" t="s">
+        <v>96</v>
+      </c>
       <c r="P17" s="9"/>
       <c r="Q17" s="9"/>
-      <c r="R17" s="9" t="b">
-        <v>1</v>
-      </c>
+      <c r="R17" s="9"/>
       <c r="S17" s="9"/>
-      <c r="T17" s="9"/>
+      <c r="T17" s="9" t="b">
+        <v>1</v>
+      </c>
       <c r="U17" s="9"/>
       <c r="V17" s="9"/>
-    </row>
-    <row r="18" spans="1:22" hidden="1">
+      <c r="W17" s="9"/>
+      <c r="X17" s="9"/>
+    </row>
+    <row r="18" spans="1:24" hidden="1">
       <c r="A18" s="22" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B18" s="22" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C18" s="22" t="b">
         <v>1</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E18" s="9"/>
       <c r="F18" s="7" t="str">
@@ -2330,986 +2387,1036 @@
         <v>home.save</v>
       </c>
       <c r="G18" s="22" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="H18" s="22" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="I18" s="22"/>
-      <c r="J18" s="9"/>
-      <c r="K18" s="9"/>
+      <c r="J18" s="22"/>
+      <c r="K18" s="22"/>
       <c r="L18" s="9"/>
       <c r="M18" s="9"/>
       <c r="N18" s="9"/>
       <c r="O18" s="9"/>
       <c r="P18" s="9"/>
       <c r="Q18" s="9"/>
-      <c r="R18" s="10" t="b">
-        <v>1</v>
-      </c>
+      <c r="R18" s="9"/>
       <c r="S18" s="9"/>
-      <c r="T18" s="9"/>
+      <c r="T18" s="10" t="b">
+        <v>1</v>
+      </c>
       <c r="U18" s="9"/>
       <c r="V18" s="9"/>
-    </row>
-    <row r="19" spans="1:22" s="21" customFormat="1">
+      <c r="W18" s="9"/>
+      <c r="X18" s="9"/>
+    </row>
+    <row r="19" spans="1:24" s="21" customFormat="1">
       <c r="A19" s="26" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B19" s="26" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C19" s="26" t="b">
         <v>1</v>
       </c>
       <c r="D19" s="27" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E19" s="28"/>
       <c r="F19" s="28"/>
       <c r="G19" s="26"/>
       <c r="H19" s="26"/>
       <c r="I19" s="26"/>
-      <c r="J19" s="28"/>
-      <c r="K19" s="28"/>
+      <c r="J19" s="26"/>
+      <c r="K19" s="26"/>
       <c r="L19" s="28"/>
       <c r="M19" s="28"/>
       <c r="N19" s="28"/>
       <c r="O19" s="28"/>
       <c r="P19" s="28"/>
       <c r="Q19" s="28"/>
-      <c r="R19" s="27" t="b">
-        <v>1</v>
-      </c>
+      <c r="R19" s="28"/>
       <c r="S19" s="28"/>
-      <c r="T19" s="28"/>
+      <c r="T19" s="27" t="b">
+        <v>1</v>
+      </c>
       <c r="U19" s="28"/>
       <c r="V19" s="28"/>
-    </row>
-    <row r="20" spans="1:22" ht="144" customHeight="1">
+      <c r="W19" s="28"/>
+      <c r="X19" s="28"/>
+    </row>
+    <row r="20" spans="1:24" ht="144" customHeight="1">
       <c r="A20" s="27" t="s">
+        <v>103</v>
+      </c>
+      <c r="B20" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C20" s="27" t="b">
+        <v>1</v>
+      </c>
+      <c r="D20" s="27" t="s">
+        <v>102</v>
+      </c>
+      <c r="E20" s="29" t="s">
         <v>101</v>
       </c>
-      <c r="B20" s="27" t="s">
-        <v>23</v>
-      </c>
-      <c r="C20" s="27" t="b">
-        <v>1</v>
-      </c>
-      <c r="D20" s="27" t="s">
-        <v>100</v>
-      </c>
-      <c r="E20" s="29" t="s">
-        <v>99</v>
-      </c>
       <c r="F20" s="29" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="G20" s="27" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="H20" s="30" t="s">
-        <v>104</v>
-      </c>
-      <c r="I20" s="27"/>
-      <c r="J20" s="29"/>
-      <c r="K20" s="29" t="s">
-        <v>93</v>
-      </c>
-      <c r="L20" s="31"/>
-      <c r="M20" s="29"/>
-      <c r="N20" s="29"/>
+        <v>106</v>
+      </c>
+      <c r="I20" s="30"/>
+      <c r="J20" s="30"/>
+      <c r="K20" s="27"/>
+      <c r="L20" s="29"/>
+      <c r="M20" s="29" t="s">
+        <v>95</v>
+      </c>
+      <c r="N20" s="31"/>
       <c r="O20" s="29"/>
       <c r="P20" s="29"/>
       <c r="Q20" s="29"/>
-      <c r="R20" s="27" t="b">
-        <v>1</v>
-      </c>
+      <c r="R20" s="29"/>
       <c r="S20" s="29"/>
-      <c r="T20" s="29"/>
+      <c r="T20" s="27" t="b">
+        <v>1</v>
+      </c>
       <c r="U20" s="29"/>
       <c r="V20" s="29"/>
-    </row>
-    <row r="21" spans="1:22" ht="37.5">
+      <c r="W20" s="29"/>
+      <c r="X20" s="29"/>
+    </row>
+    <row r="21" spans="1:24" ht="37.5">
       <c r="A21" s="27" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B21" s="27" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C21" s="27" t="b">
         <v>1</v>
       </c>
       <c r="D21" s="27" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E21" s="29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F21" s="29" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="G21" s="27" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="H21" s="30" t="s">
-        <v>109</v>
-      </c>
-      <c r="I21" s="27"/>
-      <c r="J21" s="29"/>
-      <c r="K21" s="29"/>
-      <c r="L21" s="29" t="s">
-        <v>110</v>
-      </c>
+        <v>111</v>
+      </c>
+      <c r="I21" s="37" t="s">
+        <v>112</v>
+      </c>
+      <c r="J21" s="37" t="s">
+        <v>113</v>
+      </c>
+      <c r="K21" s="27"/>
+      <c r="L21" s="29"/>
       <c r="M21" s="29"/>
-      <c r="N21" s="29"/>
+      <c r="N21" s="29" t="s">
+        <v>114</v>
+      </c>
       <c r="O21" s="29"/>
       <c r="P21" s="29"/>
       <c r="Q21" s="29"/>
-      <c r="R21" s="27" t="b">
-        <v>1</v>
-      </c>
+      <c r="R21" s="29"/>
       <c r="S21" s="29"/>
-      <c r="T21" s="29"/>
+      <c r="T21" s="27" t="b">
+        <v>1</v>
+      </c>
       <c r="U21" s="29"/>
       <c r="V21" s="29"/>
-    </row>
-    <row r="22" spans="1:22" ht="37.5">
+      <c r="W21" s="29"/>
+      <c r="X21" s="29"/>
+    </row>
+    <row r="22" spans="1:24" ht="37.5">
       <c r="A22" s="27" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="B22" s="27" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C22" s="27" t="b">
         <v>1</v>
       </c>
       <c r="D22" s="27" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E22" s="29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F22" s="29" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="G22" s="27" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="H22" s="27" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="I22" s="27"/>
-      <c r="J22" s="29"/>
-      <c r="K22" s="31"/>
+      <c r="J22" s="27"/>
+      <c r="K22" s="27"/>
       <c r="L22" s="29"/>
-      <c r="M22" s="31" t="s">
-        <v>115</v>
-      </c>
+      <c r="M22" s="31"/>
       <c r="N22" s="29"/>
-      <c r="O22" s="29"/>
+      <c r="O22" s="31" t="s">
+        <v>119</v>
+      </c>
       <c r="P22" s="29"/>
       <c r="Q22" s="29"/>
-      <c r="R22" s="27" t="b">
-        <v>1</v>
-      </c>
+      <c r="R22" s="29"/>
       <c r="S22" s="29"/>
-      <c r="T22" s="29"/>
+      <c r="T22" s="27" t="b">
+        <v>1</v>
+      </c>
       <c r="U22" s="29"/>
       <c r="V22" s="29"/>
-    </row>
-    <row r="23" spans="1:22" ht="50.25">
+      <c r="W22" s="29"/>
+      <c r="X22" s="29"/>
+    </row>
+    <row r="23" spans="1:24" ht="50.25">
       <c r="A23" s="27" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B23" s="27" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C23" s="27" t="b">
         <v>1</v>
       </c>
       <c r="D23" s="27" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E23" s="29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F23" s="29" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="G23" s="27" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="H23" s="27" t="s">
+        <v>123</v>
+      </c>
+      <c r="I23" s="27"/>
+      <c r="J23" s="27"/>
+      <c r="K23" s="27"/>
+      <c r="L23" s="29"/>
+      <c r="M23" s="31"/>
+      <c r="N23" s="29"/>
+      <c r="O23" s="31" t="s">
         <v>119</v>
       </c>
-      <c r="I23" s="27"/>
-      <c r="J23" s="29"/>
-      <c r="K23" s="31"/>
-      <c r="L23" s="29"/>
-      <c r="M23" s="31" t="s">
-        <v>115</v>
-      </c>
-      <c r="N23" s="29"/>
-      <c r="O23" s="29"/>
       <c r="P23" s="29"/>
       <c r="Q23" s="29"/>
-      <c r="R23" s="27" t="b">
-        <v>1</v>
-      </c>
+      <c r="R23" s="29"/>
       <c r="S23" s="29"/>
-      <c r="T23" s="29"/>
+      <c r="T23" s="27" t="b">
+        <v>1</v>
+      </c>
       <c r="U23" s="29"/>
       <c r="V23" s="29"/>
-    </row>
-    <row r="24" spans="1:22" ht="24.75">
+      <c r="W23" s="29"/>
+      <c r="X23" s="29"/>
+    </row>
+    <row r="24" spans="1:24" ht="24.75">
       <c r="A24" s="27" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B24" s="27" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C24" s="27" t="b">
         <v>1</v>
       </c>
       <c r="D24" s="27" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E24" s="29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F24" s="29" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="G24" s="32" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="H24" s="32" t="s">
-        <v>123</v>
-      </c>
-      <c r="I24" s="27"/>
-      <c r="J24" s="29"/>
-      <c r="K24" s="31"/>
+        <v>127</v>
+      </c>
+      <c r="I24" s="32"/>
+      <c r="J24" s="32"/>
+      <c r="K24" s="27"/>
       <c r="L24" s="29"/>
-      <c r="M24" s="31" t="s">
-        <v>115</v>
-      </c>
+      <c r="M24" s="31"/>
       <c r="N24" s="29"/>
-      <c r="O24" s="29"/>
+      <c r="O24" s="31" t="s">
+        <v>119</v>
+      </c>
       <c r="P24" s="29"/>
       <c r="Q24" s="29"/>
-      <c r="R24" s="27" t="b">
-        <v>1</v>
-      </c>
+      <c r="R24" s="29"/>
       <c r="S24" s="29"/>
-      <c r="T24" s="29"/>
+      <c r="T24" s="27" t="b">
+        <v>1</v>
+      </c>
       <c r="U24" s="29"/>
       <c r="V24" s="29"/>
-    </row>
-    <row r="25" spans="1:22" ht="24.75">
+      <c r="W24" s="29"/>
+      <c r="X24" s="29"/>
+    </row>
+    <row r="25" spans="1:24" ht="24.75">
       <c r="A25" s="27" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B25" s="27" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C25" s="27" t="b">
         <v>1</v>
       </c>
       <c r="D25" s="27" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E25" s="29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F25" s="29" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="G25" s="27" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="H25" s="27" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="I25" s="27"/>
-      <c r="J25" s="29"/>
-      <c r="K25" s="31"/>
+      <c r="J25" s="27"/>
+      <c r="K25" s="27"/>
       <c r="L25" s="29"/>
-      <c r="M25" s="31" t="s">
-        <v>115</v>
-      </c>
-      <c r="N25" s="31"/>
-      <c r="O25" s="29"/>
-      <c r="P25" s="29"/>
+      <c r="M25" s="31"/>
+      <c r="N25" s="29"/>
+      <c r="O25" s="31" t="s">
+        <v>119</v>
+      </c>
+      <c r="P25" s="31"/>
       <c r="Q25" s="29"/>
-      <c r="R25" s="27" t="b">
-        <v>1</v>
-      </c>
+      <c r="R25" s="29"/>
       <c r="S25" s="29"/>
-      <c r="T25" s="29"/>
+      <c r="T25" s="27" t="b">
+        <v>1</v>
+      </c>
       <c r="U25" s="29"/>
       <c r="V25" s="29"/>
-    </row>
-    <row r="26" spans="1:22" ht="24.75">
+      <c r="W25" s="29"/>
+      <c r="X25" s="29"/>
+    </row>
+    <row r="26" spans="1:24" ht="24.75">
       <c r="A26" s="27" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="B26" s="27" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C26" s="27" t="b">
         <v>1</v>
       </c>
       <c r="D26" s="27" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E26" s="29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F26" s="33" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="G26" s="27" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="H26" s="27" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="I26" s="27"/>
-      <c r="J26" s="29"/>
-      <c r="K26" s="31"/>
+      <c r="J26" s="27"/>
+      <c r="K26" s="27"/>
       <c r="L26" s="29"/>
-      <c r="M26" s="31" t="s">
-        <v>115</v>
-      </c>
+      <c r="M26" s="31"/>
       <c r="N26" s="29"/>
-      <c r="O26" s="29"/>
+      <c r="O26" s="31" t="s">
+        <v>119</v>
+      </c>
       <c r="P26" s="29"/>
       <c r="Q26" s="29"/>
-      <c r="R26" s="27" t="b">
-        <v>1</v>
-      </c>
+      <c r="R26" s="29"/>
       <c r="S26" s="29"/>
-      <c r="T26" s="29"/>
+      <c r="T26" s="27" t="b">
+        <v>1</v>
+      </c>
       <c r="U26" s="29"/>
       <c r="V26" s="29"/>
-    </row>
-    <row r="27" spans="1:22" ht="62.25" customHeight="1">
+      <c r="W26" s="29"/>
+      <c r="X26" s="29"/>
+    </row>
+    <row r="27" spans="1:24" ht="62.25" customHeight="1">
       <c r="A27" s="27" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="B27" s="27" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C27" s="27" t="b">
         <v>1</v>
       </c>
       <c r="D27" s="27" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E27" s="29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F27" s="29" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="G27" s="32" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="H27" s="27" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="I27" s="27"/>
-      <c r="J27" s="29"/>
-      <c r="K27" s="31"/>
+      <c r="J27" s="27"/>
+      <c r="K27" s="27"/>
       <c r="L27" s="29"/>
-      <c r="M27" s="31" t="s">
-        <v>115</v>
-      </c>
+      <c r="M27" s="31"/>
       <c r="N27" s="29"/>
-      <c r="O27" s="29"/>
+      <c r="O27" s="31" t="s">
+        <v>119</v>
+      </c>
       <c r="P27" s="29"/>
       <c r="Q27" s="29"/>
-      <c r="R27" s="27" t="b">
-        <v>1</v>
-      </c>
+      <c r="R27" s="29"/>
       <c r="S27" s="29"/>
-      <c r="T27" s="29"/>
+      <c r="T27" s="27" t="b">
+        <v>1</v>
+      </c>
       <c r="U27" s="29"/>
       <c r="V27" s="29"/>
-    </row>
-    <row r="28" spans="1:22" ht="52.5" customHeight="1">
+      <c r="W27" s="29"/>
+      <c r="X27" s="29"/>
+    </row>
+    <row r="28" spans="1:24" ht="52.5" customHeight="1">
       <c r="A28" s="27" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B28" s="27" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C28" s="27" t="b">
         <v>1</v>
       </c>
       <c r="D28" s="27" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E28" s="29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F28" s="29" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="G28" s="27" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="H28" s="27" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="I28" s="27"/>
-      <c r="J28" s="29"/>
-      <c r="K28" s="31"/>
+      <c r="J28" s="27"/>
+      <c r="K28" s="27"/>
       <c r="L28" s="29"/>
-      <c r="M28" s="31" t="s">
-        <v>115</v>
-      </c>
+      <c r="M28" s="31"/>
       <c r="N28" s="29"/>
-      <c r="O28" s="29"/>
+      <c r="O28" s="31" t="s">
+        <v>119</v>
+      </c>
       <c r="P28" s="29"/>
       <c r="Q28" s="29"/>
-      <c r="R28" s="27" t="b">
-        <v>1</v>
-      </c>
+      <c r="R28" s="29"/>
       <c r="S28" s="29"/>
-      <c r="T28" s="29"/>
+      <c r="T28" s="27" t="b">
+        <v>1</v>
+      </c>
       <c r="U28" s="29"/>
       <c r="V28" s="29"/>
-    </row>
-    <row r="29" spans="1:22" ht="50.25">
+      <c r="W28" s="29"/>
+      <c r="X28" s="29"/>
+    </row>
+    <row r="29" spans="1:24" ht="50.25">
       <c r="A29" s="27" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="B29" s="27" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="C29" s="27" t="b">
         <v>1</v>
       </c>
       <c r="D29" s="27" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E29" s="29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F29" s="29" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="G29" s="27" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="H29" s="27" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="I29" s="27"/>
-      <c r="J29" s="29"/>
-      <c r="K29" s="31"/>
-      <c r="L29" s="31"/>
-      <c r="M29" s="31" t="s">
-        <v>115</v>
-      </c>
-      <c r="N29" s="29"/>
-      <c r="O29" s="29"/>
+      <c r="J29" s="27"/>
+      <c r="K29" s="27"/>
+      <c r="L29" s="29"/>
+      <c r="M29" s="31"/>
+      <c r="N29" s="31"/>
+      <c r="O29" s="31" t="s">
+        <v>119</v>
+      </c>
       <c r="P29" s="29"/>
       <c r="Q29" s="29"/>
-      <c r="R29" s="27" t="b">
-        <v>1</v>
-      </c>
+      <c r="R29" s="29"/>
       <c r="S29" s="29"/>
-      <c r="T29" s="29"/>
+      <c r="T29" s="27" t="b">
+        <v>1</v>
+      </c>
       <c r="U29" s="29"/>
       <c r="V29" s="29"/>
-    </row>
-    <row r="30" spans="1:22" ht="37.5">
+      <c r="W29" s="29"/>
+      <c r="X29" s="29"/>
+    </row>
+    <row r="30" spans="1:24" ht="37.5">
       <c r="A30" s="27" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="B30" s="27" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C30" s="27" t="b">
         <v>1</v>
       </c>
       <c r="D30" s="27" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E30" s="29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F30" s="29" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="G30" s="27" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="H30" s="27" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="I30" s="27"/>
-      <c r="J30" s="29"/>
-      <c r="K30" s="31"/>
+      <c r="J30" s="27"/>
+      <c r="K30" s="27"/>
       <c r="L30" s="29"/>
-      <c r="M30" s="31" t="s">
-        <v>115</v>
-      </c>
+      <c r="M30" s="31"/>
       <c r="N30" s="29"/>
-      <c r="O30" s="29"/>
+      <c r="O30" s="31" t="s">
+        <v>119</v>
+      </c>
       <c r="P30" s="29"/>
       <c r="Q30" s="29"/>
-      <c r="R30" s="27" t="b">
-        <v>1</v>
-      </c>
+      <c r="R30" s="29"/>
       <c r="S30" s="29"/>
-      <c r="T30" s="29"/>
+      <c r="T30" s="27" t="b">
+        <v>1</v>
+      </c>
       <c r="U30" s="29"/>
       <c r="V30" s="29"/>
-    </row>
-    <row r="31" spans="1:22" ht="24.75">
+      <c r="W30" s="29"/>
+      <c r="X30" s="29"/>
+    </row>
+    <row r="31" spans="1:24" ht="24.75">
       <c r="A31" s="27" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="B31" s="27" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C31" s="27" t="b">
         <v>1</v>
       </c>
       <c r="D31" s="27" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E31" s="29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F31" s="29" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="G31" s="27" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="H31" s="27" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="I31" s="27"/>
-      <c r="J31" s="29"/>
-      <c r="K31" s="31"/>
+      <c r="J31" s="27"/>
+      <c r="K31" s="27"/>
       <c r="L31" s="29"/>
-      <c r="M31" s="31" t="s">
-        <v>115</v>
-      </c>
+      <c r="M31" s="31"/>
       <c r="N31" s="29"/>
-      <c r="O31" s="29"/>
+      <c r="O31" s="31" t="s">
+        <v>119</v>
+      </c>
       <c r="P31" s="29"/>
       <c r="Q31" s="29"/>
-      <c r="R31" s="27" t="b">
-        <v>1</v>
-      </c>
+      <c r="R31" s="29"/>
       <c r="S31" s="29"/>
-      <c r="T31" s="29"/>
+      <c r="T31" s="27" t="b">
+        <v>1</v>
+      </c>
       <c r="U31" s="29"/>
       <c r="V31" s="29"/>
-    </row>
-    <row r="32" spans="1:22" ht="24.75">
+      <c r="W31" s="29"/>
+      <c r="X31" s="29"/>
+    </row>
+    <row r="32" spans="1:24" ht="24.75">
       <c r="A32" s="27" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="B32" s="27" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C32" s="27" t="b">
         <v>1</v>
       </c>
       <c r="D32" s="27" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E32" s="29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F32" s="29" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="G32" s="27" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="H32" s="27" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="I32" s="27"/>
-      <c r="J32" s="29"/>
-      <c r="K32" s="31"/>
+      <c r="J32" s="27"/>
+      <c r="K32" s="27"/>
       <c r="L32" s="29"/>
-      <c r="M32" s="31" t="s">
-        <v>115</v>
-      </c>
+      <c r="M32" s="31"/>
       <c r="N32" s="29"/>
-      <c r="O32" s="29"/>
+      <c r="O32" s="31" t="s">
+        <v>119</v>
+      </c>
       <c r="P32" s="29"/>
       <c r="Q32" s="29"/>
-      <c r="R32" s="27" t="b">
-        <v>1</v>
-      </c>
+      <c r="R32" s="29"/>
       <c r="S32" s="29"/>
-      <c r="T32" s="29"/>
+      <c r="T32" s="27" t="b">
+        <v>1</v>
+      </c>
       <c r="U32" s="29"/>
       <c r="V32" s="29"/>
-    </row>
-    <row r="33" spans="1:22" ht="24.75">
+      <c r="W32" s="29"/>
+      <c r="X32" s="29"/>
+    </row>
+    <row r="33" spans="1:24" ht="24.75">
       <c r="A33" s="27" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="B33" s="27" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C33" s="27" t="b">
         <v>1</v>
       </c>
       <c r="D33" s="27" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E33" s="29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F33" s="29" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="G33" s="27" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="H33" s="27" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="I33" s="27"/>
-      <c r="J33" s="29"/>
-      <c r="K33" s="31"/>
+      <c r="J33" s="27"/>
+      <c r="K33" s="27"/>
       <c r="L33" s="29"/>
-      <c r="M33" s="29"/>
-      <c r="N33" s="31"/>
+      <c r="M33" s="31"/>
+      <c r="N33" s="29"/>
       <c r="O33" s="29"/>
-      <c r="P33" s="29"/>
+      <c r="P33" s="31"/>
       <c r="Q33" s="29"/>
-      <c r="R33" s="27" t="b">
-        <v>1</v>
-      </c>
+      <c r="R33" s="29"/>
       <c r="S33" s="29"/>
-      <c r="T33" s="29"/>
+      <c r="T33" s="27" t="b">
+        <v>1</v>
+      </c>
       <c r="U33" s="29"/>
       <c r="V33" s="29"/>
-    </row>
-    <row r="34" spans="1:22" ht="24.75">
+      <c r="W33" s="29"/>
+      <c r="X33" s="29"/>
+    </row>
+    <row r="34" spans="1:24" ht="24.75">
       <c r="A34" s="27" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="B34" s="27"/>
       <c r="C34" s="27" t="b">
         <v>0</v>
       </c>
       <c r="D34" s="27" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E34" s="29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F34" s="29" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="G34" s="32" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="H34" s="32" t="s">
-        <v>163</v>
-      </c>
-      <c r="I34" s="27"/>
-      <c r="J34" s="29"/>
-      <c r="K34" s="31"/>
+        <v>167</v>
+      </c>
+      <c r="I34" s="32"/>
+      <c r="J34" s="32"/>
+      <c r="K34" s="27"/>
       <c r="L34" s="29"/>
-      <c r="M34" s="29"/>
-      <c r="N34" s="31"/>
+      <c r="M34" s="31"/>
+      <c r="N34" s="29"/>
       <c r="O34" s="29"/>
-      <c r="P34" s="29"/>
+      <c r="P34" s="31"/>
       <c r="Q34" s="29"/>
-      <c r="R34" s="27" t="b">
-        <v>1</v>
-      </c>
+      <c r="R34" s="29"/>
       <c r="S34" s="29"/>
-      <c r="T34" s="29"/>
+      <c r="T34" s="27" t="b">
+        <v>1</v>
+      </c>
       <c r="U34" s="29"/>
       <c r="V34" s="29"/>
-    </row>
-    <row r="35" spans="1:22" ht="24.75">
+      <c r="W34" s="29"/>
+      <c r="X34" s="29"/>
+    </row>
+    <row r="35" spans="1:24" ht="24.75">
       <c r="A35" s="27" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="B35" s="27" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C35" s="27" t="b">
         <v>1</v>
       </c>
       <c r="D35" s="27" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E35" s="29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F35" s="29" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="G35" s="27" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="H35" s="27" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="I35" s="27"/>
-      <c r="J35" s="29"/>
-      <c r="K35" s="31"/>
+      <c r="J35" s="27"/>
+      <c r="K35" s="27"/>
       <c r="L35" s="29"/>
-      <c r="M35" s="29"/>
-      <c r="N35" s="31"/>
+      <c r="M35" s="31"/>
+      <c r="N35" s="29"/>
       <c r="O35" s="29"/>
-      <c r="P35" s="29"/>
+      <c r="P35" s="31"/>
       <c r="Q35" s="29"/>
-      <c r="R35" s="27" t="b">
-        <v>1</v>
-      </c>
+      <c r="R35" s="29"/>
       <c r="S35" s="29"/>
-      <c r="T35" s="29"/>
+      <c r="T35" s="27" t="b">
+        <v>1</v>
+      </c>
       <c r="U35" s="29"/>
       <c r="V35" s="29"/>
-    </row>
-    <row r="36" spans="1:22" ht="24.75">
+      <c r="W35" s="29"/>
+      <c r="X35" s="29"/>
+    </row>
+    <row r="36" spans="1:24" ht="24.75">
       <c r="A36" s="27" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="B36" s="27"/>
       <c r="C36" s="27" t="b">
         <v>0</v>
       </c>
       <c r="D36" s="27" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E36" s="29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F36" s="29" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="G36" s="32" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="H36" s="32" t="s">
-        <v>163</v>
-      </c>
-      <c r="I36" s="27"/>
-      <c r="J36" s="29"/>
-      <c r="K36" s="31"/>
+        <v>167</v>
+      </c>
+      <c r="I36" s="32"/>
+      <c r="J36" s="32"/>
+      <c r="K36" s="27"/>
       <c r="L36" s="29"/>
-      <c r="M36" s="29"/>
-      <c r="N36" s="31"/>
+      <c r="M36" s="31"/>
+      <c r="N36" s="29"/>
       <c r="O36" s="29"/>
-      <c r="P36" s="29"/>
+      <c r="P36" s="31"/>
       <c r="Q36" s="29"/>
-      <c r="R36" s="27" t="b">
-        <v>1</v>
-      </c>
+      <c r="R36" s="29"/>
       <c r="S36" s="29"/>
-      <c r="T36" s="29"/>
+      <c r="T36" s="27" t="b">
+        <v>1</v>
+      </c>
       <c r="U36" s="29"/>
       <c r="V36" s="29"/>
-    </row>
-    <row r="37" spans="1:22" ht="86.25" customHeight="1">
+      <c r="W36" s="29"/>
+      <c r="X36" s="29"/>
+    </row>
+    <row r="37" spans="1:24" ht="86.25" customHeight="1">
       <c r="A37" s="27" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="B37" s="27" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="C37" s="27" t="b">
         <v>1</v>
       </c>
       <c r="D37" s="27" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E37" s="29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F37" s="29" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="G37" s="27" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="H37" s="27" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="I37" s="27"/>
-      <c r="J37" s="29"/>
-      <c r="K37" s="31"/>
-      <c r="L37" s="31"/>
-      <c r="M37" s="31" t="s">
-        <v>115</v>
-      </c>
-      <c r="N37" s="29"/>
-      <c r="O37" s="29"/>
+      <c r="J37" s="27"/>
+      <c r="K37" s="27"/>
+      <c r="L37" s="29"/>
+      <c r="M37" s="31"/>
+      <c r="N37" s="31"/>
+      <c r="O37" s="31" t="s">
+        <v>119</v>
+      </c>
       <c r="P37" s="29"/>
       <c r="Q37" s="29"/>
-      <c r="R37" s="27" t="b">
-        <v>1</v>
-      </c>
+      <c r="R37" s="29"/>
       <c r="S37" s="29"/>
-      <c r="T37" s="29"/>
+      <c r="T37" s="27" t="b">
+        <v>1</v>
+      </c>
       <c r="U37" s="29"/>
       <c r="V37" s="29"/>
-    </row>
-    <row r="38" spans="1:22" ht="37.5">
+      <c r="W37" s="29"/>
+      <c r="X37" s="29"/>
+    </row>
+    <row r="38" spans="1:24" ht="37.5">
       <c r="A38" s="27" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="B38" s="27" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="C38" s="27" t="b">
         <v>1</v>
       </c>
       <c r="D38" s="27" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E38" s="29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F38" s="29" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="G38" s="27" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="H38" s="27" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="I38" s="27"/>
-      <c r="J38" s="29"/>
-      <c r="K38" s="31"/>
-      <c r="L38" s="31"/>
-      <c r="M38" s="31" t="s">
-        <v>115</v>
-      </c>
-      <c r="N38" s="29"/>
-      <c r="O38" s="29"/>
+      <c r="J38" s="27"/>
+      <c r="K38" s="27"/>
+      <c r="L38" s="29"/>
+      <c r="M38" s="31"/>
+      <c r="N38" s="31"/>
+      <c r="O38" s="31" t="s">
+        <v>119</v>
+      </c>
       <c r="P38" s="29"/>
       <c r="Q38" s="29"/>
-      <c r="R38" s="27" t="b">
-        <v>1</v>
-      </c>
+      <c r="R38" s="29"/>
       <c r="S38" s="29"/>
-      <c r="T38" s="29"/>
+      <c r="T38" s="27" t="b">
+        <v>1</v>
+      </c>
       <c r="U38" s="29"/>
       <c r="V38" s="29"/>
-    </row>
-    <row r="39" spans="1:22" ht="75.75">
+      <c r="W38" s="29"/>
+      <c r="X38" s="29"/>
+    </row>
+    <row r="39" spans="1:24" ht="75.75">
       <c r="A39" s="27" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B39" s="27" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="C39" s="27" t="b">
         <v>1</v>
       </c>
       <c r="D39" s="27" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E39" s="29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F39" s="29" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="G39" s="27" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="H39" s="27" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="I39" s="27"/>
-      <c r="J39" s="29"/>
-      <c r="K39" s="31"/>
-      <c r="L39" s="31"/>
-      <c r="M39" s="31" t="s">
-        <v>115</v>
-      </c>
-      <c r="N39" s="29"/>
-      <c r="O39" s="29"/>
+      <c r="J39" s="27"/>
+      <c r="K39" s="27"/>
+      <c r="L39" s="29"/>
+      <c r="M39" s="31"/>
+      <c r="N39" s="31"/>
+      <c r="O39" s="31" t="s">
+        <v>119</v>
+      </c>
       <c r="P39" s="29"/>
       <c r="Q39" s="29"/>
-      <c r="R39" s="27" t="b">
-        <v>1</v>
-      </c>
+      <c r="R39" s="29"/>
       <c r="S39" s="29"/>
-      <c r="T39" s="29"/>
+      <c r="T39" s="27" t="b">
+        <v>1</v>
+      </c>
       <c r="U39" s="29"/>
       <c r="V39" s="29"/>
-    </row>
-    <row r="40" spans="1:22" ht="37.5">
+      <c r="W39" s="29"/>
+      <c r="X39" s="29"/>
+    </row>
+    <row r="40" spans="1:24" ht="37.5">
       <c r="A40" s="27" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="B40" s="27" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="C40" s="27" t="b">
         <v>1</v>
       </c>
       <c r="D40" s="27" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E40" s="29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F40" s="29" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="G40" s="27" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="H40" s="27" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="I40" s="27"/>
-      <c r="J40" s="29"/>
-      <c r="K40" s="31"/>
-      <c r="L40" s="31"/>
-      <c r="M40" s="31" t="s">
-        <v>115</v>
-      </c>
-      <c r="N40" s="29"/>
-      <c r="O40" s="29"/>
+      <c r="J40" s="27"/>
+      <c r="K40" s="27"/>
+      <c r="L40" s="29"/>
+      <c r="M40" s="31"/>
+      <c r="N40" s="31"/>
+      <c r="O40" s="31" t="s">
+        <v>119</v>
+      </c>
       <c r="P40" s="29"/>
       <c r="Q40" s="29"/>
-      <c r="R40" s="27" t="b">
-        <v>1</v>
-      </c>
+      <c r="R40" s="29"/>
       <c r="S40" s="29"/>
-      <c r="T40" s="29"/>
+      <c r="T40" s="27" t="b">
+        <v>1</v>
+      </c>
       <c r="U40" s="29"/>
       <c r="V40" s="29"/>
-    </row>
-    <row r="41" spans="1:22" s="18" customFormat="1">
+      <c r="W40" s="29"/>
+      <c r="X40" s="29"/>
+    </row>
+    <row r="41" spans="1:24" s="18" customFormat="1">
       <c r="A41" s="34" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="B41" s="34" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C41" s="34" t="b">
         <v>1</v>
       </c>
       <c r="D41" s="34" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E41" s="35"/>
       <c r="F41" s="35" t="str">
@@ -3317,58 +3424,60 @@
         <v>household.save</v>
       </c>
       <c r="G41" s="34" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="H41" s="34" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="I41" s="34"/>
-      <c r="J41" s="35"/>
-      <c r="K41" s="35"/>
+      <c r="J41" s="34"/>
+      <c r="K41" s="34"/>
       <c r="L41" s="35"/>
       <c r="M41" s="35"/>
       <c r="N41" s="35"/>
       <c r="O41" s="35"/>
       <c r="P41" s="35"/>
       <c r="Q41" s="35"/>
-      <c r="R41" s="34" t="b">
-        <v>1</v>
-      </c>
+      <c r="R41" s="35"/>
       <c r="S41" s="35"/>
-      <c r="T41" s="35"/>
+      <c r="T41" s="34" t="b">
+        <v>1</v>
+      </c>
       <c r="U41" s="35"/>
       <c r="V41" s="35"/>
-    </row>
-    <row r="42" spans="1:22" ht="130.5" hidden="1">
+      <c r="W41" s="35"/>
+      <c r="X41" s="35"/>
+    </row>
+    <row r="42" spans="1:24" ht="130.5" hidden="1">
       <c r="A42" s="8" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C42" s="8" t="b">
         <v>1</v>
       </c>
       <c r="D42" s="8" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="F42" s="8" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="G42" s="8" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="H42" s="8" t="s">
-        <v>190</v>
-      </c>
-      <c r="J42" s="20"/>
-      <c r="K42" s="19"/>
-      <c r="R42" s="8" t="b">
+        <v>194</v>
+      </c>
+      <c r="L42" s="20"/>
+      <c r="M42" s="19"/>
+      <c r="T42" s="8" t="b">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:V42" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <autoFilter ref="A1:X42" xr:uid="{00000000-0001-0000-0000-000000000000}">
     <filterColumn colId="3">
       <filters>
         <filter val="household"/>
@@ -3393,19 +3502,19 @@
       <formula>NOT(ISERROR(SEARCH("TRUE",C42)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L42:O42">
+  <conditionalFormatting sqref="N42:Q42">
     <cfRule type="expression" dxfId="2" priority="1">
-      <formula>AND($B1048370="Custom",  $B1048370&lt;&gt;"", ROW(L1048370)&lt;&gt;1)</formula>
+      <formula>AND($B1048370="Custom",  $B1048370&lt;&gt;"", ROW(N1048370)&lt;&gt;1)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M42:N42">
+  <conditionalFormatting sqref="O42:P42">
     <cfRule type="expression" dxfId="1" priority="5">
-      <formula>AND($B42&lt;&gt;"Select", $B42&lt;&gt;"Checkbox", $B42&lt;&gt;"Radio",  $B42&lt;&gt;"", ROW(M42)&lt;&gt;1)</formula>
+      <formula>AND($B42&lt;&gt;"Select", $B42&lt;&gt;"Checkbox", $B42&lt;&gt;"Radio",  $B42&lt;&gt;"", ROW(O42)&lt;&gt;1)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O42">
+  <conditionalFormatting sqref="Q42">
     <cfRule type="expression" dxfId="0" priority="2">
-      <formula>AND($B42&lt;&gt;"Range", $B42&lt;&gt;"", ROW(O42)&lt;&gt;1)</formula>
+      <formula>AND($B42&lt;&gt;"Range", $B42&lt;&gt;"", ROW(Q42)&lt;&gt;1)</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3427,34 +3536,34 @@
   <sheetData>
     <row r="1" spans="1:6" s="6" customFormat="1">
       <c r="A1" s="14" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="C1" s="14" t="s">
         <v>5</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="E1" s="14" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="F1" s="14" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="29.25">
       <c r="A2" s="12" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="D2" s="15" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="E2" s="12">
         <v>1</v>
@@ -3463,14 +3572,14 @@
     </row>
     <row r="3" spans="1:6" ht="29.25">
       <c r="A3" s="12" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B3" s="12"/>
       <c r="C3" s="12" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="E3" s="12">
         <v>2</v>
@@ -3502,39 +3611,39 @@
         <v>3</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="G1" s="18" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="12" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="D2" s="12" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E2" s="12" t="b">
         <v>1</v>
@@ -3548,16 +3657,16 @@
     </row>
     <row r="3" spans="1:8">
       <c r="A3" s="12" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="E3" s="12" t="b">
         <v>1</v>
@@ -3571,16 +3680,16 @@
     </row>
     <row r="4" spans="1:8" ht="29.25">
       <c r="A4" s="12" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="E4" s="12" t="b">
         <v>0</v>
@@ -3612,10 +3721,10 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="3" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>6</v>
@@ -3624,136 +3733,136 @@
         <v>7</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="B2" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="C2" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="D2" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="B3" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="C3" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="D3" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="B4" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="C4" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="D4" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="C5" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="D5" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="B6" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="C6" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="D6" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E7" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E8" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="E9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="E10" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="E11" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="E12" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="E13" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
     </row>
   </sheetData>
@@ -3780,40 +3889,40 @@
   <sheetData>
     <row r="1" spans="1:12" s="5" customFormat="1">
       <c r="A1" s="4" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
   </sheetData>
@@ -3828,19 +3937,19 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="B1" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="C1" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="D1" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="E1" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add gender context for label translations with the Generator.
Add getActivePersonGender helper function to help with that.
Update the household Excel with this new method.
</commit_message>
<xml_diff>
--- a/example/demo_generator/references/Household_Travel_Generate_Survey.xlsx
+++ b/example/demo_generator/references/Household_Travel_Generate_Survey.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28928"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="978" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C0AF4DD7-5803-4D81-ABD0-4FE84017DD06}"/>
+  <xr:revisionPtr revIDLastSave="1011" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{16609EB3-8854-4224-91CB-3373A9034551}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="260">
   <si>
     <t>questionName</t>
   </si>
@@ -403,10 +403,10 @@
 __For babies under the age of 1, write "0"__</t>
   </si>
   <si>
-    <t>**Votre âge**</t>
-  </si>
-  <si>
-    <t>**Your age**</t>
+    <t>Votre **âge**</t>
+  </si>
+  <si>
+    <t>Your **age**</t>
   </si>
   <si>
     <t>ageValidation</t>
@@ -426,9 +426,6 @@
 __Sex assigned at birth or that which appears on legal documents.__</t>
   </si>
   <si>
-    <t>yesNoDontKnow</t>
-  </si>
-  <si>
     <t>personWorkerType</t>
   </si>
   <si>
@@ -443,6 +440,9 @@
 __Including self-employed, artist, on sick leave or parental leave.__</t>
   </si>
   <si>
+    <t>yesNoDontKnow</t>
+  </si>
+  <si>
     <t>personSchoolType</t>
   </si>
   <si>
@@ -461,7 +461,7 @@
     <t>studentType</t>
   </si>
   <si>
-    <t>**Étudiant**</t>
+    <t>**Étudiant{{gender:e}}**</t>
   </si>
   <si>
     <t>**Student**</t>
@@ -486,7 +486,7 @@
   </si>
   <si>
     <t>**Permis de conduire**
-__Inclure les permis d’apprenti{{suffixE}}conduct{{suffixEurRice}} et probatoires, mais ne pas inclure les permis de cyclomoteur/scooter.__</t>
+__Inclure les permis d’apprenti{{gender:e}} conduct{{gender:eur/rice}} et probatoires, mais ne pas inclure les permis de cyclomoteur/scooter.__</t>
   </si>
   <si>
     <t>**Driver's licence**
@@ -603,7 +603,7 @@
     <t>travelToWorkDays</t>
   </si>
   <si>
-    <t>Durant la dernière **semaine**, quand est-ce que {{nickname}} s'est **déplacé{{suffixE}}** pour le **travail** ?
+    <t>Durant la dernière **semaine**, quand est-ce que {{nickname}} s'est **déplacé{{gender:e}}** pour le **travail** ?
 __Pour se rendre au travail ou toute autre raison concernant le travail.__</t>
   </si>
   <si>
@@ -629,7 +629,7 @@
     <t>travelToStudyDays</t>
   </si>
   <si>
-    <t>Durant la **dernière semaine**, est-ce que {{nickname}} s'est **déplacé{{suffixE}}** pour les **études**.
+    <t>Durant la **dernière semaine**, est-ce que {{nickname}} s'est **déplacé{{gender:e}}** pour les **études**.
 __Pour se rendre à l'établissement d'enseignement ou pour toute autre raison concernant les études.__</t>
   </si>
   <si>
@@ -790,6 +790,24 @@
   </si>
   <si>
     <t>I prefer not to answer</t>
+  </si>
+  <si>
+    <t>man</t>
+  </si>
+  <si>
+    <t>Homme</t>
+  </si>
+  <si>
+    <t>Man</t>
+  </si>
+  <si>
+    <t>woman</t>
+  </si>
+  <si>
+    <t>Femme</t>
+  </si>
+  <si>
+    <t>Woman</t>
   </si>
   <si>
     <t>inputRangeName</t>
@@ -1127,10 +1145,10 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2518,10 +2536,10 @@
       <c r="H21" s="30" t="s">
         <v>111</v>
       </c>
-      <c r="I21" s="37" t="s">
+      <c r="I21" s="30" t="s">
         <v>112</v>
       </c>
-      <c r="J21" s="37" t="s">
+      <c r="J21" s="30" t="s">
         <v>113</v>
       </c>
       <c r="K21" s="27"/>
@@ -2574,8 +2592,8 @@
       <c r="L22" s="29"/>
       <c r="M22" s="31"/>
       <c r="N22" s="29"/>
-      <c r="O22" s="31" t="s">
-        <v>119</v>
+      <c r="O22" s="37" t="s">
+        <v>116</v>
       </c>
       <c r="P22" s="29"/>
       <c r="Q22" s="29"/>
@@ -2591,7 +2609,7 @@
     </row>
     <row r="23" spans="1:24" ht="50.25">
       <c r="A23" s="27" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B23" s="27" t="s">
         <v>30</v>
@@ -2606,13 +2624,13 @@
         <v>101</v>
       </c>
       <c r="F23" s="29" t="s">
+        <v>120</v>
+      </c>
+      <c r="G23" s="27" t="s">
         <v>121</v>
       </c>
-      <c r="G23" s="27" t="s">
+      <c r="H23" s="27" t="s">
         <v>122</v>
-      </c>
-      <c r="H23" s="27" t="s">
-        <v>123</v>
       </c>
       <c r="I23" s="27"/>
       <c r="J23" s="27"/>
@@ -2621,7 +2639,7 @@
       <c r="M23" s="31"/>
       <c r="N23" s="29"/>
       <c r="O23" s="31" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="P23" s="29"/>
       <c r="Q23" s="29"/>
@@ -2660,14 +2678,14 @@
       <c r="H24" s="32" t="s">
         <v>127</v>
       </c>
-      <c r="I24" s="32"/>
-      <c r="J24" s="32"/>
+      <c r="I24" s="27"/>
+      <c r="J24" s="27"/>
       <c r="K24" s="27"/>
       <c r="L24" s="29"/>
       <c r="M24" s="31"/>
       <c r="N24" s="29"/>
       <c r="O24" s="31" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="P24" s="29"/>
       <c r="Q24" s="29"/>
@@ -2713,7 +2731,7 @@
       <c r="M25" s="31"/>
       <c r="N25" s="29"/>
       <c r="O25" s="31" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="P25" s="31"/>
       <c r="Q25" s="29"/>
@@ -2759,7 +2777,7 @@
       <c r="M26" s="31"/>
       <c r="N26" s="29"/>
       <c r="O26" s="31" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="P26" s="29"/>
       <c r="Q26" s="29"/>
@@ -2805,7 +2823,7 @@
       <c r="M27" s="31"/>
       <c r="N27" s="29"/>
       <c r="O27" s="31" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="P27" s="29"/>
       <c r="Q27" s="29"/>
@@ -2851,7 +2869,7 @@
       <c r="M28" s="31"/>
       <c r="N28" s="29"/>
       <c r="O28" s="31" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="P28" s="29"/>
       <c r="Q28" s="29"/>
@@ -2897,7 +2915,7 @@
       <c r="M29" s="31"/>
       <c r="N29" s="31"/>
       <c r="O29" s="31" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="P29" s="29"/>
       <c r="Q29" s="29"/>
@@ -2943,7 +2961,7 @@
       <c r="M30" s="31"/>
       <c r="N30" s="29"/>
       <c r="O30" s="31" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="P30" s="29"/>
       <c r="Q30" s="29"/>
@@ -2989,7 +3007,7 @@
       <c r="M31" s="31"/>
       <c r="N31" s="29"/>
       <c r="O31" s="31" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="P31" s="29"/>
       <c r="Q31" s="29"/>
@@ -3035,7 +3053,7 @@
       <c r="M32" s="31"/>
       <c r="N32" s="29"/>
       <c r="O32" s="31" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="P32" s="29"/>
       <c r="Q32" s="29"/>
@@ -3253,7 +3271,7 @@
       <c r="M37" s="31"/>
       <c r="N37" s="31"/>
       <c r="O37" s="31" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="P37" s="29"/>
       <c r="Q37" s="29"/>
@@ -3299,7 +3317,7 @@
       <c r="M38" s="31"/>
       <c r="N38" s="31"/>
       <c r="O38" s="31" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="P38" s="29"/>
       <c r="Q38" s="29"/>
@@ -3345,7 +3363,7 @@
       <c r="M39" s="31"/>
       <c r="N39" s="31"/>
       <c r="O39" s="31" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="P39" s="29"/>
       <c r="Q39" s="29"/>
@@ -3391,7 +3409,7 @@
       <c r="M40" s="31"/>
       <c r="N40" s="31"/>
       <c r="O40" s="31" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="P40" s="29"/>
       <c r="Q40" s="29"/>
@@ -3708,7 +3726,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B85C046C-24FF-4202-B29D-53FEFBA5C312}">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="21.28515625" bestFit="1" customWidth="1"/>
@@ -3827,7 +3845,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="E9" t="s">
         <v>33</v>
@@ -3835,7 +3853,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="E10" t="s">
         <v>231</v>
@@ -3862,6 +3880,42 @@
         <v>96</v>
       </c>
       <c r="E13" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" t="s">
+        <v>116</v>
+      </c>
+      <c r="B14" t="s">
+        <v>237</v>
+      </c>
+      <c r="C14" t="s">
+        <v>238</v>
+      </c>
+      <c r="D14" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" t="s">
+        <v>116</v>
+      </c>
+      <c r="B15" t="s">
+        <v>240</v>
+      </c>
+      <c r="C15" t="s">
+        <v>241</v>
+      </c>
+      <c r="D15" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" t="s">
+        <v>116</v>
+      </c>
+      <c r="E16" t="s">
         <v>234</v>
       </c>
     </row>
@@ -3889,40 +3943,40 @@
   <sheetData>
     <row r="1" spans="1:12" s="5" customFormat="1">
       <c r="A1" s="4" t="s">
-        <v>237</v>
+        <v>243</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>239</v>
+        <v>245</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>243</v>
+        <v>249</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>248</v>
+        <v>254</v>
       </c>
     </row>
   </sheetData>
@@ -3937,19 +3991,19 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>249</v>
+        <v>255</v>
       </c>
       <c r="B1" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="C1" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="D1" t="s">
-        <v>252</v>
+        <v>258</v>
       </c>
       <c r="E1" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add 2 custom widgets map in household
Add custom helpers and geojson that was not possible to migrate to Evolution yet.
</commit_message>
<xml_diff>
--- a/example/demo_generator/references/Household_Travel_Generate_Survey.xlsx
+++ b/example/demo_generator/references/Household_Travel_Generate_Survey.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28928"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="1011" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{16609EB3-8854-4224-91CB-3373A9034551}"/>
+  <xr:revisionPtr revIDLastSave="1018" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{62ECE760-9A17-495C-ADE5-20B0A6087FD8}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="260">
   <si>
     <t>questionName</t>
   </si>
@@ -1148,7 +1148,7 @@
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2433,7 +2433,7 @@
       <c r="A19" s="26" t="s">
         <v>101</v>
       </c>
-      <c r="B19" s="26" t="s">
+      <c r="B19" s="37" t="s">
         <v>69</v>
       </c>
       <c r="C19" s="26" t="b">
@@ -2592,7 +2592,7 @@
       <c r="L22" s="29"/>
       <c r="M22" s="31"/>
       <c r="N22" s="29"/>
-      <c r="O22" s="37" t="s">
+      <c r="O22" s="29" t="s">
         <v>116</v>
       </c>
       <c r="P22" s="29"/>
@@ -3115,9 +3115,11 @@
       <c r="A34" s="27" t="s">
         <v>165</v>
       </c>
-      <c r="B34" s="27"/>
+      <c r="B34" s="32" t="s">
+        <v>69</v>
+      </c>
       <c r="C34" s="27" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D34" s="27" t="s">
         <v>102</v>
@@ -3201,9 +3203,11 @@
       <c r="A36" s="27" t="s">
         <v>172</v>
       </c>
-      <c r="B36" s="27"/>
+      <c r="B36" s="32" t="s">
+        <v>69</v>
+      </c>
       <c r="C36" s="27" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D36" s="27" t="s">
         <v>102</v>

</xml_diff>

<commit_message>
Generator: add a custom labels example in customLabels.ts
- Introduced a new custom labels for personSchoolType
- Updated the Household Travel Generate Survey Excel file to reflect the translation effect.
</commit_message>
<xml_diff>
--- a/example/demo_generator/references/Household_Travel_Generate_Survey.xlsx
+++ b/example/demo_generator/references/Household_Travel_Generate_Survey.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="678" uniqueCount="385">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="681" uniqueCount="385">
   <si>
     <t xml:space="preserve">questionName</t>
   </si>
@@ -465,6 +465,9 @@
     <t xml:space="preserve">**School type**</t>
   </si>
   <si>
+    <t xml:space="preserve">customLabels={{personSchoolTypeCustomLabels}}</t>
+  </si>
+  <si>
     <t xml:space="preserve">ifAge15OrLessConditional</t>
   </si>
   <si>
@@ -1226,19 +1229,16 @@
     <t xml:space="preserve">input_color</t>
   </si>
   <si>
-    <t xml:space="preserve">home.test</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test</t>
-  </si>
-  <si>
-    <t xml:space="preserve">**Test**</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mon test</t>
-  </si>
-  <si>
-    <t xml:space="preserve">**My test**</t>
+    <t xml:space="preserve">personSchoolTypeYoungChild</t>
+  </si>
+  <si>
+    <t xml:space="preserve">**Type d’école / garderie**</t>
+  </si>
+  <si>
+    <t xml:space="preserve">**School type / daycare**</t>
+  </si>
+  <si>
+    <t xml:space="preserve">personSchoolTypeOlderPerson</t>
   </si>
 </sst>
 </file>
@@ -1250,7 +1250,7 @@
     <numFmt numFmtId="165" formatCode="General"/>
     <numFmt numFmtId="166" formatCode="@"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1325,6 +1325,12 @@
       <name val="Calibri"/>
       <family val="0"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
     <font>
       <sz val="9"/>
@@ -1468,7 +1474,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="54">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1569,7 +1575,7 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1577,7 +1583,11 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1597,11 +1607,11 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1613,11 +1623,11 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1629,11 +1639,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1649,11 +1659,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1665,16 +1675,20 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -2036,7 +2050,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="31.28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="8" style="1" width="31.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="20.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="35.41"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="22.7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="19.72"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="13.57"/>
@@ -2680,7 +2694,7 @@
       <c r="Q13" s="7"/>
       <c r="R13" s="7"/>
       <c r="S13" s="7"/>
-      <c r="T13" s="8" t="b">
+      <c r="T13" s="7" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2731,7 +2745,7 @@
       <c r="Q14" s="7"/>
       <c r="R14" s="7"/>
       <c r="S14" s="7"/>
-      <c r="T14" s="8" t="b">
+      <c r="T14" s="7" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -3238,18 +3252,20 @@
       <c r="F25" s="23" t="s">
         <v>132</v>
       </c>
-      <c r="G25" s="19" t="s">
+      <c r="G25" s="25" t="s">
         <v>133</v>
       </c>
-      <c r="H25" s="19" t="s">
+      <c r="H25" s="25" t="s">
         <v>134</v>
       </c>
       <c r="I25" s="19"/>
       <c r="J25" s="19"/>
-      <c r="K25" s="19"/>
+      <c r="K25" s="26" t="s">
+        <v>135</v>
+      </c>
       <c r="L25" s="23"/>
-      <c r="M25" s="25" t="s">
-        <v>135</v>
+      <c r="M25" s="27" t="s">
+        <v>136</v>
       </c>
       <c r="N25" s="23"/>
       <c r="O25" s="23" t="s">
@@ -3264,17 +3280,17 @@
         <v>1</v>
       </c>
       <c r="U25" s="23" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="V25" s="23" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="W25" s="23"/>
       <c r="X25" s="23"/>
     </row>
     <row r="26" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="19" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B26" s="19" t="s">
         <v>30</v>
@@ -3289,25 +3305,25 @@
       <c r="E26" s="23" t="s">
         <v>101</v>
       </c>
-      <c r="F26" s="26" t="s">
-        <v>139</v>
+      <c r="F26" s="28" t="s">
+        <v>140</v>
       </c>
       <c r="G26" s="19" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H26" s="19" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="I26" s="19"/>
       <c r="J26" s="19"/>
       <c r="K26" s="19"/>
       <c r="L26" s="23"/>
       <c r="M26" s="23" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="N26" s="23"/>
       <c r="O26" s="23" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="P26" s="23"/>
       <c r="Q26" s="23"/>
@@ -3324,7 +3340,7 @@
     </row>
     <row r="27" customFormat="false" ht="62.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="19" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B27" s="19" t="s">
         <v>30</v>
@@ -3340,13 +3356,13 @@
         <v>101</v>
       </c>
       <c r="F27" s="23" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G27" s="19" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H27" s="19" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="I27" s="19"/>
       <c r="J27" s="19"/>
@@ -3357,7 +3373,7 @@
       </c>
       <c r="N27" s="23"/>
       <c r="O27" s="23" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="P27" s="23"/>
       <c r="Q27" s="23"/>
@@ -3374,7 +3390,7 @@
     </row>
     <row r="28" customFormat="false" ht="52.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="19" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B28" s="19" t="s">
         <v>30</v>
@@ -3390,30 +3406,30 @@
         <v>101</v>
       </c>
       <c r="F28" s="23" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G28" s="19" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="H28" s="19" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="I28" s="19"/>
       <c r="J28" s="19"/>
       <c r="K28" s="19"/>
       <c r="L28" s="23"/>
       <c r="M28" s="23" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="N28" s="23"/>
       <c r="O28" s="23" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="P28" s="23"/>
       <c r="Q28" s="23"/>
       <c r="R28" s="23"/>
       <c r="S28" s="23"/>
-      <c r="T28" s="21" t="b">
+      <c r="T28" s="19" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -3423,11 +3439,11 @@
       <c r="X28" s="23"/>
     </row>
     <row r="29" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="27" t="s">
-        <v>153</v>
+      <c r="A29" s="25" t="s">
+        <v>154</v>
       </c>
       <c r="B29" s="19" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C29" s="21" t="b">
         <f aca="false">FALSE()</f>
@@ -3440,24 +3456,24 @@
         <v>101</v>
       </c>
       <c r="F29" s="23" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="G29" s="19" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="H29" s="19" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="I29" s="19"/>
       <c r="J29" s="19"/>
       <c r="K29" s="19"/>
       <c r="L29" s="23"/>
       <c r="M29" s="23" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="N29" s="24"/>
       <c r="O29" s="23" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="P29" s="23"/>
       <c r="Q29" s="23"/>
@@ -3474,7 +3490,7 @@
     </row>
     <row r="30" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="19" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B30" s="19" t="s">
         <v>30</v>
@@ -3490,20 +3506,20 @@
         <v>101</v>
       </c>
       <c r="F30" s="23" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="G30" s="19" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="H30" s="19" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="I30" s="19"/>
       <c r="J30" s="19"/>
       <c r="K30" s="19"/>
       <c r="L30" s="23"/>
       <c r="M30" s="23" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="N30" s="23"/>
       <c r="O30" s="23" t="s">
@@ -3524,7 +3540,7 @@
     </row>
     <row r="31" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="19" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B31" s="19" t="s">
         <v>30</v>
@@ -3540,24 +3556,24 @@
         <v>101</v>
       </c>
       <c r="F31" s="23" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G31" s="19" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="H31" s="19" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="I31" s="19"/>
       <c r="J31" s="19"/>
       <c r="K31" s="19"/>
       <c r="L31" s="23"/>
       <c r="M31" s="23" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="N31" s="23"/>
       <c r="O31" s="23" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="P31" s="23"/>
       <c r="Q31" s="23"/>
@@ -3574,7 +3590,7 @@
     </row>
     <row r="32" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="19" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B32" s="19" t="s">
         <v>30</v>
@@ -3590,24 +3606,24 @@
         <v>101</v>
       </c>
       <c r="F32" s="23" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="G32" s="19" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H32" s="19" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="I32" s="19"/>
       <c r="J32" s="19"/>
       <c r="K32" s="19"/>
       <c r="L32" s="23"/>
       <c r="M32" s="23" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="N32" s="23"/>
       <c r="O32" s="23" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="P32" s="23"/>
       <c r="Q32" s="23"/>
@@ -3624,7 +3640,7 @@
     </row>
     <row r="33" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="19" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B33" s="19" t="s">
         <v>25</v>
@@ -3640,20 +3656,20 @@
         <v>101</v>
       </c>
       <c r="F33" s="23" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="G33" s="19" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H33" s="19" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I33" s="19"/>
       <c r="J33" s="19"/>
       <c r="K33" s="19"/>
       <c r="L33" s="23"/>
       <c r="M33" s="19" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="N33" s="23"/>
       <c r="O33" s="23"/>
@@ -3672,9 +3688,9 @@
     </row>
     <row r="34" customFormat="false" ht="85.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="19" t="s">
-        <v>181</v>
-      </c>
-      <c r="B34" s="28" t="s">
+        <v>182</v>
+      </c>
+      <c r="B34" s="29" t="s">
         <v>69</v>
       </c>
       <c r="C34" s="21" t="b">
@@ -3688,24 +3704,24 @@
         <v>101</v>
       </c>
       <c r="F34" s="23" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="G34" s="19" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="H34" s="19" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="I34" s="19" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="J34" s="19" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="K34" s="19"/>
       <c r="L34" s="23"/>
       <c r="M34" s="19" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="N34" s="23"/>
       <c r="O34" s="23"/>
@@ -3724,7 +3740,7 @@
     </row>
     <row r="35" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="19" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B35" s="19" t="s">
         <v>25</v>
@@ -3740,20 +3756,20 @@
         <v>101</v>
       </c>
       <c r="F35" s="23" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="G35" s="19" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="H35" s="19" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="I35" s="19"/>
       <c r="J35" s="19"/>
       <c r="K35" s="19"/>
       <c r="L35" s="23"/>
       <c r="M35" s="19" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="N35" s="23"/>
       <c r="O35" s="23"/>
@@ -3772,9 +3788,9 @@
     </row>
     <row r="36" customFormat="false" ht="85.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="19" t="s">
-        <v>192</v>
-      </c>
-      <c r="B36" s="28" t="s">
+        <v>193</v>
+      </c>
+      <c r="B36" s="29" t="s">
         <v>69</v>
       </c>
       <c r="C36" s="21" t="b">
@@ -3788,27 +3804,27 @@
         <v>101</v>
       </c>
       <c r="F36" s="23" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="G36" s="19" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="H36" s="19" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I36" s="19" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="J36" s="19" t="s">
-        <v>197</v>
-      </c>
-      <c r="K36" s="29"/>
-      <c r="L36" s="30"/>
-      <c r="M36" s="29"/>
-      <c r="N36" s="30"/>
-      <c r="O36" s="30"/>
-      <c r="P36" s="30"/>
-      <c r="Q36" s="30"/>
+        <v>198</v>
+      </c>
+      <c r="K36" s="30"/>
+      <c r="L36" s="31"/>
+      <c r="M36" s="30"/>
+      <c r="N36" s="31"/>
+      <c r="O36" s="31"/>
+      <c r="P36" s="31"/>
+      <c r="Q36" s="31"/>
       <c r="R36" s="23"/>
       <c r="S36" s="23"/>
       <c r="T36" s="21" t="b">
@@ -3821,11 +3837,11 @@
       <c r="X36" s="23"/>
     </row>
     <row r="37" customFormat="false" ht="86.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="27" t="s">
-        <v>198</v>
+      <c r="A37" s="25" t="s">
+        <v>199</v>
       </c>
       <c r="B37" s="19" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C37" s="21" t="b">
         <f aca="false">FALSE()</f>
@@ -3838,13 +3854,13 @@
         <v>101</v>
       </c>
       <c r="F37" s="23" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="G37" s="19" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="H37" s="19" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="I37" s="19"/>
       <c r="J37" s="19"/>
@@ -3852,14 +3868,14 @@
       <c r="L37" s="23"/>
       <c r="M37" s="24"/>
       <c r="N37" s="24"/>
-      <c r="O37" s="31" t="s">
-        <v>147</v>
+      <c r="O37" s="32" t="s">
+        <v>148</v>
       </c>
       <c r="P37" s="23"/>
       <c r="Q37" s="23"/>
       <c r="R37" s="23"/>
       <c r="S37" s="23"/>
-      <c r="T37" s="21" t="b">
+      <c r="T37" s="19" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -3869,11 +3885,11 @@
       <c r="X37" s="23"/>
     </row>
     <row r="38" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="27" t="s">
-        <v>202</v>
+      <c r="A38" s="25" t="s">
+        <v>203</v>
       </c>
       <c r="B38" s="19" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C38" s="21" t="b">
         <f aca="false">FALSE()</f>
@@ -3886,13 +3902,13 @@
         <v>101</v>
       </c>
       <c r="F38" s="23" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="G38" s="19" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="H38" s="19" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="I38" s="19"/>
       <c r="J38" s="19"/>
@@ -3900,8 +3916,8 @@
       <c r="L38" s="23"/>
       <c r="M38" s="24"/>
       <c r="N38" s="24"/>
-      <c r="O38" s="31" t="s">
-        <v>147</v>
+      <c r="O38" s="32" t="s">
+        <v>148</v>
       </c>
       <c r="P38" s="23"/>
       <c r="Q38" s="23"/>
@@ -3917,11 +3933,11 @@
       <c r="X38" s="23"/>
     </row>
     <row r="39" customFormat="false" ht="64.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="27" t="s">
-        <v>206</v>
+      <c r="A39" s="25" t="s">
+        <v>207</v>
       </c>
       <c r="B39" s="19" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C39" s="21" t="b">
         <f aca="false">FALSE()</f>
@@ -3934,13 +3950,13 @@
         <v>101</v>
       </c>
       <c r="F39" s="23" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="G39" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H39" s="19" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="I39" s="19"/>
       <c r="J39" s="19"/>
@@ -3948,8 +3964,8 @@
       <c r="L39" s="23"/>
       <c r="M39" s="24"/>
       <c r="N39" s="24"/>
-      <c r="O39" s="31" t="s">
-        <v>147</v>
+      <c r="O39" s="32" t="s">
+        <v>148</v>
       </c>
       <c r="P39" s="23"/>
       <c r="Q39" s="23"/>
@@ -3965,11 +3981,11 @@
       <c r="X39" s="23"/>
     </row>
     <row r="40" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="27" t="s">
-        <v>210</v>
+      <c r="A40" s="25" t="s">
+        <v>211</v>
       </c>
       <c r="B40" s="19" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C40" s="21" t="b">
         <f aca="false">FALSE()</f>
@@ -3982,13 +3998,13 @@
         <v>101</v>
       </c>
       <c r="F40" s="23" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="G40" s="19" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="H40" s="19" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="I40" s="19"/>
       <c r="J40" s="19"/>
@@ -3996,8 +4012,8 @@
       <c r="L40" s="23"/>
       <c r="M40" s="24"/>
       <c r="N40" s="24"/>
-      <c r="O40" s="31" t="s">
-        <v>147</v>
+      <c r="O40" s="32" t="s">
+        <v>148</v>
       </c>
       <c r="P40" s="23"/>
       <c r="Q40" s="23"/>
@@ -4013,76 +4029,76 @@
       <c r="X40" s="23"/>
     </row>
     <row r="41" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="32" t="s">
-        <v>214</v>
-      </c>
-      <c r="B41" s="32" t="s">
+      <c r="A41" s="33" t="s">
+        <v>215</v>
+      </c>
+      <c r="B41" s="33" t="s">
         <v>98</v>
       </c>
-      <c r="C41" s="33" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D41" s="32" t="s">
+      <c r="C41" s="34" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D41" s="33" t="s">
         <v>102</v>
       </c>
-      <c r="E41" s="34"/>
-      <c r="F41" s="34" t="str">
+      <c r="E41" s="35"/>
+      <c r="F41" s="35" t="str">
         <f aca="false">REPLACE(A41, FIND("_", A41), 1, ".")</f>
         <v>household.save</v>
       </c>
-      <c r="G41" s="32" t="s">
+      <c r="G41" s="33" t="s">
         <v>99</v>
       </c>
-      <c r="H41" s="32" t="s">
+      <c r="H41" s="33" t="s">
         <v>100</v>
       </c>
-      <c r="I41" s="32"/>
-      <c r="J41" s="32"/>
-      <c r="K41" s="32"/>
-      <c r="L41" s="34"/>
-      <c r="M41" s="34"/>
-      <c r="N41" s="34"/>
-      <c r="O41" s="34"/>
-      <c r="P41" s="34"/>
-      <c r="Q41" s="34"/>
-      <c r="R41" s="34"/>
-      <c r="S41" s="34"/>
-      <c r="T41" s="33" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U41" s="34"/>
-      <c r="V41" s="34"/>
-      <c r="W41" s="34"/>
-      <c r="X41" s="34"/>
+      <c r="I41" s="33"/>
+      <c r="J41" s="33"/>
+      <c r="K41" s="33"/>
+      <c r="L41" s="35"/>
+      <c r="M41" s="35"/>
+      <c r="N41" s="35"/>
+      <c r="O41" s="35"/>
+      <c r="P41" s="35"/>
+      <c r="Q41" s="35"/>
+      <c r="R41" s="35"/>
+      <c r="S41" s="35"/>
+      <c r="T41" s="34" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U41" s="35"/>
+      <c r="V41" s="35"/>
+      <c r="W41" s="35"/>
+      <c r="X41" s="35"/>
     </row>
     <row r="42" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C42" s="35" t="b">
+      <c r="C42" s="36" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="D42" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="F42" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="F42" s="1" t="s">
-        <v>215</v>
-      </c>
       <c r="G42" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>218</v>
-      </c>
-      <c r="L42" s="36"/>
-      <c r="M42" s="37"/>
-      <c r="T42" s="35" t="b">
+        <v>219</v>
+      </c>
+      <c r="L42" s="37"/>
+      <c r="M42" s="38"/>
+      <c r="T42" s="36" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -4139,486 +4155,486 @@
   <dimension ref="A1:F29"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="38" width="27.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="38" width="15.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="38" width="31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="39" width="20.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="38" width="19.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="38" width="12.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="39" width="27.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="39" width="15.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="39" width="31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="40" width="20.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="39" width="19.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="39" width="12.14"/>
   </cols>
   <sheetData>
-    <row r="1" s="42" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="40" t="s">
-        <v>219</v>
-      </c>
-      <c r="B1" s="40" t="s">
+    <row r="1" s="43" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="41" t="s">
         <v>220</v>
       </c>
-      <c r="C1" s="40" t="s">
+      <c r="B1" s="41" t="s">
+        <v>221</v>
+      </c>
+      <c r="C1" s="41" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="41" t="s">
-        <v>221</v>
-      </c>
-      <c r="E1" s="40" t="s">
+      <c r="D1" s="42" t="s">
         <v>222</v>
       </c>
-      <c r="F1" s="40" t="s">
+      <c r="E1" s="41" t="s">
         <v>223</v>
       </c>
+      <c r="F1" s="41" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="43" t="s">
-        <v>224</v>
-      </c>
-      <c r="B2" s="43"/>
-      <c r="C2" s="43" t="s">
+      <c r="A2" s="44" t="s">
         <v>225</v>
       </c>
-      <c r="D2" s="44" t="s">
+      <c r="B2" s="44"/>
+      <c r="C2" s="44" t="s">
         <v>226</v>
       </c>
-      <c r="E2" s="43" t="n">
-        <v>1</v>
-      </c>
-      <c r="F2" s="43"/>
+      <c r="D2" s="45" t="s">
+        <v>227</v>
+      </c>
+      <c r="E2" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="44"/>
     </row>
     <row r="3" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="43" t="s">
+      <c r="A3" s="44" t="s">
         <v>95</v>
       </c>
-      <c r="B3" s="43"/>
-      <c r="C3" s="43" t="s">
-        <v>225</v>
-      </c>
-      <c r="D3" s="44" t="s">
+      <c r="B3" s="44"/>
+      <c r="C3" s="44" t="s">
+        <v>226</v>
+      </c>
+      <c r="D3" s="45" t="s">
+        <v>228</v>
+      </c>
+      <c r="E3" s="44" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" s="44"/>
+    </row>
+    <row r="4" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="44" t="s">
+        <v>165</v>
+      </c>
+      <c r="B4" s="44"/>
+      <c r="C4" s="44" t="s">
+        <v>229</v>
+      </c>
+      <c r="D4" s="45" t="s">
         <v>227</v>
       </c>
-      <c r="E3" s="43" t="n">
-        <v>2</v>
-      </c>
-      <c r="F3" s="43"/>
-    </row>
-    <row r="4" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="43" t="s">
-        <v>164</v>
-      </c>
-      <c r="B4" s="43"/>
-      <c r="C4" s="43" t="s">
+      <c r="E4" s="44" t="s">
+        <v>230</v>
+      </c>
+      <c r="F4" s="44"/>
+    </row>
+    <row r="5" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="44" t="s">
+        <v>165</v>
+      </c>
+      <c r="B5" s="44" t="s">
+        <v>231</v>
+      </c>
+      <c r="C5" s="44" t="s">
+        <v>226</v>
+      </c>
+      <c r="D5" s="45" t="s">
+        <v>227</v>
+      </c>
+      <c r="E5" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="44"/>
+    </row>
+    <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="44" t="s">
+        <v>232</v>
+      </c>
+      <c r="B6" s="44"/>
+      <c r="C6" s="44" t="s">
+        <v>233</v>
+      </c>
+      <c r="D6" s="45" t="s">
         <v>228</v>
       </c>
-      <c r="D4" s="44" t="s">
-        <v>226</v>
-      </c>
-      <c r="E4" s="43" t="s">
-        <v>229</v>
-      </c>
-      <c r="F4" s="43"/>
-    </row>
-    <row r="5" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="43" t="s">
-        <v>164</v>
-      </c>
-      <c r="B5" s="43" t="s">
+      <c r="E6" s="44" t="n">
+        <v>3</v>
+      </c>
+      <c r="F6" s="44"/>
+    </row>
+    <row r="7" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="44" t="s">
+        <v>232</v>
+      </c>
+      <c r="B7" s="44" t="s">
+        <v>234</v>
+      </c>
+      <c r="C7" s="44" t="s">
+        <v>233</v>
+      </c>
+      <c r="D7" s="45" t="s">
+        <v>235</v>
+      </c>
+      <c r="E7" s="44" t="n">
+        <v>5</v>
+      </c>
+      <c r="F7" s="44"/>
+    </row>
+    <row r="8" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="44" t="s">
+        <v>236</v>
+      </c>
+      <c r="B8" s="44"/>
+      <c r="C8" s="44" t="s">
+        <v>233</v>
+      </c>
+      <c r="D8" s="45" t="s">
+        <v>228</v>
+      </c>
+      <c r="E8" s="44" t="n">
+        <v>4</v>
+      </c>
+      <c r="F8" s="44"/>
+    </row>
+    <row r="9" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="44" t="s">
+        <v>236</v>
+      </c>
+      <c r="B9" s="44" t="s">
+        <v>234</v>
+      </c>
+      <c r="C9" s="44" t="s">
+        <v>233</v>
+      </c>
+      <c r="D9" s="45" t="s">
+        <v>235</v>
+      </c>
+      <c r="E9" s="44" t="n">
+        <v>13</v>
+      </c>
+      <c r="F9" s="44"/>
+    </row>
+    <row r="10" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="44" t="s">
+        <v>237</v>
+      </c>
+      <c r="B10" s="44"/>
+      <c r="C10" s="44" t="s">
+        <v>233</v>
+      </c>
+      <c r="D10" s="45" t="s">
+        <v>235</v>
+      </c>
+      <c r="E10" s="44" t="n">
+        <v>5</v>
+      </c>
+      <c r="F10" s="44"/>
+    </row>
+    <row r="11" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="44" t="s">
+        <v>119</v>
+      </c>
+      <c r="B11" s="44"/>
+      <c r="C11" s="44" t="s">
+        <v>233</v>
+      </c>
+      <c r="D11" s="45" t="s">
+        <v>228</v>
+      </c>
+      <c r="E11" s="44" t="n">
+        <v>5</v>
+      </c>
+      <c r="F11" s="44"/>
+    </row>
+    <row r="12" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="44" t="s">
+        <v>159</v>
+      </c>
+      <c r="B12" s="44"/>
+      <c r="C12" s="44" t="s">
+        <v>233</v>
+      </c>
+      <c r="D12" s="45" t="s">
+        <v>228</v>
+      </c>
+      <c r="E12" s="44" t="n">
+        <v>6</v>
+      </c>
+      <c r="F12" s="44"/>
+    </row>
+    <row r="13" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="44" t="s">
+        <v>238</v>
+      </c>
+      <c r="B13" s="44"/>
+      <c r="C13" s="44" t="s">
+        <v>233</v>
+      </c>
+      <c r="D13" s="45" t="s">
+        <v>228</v>
+      </c>
+      <c r="E13" s="44" t="n">
+        <v>11</v>
+      </c>
+      <c r="F13" s="44"/>
+    </row>
+    <row r="14" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="44" t="s">
+        <v>124</v>
+      </c>
+      <c r="B14" s="44"/>
+      <c r="C14" s="44" t="s">
+        <v>233</v>
+      </c>
+      <c r="D14" s="45" t="s">
+        <v>228</v>
+      </c>
+      <c r="E14" s="44" t="n">
+        <v>14</v>
+      </c>
+      <c r="F14" s="44"/>
+    </row>
+    <row r="15" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="44" t="s">
+        <v>136</v>
+      </c>
+      <c r="B15" s="44"/>
+      <c r="C15" s="44" t="s">
+        <v>233</v>
+      </c>
+      <c r="D15" s="45" t="s">
+        <v>235</v>
+      </c>
+      <c r="E15" s="44" t="n">
+        <v>15</v>
+      </c>
+      <c r="F15" s="44"/>
+    </row>
+    <row r="16" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="44" t="s">
+        <v>136</v>
+      </c>
+      <c r="B16" s="44"/>
+      <c r="C16" s="44" t="s">
+        <v>233</v>
+      </c>
+      <c r="D16" s="45" t="s">
+        <v>239</v>
+      </c>
+      <c r="E16" s="44" t="s">
+        <v>240</v>
+      </c>
+      <c r="F16" s="44"/>
+    </row>
+    <row r="17" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="44" t="s">
+        <v>241</v>
+      </c>
+      <c r="B17" s="44"/>
+      <c r="C17" s="44" t="s">
+        <v>233</v>
+      </c>
+      <c r="D17" s="45" t="s">
+        <v>228</v>
+      </c>
+      <c r="E17" s="44" t="n">
+        <v>15</v>
+      </c>
+      <c r="F17" s="44"/>
+    </row>
+    <row r="18" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="44" t="s">
+        <v>130</v>
+      </c>
+      <c r="B18" s="44"/>
+      <c r="C18" s="44" t="s">
+        <v>233</v>
+      </c>
+      <c r="D18" s="45" t="s">
+        <v>228</v>
+      </c>
+      <c r="E18" s="44" t="n">
+        <v>16</v>
+      </c>
+      <c r="F18" s="44"/>
+    </row>
+    <row r="19" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="44" t="s">
+        <v>242</v>
+      </c>
+      <c r="B19" s="44"/>
+      <c r="C19" s="44" t="s">
+        <v>233</v>
+      </c>
+      <c r="D19" s="45" t="s">
+        <v>228</v>
+      </c>
+      <c r="E19" s="44" t="n">
+        <v>40</v>
+      </c>
+      <c r="F19" s="44"/>
+    </row>
+    <row r="20" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="44" t="s">
+        <v>153</v>
+      </c>
+      <c r="B20" s="44"/>
+      <c r="C20" s="44" t="s">
+        <v>243</v>
+      </c>
+      <c r="D20" s="45" t="s">
+        <v>227</v>
+      </c>
+      <c r="E20" s="44" t="s">
         <v>230</v>
       </c>
-      <c r="C5" s="43" t="s">
-        <v>225</v>
-      </c>
-      <c r="D5" s="44" t="s">
-        <v>226</v>
-      </c>
-      <c r="E5" s="43" t="n">
-        <v>1</v>
-      </c>
-      <c r="F5" s="43"/>
-    </row>
-    <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="43" t="s">
+      <c r="F20" s="44"/>
+    </row>
+    <row r="21" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="39" t="s">
+        <v>170</v>
+      </c>
+      <c r="C21" s="39" t="s">
+        <v>244</v>
+      </c>
+      <c r="D21" s="45" t="s">
+        <v>227</v>
+      </c>
+      <c r="E21" s="40" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="39" t="s">
+        <v>170</v>
+      </c>
+      <c r="B22" s="39" t="s">
         <v>231</v>
       </c>
-      <c r="B6" s="43"/>
-      <c r="C6" s="43" t="s">
-        <v>232</v>
-      </c>
-      <c r="D6" s="44" t="s">
+      <c r="C22" s="39" t="s">
+        <v>244</v>
+      </c>
+      <c r="D22" s="45" t="s">
         <v>227</v>
       </c>
-      <c r="E6" s="43" t="n">
-        <v>3</v>
-      </c>
-      <c r="F6" s="43"/>
-    </row>
-    <row r="7" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="43" t="s">
+      <c r="E22" s="40" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="39" t="s">
+        <v>170</v>
+      </c>
+      <c r="B23" s="39" t="s">
         <v>231</v>
       </c>
-      <c r="B7" s="43" t="s">
-        <v>233</v>
-      </c>
-      <c r="C7" s="43" t="s">
-        <v>232</v>
-      </c>
-      <c r="D7" s="44" t="s">
-        <v>234</v>
-      </c>
-      <c r="E7" s="43" t="n">
-        <v>5</v>
-      </c>
-      <c r="F7" s="43"/>
-    </row>
-    <row r="8" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="43" t="s">
-        <v>235</v>
-      </c>
-      <c r="B8" s="43"/>
-      <c r="C8" s="43" t="s">
-        <v>232</v>
-      </c>
-      <c r="D8" s="44" t="s">
+      <c r="C23" s="39" t="s">
+        <v>244</v>
+      </c>
+      <c r="D23" s="45" t="s">
         <v>227</v>
       </c>
-      <c r="E8" s="43" t="n">
-        <v>4</v>
-      </c>
-      <c r="F8" s="43"/>
-    </row>
-    <row r="9" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="43" t="s">
-        <v>235</v>
-      </c>
-      <c r="B9" s="43" t="s">
-        <v>233</v>
-      </c>
-      <c r="C9" s="43" t="s">
-        <v>232</v>
-      </c>
-      <c r="D9" s="44" t="s">
-        <v>234</v>
-      </c>
-      <c r="E9" s="43" t="n">
-        <v>13</v>
-      </c>
-      <c r="F9" s="43"/>
-    </row>
-    <row r="10" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="43" t="s">
-        <v>236</v>
-      </c>
-      <c r="B10" s="43"/>
-      <c r="C10" s="43" t="s">
-        <v>232</v>
-      </c>
-      <c r="D10" s="44" t="s">
-        <v>234</v>
-      </c>
-      <c r="E10" s="43" t="n">
-        <v>5</v>
-      </c>
-      <c r="F10" s="43"/>
-    </row>
-    <row r="11" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="43" t="s">
-        <v>119</v>
-      </c>
-      <c r="B11" s="43"/>
-      <c r="C11" s="43" t="s">
-        <v>232</v>
-      </c>
-      <c r="D11" s="44" t="s">
+      <c r="E23" s="40" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="39" t="s">
+        <v>175</v>
+      </c>
+      <c r="C24" s="39" t="s">
+        <v>244</v>
+      </c>
+      <c r="D24" s="45" t="s">
         <v>227</v>
       </c>
-      <c r="E11" s="43" t="n">
-        <v>5</v>
-      </c>
-      <c r="F11" s="43"/>
-    </row>
-    <row r="12" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="43" t="s">
-        <v>158</v>
-      </c>
-      <c r="B12" s="43"/>
-      <c r="C12" s="43" t="s">
-        <v>232</v>
-      </c>
-      <c r="D12" s="44" t="s">
+      <c r="E24" s="40" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="39" t="s">
+        <v>175</v>
+      </c>
+      <c r="B25" s="39" t="s">
+        <v>231</v>
+      </c>
+      <c r="C25" s="39" t="s">
+        <v>244</v>
+      </c>
+      <c r="D25" s="45" t="s">
         <v>227</v>
       </c>
-      <c r="E12" s="43" t="n">
-        <v>6</v>
-      </c>
-      <c r="F12" s="43"/>
-    </row>
-    <row r="13" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="43" t="s">
-        <v>237</v>
-      </c>
-      <c r="B13" s="43"/>
-      <c r="C13" s="43" t="s">
-        <v>232</v>
-      </c>
-      <c r="D13" s="44" t="s">
+      <c r="E25" s="40" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="39" t="s">
+        <v>175</v>
+      </c>
+      <c r="B26" s="39" t="s">
+        <v>231</v>
+      </c>
+      <c r="C26" s="39" t="s">
+        <v>244</v>
+      </c>
+      <c r="D26" s="45" t="s">
         <v>227</v>
       </c>
-      <c r="E13" s="43" t="n">
-        <v>11</v>
-      </c>
-      <c r="F13" s="43"/>
-    </row>
-    <row r="14" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="43" t="s">
-        <v>124</v>
-      </c>
-      <c r="B14" s="43"/>
-      <c r="C14" s="43" t="s">
-        <v>232</v>
-      </c>
-      <c r="D14" s="44" t="s">
+      <c r="E26" s="40" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="39" t="s">
+        <v>181</v>
+      </c>
+      <c r="C27" s="39" t="s">
+        <v>250</v>
+      </c>
+      <c r="D27" s="45" t="s">
         <v>227</v>
       </c>
-      <c r="E14" s="43" t="n">
-        <v>14</v>
-      </c>
-      <c r="F14" s="43"/>
-    </row>
-    <row r="15" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="43" t="s">
-        <v>135</v>
-      </c>
-      <c r="B15" s="43"/>
-      <c r="C15" s="43" t="s">
-        <v>232</v>
-      </c>
-      <c r="D15" s="44" t="s">
-        <v>234</v>
-      </c>
-      <c r="E15" s="43" t="n">
-        <v>15</v>
-      </c>
-      <c r="F15" s="43"/>
-    </row>
-    <row r="16" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="43" t="s">
-        <v>135</v>
-      </c>
-      <c r="B16" s="43"/>
-      <c r="C16" s="43" t="s">
-        <v>232</v>
-      </c>
-      <c r="D16" s="44" t="s">
-        <v>238</v>
-      </c>
-      <c r="E16" s="43" t="s">
-        <v>239</v>
-      </c>
-      <c r="F16" s="43"/>
-    </row>
-    <row r="17" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="43" t="s">
-        <v>240</v>
-      </c>
-      <c r="B17" s="43"/>
-      <c r="C17" s="43" t="s">
-        <v>232</v>
-      </c>
-      <c r="D17" s="44" t="s">
+      <c r="E27" s="39" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="39" t="s">
+        <v>181</v>
+      </c>
+      <c r="B28" s="39" t="s">
+        <v>231</v>
+      </c>
+      <c r="C28" s="39" t="s">
+        <v>250</v>
+      </c>
+      <c r="D28" s="45" t="s">
         <v>227</v>
       </c>
-      <c r="E17" s="43" t="n">
-        <v>15</v>
-      </c>
-      <c r="F17" s="43"/>
-    </row>
-    <row r="18" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="43" t="s">
-        <v>130</v>
-      </c>
-      <c r="B18" s="43"/>
-      <c r="C18" s="43" t="s">
-        <v>232</v>
-      </c>
-      <c r="D18" s="44" t="s">
+      <c r="E28" s="39" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="39" t="s">
+        <v>181</v>
+      </c>
+      <c r="B29" s="39" t="s">
+        <v>231</v>
+      </c>
+      <c r="C29" s="39" t="s">
+        <v>250</v>
+      </c>
+      <c r="D29" s="45" t="s">
         <v>227</v>
       </c>
-      <c r="E18" s="43" t="n">
-        <v>16</v>
-      </c>
-      <c r="F18" s="43"/>
-    </row>
-    <row r="19" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="43" t="s">
-        <v>241</v>
-      </c>
-      <c r="B19" s="43"/>
-      <c r="C19" s="43" t="s">
-        <v>232</v>
-      </c>
-      <c r="D19" s="44" t="s">
-        <v>227</v>
-      </c>
-      <c r="E19" s="43" t="n">
-        <v>40</v>
-      </c>
-      <c r="F19" s="43"/>
-    </row>
-    <row r="20" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="43" t="s">
-        <v>152</v>
-      </c>
-      <c r="B20" s="43"/>
-      <c r="C20" s="43" t="s">
-        <v>242</v>
-      </c>
-      <c r="D20" s="44" t="s">
-        <v>226</v>
-      </c>
-      <c r="E20" s="43" t="s">
-        <v>229</v>
-      </c>
-      <c r="F20" s="43"/>
-    </row>
-    <row r="21" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="38" t="s">
-        <v>169</v>
-      </c>
-      <c r="C21" s="38" t="s">
-        <v>243</v>
-      </c>
-      <c r="D21" s="44" t="s">
-        <v>226</v>
-      </c>
-      <c r="E21" s="39" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="38" t="s">
-        <v>169</v>
-      </c>
-      <c r="B22" s="38" t="s">
-        <v>230</v>
-      </c>
-      <c r="C22" s="38" t="s">
-        <v>243</v>
-      </c>
-      <c r="D22" s="44" t="s">
-        <v>226</v>
-      </c>
-      <c r="E22" s="39" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="38" t="s">
-        <v>169</v>
-      </c>
-      <c r="B23" s="38" t="s">
-        <v>230</v>
-      </c>
-      <c r="C23" s="38" t="s">
-        <v>243</v>
-      </c>
-      <c r="D23" s="44" t="s">
-        <v>226</v>
-      </c>
-      <c r="E23" s="39" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="38" t="s">
-        <v>174</v>
-      </c>
-      <c r="C24" s="38" t="s">
-        <v>243</v>
-      </c>
-      <c r="D24" s="44" t="s">
-        <v>226</v>
-      </c>
-      <c r="E24" s="39" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="38" t="s">
-        <v>174</v>
-      </c>
-      <c r="B25" s="38" t="s">
-        <v>230</v>
-      </c>
-      <c r="C25" s="38" t="s">
-        <v>243</v>
-      </c>
-      <c r="D25" s="44" t="s">
-        <v>226</v>
-      </c>
-      <c r="E25" s="39" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="38" t="s">
-        <v>174</v>
-      </c>
-      <c r="B26" s="38" t="s">
-        <v>230</v>
-      </c>
-      <c r="C26" s="38" t="s">
-        <v>243</v>
-      </c>
-      <c r="D26" s="44" t="s">
-        <v>226</v>
-      </c>
-      <c r="E26" s="39" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="38" t="s">
-        <v>180</v>
-      </c>
-      <c r="C27" s="38" t="s">
-        <v>249</v>
-      </c>
-      <c r="D27" s="44" t="s">
-        <v>226</v>
-      </c>
-      <c r="E27" s="38" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="38" t="s">
-        <v>180</v>
-      </c>
-      <c r="B28" s="38" t="s">
-        <v>230</v>
-      </c>
-      <c r="C28" s="38" t="s">
-        <v>249</v>
-      </c>
-      <c r="D28" s="44" t="s">
-        <v>226</v>
-      </c>
-      <c r="E28" s="38" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="38" t="s">
-        <v>180</v>
-      </c>
-      <c r="B29" s="38" t="s">
-        <v>230</v>
-      </c>
-      <c r="C29" s="38" t="s">
-        <v>249</v>
-      </c>
-      <c r="D29" s="44" t="s">
-        <v>226</v>
-      </c>
-      <c r="E29" s="38" t="s">
-        <v>252</v>
+      <c r="E29" s="39" t="s">
+        <v>253</v>
       </c>
     </row>
   </sheetData>
@@ -4638,118 +4654,118 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H4"/>
-  <sheetFormatPr defaultColWidth="10.70703125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.69921875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="43" width="10.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="43" width="12.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="43" width="13.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="43" width="12.57"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="6" min="5" style="43" width="10.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="43" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="43" width="15.43"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="9" style="43" width="10.7"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="44" width="10.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="44" width="12.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="44" width="13.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="44" width="12.57"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="6" min="5" style="44" width="10.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="44" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="44" width="15.43"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="9" style="44" width="10.7"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="46" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="46" t="s">
-        <v>253</v>
-      </c>
-      <c r="C1" s="45" t="s">
+      <c r="B1" s="47" t="s">
         <v>254</v>
       </c>
-      <c r="D1" s="45" t="s">
+      <c r="C1" s="46" t="s">
         <v>255</v>
       </c>
-      <c r="E1" s="45" t="s">
+      <c r="D1" s="46" t="s">
         <v>256</v>
       </c>
-      <c r="F1" s="45" t="s">
+      <c r="E1" s="46" t="s">
         <v>257</v>
       </c>
+      <c r="F1" s="46" t="s">
+        <v>258</v>
+      </c>
       <c r="G1" s="6" t="s">
-        <v>258</v>
-      </c>
-      <c r="H1" s="45" t="s">
         <v>259</v>
       </c>
+      <c r="H1" s="46" t="s">
+        <v>260</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="43" t="s">
+      <c r="A2" s="44" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="43" t="s">
-        <v>260</v>
-      </c>
-      <c r="C2" s="43" t="s">
+      <c r="B2" s="44" t="s">
         <v>261</v>
       </c>
-      <c r="D2" s="43" t="s">
+      <c r="C2" s="44" t="s">
         <v>262</v>
       </c>
-      <c r="E2" s="47" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="F2" s="47" t="b">
+      <c r="D2" s="44" t="s">
+        <v>263</v>
+      </c>
+      <c r="E2" s="48" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="F2" s="48" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="G2" s="47" t="b">
+      <c r="G2" s="48" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="43" t="s">
+      <c r="A3" s="44" t="s">
         <v>102</v>
       </c>
-      <c r="B3" s="43" t="s">
-        <v>263</v>
-      </c>
-      <c r="C3" s="43" t="s">
+      <c r="B3" s="44" t="s">
         <v>264</v>
       </c>
-      <c r="D3" s="43" t="s">
+      <c r="C3" s="44" t="s">
         <v>265</v>
       </c>
-      <c r="E3" s="47" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="F3" s="47" t="b">
+      <c r="D3" s="44" t="s">
+        <v>266</v>
+      </c>
+      <c r="E3" s="48" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="F3" s="48" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="G3" s="47" t="b">
+      <c r="G3" s="48" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="43" t="s">
-        <v>216</v>
-      </c>
-      <c r="B4" s="43" t="s">
-        <v>266</v>
-      </c>
-      <c r="C4" s="43" t="s">
+      <c r="A4" s="44" t="s">
+        <v>217</v>
+      </c>
+      <c r="B4" s="44" t="s">
         <v>267</v>
       </c>
-      <c r="D4" s="43" t="s">
+      <c r="C4" s="44" t="s">
         <v>268</v>
       </c>
-      <c r="E4" s="47" t="b">
+      <c r="D4" s="44" t="s">
+        <v>269</v>
+      </c>
+      <c r="E4" s="48" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="F4" s="47" t="b">
+      <c r="F4" s="48" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="G4" s="47" t="b">
+      <c r="G4" s="48" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -4773,126 +4789,126 @@
   <dimension ref="A1:F51"/>
   <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="48" width="21.3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="48" width="15.72"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="48" width="23.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="48" width="19.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="48" width="24.29"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="7" style="48" width="9.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="49" width="21.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="49" width="15.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="49" width="23.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="49" width="19.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="49" width="24.29"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="7" style="49" width="9.14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="49" t="s">
-        <v>269</v>
-      </c>
-      <c r="B1" s="49" t="s">
-        <v>222</v>
-      </c>
-      <c r="C1" s="49" t="s">
+      <c r="A1" s="50" t="s">
+        <v>270</v>
+      </c>
+      <c r="B1" s="50" t="s">
+        <v>223</v>
+      </c>
+      <c r="C1" s="50" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="49" t="s">
+      <c r="D1" s="50" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="49" t="s">
-        <v>270</v>
-      </c>
-      <c r="F1" s="49" t="s">
+      <c r="E1" s="50" t="s">
+        <v>271</v>
+      </c>
+      <c r="F1" s="50" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
     </row>
     <row r="4" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
     </row>
     <row r="5" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
     </row>
     <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
     </row>
     <row r="7" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
@@ -4905,7 +4921,7 @@
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
       <c r="E8" s="1" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="F8" s="1"/>
     </row>
@@ -4917,13 +4933,13 @@
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
       <c r="E9" s="1" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F9" s="1"/>
     </row>
     <row r="10" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
@@ -4935,13 +4951,13 @@
     </row>
     <row r="11" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
       <c r="E11" s="1" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="F11" s="1"/>
     </row>
@@ -4953,7 +4969,7 @@
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
       <c r="E12" s="1" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="F12" s="1"/>
     </row>
@@ -4965,7 +4981,7 @@
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
       <c r="E13" s="1" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F13" s="1"/>
     </row>
@@ -4977,7 +4993,7 @@
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
       <c r="E14" s="1" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="F14" s="1"/>
     </row>
@@ -4986,13 +5002,13 @@
         <v>116</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
@@ -5002,13 +5018,13 @@
         <v>116</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
@@ -5021,7 +5037,7 @@
       <c r="C17" s="1"/>
       <c r="D17" s="1"/>
       <c r="E17" s="1" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="F17" s="1"/>
     </row>
@@ -5030,13 +5046,13 @@
         <v>125</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
@@ -5046,13 +5062,13 @@
         <v>125</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E19" s="1"/>
       <c r="F19" s="1"/>
@@ -5065,7 +5081,7 @@
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
       <c r="E20" s="1" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F20" s="1"/>
     </row>
@@ -5074,17 +5090,17 @@
         <v>132</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="E21" s="1"/>
       <c r="F21" s="1" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5092,17 +5108,17 @@
         <v>132</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="E22" s="1"/>
       <c r="F22" s="1" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5110,17 +5126,17 @@
         <v>132</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="E23" s="1"/>
       <c r="F23" s="1" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5128,13 +5144,13 @@
         <v>132</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E24" s="1"/>
       <c r="F24" s="1"/>
@@ -5144,17 +5160,17 @@
         <v>132</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E25" s="1"/>
       <c r="F25" s="1" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5165,396 +5181,396 @@
       <c r="C26" s="1"/>
       <c r="D26" s="1"/>
       <c r="E26" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F26" s="1"/>
     </row>
     <row r="27" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
     </row>
     <row r="28" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="E28" s="1"/>
       <c r="F28" s="1"/>
     </row>
     <row r="29" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="E29" s="1"/>
       <c r="F29" s="1"/>
     </row>
     <row r="30" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="E30" s="1"/>
       <c r="F30" s="1"/>
     </row>
     <row r="31" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="E31" s="1"/>
       <c r="F31" s="1"/>
     </row>
     <row r="32" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E32" s="1"/>
       <c r="F32" s="1" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="E33" s="1"/>
       <c r="F33" s="1"/>
     </row>
     <row r="34" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="E34" s="1"/>
       <c r="F34" s="1"/>
     </row>
     <row r="35" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="E35" s="1"/>
       <c r="F35" s="1"/>
     </row>
     <row r="36" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="E36" s="1"/>
       <c r="F36" s="1"/>
     </row>
     <row r="37" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="E37" s="1"/>
       <c r="F37" s="1"/>
     </row>
     <row r="38" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="B38" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="B38" s="1" t="s">
-        <v>137</v>
-      </c>
       <c r="C38" s="1" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E38" s="1"/>
       <c r="F38" s="1"/>
     </row>
     <row r="39" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E39" s="1"/>
       <c r="F39" s="1"/>
     </row>
     <row r="40" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B40" s="1"/>
       <c r="C40" s="1"/>
       <c r="D40" s="1"/>
       <c r="E40" s="1" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F40" s="1"/>
     </row>
     <row r="41" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="E41" s="1"/>
       <c r="F41" s="1"/>
     </row>
     <row r="42" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="E42" s="1"/>
       <c r="F42" s="1"/>
     </row>
     <row r="43" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B43" s="1"/>
       <c r="C43" s="1"/>
       <c r="D43" s="1"/>
       <c r="E43" s="1" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="F43" s="1"/>
     </row>
     <row r="44" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E44" s="1"/>
       <c r="F44" s="1"/>
     </row>
     <row r="45" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="E45" s="1"/>
       <c r="F45" s="1"/>
     </row>
     <row r="46" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="E46" s="1"/>
       <c r="F46" s="1"/>
     </row>
     <row r="47" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="E47" s="1"/>
       <c r="F47" s="1"/>
     </row>
     <row r="48" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="E48" s="1"/>
       <c r="F48" s="1"/>
     </row>
     <row r="49" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="48" t="s">
-        <v>175</v>
-      </c>
-      <c r="B49" s="48" t="s">
-        <v>250</v>
-      </c>
-      <c r="C49" s="48" t="s">
-        <v>363</v>
-      </c>
-      <c r="D49" s="48" t="s">
-        <v>352</v>
+      <c r="A49" s="49" t="s">
+        <v>176</v>
+      </c>
+      <c r="B49" s="49" t="s">
+        <v>251</v>
+      </c>
+      <c r="C49" s="49" t="s">
+        <v>364</v>
+      </c>
+      <c r="D49" s="49" t="s">
+        <v>353</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="48" t="s">
-        <v>175</v>
-      </c>
-      <c r="B50" s="48" t="s">
-        <v>251</v>
-      </c>
-      <c r="C50" s="48" t="s">
-        <v>364</v>
-      </c>
-      <c r="D50" s="48" t="s">
+      <c r="A50" s="49" t="s">
+        <v>176</v>
+      </c>
+      <c r="B50" s="49" t="s">
+        <v>252</v>
+      </c>
+      <c r="C50" s="49" t="s">
         <v>365</v>
       </c>
+      <c r="D50" s="49" t="s">
+        <v>366</v>
+      </c>
     </row>
     <row r="51" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="48" t="s">
-        <v>175</v>
-      </c>
-      <c r="B51" s="48" t="s">
-        <v>360</v>
-      </c>
-      <c r="C51" s="48" t="s">
-        <v>366</v>
-      </c>
-      <c r="D51" s="48" t="s">
+      <c r="A51" s="49" t="s">
+        <v>176</v>
+      </c>
+      <c r="B51" s="49" t="s">
+        <v>361</v>
+      </c>
+      <c r="C51" s="49" t="s">
         <v>367</v>
+      </c>
+      <c r="D51" s="49" t="s">
+        <v>368</v>
       </c>
     </row>
   </sheetData>
@@ -5576,54 +5592,54 @@
   <dimension ref="A1:L1"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="38" width="18.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="38" width="17.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="38" width="13.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="38" width="12.72"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="38" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="38" width="13.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="38" width="14.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="38" width="11.28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="38" width="13.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="38" width="14.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="39" width="18.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="39" width="17.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="39" width="13.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="39" width="12.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="39" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="39" width="13.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="39" width="14.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="39" width="11.28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="39" width="13.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="39" width="14.43"/>
   </cols>
   <sheetData>
-    <row r="1" s="49" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="50" t="s">
-        <v>368</v>
-      </c>
-      <c r="B1" s="50" t="s">
+    <row r="1" s="50" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="51" t="s">
         <v>369</v>
       </c>
-      <c r="C1" s="50" t="s">
+      <c r="B1" s="51" t="s">
         <v>370</v>
       </c>
-      <c r="D1" s="50" t="s">
+      <c r="C1" s="51" t="s">
         <v>371</v>
       </c>
-      <c r="E1" s="50" t="s">
+      <c r="D1" s="51" t="s">
         <v>372</v>
       </c>
-      <c r="F1" s="50" t="s">
+      <c r="E1" s="51" t="s">
         <v>373</v>
       </c>
-      <c r="G1" s="50" t="s">
+      <c r="F1" s="51" t="s">
         <v>374</v>
       </c>
-      <c r="H1" s="50" t="s">
+      <c r="G1" s="51" t="s">
         <v>375</v>
       </c>
-      <c r="I1" s="50" t="s">
+      <c r="H1" s="51" t="s">
         <v>376</v>
       </c>
-      <c r="J1" s="50" t="s">
+      <c r="I1" s="51" t="s">
         <v>377</v>
       </c>
-      <c r="K1" s="50" t="s">
+      <c r="J1" s="51" t="s">
         <v>378</v>
       </c>
-      <c r="L1" s="49" t="s">
+      <c r="K1" s="51" t="s">
         <v>379</v>
+      </c>
+      <c r="L1" s="50" t="s">
+        <v>380</v>
       </c>
     </row>
   </sheetData>
@@ -5642,11 +5658,14 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="9.84"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="3" style="0" width="28.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="39" width="32.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="39" width="43.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="39" width="46.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="39" width="28.55"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5668,27 +5687,39 @@
       <c r="F1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="38"/>
+      <c r="G1" s="39"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="51" t="s">
-        <v>26</v>
-      </c>
-      <c r="B2" s="51" t="s">
-        <v>380</v>
-      </c>
-      <c r="C2" s="51" t="s">
+      <c r="A2" s="52" t="s">
+        <v>102</v>
+      </c>
+      <c r="B2" s="53" t="s">
         <v>381</v>
       </c>
-      <c r="D2" s="51" t="s">
+      <c r="C2" s="52" t="s">
         <v>382</v>
       </c>
-      <c r="E2" s="51" t="s">
+      <c r="D2" s="52" t="s">
         <v>383</v>
       </c>
-      <c r="F2" s="51" t="s">
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="52" t="s">
+        <v>102</v>
+      </c>
+      <c r="B3" s="53" t="s">
         <v>384</v>
       </c>
+      <c r="C3" s="52" t="s">
+        <v>133</v>
+      </c>
+      <c r="D3" s="52" t="s">
+        <v>134</v>
+      </c>
+      <c r="E3" s="52"/>
+      <c r="F3" s="52"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Generator: Add support for custom labels in widget generation
Fix: #1035
Note: we are doing this so we don't need a full custom widget if we only want a custom label.
- Updated the generate_import_statements function to include custom labels import.
- Enhanced the generate_label function to handle custom labels in parameters, with validation for format.
- Updated the Household Travel Generate Survey Excel file example to reflect these changes.
- Updated the Generator README with custom label.
</commit_message>
<xml_diff>
--- a/example/demo_generator/references/Household_Travel_Generate_Survey.xlsx
+++ b/example/demo_generator/references/Household_Travel_Generate_Survey.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Widgets" sheetId="1" state="visible" r:id="rId3"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="681" uniqueCount="385">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="679" uniqueCount="385">
   <si>
     <t xml:space="preserve">questionName</t>
   </si>
@@ -459,12 +459,6 @@
     <t xml:space="preserve">schoolType</t>
   </si>
   <si>
-    <t xml:space="preserve">**Établissement d'enseignement / type d'école**</t>
-  </si>
-  <si>
-    <t xml:space="preserve">**School type**</t>
-  </si>
-  <si>
     <t xml:space="preserve">customLabels={{personSchoolTypeCustomLabels}}</t>
   </si>
   <si>
@@ -1239,6 +1233,12 @@
   </si>
   <si>
     <t xml:space="preserve">personSchoolTypeOlderPerson</t>
+  </si>
+  <si>
+    <t xml:space="preserve">**Établissement d'enseignement / type d'école**</t>
+  </si>
+  <si>
+    <t xml:space="preserve">**School type**</t>
   </si>
 </sst>
 </file>
@@ -1474,7 +1474,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="55">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1575,7 +1575,7 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1588,6 +1588,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3252,20 +3256,16 @@
       <c r="F25" s="23" t="s">
         <v>132</v>
       </c>
-      <c r="G25" s="25" t="s">
-        <v>133</v>
-      </c>
-      <c r="H25" s="25" t="s">
-        <v>134</v>
-      </c>
+      <c r="G25" s="25"/>
+      <c r="H25" s="25"/>
       <c r="I25" s="19"/>
       <c r="J25" s="19"/>
       <c r="K25" s="26" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="L25" s="23"/>
       <c r="M25" s="27" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="N25" s="23"/>
       <c r="O25" s="23" t="s">
@@ -3280,17 +3280,17 @@
         <v>1</v>
       </c>
       <c r="U25" s="23" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="V25" s="23" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="W25" s="23"/>
       <c r="X25" s="23"/>
     </row>
     <row r="26" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="19" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B26" s="19" t="s">
         <v>30</v>
@@ -3306,24 +3306,24 @@
         <v>101</v>
       </c>
       <c r="F26" s="28" t="s">
+        <v>138</v>
+      </c>
+      <c r="G26" s="19" t="s">
+        <v>139</v>
+      </c>
+      <c r="H26" s="19" t="s">
         <v>140</v>
-      </c>
-      <c r="G26" s="19" t="s">
-        <v>141</v>
-      </c>
-      <c r="H26" s="19" t="s">
-        <v>142</v>
       </c>
       <c r="I26" s="19"/>
       <c r="J26" s="19"/>
       <c r="K26" s="19"/>
       <c r="L26" s="23"/>
       <c r="M26" s="23" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="N26" s="23"/>
       <c r="O26" s="23" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="P26" s="23"/>
       <c r="Q26" s="23"/>
@@ -3340,7 +3340,7 @@
     </row>
     <row r="27" customFormat="false" ht="62.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="19" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B27" s="19" t="s">
         <v>30</v>
@@ -3356,13 +3356,13 @@
         <v>101</v>
       </c>
       <c r="F27" s="23" t="s">
+        <v>143</v>
+      </c>
+      <c r="G27" s="19" t="s">
+        <v>144</v>
+      </c>
+      <c r="H27" s="19" t="s">
         <v>145</v>
-      </c>
-      <c r="G27" s="19" t="s">
-        <v>146</v>
-      </c>
-      <c r="H27" s="19" t="s">
-        <v>147</v>
       </c>
       <c r="I27" s="19"/>
       <c r="J27" s="19"/>
@@ -3373,7 +3373,7 @@
       </c>
       <c r="N27" s="23"/>
       <c r="O27" s="23" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="P27" s="23"/>
       <c r="Q27" s="23"/>
@@ -3390,7 +3390,7 @@
     </row>
     <row r="28" customFormat="false" ht="52.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="19" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B28" s="19" t="s">
         <v>30</v>
@@ -3406,24 +3406,24 @@
         <v>101</v>
       </c>
       <c r="F28" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="G28" s="19" t="s">
+        <v>149</v>
+      </c>
+      <c r="H28" s="19" t="s">
         <v>150</v>
-      </c>
-      <c r="G28" s="19" t="s">
-        <v>151</v>
-      </c>
-      <c r="H28" s="19" t="s">
-        <v>152</v>
       </c>
       <c r="I28" s="19"/>
       <c r="J28" s="19"/>
       <c r="K28" s="19"/>
       <c r="L28" s="23"/>
       <c r="M28" s="23" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="N28" s="23"/>
       <c r="O28" s="23" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="P28" s="23"/>
       <c r="Q28" s="23"/>
@@ -3439,11 +3439,11 @@
       <c r="X28" s="23"/>
     </row>
     <row r="29" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="25" t="s">
-        <v>154</v>
+      <c r="A29" s="29" t="s">
+        <v>152</v>
       </c>
       <c r="B29" s="19" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C29" s="21" t="b">
         <f aca="false">FALSE()</f>
@@ -3456,24 +3456,24 @@
         <v>101</v>
       </c>
       <c r="F29" s="23" t="s">
+        <v>154</v>
+      </c>
+      <c r="G29" s="19" t="s">
+        <v>155</v>
+      </c>
+      <c r="H29" s="19" t="s">
         <v>156</v>
-      </c>
-      <c r="G29" s="19" t="s">
-        <v>157</v>
-      </c>
-      <c r="H29" s="19" t="s">
-        <v>158</v>
       </c>
       <c r="I29" s="19"/>
       <c r="J29" s="19"/>
       <c r="K29" s="19"/>
       <c r="L29" s="23"/>
       <c r="M29" s="23" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="N29" s="24"/>
       <c r="O29" s="23" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="P29" s="23"/>
       <c r="Q29" s="23"/>
@@ -3490,7 +3490,7 @@
     </row>
     <row r="30" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="19" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B30" s="19" t="s">
         <v>30</v>
@@ -3506,20 +3506,20 @@
         <v>101</v>
       </c>
       <c r="F30" s="23" t="s">
+        <v>160</v>
+      </c>
+      <c r="G30" s="19" t="s">
+        <v>161</v>
+      </c>
+      <c r="H30" s="19" t="s">
         <v>162</v>
-      </c>
-      <c r="G30" s="19" t="s">
-        <v>163</v>
-      </c>
-      <c r="H30" s="19" t="s">
-        <v>164</v>
       </c>
       <c r="I30" s="19"/>
       <c r="J30" s="19"/>
       <c r="K30" s="19"/>
       <c r="L30" s="23"/>
       <c r="M30" s="23" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="N30" s="23"/>
       <c r="O30" s="23" t="s">
@@ -3540,7 +3540,7 @@
     </row>
     <row r="31" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="19" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B31" s="19" t="s">
         <v>30</v>
@@ -3556,24 +3556,24 @@
         <v>101</v>
       </c>
       <c r="F31" s="23" t="s">
+        <v>165</v>
+      </c>
+      <c r="G31" s="19" t="s">
+        <v>166</v>
+      </c>
+      <c r="H31" s="19" t="s">
         <v>167</v>
-      </c>
-      <c r="G31" s="19" t="s">
-        <v>168</v>
-      </c>
-      <c r="H31" s="19" t="s">
-        <v>169</v>
       </c>
       <c r="I31" s="19"/>
       <c r="J31" s="19"/>
       <c r="K31" s="19"/>
       <c r="L31" s="23"/>
       <c r="M31" s="23" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="N31" s="23"/>
       <c r="O31" s="23" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="P31" s="23"/>
       <c r="Q31" s="23"/>
@@ -3590,7 +3590,7 @@
     </row>
     <row r="32" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="19" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B32" s="19" t="s">
         <v>30</v>
@@ -3606,24 +3606,24 @@
         <v>101</v>
       </c>
       <c r="F32" s="23" t="s">
+        <v>170</v>
+      </c>
+      <c r="G32" s="19" t="s">
+        <v>171</v>
+      </c>
+      <c r="H32" s="19" t="s">
         <v>172</v>
-      </c>
-      <c r="G32" s="19" t="s">
-        <v>173</v>
-      </c>
-      <c r="H32" s="19" t="s">
-        <v>174</v>
       </c>
       <c r="I32" s="19"/>
       <c r="J32" s="19"/>
       <c r="K32" s="19"/>
       <c r="L32" s="23"/>
       <c r="M32" s="23" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="N32" s="23"/>
       <c r="O32" s="23" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="P32" s="23"/>
       <c r="Q32" s="23"/>
@@ -3640,7 +3640,7 @@
     </row>
     <row r="33" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="19" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B33" s="19" t="s">
         <v>25</v>
@@ -3656,20 +3656,20 @@
         <v>101</v>
       </c>
       <c r="F33" s="23" t="s">
+        <v>176</v>
+      </c>
+      <c r="G33" s="19" t="s">
+        <v>177</v>
+      </c>
+      <c r="H33" s="19" t="s">
         <v>178</v>
-      </c>
-      <c r="G33" s="19" t="s">
-        <v>179</v>
-      </c>
-      <c r="H33" s="19" t="s">
-        <v>180</v>
       </c>
       <c r="I33" s="19"/>
       <c r="J33" s="19"/>
       <c r="K33" s="19"/>
       <c r="L33" s="23"/>
       <c r="M33" s="19" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="N33" s="23"/>
       <c r="O33" s="23"/>
@@ -3688,9 +3688,9 @@
     </row>
     <row r="34" customFormat="false" ht="85.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="19" t="s">
-        <v>182</v>
-      </c>
-      <c r="B34" s="29" t="s">
+        <v>180</v>
+      </c>
+      <c r="B34" s="30" t="s">
         <v>69</v>
       </c>
       <c r="C34" s="21" t="b">
@@ -3704,24 +3704,24 @@
         <v>101</v>
       </c>
       <c r="F34" s="23" t="s">
+        <v>181</v>
+      </c>
+      <c r="G34" s="19" t="s">
+        <v>182</v>
+      </c>
+      <c r="H34" s="19" t="s">
         <v>183</v>
       </c>
-      <c r="G34" s="19" t="s">
+      <c r="I34" s="19" t="s">
         <v>184</v>
       </c>
-      <c r="H34" s="19" t="s">
+      <c r="J34" s="19" t="s">
         <v>185</v>
-      </c>
-      <c r="I34" s="19" t="s">
-        <v>186</v>
-      </c>
-      <c r="J34" s="19" t="s">
-        <v>187</v>
       </c>
       <c r="K34" s="19"/>
       <c r="L34" s="23"/>
       <c r="M34" s="19" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="N34" s="23"/>
       <c r="O34" s="23"/>
@@ -3740,7 +3740,7 @@
     </row>
     <row r="35" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="19" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B35" s="19" t="s">
         <v>25</v>
@@ -3756,20 +3756,20 @@
         <v>101</v>
       </c>
       <c r="F35" s="23" t="s">
+        <v>187</v>
+      </c>
+      <c r="G35" s="19" t="s">
+        <v>188</v>
+      </c>
+      <c r="H35" s="19" t="s">
         <v>189</v>
-      </c>
-      <c r="G35" s="19" t="s">
-        <v>190</v>
-      </c>
-      <c r="H35" s="19" t="s">
-        <v>191</v>
       </c>
       <c r="I35" s="19"/>
       <c r="J35" s="19"/>
       <c r="K35" s="19"/>
       <c r="L35" s="23"/>
       <c r="M35" s="19" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="N35" s="23"/>
       <c r="O35" s="23"/>
@@ -3788,9 +3788,9 @@
     </row>
     <row r="36" customFormat="false" ht="85.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="19" t="s">
-        <v>193</v>
-      </c>
-      <c r="B36" s="29" t="s">
+        <v>191</v>
+      </c>
+      <c r="B36" s="30" t="s">
         <v>69</v>
       </c>
       <c r="C36" s="21" t="b">
@@ -3804,27 +3804,27 @@
         <v>101</v>
       </c>
       <c r="F36" s="23" t="s">
+        <v>192</v>
+      </c>
+      <c r="G36" s="19" t="s">
+        <v>193</v>
+      </c>
+      <c r="H36" s="19" t="s">
         <v>194</v>
       </c>
-      <c r="G36" s="19" t="s">
+      <c r="I36" s="19" t="s">
         <v>195</v>
       </c>
-      <c r="H36" s="19" t="s">
+      <c r="J36" s="19" t="s">
         <v>196</v>
       </c>
-      <c r="I36" s="19" t="s">
-        <v>197</v>
-      </c>
-      <c r="J36" s="19" t="s">
-        <v>198</v>
-      </c>
-      <c r="K36" s="30"/>
-      <c r="L36" s="31"/>
-      <c r="M36" s="30"/>
-      <c r="N36" s="31"/>
-      <c r="O36" s="31"/>
-      <c r="P36" s="31"/>
-      <c r="Q36" s="31"/>
+      <c r="K36" s="31"/>
+      <c r="L36" s="32"/>
+      <c r="M36" s="31"/>
+      <c r="N36" s="32"/>
+      <c r="O36" s="32"/>
+      <c r="P36" s="32"/>
+      <c r="Q36" s="32"/>
       <c r="R36" s="23"/>
       <c r="S36" s="23"/>
       <c r="T36" s="21" t="b">
@@ -3837,11 +3837,11 @@
       <c r="X36" s="23"/>
     </row>
     <row r="37" customFormat="false" ht="86.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="25" t="s">
-        <v>199</v>
+      <c r="A37" s="29" t="s">
+        <v>197</v>
       </c>
       <c r="B37" s="19" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C37" s="21" t="b">
         <f aca="false">FALSE()</f>
@@ -3854,13 +3854,13 @@
         <v>101</v>
       </c>
       <c r="F37" s="23" t="s">
+        <v>198</v>
+      </c>
+      <c r="G37" s="19" t="s">
+        <v>199</v>
+      </c>
+      <c r="H37" s="19" t="s">
         <v>200</v>
-      </c>
-      <c r="G37" s="19" t="s">
-        <v>201</v>
-      </c>
-      <c r="H37" s="19" t="s">
-        <v>202</v>
       </c>
       <c r="I37" s="19"/>
       <c r="J37" s="19"/>
@@ -3868,8 +3868,8 @@
       <c r="L37" s="23"/>
       <c r="M37" s="24"/>
       <c r="N37" s="24"/>
-      <c r="O37" s="32" t="s">
-        <v>148</v>
+      <c r="O37" s="33" t="s">
+        <v>146</v>
       </c>
       <c r="P37" s="23"/>
       <c r="Q37" s="23"/>
@@ -3885,11 +3885,11 @@
       <c r="X37" s="23"/>
     </row>
     <row r="38" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="25" t="s">
-        <v>203</v>
+      <c r="A38" s="29" t="s">
+        <v>201</v>
       </c>
       <c r="B38" s="19" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C38" s="21" t="b">
         <f aca="false">FALSE()</f>
@@ -3902,13 +3902,13 @@
         <v>101</v>
       </c>
       <c r="F38" s="23" t="s">
+        <v>202</v>
+      </c>
+      <c r="G38" s="19" t="s">
+        <v>203</v>
+      </c>
+      <c r="H38" s="19" t="s">
         <v>204</v>
-      </c>
-      <c r="G38" s="19" t="s">
-        <v>205</v>
-      </c>
-      <c r="H38" s="19" t="s">
-        <v>206</v>
       </c>
       <c r="I38" s="19"/>
       <c r="J38" s="19"/>
@@ -3916,8 +3916,8 @@
       <c r="L38" s="23"/>
       <c r="M38" s="24"/>
       <c r="N38" s="24"/>
-      <c r="O38" s="32" t="s">
-        <v>148</v>
+      <c r="O38" s="33" t="s">
+        <v>146</v>
       </c>
       <c r="P38" s="23"/>
       <c r="Q38" s="23"/>
@@ -3933,11 +3933,11 @@
       <c r="X38" s="23"/>
     </row>
     <row r="39" customFormat="false" ht="64.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="25" t="s">
-        <v>207</v>
+      <c r="A39" s="29" t="s">
+        <v>205</v>
       </c>
       <c r="B39" s="19" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C39" s="21" t="b">
         <f aca="false">FALSE()</f>
@@ -3950,13 +3950,13 @@
         <v>101</v>
       </c>
       <c r="F39" s="23" t="s">
+        <v>206</v>
+      </c>
+      <c r="G39" s="19" t="s">
+        <v>207</v>
+      </c>
+      <c r="H39" s="19" t="s">
         <v>208</v>
-      </c>
-      <c r="G39" s="19" t="s">
-        <v>209</v>
-      </c>
-      <c r="H39" s="19" t="s">
-        <v>210</v>
       </c>
       <c r="I39" s="19"/>
       <c r="J39" s="19"/>
@@ -3964,8 +3964,8 @@
       <c r="L39" s="23"/>
       <c r="M39" s="24"/>
       <c r="N39" s="24"/>
-      <c r="O39" s="32" t="s">
-        <v>148</v>
+      <c r="O39" s="33" t="s">
+        <v>146</v>
       </c>
       <c r="P39" s="23"/>
       <c r="Q39" s="23"/>
@@ -3981,11 +3981,11 @@
       <c r="X39" s="23"/>
     </row>
     <row r="40" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="25" t="s">
-        <v>211</v>
+      <c r="A40" s="29" t="s">
+        <v>209</v>
       </c>
       <c r="B40" s="19" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C40" s="21" t="b">
         <f aca="false">FALSE()</f>
@@ -3998,13 +3998,13 @@
         <v>101</v>
       </c>
       <c r="F40" s="23" t="s">
+        <v>210</v>
+      </c>
+      <c r="G40" s="19" t="s">
+        <v>211</v>
+      </c>
+      <c r="H40" s="19" t="s">
         <v>212</v>
-      </c>
-      <c r="G40" s="19" t="s">
-        <v>213</v>
-      </c>
-      <c r="H40" s="19" t="s">
-        <v>214</v>
       </c>
       <c r="I40" s="19"/>
       <c r="J40" s="19"/>
@@ -4012,8 +4012,8 @@
       <c r="L40" s="23"/>
       <c r="M40" s="24"/>
       <c r="N40" s="24"/>
-      <c r="O40" s="32" t="s">
-        <v>148</v>
+      <c r="O40" s="33" t="s">
+        <v>146</v>
       </c>
       <c r="P40" s="23"/>
       <c r="Q40" s="23"/>
@@ -4029,76 +4029,76 @@
       <c r="X40" s="23"/>
     </row>
     <row r="41" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="33" t="s">
-        <v>215</v>
-      </c>
-      <c r="B41" s="33" t="s">
+      <c r="A41" s="34" t="s">
+        <v>213</v>
+      </c>
+      <c r="B41" s="34" t="s">
         <v>98</v>
       </c>
-      <c r="C41" s="34" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D41" s="33" t="s">
+      <c r="C41" s="35" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D41" s="34" t="s">
         <v>102</v>
       </c>
-      <c r="E41" s="35"/>
-      <c r="F41" s="35" t="str">
+      <c r="E41" s="36"/>
+      <c r="F41" s="36" t="str">
         <f aca="false">REPLACE(A41, FIND("_", A41), 1, ".")</f>
         <v>household.save</v>
       </c>
-      <c r="G41" s="33" t="s">
+      <c r="G41" s="34" t="s">
         <v>99</v>
       </c>
-      <c r="H41" s="33" t="s">
+      <c r="H41" s="34" t="s">
         <v>100</v>
       </c>
-      <c r="I41" s="33"/>
-      <c r="J41" s="33"/>
-      <c r="K41" s="33"/>
-      <c r="L41" s="35"/>
-      <c r="M41" s="35"/>
-      <c r="N41" s="35"/>
-      <c r="O41" s="35"/>
-      <c r="P41" s="35"/>
-      <c r="Q41" s="35"/>
-      <c r="R41" s="35"/>
-      <c r="S41" s="35"/>
-      <c r="T41" s="34" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U41" s="35"/>
-      <c r="V41" s="35"/>
-      <c r="W41" s="35"/>
-      <c r="X41" s="35"/>
+      <c r="I41" s="34"/>
+      <c r="J41" s="34"/>
+      <c r="K41" s="34"/>
+      <c r="L41" s="36"/>
+      <c r="M41" s="36"/>
+      <c r="N41" s="36"/>
+      <c r="O41" s="36"/>
+      <c r="P41" s="36"/>
+      <c r="Q41" s="36"/>
+      <c r="R41" s="36"/>
+      <c r="S41" s="36"/>
+      <c r="T41" s="35" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U41" s="36"/>
+      <c r="V41" s="36"/>
+      <c r="W41" s="36"/>
+      <c r="X41" s="36"/>
     </row>
     <row r="42" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C42" s="36" t="b">
+      <c r="C42" s="37" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="D42" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="G42" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="H42" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="F42" s="1" t="s">
-        <v>216</v>
-      </c>
-      <c r="G42" s="1" t="s">
-        <v>218</v>
-      </c>
-      <c r="H42" s="1" t="s">
-        <v>219</v>
-      </c>
-      <c r="L42" s="37"/>
-      <c r="M42" s="38"/>
-      <c r="T42" s="36" t="b">
+      <c r="L42" s="38"/>
+      <c r="M42" s="39"/>
+      <c r="T42" s="37" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -4155,486 +4155,486 @@
   <dimension ref="A1:F29"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="39" width="27.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="39" width="15.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="39" width="31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="40" width="20.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="39" width="19.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="39" width="12.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="40" width="27.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="40" width="15.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="40" width="31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="41" width="20.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="40" width="19.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="40" width="12.14"/>
   </cols>
   <sheetData>
-    <row r="1" s="43" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="41" t="s">
+    <row r="1" s="44" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="42" t="s">
+        <v>218</v>
+      </c>
+      <c r="B1" s="42" t="s">
+        <v>219</v>
+      </c>
+      <c r="C1" s="42" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" s="43" t="s">
         <v>220</v>
       </c>
-      <c r="B1" s="41" t="s">
+      <c r="E1" s="42" t="s">
         <v>221</v>
       </c>
-      <c r="C1" s="41" t="s">
+      <c r="F1" s="42" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="45" t="s">
+        <v>223</v>
+      </c>
+      <c r="B2" s="45"/>
+      <c r="C2" s="45" t="s">
+        <v>224</v>
+      </c>
+      <c r="D2" s="46" t="s">
+        <v>225</v>
+      </c>
+      <c r="E2" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="45"/>
+    </row>
+    <row r="3" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="45" t="s">
+        <v>95</v>
+      </c>
+      <c r="B3" s="45"/>
+      <c r="C3" s="45" t="s">
+        <v>224</v>
+      </c>
+      <c r="D3" s="46" t="s">
+        <v>226</v>
+      </c>
+      <c r="E3" s="45" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" s="45"/>
+    </row>
+    <row r="4" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="45" t="s">
+        <v>163</v>
+      </c>
+      <c r="B4" s="45"/>
+      <c r="C4" s="45" t="s">
+        <v>227</v>
+      </c>
+      <c r="D4" s="46" t="s">
+        <v>225</v>
+      </c>
+      <c r="E4" s="45" t="s">
+        <v>228</v>
+      </c>
+      <c r="F4" s="45"/>
+    </row>
+    <row r="5" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="45" t="s">
+        <v>163</v>
+      </c>
+      <c r="B5" s="45" t="s">
+        <v>229</v>
+      </c>
+      <c r="C5" s="45" t="s">
+        <v>224</v>
+      </c>
+      <c r="D5" s="46" t="s">
+        <v>225</v>
+      </c>
+      <c r="E5" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="45"/>
+    </row>
+    <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="45" t="s">
+        <v>230</v>
+      </c>
+      <c r="B6" s="45"/>
+      <c r="C6" s="45" t="s">
+        <v>231</v>
+      </c>
+      <c r="D6" s="46" t="s">
+        <v>226</v>
+      </c>
+      <c r="E6" s="45" t="n">
+        <v>3</v>
+      </c>
+      <c r="F6" s="45"/>
+    </row>
+    <row r="7" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="45" t="s">
+        <v>230</v>
+      </c>
+      <c r="B7" s="45" t="s">
+        <v>232</v>
+      </c>
+      <c r="C7" s="45" t="s">
+        <v>231</v>
+      </c>
+      <c r="D7" s="46" t="s">
+        <v>233</v>
+      </c>
+      <c r="E7" s="45" t="n">
         <v>5</v>
       </c>
-      <c r="D1" s="42" t="s">
-        <v>222</v>
-      </c>
-      <c r="E1" s="41" t="s">
-        <v>223</v>
-      </c>
-      <c r="F1" s="41" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="44" t="s">
+      <c r="F7" s="45"/>
+    </row>
+    <row r="8" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="45" t="s">
+        <v>234</v>
+      </c>
+      <c r="B8" s="45"/>
+      <c r="C8" s="45" t="s">
+        <v>231</v>
+      </c>
+      <c r="D8" s="46" t="s">
+        <v>226</v>
+      </c>
+      <c r="E8" s="45" t="n">
+        <v>4</v>
+      </c>
+      <c r="F8" s="45"/>
+    </row>
+    <row r="9" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="45" t="s">
+        <v>234</v>
+      </c>
+      <c r="B9" s="45" t="s">
+        <v>232</v>
+      </c>
+      <c r="C9" s="45" t="s">
+        <v>231</v>
+      </c>
+      <c r="D9" s="46" t="s">
+        <v>233</v>
+      </c>
+      <c r="E9" s="45" t="n">
+        <v>13</v>
+      </c>
+      <c r="F9" s="45"/>
+    </row>
+    <row r="10" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="45" t="s">
+        <v>235</v>
+      </c>
+      <c r="B10" s="45"/>
+      <c r="C10" s="45" t="s">
+        <v>231</v>
+      </c>
+      <c r="D10" s="46" t="s">
+        <v>233</v>
+      </c>
+      <c r="E10" s="45" t="n">
+        <v>5</v>
+      </c>
+      <c r="F10" s="45"/>
+    </row>
+    <row r="11" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="45" t="s">
+        <v>119</v>
+      </c>
+      <c r="B11" s="45"/>
+      <c r="C11" s="45" t="s">
+        <v>231</v>
+      </c>
+      <c r="D11" s="46" t="s">
+        <v>226</v>
+      </c>
+      <c r="E11" s="45" t="n">
+        <v>5</v>
+      </c>
+      <c r="F11" s="45"/>
+    </row>
+    <row r="12" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="45" t="s">
+        <v>157</v>
+      </c>
+      <c r="B12" s="45"/>
+      <c r="C12" s="45" t="s">
+        <v>231</v>
+      </c>
+      <c r="D12" s="46" t="s">
+        <v>226</v>
+      </c>
+      <c r="E12" s="45" t="n">
+        <v>6</v>
+      </c>
+      <c r="F12" s="45"/>
+    </row>
+    <row r="13" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="45" t="s">
+        <v>236</v>
+      </c>
+      <c r="B13" s="45"/>
+      <c r="C13" s="45" t="s">
+        <v>231</v>
+      </c>
+      <c r="D13" s="46" t="s">
+        <v>226</v>
+      </c>
+      <c r="E13" s="45" t="n">
+        <v>11</v>
+      </c>
+      <c r="F13" s="45"/>
+    </row>
+    <row r="14" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="45" t="s">
+        <v>124</v>
+      </c>
+      <c r="B14" s="45"/>
+      <c r="C14" s="45" t="s">
+        <v>231</v>
+      </c>
+      <c r="D14" s="46" t="s">
+        <v>226</v>
+      </c>
+      <c r="E14" s="45" t="n">
+        <v>14</v>
+      </c>
+      <c r="F14" s="45"/>
+    </row>
+    <row r="15" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="45" t="s">
+        <v>134</v>
+      </c>
+      <c r="B15" s="45"/>
+      <c r="C15" s="45" t="s">
+        <v>231</v>
+      </c>
+      <c r="D15" s="46" t="s">
+        <v>233</v>
+      </c>
+      <c r="E15" s="45" t="n">
+        <v>15</v>
+      </c>
+      <c r="F15" s="45"/>
+    </row>
+    <row r="16" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="45" t="s">
+        <v>134</v>
+      </c>
+      <c r="B16" s="45"/>
+      <c r="C16" s="45" t="s">
+        <v>231</v>
+      </c>
+      <c r="D16" s="46" t="s">
+        <v>237</v>
+      </c>
+      <c r="E16" s="45" t="s">
+        <v>238</v>
+      </c>
+      <c r="F16" s="45"/>
+    </row>
+    <row r="17" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="45" t="s">
+        <v>239</v>
+      </c>
+      <c r="B17" s="45"/>
+      <c r="C17" s="45" t="s">
+        <v>231</v>
+      </c>
+      <c r="D17" s="46" t="s">
+        <v>226</v>
+      </c>
+      <c r="E17" s="45" t="n">
+        <v>15</v>
+      </c>
+      <c r="F17" s="45"/>
+    </row>
+    <row r="18" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="45" t="s">
+        <v>130</v>
+      </c>
+      <c r="B18" s="45"/>
+      <c r="C18" s="45" t="s">
+        <v>231</v>
+      </c>
+      <c r="D18" s="46" t="s">
+        <v>226</v>
+      </c>
+      <c r="E18" s="45" t="n">
+        <v>16</v>
+      </c>
+      <c r="F18" s="45"/>
+    </row>
+    <row r="19" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="45" t="s">
+        <v>240</v>
+      </c>
+      <c r="B19" s="45"/>
+      <c r="C19" s="45" t="s">
+        <v>231</v>
+      </c>
+      <c r="D19" s="46" t="s">
+        <v>226</v>
+      </c>
+      <c r="E19" s="45" t="n">
+        <v>40</v>
+      </c>
+      <c r="F19" s="45"/>
+    </row>
+    <row r="20" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="45" t="s">
+        <v>151</v>
+      </c>
+      <c r="B20" s="45"/>
+      <c r="C20" s="45" t="s">
+        <v>241</v>
+      </c>
+      <c r="D20" s="46" t="s">
         <v>225</v>
       </c>
-      <c r="B2" s="44"/>
-      <c r="C2" s="44" t="s">
-        <v>226</v>
-      </c>
-      <c r="D2" s="45" t="s">
-        <v>227</v>
-      </c>
-      <c r="E2" s="44" t="n">
-        <v>1</v>
-      </c>
-      <c r="F2" s="44"/>
-    </row>
-    <row r="3" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="44" t="s">
-        <v>95</v>
-      </c>
-      <c r="B3" s="44"/>
-      <c r="C3" s="44" t="s">
-        <v>226</v>
-      </c>
-      <c r="D3" s="45" t="s">
+      <c r="E20" s="45" t="s">
         <v>228</v>
       </c>
-      <c r="E3" s="44" t="n">
-        <v>2</v>
-      </c>
-      <c r="F3" s="44"/>
-    </row>
-    <row r="4" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="44" t="s">
-        <v>165</v>
-      </c>
-      <c r="B4" s="44"/>
-      <c r="C4" s="44" t="s">
+      <c r="F20" s="45"/>
+    </row>
+    <row r="21" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="40" t="s">
+        <v>168</v>
+      </c>
+      <c r="C21" s="40" t="s">
+        <v>242</v>
+      </c>
+      <c r="D21" s="46" t="s">
+        <v>225</v>
+      </c>
+      <c r="E21" s="41" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="40" t="s">
+        <v>168</v>
+      </c>
+      <c r="B22" s="40" t="s">
         <v>229</v>
       </c>
-      <c r="D4" s="45" t="s">
-        <v>227</v>
-      </c>
-      <c r="E4" s="44" t="s">
-        <v>230</v>
-      </c>
-      <c r="F4" s="44"/>
-    </row>
-    <row r="5" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="44" t="s">
-        <v>165</v>
-      </c>
-      <c r="B5" s="44" t="s">
-        <v>231</v>
-      </c>
-      <c r="C5" s="44" t="s">
-        <v>226</v>
-      </c>
-      <c r="D5" s="45" t="s">
-        <v>227</v>
-      </c>
-      <c r="E5" s="44" t="n">
-        <v>1</v>
-      </c>
-      <c r="F5" s="44"/>
-    </row>
-    <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="B6" s="44"/>
-      <c r="C6" s="44" t="s">
-        <v>233</v>
-      </c>
-      <c r="D6" s="45" t="s">
-        <v>228</v>
-      </c>
-      <c r="E6" s="44" t="n">
-        <v>3</v>
-      </c>
-      <c r="F6" s="44"/>
-    </row>
-    <row r="7" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="B7" s="44" t="s">
-        <v>234</v>
-      </c>
-      <c r="C7" s="44" t="s">
-        <v>233</v>
-      </c>
-      <c r="D7" s="45" t="s">
-        <v>235</v>
-      </c>
-      <c r="E7" s="44" t="n">
-        <v>5</v>
-      </c>
-      <c r="F7" s="44"/>
-    </row>
-    <row r="8" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="44" t="s">
-        <v>236</v>
-      </c>
-      <c r="B8" s="44"/>
-      <c r="C8" s="44" t="s">
-        <v>233</v>
-      </c>
-      <c r="D8" s="45" t="s">
-        <v>228</v>
-      </c>
-      <c r="E8" s="44" t="n">
-        <v>4</v>
-      </c>
-      <c r="F8" s="44"/>
-    </row>
-    <row r="9" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="44" t="s">
-        <v>236</v>
-      </c>
-      <c r="B9" s="44" t="s">
-        <v>234</v>
-      </c>
-      <c r="C9" s="44" t="s">
-        <v>233</v>
-      </c>
-      <c r="D9" s="45" t="s">
-        <v>235</v>
-      </c>
-      <c r="E9" s="44" t="n">
-        <v>13</v>
-      </c>
-      <c r="F9" s="44"/>
-    </row>
-    <row r="10" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="44" t="s">
-        <v>237</v>
-      </c>
-      <c r="B10" s="44"/>
-      <c r="C10" s="44" t="s">
-        <v>233</v>
-      </c>
-      <c r="D10" s="45" t="s">
-        <v>235</v>
-      </c>
-      <c r="E10" s="44" t="n">
-        <v>5</v>
-      </c>
-      <c r="F10" s="44"/>
-    </row>
-    <row r="11" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="44" t="s">
-        <v>119</v>
-      </c>
-      <c r="B11" s="44"/>
-      <c r="C11" s="44" t="s">
-        <v>233</v>
-      </c>
-      <c r="D11" s="45" t="s">
-        <v>228</v>
-      </c>
-      <c r="E11" s="44" t="n">
-        <v>5</v>
-      </c>
-      <c r="F11" s="44"/>
-    </row>
-    <row r="12" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="44" t="s">
-        <v>159</v>
-      </c>
-      <c r="B12" s="44"/>
-      <c r="C12" s="44" t="s">
-        <v>233</v>
-      </c>
-      <c r="D12" s="45" t="s">
-        <v>228</v>
-      </c>
-      <c r="E12" s="44" t="n">
-        <v>6</v>
-      </c>
-      <c r="F12" s="44"/>
-    </row>
-    <row r="13" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="44" t="s">
-        <v>238</v>
-      </c>
-      <c r="B13" s="44"/>
-      <c r="C13" s="44" t="s">
-        <v>233</v>
-      </c>
-      <c r="D13" s="45" t="s">
-        <v>228</v>
-      </c>
-      <c r="E13" s="44" t="n">
-        <v>11</v>
-      </c>
-      <c r="F13" s="44"/>
-    </row>
-    <row r="14" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="44" t="s">
-        <v>124</v>
-      </c>
-      <c r="B14" s="44"/>
-      <c r="C14" s="44" t="s">
-        <v>233</v>
-      </c>
-      <c r="D14" s="45" t="s">
-        <v>228</v>
-      </c>
-      <c r="E14" s="44" t="n">
-        <v>14</v>
-      </c>
-      <c r="F14" s="44"/>
-    </row>
-    <row r="15" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="44" t="s">
-        <v>136</v>
-      </c>
-      <c r="B15" s="44"/>
-      <c r="C15" s="44" t="s">
-        <v>233</v>
-      </c>
-      <c r="D15" s="45" t="s">
-        <v>235</v>
-      </c>
-      <c r="E15" s="44" t="n">
-        <v>15</v>
-      </c>
-      <c r="F15" s="44"/>
-    </row>
-    <row r="16" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="44" t="s">
-        <v>136</v>
-      </c>
-      <c r="B16" s="44"/>
-      <c r="C16" s="44" t="s">
-        <v>233</v>
-      </c>
-      <c r="D16" s="45" t="s">
-        <v>239</v>
-      </c>
-      <c r="E16" s="44" t="s">
-        <v>240</v>
-      </c>
-      <c r="F16" s="44"/>
-    </row>
-    <row r="17" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="44" t="s">
-        <v>241</v>
-      </c>
-      <c r="B17" s="44"/>
-      <c r="C17" s="44" t="s">
-        <v>233</v>
-      </c>
-      <c r="D17" s="45" t="s">
-        <v>228</v>
-      </c>
-      <c r="E17" s="44" t="n">
-        <v>15</v>
-      </c>
-      <c r="F17" s="44"/>
-    </row>
-    <row r="18" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="44" t="s">
-        <v>130</v>
-      </c>
-      <c r="B18" s="44"/>
-      <c r="C18" s="44" t="s">
-        <v>233</v>
-      </c>
-      <c r="D18" s="45" t="s">
-        <v>228</v>
-      </c>
-      <c r="E18" s="44" t="n">
-        <v>16</v>
-      </c>
-      <c r="F18" s="44"/>
-    </row>
-    <row r="19" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="44" t="s">
+      <c r="C22" s="40" t="s">
         <v>242</v>
       </c>
-      <c r="B19" s="44"/>
-      <c r="C19" s="44" t="s">
-        <v>233</v>
-      </c>
-      <c r="D19" s="45" t="s">
-        <v>228</v>
-      </c>
-      <c r="E19" s="44" t="n">
-        <v>40</v>
-      </c>
-      <c r="F19" s="44"/>
-    </row>
-    <row r="20" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="44" t="s">
-        <v>153</v>
-      </c>
-      <c r="B20" s="44"/>
-      <c r="C20" s="44" t="s">
-        <v>243</v>
-      </c>
-      <c r="D20" s="45" t="s">
-        <v>227</v>
-      </c>
-      <c r="E20" s="44" t="s">
-        <v>230</v>
-      </c>
-      <c r="F20" s="44"/>
-    </row>
-    <row r="21" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="39" t="s">
-        <v>170</v>
-      </c>
-      <c r="C21" s="39" t="s">
+      <c r="D22" s="46" t="s">
+        <v>225</v>
+      </c>
+      <c r="E22" s="41" t="s">
         <v>244</v>
       </c>
-      <c r="D21" s="45" t="s">
-        <v>227</v>
-      </c>
-      <c r="E21" s="40" t="s">
+    </row>
+    <row r="23" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="40" t="s">
+        <v>168</v>
+      </c>
+      <c r="B23" s="40" t="s">
+        <v>229</v>
+      </c>
+      <c r="C23" s="40" t="s">
+        <v>242</v>
+      </c>
+      <c r="D23" s="46" t="s">
+        <v>225</v>
+      </c>
+      <c r="E23" s="41" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="39" t="s">
-        <v>170</v>
-      </c>
-      <c r="B22" s="39" t="s">
-        <v>231</v>
-      </c>
-      <c r="C22" s="39" t="s">
-        <v>244</v>
-      </c>
-      <c r="D22" s="45" t="s">
-        <v>227</v>
-      </c>
-      <c r="E22" s="40" t="s">
+    <row r="24" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="40" t="s">
+        <v>173</v>
+      </c>
+      <c r="C24" s="40" t="s">
+        <v>242</v>
+      </c>
+      <c r="D24" s="46" t="s">
+        <v>225</v>
+      </c>
+      <c r="E24" s="41" t="s">
         <v>246</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="39" t="s">
-        <v>170</v>
-      </c>
-      <c r="B23" s="39" t="s">
-        <v>231</v>
-      </c>
-      <c r="C23" s="39" t="s">
-        <v>244</v>
-      </c>
-      <c r="D23" s="45" t="s">
-        <v>227</v>
-      </c>
-      <c r="E23" s="40" t="s">
+    <row r="25" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="40" t="s">
+        <v>173</v>
+      </c>
+      <c r="B25" s="40" t="s">
+        <v>229</v>
+      </c>
+      <c r="C25" s="40" t="s">
+        <v>242</v>
+      </c>
+      <c r="D25" s="46" t="s">
+        <v>225</v>
+      </c>
+      <c r="E25" s="41" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="39" t="s">
-        <v>175</v>
-      </c>
-      <c r="C24" s="39" t="s">
-        <v>244</v>
-      </c>
-      <c r="D24" s="45" t="s">
-        <v>227</v>
-      </c>
-      <c r="E24" s="40" t="s">
+    <row r="26" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="40" t="s">
+        <v>173</v>
+      </c>
+      <c r="B26" s="40" t="s">
+        <v>229</v>
+      </c>
+      <c r="C26" s="40" t="s">
+        <v>242</v>
+      </c>
+      <c r="D26" s="46" t="s">
+        <v>225</v>
+      </c>
+      <c r="E26" s="41" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="40" t="s">
+        <v>179</v>
+      </c>
+      <c r="C27" s="40" t="s">
         <v>248</v>
       </c>
-    </row>
-    <row r="25" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="39" t="s">
-        <v>175</v>
-      </c>
-      <c r="B25" s="39" t="s">
-        <v>231</v>
-      </c>
-      <c r="C25" s="39" t="s">
-        <v>244</v>
-      </c>
-      <c r="D25" s="45" t="s">
-        <v>227</v>
-      </c>
-      <c r="E25" s="40" t="s">
+      <c r="D27" s="46" t="s">
+        <v>225</v>
+      </c>
+      <c r="E27" s="40" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="39" t="s">
-        <v>175</v>
-      </c>
-      <c r="B26" s="39" t="s">
-        <v>231</v>
-      </c>
-      <c r="C26" s="39" t="s">
-        <v>244</v>
-      </c>
-      <c r="D26" s="45" t="s">
-        <v>227</v>
-      </c>
-      <c r="E26" s="40" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="39" t="s">
-        <v>181</v>
-      </c>
-      <c r="C27" s="39" t="s">
+    <row r="28" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="40" t="s">
+        <v>179</v>
+      </c>
+      <c r="B28" s="40" t="s">
+        <v>229</v>
+      </c>
+      <c r="C28" s="40" t="s">
+        <v>248</v>
+      </c>
+      <c r="D28" s="46" t="s">
+        <v>225</v>
+      </c>
+      <c r="E28" s="40" t="s">
         <v>250</v>
       </c>
-      <c r="D27" s="45" t="s">
-        <v>227</v>
-      </c>
-      <c r="E27" s="39" t="s">
+    </row>
+    <row r="29" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="40" t="s">
+        <v>179</v>
+      </c>
+      <c r="B29" s="40" t="s">
+        <v>229</v>
+      </c>
+      <c r="C29" s="40" t="s">
+        <v>248</v>
+      </c>
+      <c r="D29" s="46" t="s">
+        <v>225</v>
+      </c>
+      <c r="E29" s="40" t="s">
         <v>251</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="39" t="s">
-        <v>181</v>
-      </c>
-      <c r="B28" s="39" t="s">
-        <v>231</v>
-      </c>
-      <c r="C28" s="39" t="s">
-        <v>250</v>
-      </c>
-      <c r="D28" s="45" t="s">
-        <v>227</v>
-      </c>
-      <c r="E28" s="39" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="39" t="s">
-        <v>181</v>
-      </c>
-      <c r="B29" s="39" t="s">
-        <v>231</v>
-      </c>
-      <c r="C29" s="39" t="s">
-        <v>250</v>
-      </c>
-      <c r="D29" s="45" t="s">
-        <v>227</v>
-      </c>
-      <c r="E29" s="39" t="s">
-        <v>253</v>
       </c>
     </row>
   </sheetData>
@@ -4656,116 +4656,116 @@
   <dimension ref="A1:H4"/>
   <sheetFormatPr defaultColWidth="10.69921875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="44" width="10.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="44" width="12.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="44" width="13.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="44" width="12.57"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="6" min="5" style="44" width="10.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="44" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="44" width="15.43"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="9" style="44" width="10.7"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="45" width="10.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="45" width="12.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="45" width="13.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="45" width="12.57"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="6" min="5" style="45" width="10.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="45" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="45" width="15.43"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="9" style="45" width="10.7"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="47" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="47" t="s">
+      <c r="B1" s="48" t="s">
+        <v>252</v>
+      </c>
+      <c r="C1" s="47" t="s">
+        <v>253</v>
+      </c>
+      <c r="D1" s="47" t="s">
         <v>254</v>
       </c>
-      <c r="C1" s="46" t="s">
+      <c r="E1" s="47" t="s">
         <v>255</v>
       </c>
-      <c r="D1" s="46" t="s">
+      <c r="F1" s="47" t="s">
         <v>256</v>
       </c>
-      <c r="E1" s="46" t="s">
+      <c r="G1" s="6" t="s">
         <v>257</v>
       </c>
-      <c r="F1" s="46" t="s">
+      <c r="H1" s="47" t="s">
         <v>258</v>
       </c>
-      <c r="G1" s="6" t="s">
+    </row>
+    <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="45" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" s="45" t="s">
         <v>259</v>
       </c>
-      <c r="H1" s="46" t="s">
+      <c r="C2" s="45" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="44" t="s">
-        <v>26</v>
-      </c>
-      <c r="B2" s="44" t="s">
+      <c r="D2" s="45" t="s">
         <v>261</v>
       </c>
-      <c r="C2" s="44" t="s">
-        <v>262</v>
-      </c>
-      <c r="D2" s="44" t="s">
-        <v>263</v>
-      </c>
-      <c r="E2" s="48" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="F2" s="48" t="b">
+      <c r="E2" s="49" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="F2" s="49" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="G2" s="48" t="b">
+      <c r="G2" s="49" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="44" t="s">
+      <c r="A3" s="45" t="s">
         <v>102</v>
       </c>
-      <c r="B3" s="44" t="s">
+      <c r="B3" s="45" t="s">
+        <v>262</v>
+      </c>
+      <c r="C3" s="45" t="s">
+        <v>263</v>
+      </c>
+      <c r="D3" s="45" t="s">
         <v>264</v>
       </c>
-      <c r="C3" s="44" t="s">
-        <v>265</v>
-      </c>
-      <c r="D3" s="44" t="s">
-        <v>266</v>
-      </c>
-      <c r="E3" s="48" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="F3" s="48" t="b">
+      <c r="E3" s="49" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="F3" s="49" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="G3" s="48" t="b">
+      <c r="G3" s="49" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="44" t="s">
-        <v>217</v>
-      </c>
-      <c r="B4" s="44" t="s">
+      <c r="A4" s="45" t="s">
+        <v>215</v>
+      </c>
+      <c r="B4" s="45" t="s">
+        <v>265</v>
+      </c>
+      <c r="C4" s="45" t="s">
+        <v>266</v>
+      </c>
+      <c r="D4" s="45" t="s">
         <v>267</v>
       </c>
-      <c r="C4" s="44" t="s">
-        <v>268</v>
-      </c>
-      <c r="D4" s="44" t="s">
-        <v>269</v>
-      </c>
-      <c r="E4" s="48" t="b">
+      <c r="E4" s="49" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="F4" s="48" t="b">
+      <c r="F4" s="49" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="G4" s="48" t="b">
+      <c r="G4" s="49" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -4789,126 +4789,126 @@
   <dimension ref="A1:F51"/>
   <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="49" width="21.3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="49" width="15.72"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="49" width="23.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="49" width="19.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="49" width="24.29"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="7" style="49" width="9.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="50" width="21.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="50" width="15.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="50" width="23.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="50" width="19.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="50" width="24.29"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="7" style="50" width="9.14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="50" t="s">
-        <v>270</v>
-      </c>
-      <c r="B1" s="50" t="s">
-        <v>223</v>
-      </c>
-      <c r="C1" s="50" t="s">
+      <c r="A1" s="51" t="s">
+        <v>268</v>
+      </c>
+      <c r="B1" s="51" t="s">
+        <v>221</v>
+      </c>
+      <c r="C1" s="51" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="50" t="s">
+      <c r="D1" s="51" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="50" t="s">
-        <v>271</v>
-      </c>
-      <c r="F1" s="50" t="s">
+      <c r="E1" s="51" t="s">
+        <v>269</v>
+      </c>
+      <c r="F1" s="51" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>274</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>274</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>275</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>276</v>
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
     </row>
     <row r="4" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
     </row>
     <row r="5" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>279</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>280</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>281</v>
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
     </row>
     <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>282</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>282</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>283</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>284</v>
       </c>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
     </row>
     <row r="7" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>285</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>285</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>286</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>287</v>
       </c>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
@@ -4921,7 +4921,7 @@
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
       <c r="E8" s="1" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="F8" s="1"/>
     </row>
@@ -4933,13 +4933,13 @@
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
       <c r="E9" s="1" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="F9" s="1"/>
     </row>
     <row r="10" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
@@ -4951,13 +4951,13 @@
     </row>
     <row r="11" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
       <c r="E11" s="1" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="F11" s="1"/>
     </row>
@@ -4969,7 +4969,7 @@
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
       <c r="E12" s="1" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="F12" s="1"/>
     </row>
@@ -4981,7 +4981,7 @@
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
       <c r="E13" s="1" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="F13" s="1"/>
     </row>
@@ -4993,7 +4993,7 @@
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
       <c r="E14" s="1" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="F14" s="1"/>
     </row>
@@ -5002,13 +5002,13 @@
         <v>116</v>
       </c>
       <c r="B15" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="D15" s="1" t="s">
         <v>288</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>289</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>290</v>
       </c>
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
@@ -5018,13 +5018,13 @@
         <v>116</v>
       </c>
       <c r="B16" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="D16" s="1" t="s">
         <v>291</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>292</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>293</v>
       </c>
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
@@ -5037,7 +5037,7 @@
       <c r="C17" s="1"/>
       <c r="D17" s="1"/>
       <c r="E17" s="1" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="F17" s="1"/>
     </row>
@@ -5046,13 +5046,13 @@
         <v>125</v>
       </c>
       <c r="B18" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="D18" s="1" t="s">
         <v>294</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>295</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>296</v>
       </c>
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
@@ -5062,13 +5062,13 @@
         <v>125</v>
       </c>
       <c r="B19" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="D19" s="1" t="s">
         <v>297</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>298</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>299</v>
       </c>
       <c r="E19" s="1"/>
       <c r="F19" s="1"/>
@@ -5081,7 +5081,7 @@
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
       <c r="E20" s="1" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="F20" s="1"/>
     </row>
@@ -5090,17 +5090,17 @@
         <v>132</v>
       </c>
       <c r="B21" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="D21" s="1" t="s">
         <v>300</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>302</v>
       </c>
       <c r="E21" s="1"/>
       <c r="F21" s="1" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5108,17 +5108,17 @@
         <v>132</v>
       </c>
       <c r="B22" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="D22" s="1" t="s">
         <v>303</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>304</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>305</v>
       </c>
       <c r="E22" s="1"/>
       <c r="F22" s="1" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5126,17 +5126,17 @@
         <v>132</v>
       </c>
       <c r="B23" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="D23" s="1" t="s">
         <v>306</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>307</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>308</v>
       </c>
       <c r="E23" s="1"/>
       <c r="F23" s="1" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5144,13 +5144,13 @@
         <v>132</v>
       </c>
       <c r="B24" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="D24" s="1" t="s">
         <v>309</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>310</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>311</v>
       </c>
       <c r="E24" s="1"/>
       <c r="F24" s="1"/>
@@ -5160,17 +5160,17 @@
         <v>132</v>
       </c>
       <c r="B25" s="1" t="s">
+        <v>310</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>311</v>
+      </c>
+      <c r="D25" s="1" t="s">
         <v>312</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>313</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>314</v>
       </c>
       <c r="E25" s="1"/>
       <c r="F25" s="1" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5181,396 +5181,396 @@
       <c r="C26" s="1"/>
       <c r="D26" s="1"/>
       <c r="E26" s="1" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="F26" s="1"/>
     </row>
     <row r="27" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
     </row>
     <row r="28" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="E28" s="1"/>
       <c r="F28" s="1"/>
     </row>
     <row r="29" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="E29" s="1"/>
       <c r="F29" s="1"/>
     </row>
     <row r="30" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="E30" s="1"/>
       <c r="F30" s="1"/>
     </row>
     <row r="31" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="E31" s="1"/>
       <c r="F31" s="1"/>
     </row>
     <row r="32" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B32" s="1" t="s">
+        <v>323</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="D32" s="1" t="s">
         <v>325</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>326</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>327</v>
       </c>
       <c r="E32" s="1"/>
       <c r="F32" s="1" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B33" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="D33" s="1" t="s">
         <v>328</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>329</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>330</v>
       </c>
       <c r="E33" s="1"/>
       <c r="F33" s="1"/>
     </row>
     <row r="34" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B34" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="D34" s="1" t="s">
         <v>331</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>332</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>333</v>
       </c>
       <c r="E34" s="1"/>
       <c r="F34" s="1"/>
     </row>
     <row r="35" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B35" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>333</v>
+      </c>
+      <c r="D35" s="1" t="s">
         <v>334</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>335</v>
-      </c>
-      <c r="D35" s="1" t="s">
-        <v>336</v>
       </c>
       <c r="E35" s="1"/>
       <c r="F35" s="1"/>
     </row>
     <row r="36" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B36" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>336</v>
+      </c>
+      <c r="D36" s="1" t="s">
         <v>337</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>338</v>
-      </c>
-      <c r="D36" s="1" t="s">
-        <v>339</v>
       </c>
       <c r="E36" s="1"/>
       <c r="F36" s="1"/>
     </row>
     <row r="37" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B37" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="D37" s="1" t="s">
         <v>340</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>341</v>
-      </c>
-      <c r="D37" s="1" t="s">
-        <v>342</v>
       </c>
       <c r="E37" s="1"/>
       <c r="F37" s="1"/>
     </row>
     <row r="38" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="E38" s="1"/>
       <c r="F38" s="1"/>
     </row>
     <row r="39" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B39" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="D39" s="1" t="s">
         <v>343</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>344</v>
-      </c>
-      <c r="D39" s="1" t="s">
-        <v>345</v>
       </c>
       <c r="E39" s="1"/>
       <c r="F39" s="1"/>
     </row>
     <row r="40" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="B40" s="1"/>
       <c r="C40" s="1"/>
       <c r="D40" s="1"/>
       <c r="E40" s="1" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="F40" s="1"/>
     </row>
     <row r="41" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="B41" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="D41" s="1" t="s">
         <v>346</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>347</v>
-      </c>
-      <c r="D41" s="1" t="s">
-        <v>348</v>
       </c>
       <c r="E41" s="1"/>
       <c r="F41" s="1"/>
     </row>
     <row r="42" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="B42" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="D42" s="1" t="s">
         <v>349</v>
-      </c>
-      <c r="C42" s="1" t="s">
-        <v>350</v>
-      </c>
-      <c r="D42" s="1" t="s">
-        <v>351</v>
       </c>
       <c r="E42" s="1"/>
       <c r="F42" s="1"/>
     </row>
     <row r="43" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="B43" s="1"/>
       <c r="C43" s="1"/>
       <c r="D43" s="1"/>
       <c r="E43" s="1" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="F43" s="1"/>
     </row>
     <row r="44" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="E44" s="1"/>
       <c r="F44" s="1"/>
     </row>
     <row r="45" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="E45" s="1"/>
       <c r="F45" s="1"/>
     </row>
     <row r="46" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="E46" s="1"/>
       <c r="F46" s="1"/>
     </row>
     <row r="47" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B47" s="1" t="s">
+        <v>356</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>357</v>
+      </c>
+      <c r="D47" s="1" t="s">
         <v>358</v>
-      </c>
-      <c r="C47" s="1" t="s">
-        <v>359</v>
-      </c>
-      <c r="D47" s="1" t="s">
-        <v>360</v>
       </c>
       <c r="E47" s="1"/>
       <c r="F47" s="1"/>
     </row>
     <row r="48" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B48" s="1" t="s">
+        <v>359</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="D48" s="1" t="s">
         <v>361</v>
-      </c>
-      <c r="C48" s="1" t="s">
-        <v>362</v>
-      </c>
-      <c r="D48" s="1" t="s">
-        <v>363</v>
       </c>
       <c r="E48" s="1"/>
       <c r="F48" s="1"/>
     </row>
     <row r="49" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="49" t="s">
-        <v>176</v>
-      </c>
-      <c r="B49" s="49" t="s">
-        <v>251</v>
-      </c>
-      <c r="C49" s="49" t="s">
+      <c r="A49" s="50" t="s">
+        <v>174</v>
+      </c>
+      <c r="B49" s="50" t="s">
+        <v>249</v>
+      </c>
+      <c r="C49" s="50" t="s">
+        <v>362</v>
+      </c>
+      <c r="D49" s="50" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="50" t="s">
+        <v>174</v>
+      </c>
+      <c r="B50" s="50" t="s">
+        <v>250</v>
+      </c>
+      <c r="C50" s="50" t="s">
+        <v>363</v>
+      </c>
+      <c r="D50" s="50" t="s">
         <v>364</v>
       </c>
-      <c r="D49" s="49" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="49" t="s">
-        <v>176</v>
-      </c>
-      <c r="B50" s="49" t="s">
-        <v>252</v>
-      </c>
-      <c r="C50" s="49" t="s">
+    </row>
+    <row r="51" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="50" t="s">
+        <v>174</v>
+      </c>
+      <c r="B51" s="50" t="s">
+        <v>359</v>
+      </c>
+      <c r="C51" s="50" t="s">
         <v>365</v>
       </c>
-      <c r="D50" s="49" t="s">
+      <c r="D51" s="50" t="s">
         <v>366</v>
-      </c>
-    </row>
-    <row r="51" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="49" t="s">
-        <v>176</v>
-      </c>
-      <c r="B51" s="49" t="s">
-        <v>361</v>
-      </c>
-      <c r="C51" s="49" t="s">
-        <v>367</v>
-      </c>
-      <c r="D51" s="49" t="s">
-        <v>368</v>
       </c>
     </row>
   </sheetData>
@@ -5592,54 +5592,54 @@
   <dimension ref="A1:L1"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="39" width="18.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="39" width="17.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="39" width="13.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="39" width="12.72"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="39" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="39" width="13.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="39" width="14.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="39" width="11.28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="39" width="13.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="39" width="14.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="40" width="18.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="40" width="17.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="40" width="13.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="40" width="12.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="40" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="40" width="13.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="40" width="14.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="40" width="11.28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="40" width="13.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="40" width="14.43"/>
   </cols>
   <sheetData>
-    <row r="1" s="50" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="51" t="s">
+    <row r="1" s="51" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="52" t="s">
+        <v>367</v>
+      </c>
+      <c r="B1" s="52" t="s">
+        <v>368</v>
+      </c>
+      <c r="C1" s="52" t="s">
         <v>369</v>
       </c>
-      <c r="B1" s="51" t="s">
+      <c r="D1" s="52" t="s">
         <v>370</v>
       </c>
-      <c r="C1" s="51" t="s">
+      <c r="E1" s="52" t="s">
         <v>371</v>
       </c>
-      <c r="D1" s="51" t="s">
+      <c r="F1" s="52" t="s">
         <v>372</v>
       </c>
-      <c r="E1" s="51" t="s">
+      <c r="G1" s="52" t="s">
         <v>373</v>
       </c>
-      <c r="F1" s="51" t="s">
+      <c r="H1" s="52" t="s">
         <v>374</v>
       </c>
-      <c r="G1" s="51" t="s">
+      <c r="I1" s="52" t="s">
         <v>375</v>
       </c>
-      <c r="H1" s="51" t="s">
+      <c r="J1" s="52" t="s">
         <v>376</v>
       </c>
-      <c r="I1" s="51" t="s">
+      <c r="K1" s="52" t="s">
         <v>377</v>
       </c>
-      <c r="J1" s="51" t="s">
+      <c r="L1" s="51" t="s">
         <v>378</v>
-      </c>
-      <c r="K1" s="51" t="s">
-        <v>379</v>
-      </c>
-      <c r="L1" s="50" t="s">
-        <v>380</v>
       </c>
     </row>
   </sheetData>
@@ -5662,10 +5662,10 @@
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10.34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="39" width="32.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="39" width="43.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="39" width="46.08"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="39" width="28.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="40" width="32.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="40" width="43.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="40" width="46.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="40" width="28.55"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5687,39 +5687,39 @@
       <c r="F1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="39"/>
+      <c r="G1" s="40"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="52" t="s">
+      <c r="A2" s="53" t="s">
         <v>102</v>
       </c>
-      <c r="B2" s="53" t="s">
+      <c r="B2" s="54" t="s">
+        <v>379</v>
+      </c>
+      <c r="C2" s="53" t="s">
+        <v>380</v>
+      </c>
+      <c r="D2" s="53" t="s">
         <v>381</v>
       </c>
-      <c r="C2" s="52" t="s">
+      <c r="E2" s="53"/>
+      <c r="F2" s="53"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="53" t="s">
+        <v>102</v>
+      </c>
+      <c r="B3" s="54" t="s">
         <v>382</v>
       </c>
-      <c r="D2" s="52" t="s">
+      <c r="C3" s="53" t="s">
         <v>383</v>
       </c>
-      <c r="E2" s="52"/>
-      <c r="F2" s="52"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="52" t="s">
-        <v>102</v>
-      </c>
-      <c r="B3" s="53" t="s">
+      <c r="D3" s="53" t="s">
         <v>384</v>
       </c>
-      <c r="C3" s="52" t="s">
-        <v>133</v>
-      </c>
-      <c r="D3" s="52" t="s">
-        <v>134</v>
-      </c>
-      <c r="E3" s="52"/>
-      <c r="F3" s="52"/>
+      <c r="E3" s="53"/>
+      <c r="F3" s="53"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Generator: Support label_one support with choices YAML generation
- Refactored the `generate_choices` and `generate_choices_yaml_locales` functions to include support for an additional label field, `label_one`, allowing for number of persons in the household support.
- Modified tests to validate the inclusion of `label_one` in the generated YAML files and adjusted existing test cases to accommodate the new structure.
</commit_message>
<xml_diff>
--- a/example/demo_generator/references/Household_Travel_Generate_Survey.xlsx
+++ b/example/demo_generator/references/Household_Travel_Generate_Survey.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Widgets" sheetId="1" state="visible" r:id="rId3"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="679" uniqueCount="385">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="681" uniqueCount="385">
   <si>
     <t xml:space="preserve">questionName</t>
   </si>
@@ -1331,6 +1331,7 @@
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="9"/>
@@ -1474,7 +1475,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="53">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1572,10 +1573,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1689,10 +1686,6 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -2647,7 +2640,7 @@
       <c r="Q12" s="7"/>
       <c r="R12" s="7"/>
       <c r="S12" s="7"/>
-      <c r="T12" s="7" t="b">
+      <c r="T12" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2698,7 +2691,7 @@
       <c r="Q13" s="7"/>
       <c r="R13" s="7"/>
       <c r="S13" s="7"/>
-      <c r="T13" s="7" t="b">
+      <c r="T13" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2749,7 +2742,7 @@
       <c r="Q14" s="7"/>
       <c r="R14" s="7"/>
       <c r="S14" s="7"/>
-      <c r="T14" s="7" t="b">
+      <c r="T14" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2798,7 +2791,7 @@
       <c r="Q15" s="7"/>
       <c r="R15" s="7"/>
       <c r="S15" s="7"/>
-      <c r="T15" s="7" t="b">
+      <c r="T15" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2894,7 +2887,7 @@
       <c r="Q17" s="7"/>
       <c r="R17" s="7"/>
       <c r="S17" s="7"/>
-      <c r="T17" s="7" t="b">
+      <c r="T17" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -3025,7 +3018,7 @@
       <c r="Q20" s="23"/>
       <c r="R20" s="23"/>
       <c r="S20" s="23"/>
-      <c r="T20" s="19" t="b">
+      <c r="T20" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -3256,15 +3249,15 @@
       <c r="F25" s="23" t="s">
         <v>132</v>
       </c>
-      <c r="G25" s="25"/>
-      <c r="H25" s="25"/>
+      <c r="G25" s="19"/>
+      <c r="H25" s="19"/>
       <c r="I25" s="19"/>
       <c r="J25" s="19"/>
-      <c r="K25" s="26" t="s">
+      <c r="K25" s="25" t="s">
         <v>133</v>
       </c>
       <c r="L25" s="23"/>
-      <c r="M25" s="27" t="s">
+      <c r="M25" s="26" t="s">
         <v>134</v>
       </c>
       <c r="N25" s="23"/>
@@ -3305,7 +3298,7 @@
       <c r="E26" s="23" t="s">
         <v>101</v>
       </c>
-      <c r="F26" s="28" t="s">
+      <c r="F26" s="27" t="s">
         <v>138</v>
       </c>
       <c r="G26" s="19" t="s">
@@ -3429,7 +3422,7 @@
       <c r="Q28" s="23"/>
       <c r="R28" s="23"/>
       <c r="S28" s="23"/>
-      <c r="T28" s="19" t="b">
+      <c r="T28" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -3439,7 +3432,7 @@
       <c r="X28" s="23"/>
     </row>
     <row r="29" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="29" t="s">
+      <c r="A29" s="28" t="s">
         <v>152</v>
       </c>
       <c r="B29" s="19" t="s">
@@ -3690,7 +3683,7 @@
       <c r="A34" s="19" t="s">
         <v>180</v>
       </c>
-      <c r="B34" s="30" t="s">
+      <c r="B34" s="29" t="s">
         <v>69</v>
       </c>
       <c r="C34" s="21" t="b">
@@ -3790,7 +3783,7 @@
       <c r="A36" s="19" t="s">
         <v>191</v>
       </c>
-      <c r="B36" s="30" t="s">
+      <c r="B36" s="29" t="s">
         <v>69</v>
       </c>
       <c r="C36" s="21" t="b">
@@ -3818,13 +3811,13 @@
       <c r="J36" s="19" t="s">
         <v>196</v>
       </c>
-      <c r="K36" s="31"/>
-      <c r="L36" s="32"/>
-      <c r="M36" s="31"/>
-      <c r="N36" s="32"/>
-      <c r="O36" s="32"/>
-      <c r="P36" s="32"/>
-      <c r="Q36" s="32"/>
+      <c r="K36" s="30"/>
+      <c r="L36" s="31"/>
+      <c r="M36" s="30"/>
+      <c r="N36" s="31"/>
+      <c r="O36" s="31"/>
+      <c r="P36" s="31"/>
+      <c r="Q36" s="31"/>
       <c r="R36" s="23"/>
       <c r="S36" s="23"/>
       <c r="T36" s="21" t="b">
@@ -3837,7 +3830,7 @@
       <c r="X36" s="23"/>
     </row>
     <row r="37" customFormat="false" ht="86.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="29" t="s">
+      <c r="A37" s="28" t="s">
         <v>197</v>
       </c>
       <c r="B37" s="19" t="s">
@@ -3868,14 +3861,14 @@
       <c r="L37" s="23"/>
       <c r="M37" s="24"/>
       <c r="N37" s="24"/>
-      <c r="O37" s="33" t="s">
+      <c r="O37" s="32" t="s">
         <v>146</v>
       </c>
       <c r="P37" s="23"/>
       <c r="Q37" s="23"/>
       <c r="R37" s="23"/>
       <c r="S37" s="23"/>
-      <c r="T37" s="19" t="b">
+      <c r="T37" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -3885,7 +3878,7 @@
       <c r="X37" s="23"/>
     </row>
     <row r="38" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="29" t="s">
+      <c r="A38" s="28" t="s">
         <v>201</v>
       </c>
       <c r="B38" s="19" t="s">
@@ -3916,7 +3909,7 @@
       <c r="L38" s="23"/>
       <c r="M38" s="24"/>
       <c r="N38" s="24"/>
-      <c r="O38" s="33" t="s">
+      <c r="O38" s="32" t="s">
         <v>146</v>
       </c>
       <c r="P38" s="23"/>
@@ -3933,7 +3926,7 @@
       <c r="X38" s="23"/>
     </row>
     <row r="39" customFormat="false" ht="64.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="29" t="s">
+      <c r="A39" s="28" t="s">
         <v>205</v>
       </c>
       <c r="B39" s="19" t="s">
@@ -3964,7 +3957,7 @@
       <c r="L39" s="23"/>
       <c r="M39" s="24"/>
       <c r="N39" s="24"/>
-      <c r="O39" s="33" t="s">
+      <c r="O39" s="32" t="s">
         <v>146</v>
       </c>
       <c r="P39" s="23"/>
@@ -3981,7 +3974,7 @@
       <c r="X39" s="23"/>
     </row>
     <row r="40" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="29" t="s">
+      <c r="A40" s="28" t="s">
         <v>209</v>
       </c>
       <c r="B40" s="19" t="s">
@@ -4012,7 +4005,7 @@
       <c r="L40" s="23"/>
       <c r="M40" s="24"/>
       <c r="N40" s="24"/>
-      <c r="O40" s="33" t="s">
+      <c r="O40" s="32" t="s">
         <v>146</v>
       </c>
       <c r="P40" s="23"/>
@@ -4029,49 +4022,49 @@
       <c r="X40" s="23"/>
     </row>
     <row r="41" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="34" t="s">
+      <c r="A41" s="33" t="s">
         <v>213</v>
       </c>
-      <c r="B41" s="34" t="s">
+      <c r="B41" s="33" t="s">
         <v>98</v>
       </c>
-      <c r="C41" s="35" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D41" s="34" t="s">
+      <c r="C41" s="34" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D41" s="33" t="s">
         <v>102</v>
       </c>
-      <c r="E41" s="36"/>
-      <c r="F41" s="36" t="str">
+      <c r="E41" s="35"/>
+      <c r="F41" s="35" t="str">
         <f aca="false">REPLACE(A41, FIND("_", A41), 1, ".")</f>
         <v>household.save</v>
       </c>
-      <c r="G41" s="34" t="s">
+      <c r="G41" s="33" t="s">
         <v>99</v>
       </c>
-      <c r="H41" s="34" t="s">
+      <c r="H41" s="33" t="s">
         <v>100</v>
       </c>
-      <c r="I41" s="34"/>
-      <c r="J41" s="34"/>
-      <c r="K41" s="34"/>
-      <c r="L41" s="36"/>
-      <c r="M41" s="36"/>
-      <c r="N41" s="36"/>
-      <c r="O41" s="36"/>
-      <c r="P41" s="36"/>
-      <c r="Q41" s="36"/>
-      <c r="R41" s="36"/>
-      <c r="S41" s="36"/>
-      <c r="T41" s="35" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U41" s="36"/>
-      <c r="V41" s="36"/>
-      <c r="W41" s="36"/>
-      <c r="X41" s="36"/>
+      <c r="I41" s="33"/>
+      <c r="J41" s="33"/>
+      <c r="K41" s="33"/>
+      <c r="L41" s="35"/>
+      <c r="M41" s="35"/>
+      <c r="N41" s="35"/>
+      <c r="O41" s="35"/>
+      <c r="P41" s="35"/>
+      <c r="Q41" s="35"/>
+      <c r="R41" s="35"/>
+      <c r="S41" s="35"/>
+      <c r="T41" s="34" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U41" s="35"/>
+      <c r="V41" s="35"/>
+      <c r="W41" s="35"/>
+      <c r="X41" s="35"/>
     </row>
     <row r="42" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
@@ -4080,7 +4073,7 @@
       <c r="B42" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C42" s="37" t="b">
+      <c r="C42" s="36" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -4096,9 +4089,9 @@
       <c r="H42" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="L42" s="38"/>
-      <c r="M42" s="39"/>
-      <c r="T42" s="37" t="b">
+      <c r="L42" s="37"/>
+      <c r="M42" s="38"/>
+      <c r="T42" s="36" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -4155,485 +4148,485 @@
   <dimension ref="A1:F29"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="40" width="27.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="40" width="15.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="40" width="31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="41" width="20.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="40" width="19.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="40" width="12.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="39" width="27.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="39" width="15.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="39" width="31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="40" width="20.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="39" width="19.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="39" width="12.14"/>
   </cols>
   <sheetData>
-    <row r="1" s="44" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="42" t="s">
+    <row r="1" s="43" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="41" t="s">
         <v>218</v>
       </c>
-      <c r="B1" s="42" t="s">
+      <c r="B1" s="41" t="s">
         <v>219</v>
       </c>
-      <c r="C1" s="42" t="s">
+      <c r="C1" s="41" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="43" t="s">
+      <c r="D1" s="42" t="s">
         <v>220</v>
       </c>
-      <c r="E1" s="42" t="s">
+      <c r="E1" s="41" t="s">
         <v>221</v>
       </c>
-      <c r="F1" s="42" t="s">
+      <c r="F1" s="41" t="s">
         <v>222</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="45" t="s">
+      <c r="A2" s="44" t="s">
         <v>223</v>
       </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45" t="s">
+      <c r="B2" s="44"/>
+      <c r="C2" s="44" t="s">
         <v>224</v>
       </c>
-      <c r="D2" s="46" t="s">
+      <c r="D2" s="45" t="s">
         <v>225</v>
       </c>
-      <c r="E2" s="45" t="n">
-        <v>1</v>
-      </c>
-      <c r="F2" s="45"/>
+      <c r="E2" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="44"/>
     </row>
     <row r="3" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="45" t="s">
+      <c r="A3" s="44" t="s">
         <v>95</v>
       </c>
-      <c r="B3" s="45"/>
-      <c r="C3" s="45" t="s">
+      <c r="B3" s="44"/>
+      <c r="C3" s="44" t="s">
         <v>224</v>
       </c>
-      <c r="D3" s="46" t="s">
+      <c r="D3" s="45" t="s">
         <v>226</v>
       </c>
-      <c r="E3" s="45" t="n">
+      <c r="E3" s="44" t="n">
         <v>2</v>
       </c>
-      <c r="F3" s="45"/>
+      <c r="F3" s="44"/>
     </row>
     <row r="4" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="45" t="s">
+      <c r="A4" s="44" t="s">
         <v>163</v>
       </c>
-      <c r="B4" s="45"/>
-      <c r="C4" s="45" t="s">
+      <c r="B4" s="44"/>
+      <c r="C4" s="44" t="s">
         <v>227</v>
       </c>
-      <c r="D4" s="46" t="s">
+      <c r="D4" s="45" t="s">
         <v>225</v>
       </c>
-      <c r="E4" s="45" t="s">
+      <c r="E4" s="44" t="s">
         <v>228</v>
       </c>
-      <c r="F4" s="45"/>
+      <c r="F4" s="44"/>
     </row>
     <row r="5" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="45" t="s">
+      <c r="A5" s="44" t="s">
         <v>163</v>
       </c>
-      <c r="B5" s="45" t="s">
+      <c r="B5" s="44" t="s">
         <v>229</v>
       </c>
-      <c r="C5" s="45" t="s">
+      <c r="C5" s="44" t="s">
         <v>224</v>
       </c>
-      <c r="D5" s="46" t="s">
+      <c r="D5" s="45" t="s">
         <v>225</v>
       </c>
-      <c r="E5" s="45" t="n">
-        <v>1</v>
-      </c>
-      <c r="F5" s="45"/>
+      <c r="E5" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="44"/>
     </row>
     <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="45" t="s">
+      <c r="A6" s="44" t="s">
         <v>230</v>
       </c>
-      <c r="B6" s="45"/>
-      <c r="C6" s="45" t="s">
+      <c r="B6" s="44"/>
+      <c r="C6" s="44" t="s">
         <v>231</v>
       </c>
-      <c r="D6" s="46" t="s">
+      <c r="D6" s="45" t="s">
         <v>226</v>
       </c>
-      <c r="E6" s="45" t="n">
+      <c r="E6" s="44" t="n">
         <v>3</v>
       </c>
-      <c r="F6" s="45"/>
+      <c r="F6" s="44"/>
     </row>
     <row r="7" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="45" t="s">
+      <c r="A7" s="44" t="s">
         <v>230</v>
       </c>
-      <c r="B7" s="45" t="s">
+      <c r="B7" s="44" t="s">
         <v>232</v>
       </c>
-      <c r="C7" s="45" t="s">
+      <c r="C7" s="44" t="s">
         <v>231</v>
       </c>
-      <c r="D7" s="46" t="s">
+      <c r="D7" s="45" t="s">
         <v>233</v>
       </c>
-      <c r="E7" s="45" t="n">
+      <c r="E7" s="44" t="n">
         <v>5</v>
       </c>
-      <c r="F7" s="45"/>
+      <c r="F7" s="44"/>
     </row>
     <row r="8" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="45" t="s">
+      <c r="A8" s="44" t="s">
         <v>234</v>
       </c>
-      <c r="B8" s="45"/>
-      <c r="C8" s="45" t="s">
+      <c r="B8" s="44"/>
+      <c r="C8" s="44" t="s">
         <v>231</v>
       </c>
-      <c r="D8" s="46" t="s">
+      <c r="D8" s="45" t="s">
         <v>226</v>
       </c>
-      <c r="E8" s="45" t="n">
+      <c r="E8" s="44" t="n">
         <v>4</v>
       </c>
-      <c r="F8" s="45"/>
+      <c r="F8" s="44"/>
     </row>
     <row r="9" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="45" t="s">
+      <c r="A9" s="44" t="s">
         <v>234</v>
       </c>
-      <c r="B9" s="45" t="s">
+      <c r="B9" s="44" t="s">
         <v>232</v>
       </c>
-      <c r="C9" s="45" t="s">
+      <c r="C9" s="44" t="s">
         <v>231</v>
       </c>
-      <c r="D9" s="46" t="s">
+      <c r="D9" s="45" t="s">
         <v>233</v>
       </c>
-      <c r="E9" s="45" t="n">
+      <c r="E9" s="44" t="n">
         <v>13</v>
       </c>
-      <c r="F9" s="45"/>
+      <c r="F9" s="44"/>
     </row>
     <row r="10" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="45" t="s">
+      <c r="A10" s="44" t="s">
         <v>235</v>
       </c>
-      <c r="B10" s="45"/>
-      <c r="C10" s="45" t="s">
+      <c r="B10" s="44"/>
+      <c r="C10" s="44" t="s">
         <v>231</v>
       </c>
-      <c r="D10" s="46" t="s">
+      <c r="D10" s="45" t="s">
         <v>233</v>
       </c>
-      <c r="E10" s="45" t="n">
+      <c r="E10" s="44" t="n">
         <v>5</v>
       </c>
-      <c r="F10" s="45"/>
+      <c r="F10" s="44"/>
     </row>
     <row r="11" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="45" t="s">
+      <c r="A11" s="44" t="s">
         <v>119</v>
       </c>
-      <c r="B11" s="45"/>
-      <c r="C11" s="45" t="s">
+      <c r="B11" s="44"/>
+      <c r="C11" s="44" t="s">
         <v>231</v>
       </c>
-      <c r="D11" s="46" t="s">
+      <c r="D11" s="45" t="s">
         <v>226</v>
       </c>
-      <c r="E11" s="45" t="n">
+      <c r="E11" s="44" t="n">
         <v>5</v>
       </c>
-      <c r="F11" s="45"/>
+      <c r="F11" s="44"/>
     </row>
     <row r="12" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="45" t="s">
+      <c r="A12" s="44" t="s">
         <v>157</v>
       </c>
-      <c r="B12" s="45"/>
-      <c r="C12" s="45" t="s">
+      <c r="B12" s="44"/>
+      <c r="C12" s="44" t="s">
         <v>231</v>
       </c>
-      <c r="D12" s="46" t="s">
+      <c r="D12" s="45" t="s">
         <v>226</v>
       </c>
-      <c r="E12" s="45" t="n">
+      <c r="E12" s="44" t="n">
         <v>6</v>
       </c>
-      <c r="F12" s="45"/>
+      <c r="F12" s="44"/>
     </row>
     <row r="13" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="45" t="s">
+      <c r="A13" s="44" t="s">
         <v>236</v>
       </c>
-      <c r="B13" s="45"/>
-      <c r="C13" s="45" t="s">
+      <c r="B13" s="44"/>
+      <c r="C13" s="44" t="s">
         <v>231</v>
       </c>
-      <c r="D13" s="46" t="s">
+      <c r="D13" s="45" t="s">
         <v>226</v>
       </c>
-      <c r="E13" s="45" t="n">
+      <c r="E13" s="44" t="n">
         <v>11</v>
       </c>
-      <c r="F13" s="45"/>
+      <c r="F13" s="44"/>
     </row>
     <row r="14" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="45" t="s">
+      <c r="A14" s="44" t="s">
         <v>124</v>
       </c>
-      <c r="B14" s="45"/>
-      <c r="C14" s="45" t="s">
+      <c r="B14" s="44"/>
+      <c r="C14" s="44" t="s">
         <v>231</v>
       </c>
-      <c r="D14" s="46" t="s">
+      <c r="D14" s="45" t="s">
         <v>226</v>
       </c>
-      <c r="E14" s="45" t="n">
+      <c r="E14" s="44" t="n">
         <v>14</v>
       </c>
-      <c r="F14" s="45"/>
+      <c r="F14" s="44"/>
     </row>
     <row r="15" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="45" t="s">
+      <c r="A15" s="44" t="s">
         <v>134</v>
       </c>
-      <c r="B15" s="45"/>
-      <c r="C15" s="45" t="s">
+      <c r="B15" s="44"/>
+      <c r="C15" s="44" t="s">
         <v>231</v>
       </c>
-      <c r="D15" s="46" t="s">
+      <c r="D15" s="45" t="s">
         <v>233</v>
       </c>
-      <c r="E15" s="45" t="n">
+      <c r="E15" s="44" t="n">
         <v>15</v>
       </c>
-      <c r="F15" s="45"/>
+      <c r="F15" s="44"/>
     </row>
     <row r="16" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="45" t="s">
+      <c r="A16" s="44" t="s">
         <v>134</v>
       </c>
-      <c r="B16" s="45"/>
-      <c r="C16" s="45" t="s">
+      <c r="B16" s="44"/>
+      <c r="C16" s="44" t="s">
         <v>231</v>
       </c>
-      <c r="D16" s="46" t="s">
+      <c r="D16" s="45" t="s">
         <v>237</v>
       </c>
-      <c r="E16" s="45" t="s">
+      <c r="E16" s="44" t="s">
         <v>238</v>
       </c>
-      <c r="F16" s="45"/>
+      <c r="F16" s="44"/>
     </row>
     <row r="17" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="45" t="s">
+      <c r="A17" s="44" t="s">
         <v>239</v>
       </c>
-      <c r="B17" s="45"/>
-      <c r="C17" s="45" t="s">
+      <c r="B17" s="44"/>
+      <c r="C17" s="44" t="s">
         <v>231</v>
       </c>
-      <c r="D17" s="46" t="s">
+      <c r="D17" s="45" t="s">
         <v>226</v>
       </c>
-      <c r="E17" s="45" t="n">
+      <c r="E17" s="44" t="n">
         <v>15</v>
       </c>
-      <c r="F17" s="45"/>
+      <c r="F17" s="44"/>
     </row>
     <row r="18" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="45" t="s">
+      <c r="A18" s="44" t="s">
         <v>130</v>
       </c>
-      <c r="B18" s="45"/>
-      <c r="C18" s="45" t="s">
+      <c r="B18" s="44"/>
+      <c r="C18" s="44" t="s">
         <v>231</v>
       </c>
-      <c r="D18" s="46" t="s">
+      <c r="D18" s="45" t="s">
         <v>226</v>
       </c>
-      <c r="E18" s="45" t="n">
+      <c r="E18" s="44" t="n">
         <v>16</v>
       </c>
-      <c r="F18" s="45"/>
+      <c r="F18" s="44"/>
     </row>
     <row r="19" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="45" t="s">
+      <c r="A19" s="44" t="s">
         <v>240</v>
       </c>
-      <c r="B19" s="45"/>
-      <c r="C19" s="45" t="s">
+      <c r="B19" s="44"/>
+      <c r="C19" s="44" t="s">
         <v>231</v>
       </c>
-      <c r="D19" s="46" t="s">
+      <c r="D19" s="45" t="s">
         <v>226</v>
       </c>
-      <c r="E19" s="45" t="n">
+      <c r="E19" s="44" t="n">
         <v>40</v>
       </c>
-      <c r="F19" s="45"/>
+      <c r="F19" s="44"/>
     </row>
     <row r="20" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="45" t="s">
+      <c r="A20" s="44" t="s">
         <v>151</v>
       </c>
-      <c r="B20" s="45"/>
-      <c r="C20" s="45" t="s">
+      <c r="B20" s="44"/>
+      <c r="C20" s="44" t="s">
         <v>241</v>
       </c>
-      <c r="D20" s="46" t="s">
+      <c r="D20" s="45" t="s">
         <v>225</v>
       </c>
-      <c r="E20" s="45" t="s">
+      <c r="E20" s="44" t="s">
         <v>228</v>
       </c>
-      <c r="F20" s="45"/>
+      <c r="F20" s="44"/>
     </row>
     <row r="21" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="40" t="s">
+      <c r="A21" s="39" t="s">
         <v>168</v>
       </c>
-      <c r="C21" s="40" t="s">
+      <c r="C21" s="39" t="s">
         <v>242</v>
       </c>
-      <c r="D21" s="46" t="s">
+      <c r="D21" s="45" t="s">
         <v>225</v>
       </c>
-      <c r="E21" s="41" t="s">
+      <c r="E21" s="40" t="s">
         <v>243</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="40" t="s">
+      <c r="A22" s="39" t="s">
         <v>168</v>
       </c>
-      <c r="B22" s="40" t="s">
+      <c r="B22" s="39" t="s">
         <v>229</v>
       </c>
-      <c r="C22" s="40" t="s">
+      <c r="C22" s="39" t="s">
         <v>242</v>
       </c>
-      <c r="D22" s="46" t="s">
+      <c r="D22" s="45" t="s">
         <v>225</v>
       </c>
-      <c r="E22" s="41" t="s">
+      <c r="E22" s="40" t="s">
         <v>244</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="40" t="s">
+      <c r="A23" s="39" t="s">
         <v>168</v>
       </c>
-      <c r="B23" s="40" t="s">
+      <c r="B23" s="39" t="s">
         <v>229</v>
       </c>
-      <c r="C23" s="40" t="s">
+      <c r="C23" s="39" t="s">
         <v>242</v>
       </c>
-      <c r="D23" s="46" t="s">
+      <c r="D23" s="45" t="s">
         <v>225</v>
       </c>
-      <c r="E23" s="41" t="s">
+      <c r="E23" s="40" t="s">
         <v>245</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="40" t="s">
+      <c r="A24" s="39" t="s">
         <v>173</v>
       </c>
-      <c r="C24" s="40" t="s">
+      <c r="C24" s="39" t="s">
         <v>242</v>
       </c>
-      <c r="D24" s="46" t="s">
+      <c r="D24" s="45" t="s">
         <v>225</v>
       </c>
-      <c r="E24" s="41" t="s">
+      <c r="E24" s="40" t="s">
         <v>246</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="40" t="s">
+      <c r="A25" s="39" t="s">
         <v>173</v>
       </c>
-      <c r="B25" s="40" t="s">
+      <c r="B25" s="39" t="s">
         <v>229</v>
       </c>
-      <c r="C25" s="40" t="s">
+      <c r="C25" s="39" t="s">
         <v>242</v>
       </c>
-      <c r="D25" s="46" t="s">
+      <c r="D25" s="45" t="s">
         <v>225</v>
       </c>
-      <c r="E25" s="41" t="s">
+      <c r="E25" s="40" t="s">
         <v>247</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="40" t="s">
+      <c r="A26" s="39" t="s">
         <v>173</v>
       </c>
-      <c r="B26" s="40" t="s">
+      <c r="B26" s="39" t="s">
         <v>229</v>
       </c>
-      <c r="C26" s="40" t="s">
+      <c r="C26" s="39" t="s">
         <v>242</v>
       </c>
-      <c r="D26" s="46" t="s">
+      <c r="D26" s="45" t="s">
         <v>225</v>
       </c>
-      <c r="E26" s="41" t="s">
+      <c r="E26" s="40" t="s">
         <v>245</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="40" t="s">
+      <c r="A27" s="39" t="s">
         <v>179</v>
       </c>
-      <c r="C27" s="40" t="s">
+      <c r="C27" s="39" t="s">
         <v>248</v>
       </c>
-      <c r="D27" s="46" t="s">
+      <c r="D27" s="45" t="s">
         <v>225</v>
       </c>
-      <c r="E27" s="40" t="s">
+      <c r="E27" s="39" t="s">
         <v>249</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="40" t="s">
+      <c r="A28" s="39" t="s">
         <v>179</v>
       </c>
-      <c r="B28" s="40" t="s">
+      <c r="B28" s="39" t="s">
         <v>229</v>
       </c>
-      <c r="C28" s="40" t="s">
+      <c r="C28" s="39" t="s">
         <v>248</v>
       </c>
-      <c r="D28" s="46" t="s">
+      <c r="D28" s="45" t="s">
         <v>225</v>
       </c>
-      <c r="E28" s="40" t="s">
+      <c r="E28" s="39" t="s">
         <v>250</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="40" t="s">
+      <c r="A29" s="39" t="s">
         <v>179</v>
       </c>
-      <c r="B29" s="40" t="s">
+      <c r="B29" s="39" t="s">
         <v>229</v>
       </c>
-      <c r="C29" s="40" t="s">
+      <c r="C29" s="39" t="s">
         <v>248</v>
       </c>
-      <c r="D29" s="46" t="s">
+      <c r="D29" s="45" t="s">
         <v>225</v>
       </c>
-      <c r="E29" s="40" t="s">
+      <c r="E29" s="39" t="s">
         <v>251</v>
       </c>
     </row>
@@ -4656,116 +4649,116 @@
   <dimension ref="A1:H4"/>
   <sheetFormatPr defaultColWidth="10.69921875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="45" width="10.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="45" width="12.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="45" width="13.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="45" width="12.57"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="6" min="5" style="45" width="10.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="45" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="45" width="15.43"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="9" style="45" width="10.7"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="44" width="10.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="44" width="12.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="44" width="13.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="44" width="12.57"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="6" min="5" style="44" width="10.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="44" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="44" width="15.43"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="9" style="44" width="10.7"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="47" t="s">
+      <c r="A1" s="46" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="48" t="s">
+      <c r="B1" s="47" t="s">
         <v>252</v>
       </c>
-      <c r="C1" s="47" t="s">
+      <c r="C1" s="46" t="s">
         <v>253</v>
       </c>
-      <c r="D1" s="47" t="s">
+      <c r="D1" s="46" t="s">
         <v>254</v>
       </c>
-      <c r="E1" s="47" t="s">
+      <c r="E1" s="46" t="s">
         <v>255</v>
       </c>
-      <c r="F1" s="47" t="s">
+      <c r="F1" s="46" t="s">
         <v>256</v>
       </c>
       <c r="G1" s="6" t="s">
         <v>257</v>
       </c>
-      <c r="H1" s="47" t="s">
+      <c r="H1" s="46" t="s">
         <v>258</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="45" t="s">
+      <c r="A2" s="44" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="45" t="s">
+      <c r="B2" s="44" t="s">
         <v>259</v>
       </c>
-      <c r="C2" s="45" t="s">
+      <c r="C2" s="44" t="s">
         <v>260</v>
       </c>
-      <c r="D2" s="45" t="s">
+      <c r="D2" s="44" t="s">
         <v>261</v>
       </c>
-      <c r="E2" s="49" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="F2" s="49" t="b">
+      <c r="E2" s="48" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="F2" s="48" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="G2" s="49" t="b">
+      <c r="G2" s="48" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="45" t="s">
+      <c r="A3" s="44" t="s">
         <v>102</v>
       </c>
-      <c r="B3" s="45" t="s">
+      <c r="B3" s="44" t="s">
         <v>262</v>
       </c>
-      <c r="C3" s="45" t="s">
+      <c r="C3" s="44" t="s">
         <v>263</v>
       </c>
-      <c r="D3" s="45" t="s">
+      <c r="D3" s="44" t="s">
         <v>264</v>
       </c>
-      <c r="E3" s="49" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="F3" s="49" t="b">
+      <c r="E3" s="48" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="F3" s="48" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="G3" s="49" t="b">
+      <c r="G3" s="48" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="45" t="s">
+      <c r="A4" s="44" t="s">
         <v>215</v>
       </c>
-      <c r="B4" s="45" t="s">
+      <c r="B4" s="44" t="s">
         <v>265</v>
       </c>
-      <c r="C4" s="45" t="s">
+      <c r="C4" s="44" t="s">
         <v>266</v>
       </c>
-      <c r="D4" s="45" t="s">
+      <c r="D4" s="44" t="s">
         <v>267</v>
       </c>
-      <c r="E4" s="49" t="b">
+      <c r="E4" s="48" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="F4" s="49" t="b">
+      <c r="F4" s="48" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="G4" s="49" t="b">
+      <c r="G4" s="48" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -4786,34 +4779,41 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="50" width="21.3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="50" width="15.72"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="50" width="23.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="50" width="19.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="50" width="24.29"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="7" style="50" width="9.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="49" width="21.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="49" width="15.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="49" width="23.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="49" width="19.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="49" width="21.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="49" width="24.29"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="9" style="49" width="9.14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="51" t="s">
+      <c r="A1" s="50" t="s">
         <v>268</v>
       </c>
-      <c r="B1" s="51" t="s">
+      <c r="B1" s="50" t="s">
         <v>221</v>
       </c>
-      <c r="C1" s="51" t="s">
+      <c r="C1" s="50" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="51" t="s">
+      <c r="D1" s="50" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="51" t="s">
+      <c r="E1" s="50" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" s="50" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" s="50" t="s">
         <v>269</v>
       </c>
-      <c r="F1" s="51" t="s">
+      <c r="H1" s="50" t="s">
         <v>12</v>
       </c>
     </row>
@@ -4832,6 +4832,8 @@
       </c>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
@@ -4848,6 +4850,8 @@
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+      <c r="H3" s="1"/>
     </row>
     <row r="4" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
@@ -4864,6 +4868,8 @@
       </c>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
     </row>
     <row r="5" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
@@ -4880,6 +4886,8 @@
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
     </row>
     <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
@@ -4896,6 +4904,8 @@
       </c>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
     </row>
     <row r="7" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
@@ -4912,6 +4922,8 @@
       </c>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
     </row>
     <row r="8" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
@@ -4920,10 +4932,12 @@
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
-      <c r="E8" s="1" t="s">
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="F8" s="1"/>
+      <c r="H8" s="1"/>
     </row>
     <row r="9" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
@@ -4932,10 +4946,12 @@
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
-      <c r="E9" s="1" t="s">
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1" t="s">
         <v>272</v>
       </c>
-      <c r="F9" s="1"/>
+      <c r="H9" s="1"/>
     </row>
     <row r="10" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
@@ -4944,10 +4960,12 @@
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
-      <c r="E10" s="1" t="s">
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="F10" s="1"/>
+      <c r="H10" s="1"/>
     </row>
     <row r="11" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
@@ -4956,10 +4974,12 @@
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
-      <c r="E11" s="1" t="s">
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="F11" s="1"/>
+      <c r="H11" s="1"/>
     </row>
     <row r="12" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
@@ -4968,10 +4988,12 @@
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
-      <c r="E12" s="1" t="s">
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="F12" s="1"/>
+      <c r="H12" s="1"/>
     </row>
     <row r="13" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
@@ -4980,10 +5002,12 @@
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
-      <c r="E13" s="1" t="s">
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="1" t="s">
         <v>272</v>
       </c>
-      <c r="F13" s="1"/>
+      <c r="H13" s="1"/>
     </row>
     <row r="14" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
@@ -4992,10 +5016,12 @@
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
-      <c r="E14" s="1" t="s">
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1" t="s">
         <v>283</v>
       </c>
-      <c r="F14" s="1"/>
+      <c r="H14" s="1"/>
     </row>
     <row r="15" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
@@ -5012,6 +5038,8 @@
       </c>
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
+      <c r="H15" s="1"/>
     </row>
     <row r="16" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
@@ -5028,6 +5056,8 @@
       </c>
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
+      <c r="H16" s="1"/>
     </row>
     <row r="17" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
@@ -5036,10 +5066,12 @@
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
       <c r="D17" s="1"/>
-      <c r="E17" s="1" t="s">
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1" t="s">
         <v>283</v>
       </c>
-      <c r="F17" s="1"/>
+      <c r="H17" s="1"/>
     </row>
     <row r="18" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
@@ -5056,6 +5088,8 @@
       </c>
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
+      <c r="G18" s="1"/>
+      <c r="H18" s="1"/>
     </row>
     <row r="19" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
@@ -5072,6 +5106,8 @@
       </c>
       <c r="E19" s="1"/>
       <c r="F19" s="1"/>
+      <c r="G19" s="1"/>
+      <c r="H19" s="1"/>
     </row>
     <row r="20" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
@@ -5080,10 +5116,12 @@
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
-      <c r="E20" s="1" t="s">
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
+      <c r="G20" s="1" t="s">
         <v>272</v>
       </c>
-      <c r="F20" s="1"/>
+      <c r="H20" s="1"/>
     </row>
     <row r="21" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
@@ -5099,7 +5137,9 @@
         <v>300</v>
       </c>
       <c r="E21" s="1"/>
-      <c r="F21" s="1" t="s">
+      <c r="F21" s="1"/>
+      <c r="G21" s="1"/>
+      <c r="H21" s="1" t="s">
         <v>235</v>
       </c>
     </row>
@@ -5117,7 +5157,9 @@
         <v>303</v>
       </c>
       <c r="E22" s="1"/>
-      <c r="F22" s="1" t="s">
+      <c r="F22" s="1"/>
+      <c r="G22" s="1"/>
+      <c r="H22" s="1" t="s">
         <v>234</v>
       </c>
     </row>
@@ -5135,7 +5177,9 @@
         <v>306</v>
       </c>
       <c r="E23" s="1"/>
-      <c r="F23" s="1" t="s">
+      <c r="F23" s="1"/>
+      <c r="G23" s="1"/>
+      <c r="H23" s="1" t="s">
         <v>236</v>
       </c>
     </row>
@@ -5154,6 +5198,8 @@
       </c>
       <c r="E24" s="1"/>
       <c r="F24" s="1"/>
+      <c r="G24" s="1"/>
+      <c r="H24" s="1"/>
     </row>
     <row r="25" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
@@ -5169,7 +5215,9 @@
         <v>312</v>
       </c>
       <c r="E25" s="1"/>
-      <c r="F25" s="1" t="s">
+      <c r="F25" s="1"/>
+      <c r="G25" s="1"/>
+      <c r="H25" s="1" t="s">
         <v>239</v>
       </c>
     </row>
@@ -5180,10 +5228,12 @@
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
       <c r="D26" s="1"/>
-      <c r="E26" s="1" t="s">
+      <c r="E26" s="1"/>
+      <c r="F26" s="1"/>
+      <c r="G26" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="F26" s="1"/>
+      <c r="H26" s="1"/>
     </row>
     <row r="27" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
@@ -5200,6 +5250,8 @@
       </c>
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
+      <c r="G27" s="1"/>
+      <c r="H27" s="1"/>
     </row>
     <row r="28" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
@@ -5216,6 +5268,8 @@
       </c>
       <c r="E28" s="1"/>
       <c r="F28" s="1"/>
+      <c r="G28" s="1"/>
+      <c r="H28" s="1"/>
     </row>
     <row r="29" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
@@ -5232,6 +5286,8 @@
       </c>
       <c r="E29" s="1"/>
       <c r="F29" s="1"/>
+      <c r="G29" s="1"/>
+      <c r="H29" s="1"/>
     </row>
     <row r="30" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
@@ -5248,6 +5304,8 @@
       </c>
       <c r="E30" s="1"/>
       <c r="F30" s="1"/>
+      <c r="G30" s="1"/>
+      <c r="H30" s="1"/>
     </row>
     <row r="31" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
@@ -5264,6 +5322,8 @@
       </c>
       <c r="E31" s="1"/>
       <c r="F31" s="1"/>
+      <c r="G31" s="1"/>
+      <c r="H31" s="1"/>
     </row>
     <row r="32" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
@@ -5279,7 +5339,9 @@
         <v>325</v>
       </c>
       <c r="E32" s="1"/>
-      <c r="F32" s="1" t="s">
+      <c r="F32" s="1"/>
+      <c r="G32" s="1"/>
+      <c r="H32" s="1" t="s">
         <v>240</v>
       </c>
     </row>
@@ -5298,6 +5360,8 @@
       </c>
       <c r="E33" s="1"/>
       <c r="F33" s="1"/>
+      <c r="G33" s="1"/>
+      <c r="H33" s="1"/>
     </row>
     <row r="34" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
@@ -5314,6 +5378,8 @@
       </c>
       <c r="E34" s="1"/>
       <c r="F34" s="1"/>
+      <c r="G34" s="1"/>
+      <c r="H34" s="1"/>
     </row>
     <row r="35" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
@@ -5330,6 +5396,8 @@
       </c>
       <c r="E35" s="1"/>
       <c r="F35" s="1"/>
+      <c r="G35" s="1"/>
+      <c r="H35" s="1"/>
     </row>
     <row r="36" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
@@ -5346,6 +5414,8 @@
       </c>
       <c r="E36" s="1"/>
       <c r="F36" s="1"/>
+      <c r="G36" s="1"/>
+      <c r="H36" s="1"/>
     </row>
     <row r="37" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
@@ -5362,6 +5432,8 @@
       </c>
       <c r="E37" s="1"/>
       <c r="F37" s="1"/>
+      <c r="G37" s="1"/>
+      <c r="H37" s="1"/>
     </row>
     <row r="38" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
@@ -5378,6 +5450,8 @@
       </c>
       <c r="E38" s="1"/>
       <c r="F38" s="1"/>
+      <c r="G38" s="1"/>
+      <c r="H38" s="1"/>
     </row>
     <row r="39" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
@@ -5394,6 +5468,8 @@
       </c>
       <c r="E39" s="1"/>
       <c r="F39" s="1"/>
+      <c r="G39" s="1"/>
+      <c r="H39" s="1"/>
     </row>
     <row r="40" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
@@ -5402,10 +5478,12 @@
       <c r="B40" s="1"/>
       <c r="C40" s="1"/>
       <c r="D40" s="1"/>
-      <c r="E40" s="1" t="s">
+      <c r="E40" s="1"/>
+      <c r="F40" s="1"/>
+      <c r="G40" s="1" t="s">
         <v>272</v>
       </c>
-      <c r="F40" s="1"/>
+      <c r="H40" s="1"/>
     </row>
     <row r="41" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
@@ -5422,6 +5500,8 @@
       </c>
       <c r="E41" s="1"/>
       <c r="F41" s="1"/>
+      <c r="G41" s="1"/>
+      <c r="H41" s="1"/>
     </row>
     <row r="42" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
@@ -5438,6 +5518,8 @@
       </c>
       <c r="E42" s="1"/>
       <c r="F42" s="1"/>
+      <c r="G42" s="1"/>
+      <c r="H42" s="1"/>
     </row>
     <row r="43" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
@@ -5446,10 +5528,12 @@
       <c r="B43" s="1"/>
       <c r="C43" s="1"/>
       <c r="D43" s="1"/>
-      <c r="E43" s="1" t="s">
+      <c r="E43" s="1"/>
+      <c r="F43" s="1"/>
+      <c r="G43" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="F43" s="1"/>
+      <c r="H43" s="1"/>
     </row>
     <row r="44" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
@@ -5466,6 +5550,8 @@
       </c>
       <c r="E44" s="1"/>
       <c r="F44" s="1"/>
+      <c r="G44" s="1"/>
+      <c r="H44" s="1"/>
     </row>
     <row r="45" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
@@ -5482,6 +5568,8 @@
       </c>
       <c r="E45" s="1"/>
       <c r="F45" s="1"/>
+      <c r="G45" s="1"/>
+      <c r="H45" s="1"/>
     </row>
     <row r="46" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
@@ -5498,6 +5586,8 @@
       </c>
       <c r="E46" s="1"/>
       <c r="F46" s="1"/>
+      <c r="G46" s="1"/>
+      <c r="H46" s="1"/>
     </row>
     <row r="47" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
@@ -5514,6 +5604,8 @@
       </c>
       <c r="E47" s="1"/>
       <c r="F47" s="1"/>
+      <c r="G47" s="1"/>
+      <c r="H47" s="1"/>
     </row>
     <row r="48" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
@@ -5530,46 +5622,48 @@
       </c>
       <c r="E48" s="1"/>
       <c r="F48" s="1"/>
+      <c r="G48" s="1"/>
+      <c r="H48" s="1"/>
     </row>
     <row r="49" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="50" t="s">
+      <c r="A49" s="49" t="s">
         <v>174</v>
       </c>
-      <c r="B49" s="50" t="s">
+      <c r="B49" s="49" t="s">
         <v>249</v>
       </c>
-      <c r="C49" s="50" t="s">
+      <c r="C49" s="49" t="s">
         <v>362</v>
       </c>
-      <c r="D49" s="50" t="s">
+      <c r="D49" s="49" t="s">
         <v>351</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="50" t="s">
+      <c r="A50" s="49" t="s">
         <v>174</v>
       </c>
-      <c r="B50" s="50" t="s">
+      <c r="B50" s="49" t="s">
         <v>250</v>
       </c>
-      <c r="C50" s="50" t="s">
+      <c r="C50" s="49" t="s">
         <v>363</v>
       </c>
-      <c r="D50" s="50" t="s">
+      <c r="D50" s="49" t="s">
         <v>364</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="50" t="s">
+      <c r="A51" s="49" t="s">
         <v>174</v>
       </c>
-      <c r="B51" s="50" t="s">
+      <c r="B51" s="49" t="s">
         <v>359</v>
       </c>
-      <c r="C51" s="50" t="s">
+      <c r="C51" s="49" t="s">
         <v>365</v>
       </c>
-      <c r="D51" s="50" t="s">
+      <c r="D51" s="49" t="s">
         <v>366</v>
       </c>
     </row>
@@ -5592,53 +5686,53 @@
   <dimension ref="A1:L1"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="40" width="18.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="40" width="17.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="40" width="13.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="40" width="12.72"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="40" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="40" width="13.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="40" width="14.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="40" width="11.28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="40" width="13.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="40" width="14.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="39" width="18.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="39" width="17.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="39" width="13.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="39" width="12.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="39" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="39" width="13.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="39" width="14.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="39" width="11.28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="39" width="13.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="39" width="14.43"/>
   </cols>
   <sheetData>
-    <row r="1" s="51" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="52" t="s">
+    <row r="1" s="50" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="51" t="s">
         <v>367</v>
       </c>
-      <c r="B1" s="52" t="s">
+      <c r="B1" s="51" t="s">
         <v>368</v>
       </c>
-      <c r="C1" s="52" t="s">
+      <c r="C1" s="51" t="s">
         <v>369</v>
       </c>
-      <c r="D1" s="52" t="s">
+      <c r="D1" s="51" t="s">
         <v>370</v>
       </c>
-      <c r="E1" s="52" t="s">
+      <c r="E1" s="51" t="s">
         <v>371</v>
       </c>
-      <c r="F1" s="52" t="s">
+      <c r="F1" s="51" t="s">
         <v>372</v>
       </c>
-      <c r="G1" s="52" t="s">
+      <c r="G1" s="51" t="s">
         <v>373</v>
       </c>
-      <c r="H1" s="52" t="s">
+      <c r="H1" s="51" t="s">
         <v>374</v>
       </c>
-      <c r="I1" s="52" t="s">
+      <c r="I1" s="51" t="s">
         <v>375</v>
       </c>
-      <c r="J1" s="52" t="s">
+      <c r="J1" s="51" t="s">
         <v>376</v>
       </c>
-      <c r="K1" s="52" t="s">
+      <c r="K1" s="51" t="s">
         <v>377</v>
       </c>
-      <c r="L1" s="51" t="s">
+      <c r="L1" s="50" t="s">
         <v>378</v>
       </c>
     </row>
@@ -5661,11 +5755,11 @@
   <dimension ref="A1:G3"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10.34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="40" width="32.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="40" width="43.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="40" width="46.08"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="40" width="28.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="39" width="10.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="39" width="32.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="39" width="43.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="39" width="46.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="39" width="28.55"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5687,39 +5781,39 @@
       <c r="F1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="40"/>
+      <c r="G1" s="39"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="53" t="s">
+      <c r="A2" s="52" t="s">
         <v>102</v>
       </c>
-      <c r="B2" s="54" t="s">
+      <c r="B2" s="44" t="s">
         <v>379</v>
       </c>
-      <c r="C2" s="53" t="s">
+      <c r="C2" s="52" t="s">
         <v>380</v>
       </c>
-      <c r="D2" s="53" t="s">
+      <c r="D2" s="52" t="s">
         <v>381</v>
       </c>
-      <c r="E2" s="53"/>
-      <c r="F2" s="53"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="53" t="s">
+      <c r="A3" s="52" t="s">
         <v>102</v>
       </c>
-      <c r="B3" s="54" t="s">
+      <c r="B3" s="44" t="s">
         <v>382</v>
       </c>
-      <c r="C3" s="53" t="s">
+      <c r="C3" s="52" t="s">
         <v>383</v>
       </c>
-      <c r="D3" s="53" t="s">
+      <c r="D3" s="52" t="s">
         <v>384</v>
       </c>
-      <c r="E3" s="53"/>
-      <c r="F3" s="53"/>
+      <c r="E3" s="52"/>
+      <c r="F3" s="52"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Refactor: Introduce `get_label_context_flags` for dynamic label context detection
- Added a new helper function `get_label_context_flags` to identify the presence of nickname, count, gender context, and label_one in label strings.
- Refactored existing code in `generate_choices.py`, `generate_widgets.py`, and `labels_generator.py` to utilize the new function, improving code clarity and reducing redundancy.
- Created unit tests for `get_label_context_flags` to ensure accurate detection of context flags across various label formats.
</commit_message>
<xml_diff>
--- a/example/demo_generator/references/Household_Travel_Generate_Survey.xlsx
+++ b/example/demo_generator/references/Household_Travel_Generate_Survey.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Widgets" sheetId="1" state="visible" r:id="rId3"/>
@@ -1250,7 +1250,7 @@
     <numFmt numFmtId="165" formatCode="General"/>
     <numFmt numFmtId="166" formatCode="@"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1372,6 +1372,13 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <b val="true"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -1438,15 +1445,15 @@
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
-      <top/>
-      <bottom style="thin"/>
+      <top style="thin"/>
+      <bottom/>
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
-      <top style="thin"/>
-      <bottom/>
+      <top/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
   </borders>
@@ -1475,7 +1482,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="54">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1520,6 +1527,10 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1528,7 +1539,7 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1536,19 +1547,19 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1556,15 +1567,11 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1608,15 +1615,15 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1681,6 +1688,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2847,7 +2858,7 @@
       <c r="W16" s="7"/>
       <c r="X16" s="7"/>
     </row>
-    <row r="17" customFormat="false" ht="76.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="17" s="11" customFormat="true" ht="76.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
         <v>92</v>
       </c>
@@ -2897,33 +2908,33 @@
       <c r="X17" s="7"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="11" t="s">
+      <c r="A18" s="12" t="s">
         <v>97</v>
       </c>
-      <c r="B18" s="11" t="s">
+      <c r="B18" s="12" t="s">
         <v>98</v>
       </c>
-      <c r="C18" s="12" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D18" s="13" t="s">
+      <c r="C18" s="13" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D18" s="14" t="s">
         <v>26</v>
       </c>
       <c r="E18" s="7"/>
-      <c r="F18" s="14" t="str">
+      <c r="F18" s="15" t="str">
         <f aca="false">REPLACE(A18, FIND("_", A18), 1, ".")</f>
         <v>home.save</v>
       </c>
-      <c r="G18" s="11" t="s">
+      <c r="G18" s="12" t="s">
         <v>99</v>
       </c>
-      <c r="H18" s="11" t="s">
+      <c r="H18" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="I18" s="11"/>
-      <c r="J18" s="11"/>
-      <c r="K18" s="11"/>
+      <c r="I18" s="12"/>
+      <c r="J18" s="12"/>
+      <c r="K18" s="12"/>
       <c r="L18" s="7"/>
       <c r="M18" s="7"/>
       <c r="N18" s="7"/>
@@ -2932,7 +2943,7 @@
       <c r="Q18" s="7"/>
       <c r="R18" s="7"/>
       <c r="S18" s="7"/>
-      <c r="T18" s="15" t="b">
+      <c r="T18" s="16" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2941,56 +2952,56 @@
       <c r="W18" s="7"/>
       <c r="X18" s="7"/>
     </row>
-    <row r="19" s="22" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="16" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="17" t="s">
         <v>101</v>
       </c>
-      <c r="B19" s="17" t="s">
+      <c r="B19" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="C19" s="18" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D19" s="19" t="s">
+      <c r="C19" s="19" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D19" s="20" t="s">
         <v>102</v>
       </c>
-      <c r="E19" s="20"/>
-      <c r="F19" s="20"/>
-      <c r="G19" s="16"/>
-      <c r="H19" s="16"/>
-      <c r="I19" s="16"/>
-      <c r="J19" s="16"/>
-      <c r="K19" s="16"/>
-      <c r="L19" s="20"/>
-      <c r="M19" s="20"/>
-      <c r="N19" s="20"/>
-      <c r="O19" s="20"/>
-      <c r="P19" s="20"/>
-      <c r="Q19" s="20"/>
-      <c r="R19" s="20"/>
-      <c r="S19" s="20"/>
-      <c r="T19" s="21" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U19" s="20"/>
-      <c r="V19" s="20"/>
-      <c r="W19" s="20"/>
-      <c r="X19" s="20"/>
+      <c r="E19" s="21"/>
+      <c r="F19" s="21"/>
+      <c r="G19" s="17"/>
+      <c r="H19" s="17"/>
+      <c r="I19" s="17"/>
+      <c r="J19" s="17"/>
+      <c r="K19" s="17"/>
+      <c r="L19" s="21"/>
+      <c r="M19" s="21"/>
+      <c r="N19" s="21"/>
+      <c r="O19" s="21"/>
+      <c r="P19" s="21"/>
+      <c r="Q19" s="21"/>
+      <c r="R19" s="21"/>
+      <c r="S19" s="21"/>
+      <c r="T19" s="22" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U19" s="21"/>
+      <c r="V19" s="21"/>
+      <c r="W19" s="21"/>
+      <c r="X19" s="21"/>
     </row>
     <row r="20" customFormat="false" ht="144" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="19" t="s">
+      <c r="A20" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="B20" s="19" t="s">
+      <c r="B20" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="C20" s="21" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D20" s="19" t="s">
+      <c r="C20" s="22" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D20" s="20" t="s">
         <v>102</v>
       </c>
       <c r="E20" s="23" t="s">
@@ -2999,15 +3010,15 @@
       <c r="F20" s="23" t="s">
         <v>104</v>
       </c>
-      <c r="G20" s="19" t="s">
+      <c r="G20" s="20" t="s">
         <v>105</v>
       </c>
-      <c r="H20" s="19" t="s">
+      <c r="H20" s="20" t="s">
         <v>106</v>
       </c>
-      <c r="I20" s="19"/>
-      <c r="J20" s="19"/>
-      <c r="K20" s="19"/>
+      <c r="I20" s="20"/>
+      <c r="J20" s="20"/>
+      <c r="K20" s="20"/>
       <c r="L20" s="23"/>
       <c r="M20" s="23" t="s">
         <v>95</v>
@@ -3018,7 +3029,7 @@
       <c r="Q20" s="23"/>
       <c r="R20" s="23"/>
       <c r="S20" s="23"/>
-      <c r="T20" s="21" t="b">
+      <c r="T20" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -3028,17 +3039,17 @@
       <c r="X20" s="23"/>
     </row>
     <row r="21" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="19" t="s">
+      <c r="A21" s="20" t="s">
         <v>107</v>
       </c>
-      <c r="B21" s="19" t="s">
+      <c r="B21" s="20" t="s">
         <v>108</v>
       </c>
-      <c r="C21" s="21" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D21" s="19" t="s">
+      <c r="C21" s="22" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D21" s="20" t="s">
         <v>102</v>
       </c>
       <c r="E21" s="23" t="s">
@@ -3047,19 +3058,19 @@
       <c r="F21" s="23" t="s">
         <v>109</v>
       </c>
-      <c r="G21" s="19" t="s">
+      <c r="G21" s="20" t="s">
         <v>110</v>
       </c>
-      <c r="H21" s="19" t="s">
+      <c r="H21" s="20" t="s">
         <v>111</v>
       </c>
-      <c r="I21" s="19" t="s">
+      <c r="I21" s="20" t="s">
         <v>112</v>
       </c>
-      <c r="J21" s="19" t="s">
+      <c r="J21" s="20" t="s">
         <v>113</v>
       </c>
-      <c r="K21" s="19"/>
+      <c r="K21" s="20"/>
       <c r="L21" s="23"/>
       <c r="M21" s="23"/>
       <c r="N21" s="23" t="s">
@@ -3070,7 +3081,7 @@
       <c r="Q21" s="23"/>
       <c r="R21" s="23"/>
       <c r="S21" s="23"/>
-      <c r="T21" s="21" t="b">
+      <c r="T21" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -3080,17 +3091,17 @@
       <c r="X21" s="23"/>
     </row>
     <row r="22" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="19" t="s">
+      <c r="A22" s="20" t="s">
         <v>115</v>
       </c>
-      <c r="B22" s="19" t="s">
+      <c r="B22" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="C22" s="21" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D22" s="19" t="s">
+      <c r="C22" s="22" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D22" s="20" t="s">
         <v>102</v>
       </c>
       <c r="E22" s="23" t="s">
@@ -3099,15 +3110,15 @@
       <c r="F22" s="23" t="s">
         <v>116</v>
       </c>
-      <c r="G22" s="19" t="s">
+      <c r="G22" s="20" t="s">
         <v>117</v>
       </c>
-      <c r="H22" s="19" t="s">
+      <c r="H22" s="20" t="s">
         <v>118</v>
       </c>
-      <c r="I22" s="19"/>
-      <c r="J22" s="19"/>
-      <c r="K22" s="19"/>
+      <c r="I22" s="20"/>
+      <c r="J22" s="20"/>
+      <c r="K22" s="20"/>
       <c r="L22" s="23"/>
       <c r="M22" s="23" t="s">
         <v>119</v>
@@ -3120,7 +3131,7 @@
       <c r="Q22" s="23"/>
       <c r="R22" s="23"/>
       <c r="S22" s="23"/>
-      <c r="T22" s="21" t="b">
+      <c r="T22" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -3130,17 +3141,17 @@
       <c r="X22" s="23"/>
     </row>
     <row r="23" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="19" t="s">
+      <c r="A23" s="20" t="s">
         <v>120</v>
       </c>
-      <c r="B23" s="19" t="s">
+      <c r="B23" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="C23" s="21" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D23" s="19" t="s">
+      <c r="C23" s="22" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D23" s="20" t="s">
         <v>102</v>
       </c>
       <c r="E23" s="23" t="s">
@@ -3149,15 +3160,15 @@
       <c r="F23" s="23" t="s">
         <v>121</v>
       </c>
-      <c r="G23" s="19" t="s">
+      <c r="G23" s="20" t="s">
         <v>122</v>
       </c>
-      <c r="H23" s="19" t="s">
+      <c r="H23" s="20" t="s">
         <v>123</v>
       </c>
-      <c r="I23" s="19"/>
-      <c r="J23" s="19"/>
-      <c r="K23" s="19"/>
+      <c r="I23" s="20"/>
+      <c r="J23" s="20"/>
+      <c r="K23" s="20"/>
       <c r="L23" s="23"/>
       <c r="M23" s="23" t="s">
         <v>124</v>
@@ -3170,7 +3181,7 @@
       <c r="Q23" s="23"/>
       <c r="R23" s="23"/>
       <c r="S23" s="23"/>
-      <c r="T23" s="21" t="b">
+      <c r="T23" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -3180,17 +3191,17 @@
       <c r="X23" s="23"/>
     </row>
     <row r="24" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="19" t="s">
+      <c r="A24" s="20" t="s">
         <v>126</v>
       </c>
-      <c r="B24" s="19" t="s">
+      <c r="B24" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="C24" s="21" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D24" s="19" t="s">
+      <c r="C24" s="22" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D24" s="20" t="s">
         <v>102</v>
       </c>
       <c r="E24" s="23" t="s">
@@ -3199,15 +3210,15 @@
       <c r="F24" s="23" t="s">
         <v>127</v>
       </c>
-      <c r="G24" s="19" t="s">
+      <c r="G24" s="20" t="s">
         <v>128</v>
       </c>
-      <c r="H24" s="19" t="s">
+      <c r="H24" s="20" t="s">
         <v>129</v>
       </c>
-      <c r="I24" s="19"/>
-      <c r="J24" s="19"/>
-      <c r="K24" s="19"/>
+      <c r="I24" s="20"/>
+      <c r="J24" s="20"/>
+      <c r="K24" s="20"/>
       <c r="L24" s="23"/>
       <c r="M24" s="23" t="s">
         <v>130</v>
@@ -3220,7 +3231,7 @@
       <c r="Q24" s="23"/>
       <c r="R24" s="23"/>
       <c r="S24" s="23"/>
-      <c r="T24" s="21" t="b">
+      <c r="T24" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -3230,17 +3241,17 @@
       <c r="X24" s="23"/>
     </row>
     <row r="25" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="19" t="s">
+      <c r="A25" s="20" t="s">
         <v>131</v>
       </c>
-      <c r="B25" s="19" t="s">
+      <c r="B25" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="C25" s="21" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D25" s="19" t="s">
+      <c r="C25" s="22" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D25" s="20" t="s">
         <v>102</v>
       </c>
       <c r="E25" s="23" t="s">
@@ -3249,10 +3260,10 @@
       <c r="F25" s="23" t="s">
         <v>132</v>
       </c>
-      <c r="G25" s="19"/>
-      <c r="H25" s="19"/>
-      <c r="I25" s="19"/>
-      <c r="J25" s="19"/>
+      <c r="G25" s="20"/>
+      <c r="H25" s="20"/>
+      <c r="I25" s="20"/>
+      <c r="J25" s="20"/>
       <c r="K25" s="25" t="s">
         <v>133</v>
       </c>
@@ -3268,7 +3279,7 @@
       <c r="Q25" s="23"/>
       <c r="R25" s="23"/>
       <c r="S25" s="23"/>
-      <c r="T25" s="21" t="b">
+      <c r="T25" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -3282,17 +3293,17 @@
       <c r="X25" s="23"/>
     </row>
     <row r="26" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="19" t="s">
+      <c r="A26" s="20" t="s">
         <v>137</v>
       </c>
-      <c r="B26" s="19" t="s">
+      <c r="B26" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="C26" s="21" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D26" s="19" t="s">
+      <c r="C26" s="22" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D26" s="20" t="s">
         <v>102</v>
       </c>
       <c r="E26" s="23" t="s">
@@ -3301,15 +3312,15 @@
       <c r="F26" s="27" t="s">
         <v>138</v>
       </c>
-      <c r="G26" s="19" t="s">
+      <c r="G26" s="20" t="s">
         <v>139</v>
       </c>
-      <c r="H26" s="19" t="s">
+      <c r="H26" s="20" t="s">
         <v>140</v>
       </c>
-      <c r="I26" s="19"/>
-      <c r="J26" s="19"/>
-      <c r="K26" s="19"/>
+      <c r="I26" s="20"/>
+      <c r="J26" s="20"/>
+      <c r="K26" s="20"/>
       <c r="L26" s="23"/>
       <c r="M26" s="23" t="s">
         <v>141</v>
@@ -3322,7 +3333,7 @@
       <c r="Q26" s="23"/>
       <c r="R26" s="23"/>
       <c r="S26" s="23"/>
-      <c r="T26" s="21" t="b">
+      <c r="T26" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -3332,17 +3343,17 @@
       <c r="X26" s="23"/>
     </row>
     <row r="27" customFormat="false" ht="62.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="19" t="s">
+      <c r="A27" s="20" t="s">
         <v>142</v>
       </c>
-      <c r="B27" s="19" t="s">
+      <c r="B27" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="C27" s="21" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D27" s="19" t="s">
+      <c r="C27" s="22" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D27" s="20" t="s">
         <v>102</v>
       </c>
       <c r="E27" s="23" t="s">
@@ -3351,15 +3362,15 @@
       <c r="F27" s="23" t="s">
         <v>143</v>
       </c>
-      <c r="G27" s="19" t="s">
+      <c r="G27" s="20" t="s">
         <v>144</v>
       </c>
-      <c r="H27" s="19" t="s">
+      <c r="H27" s="20" t="s">
         <v>145</v>
       </c>
-      <c r="I27" s="19"/>
-      <c r="J27" s="19"/>
-      <c r="K27" s="19"/>
+      <c r="I27" s="20"/>
+      <c r="J27" s="20"/>
+      <c r="K27" s="20"/>
       <c r="L27" s="23"/>
       <c r="M27" s="23" t="s">
         <v>130</v>
@@ -3372,7 +3383,7 @@
       <c r="Q27" s="23"/>
       <c r="R27" s="23"/>
       <c r="S27" s="23"/>
-      <c r="T27" s="21" t="b">
+      <c r="T27" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -3382,17 +3393,17 @@
       <c r="X27" s="23"/>
     </row>
     <row r="28" customFormat="false" ht="52.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="19" t="s">
+      <c r="A28" s="20" t="s">
         <v>147</v>
       </c>
-      <c r="B28" s="19" t="s">
+      <c r="B28" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="C28" s="21" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D28" s="19" t="s">
+      <c r="C28" s="22" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D28" s="20" t="s">
         <v>102</v>
       </c>
       <c r="E28" s="23" t="s">
@@ -3401,15 +3412,15 @@
       <c r="F28" s="23" t="s">
         <v>148</v>
       </c>
-      <c r="G28" s="19" t="s">
+      <c r="G28" s="20" t="s">
         <v>149</v>
       </c>
-      <c r="H28" s="19" t="s">
+      <c r="H28" s="20" t="s">
         <v>150</v>
       </c>
-      <c r="I28" s="19"/>
-      <c r="J28" s="19"/>
-      <c r="K28" s="19"/>
+      <c r="I28" s="20"/>
+      <c r="J28" s="20"/>
+      <c r="K28" s="20"/>
       <c r="L28" s="23"/>
       <c r="M28" s="23" t="s">
         <v>151</v>
@@ -3422,7 +3433,7 @@
       <c r="Q28" s="23"/>
       <c r="R28" s="23"/>
       <c r="S28" s="23"/>
-      <c r="T28" s="21" t="b">
+      <c r="T28" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -3435,14 +3446,14 @@
       <c r="A29" s="28" t="s">
         <v>152</v>
       </c>
-      <c r="B29" s="19" t="s">
+      <c r="B29" s="20" t="s">
         <v>153</v>
       </c>
-      <c r="C29" s="21" t="b">
+      <c r="C29" s="22" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="D29" s="19" t="s">
+      <c r="D29" s="20" t="s">
         <v>102</v>
       </c>
       <c r="E29" s="23" t="s">
@@ -3451,15 +3462,15 @@
       <c r="F29" s="23" t="s">
         <v>154</v>
       </c>
-      <c r="G29" s="19" t="s">
+      <c r="G29" s="20" t="s">
         <v>155</v>
       </c>
-      <c r="H29" s="19" t="s">
+      <c r="H29" s="20" t="s">
         <v>156</v>
       </c>
-      <c r="I29" s="19"/>
-      <c r="J29" s="19"/>
-      <c r="K29" s="19"/>
+      <c r="I29" s="20"/>
+      <c r="J29" s="20"/>
+      <c r="K29" s="20"/>
       <c r="L29" s="23"/>
       <c r="M29" s="23" t="s">
         <v>157</v>
@@ -3472,7 +3483,7 @@
       <c r="Q29" s="23"/>
       <c r="R29" s="23"/>
       <c r="S29" s="23"/>
-      <c r="T29" s="21" t="b">
+      <c r="T29" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -3482,17 +3493,17 @@
       <c r="X29" s="23"/>
     </row>
     <row r="30" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="19" t="s">
+      <c r="A30" s="20" t="s">
         <v>159</v>
       </c>
-      <c r="B30" s="19" t="s">
+      <c r="B30" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="C30" s="21" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D30" s="19" t="s">
+      <c r="C30" s="22" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D30" s="20" t="s">
         <v>102</v>
       </c>
       <c r="E30" s="23" t="s">
@@ -3501,15 +3512,15 @@
       <c r="F30" s="23" t="s">
         <v>160</v>
       </c>
-      <c r="G30" s="19" t="s">
+      <c r="G30" s="20" t="s">
         <v>161</v>
       </c>
-      <c r="H30" s="19" t="s">
+      <c r="H30" s="20" t="s">
         <v>162</v>
       </c>
-      <c r="I30" s="19"/>
-      <c r="J30" s="19"/>
-      <c r="K30" s="19"/>
+      <c r="I30" s="20"/>
+      <c r="J30" s="20"/>
+      <c r="K30" s="20"/>
       <c r="L30" s="23"/>
       <c r="M30" s="23" t="s">
         <v>163</v>
@@ -3522,7 +3533,7 @@
       <c r="Q30" s="23"/>
       <c r="R30" s="23"/>
       <c r="S30" s="23"/>
-      <c r="T30" s="21" t="b">
+      <c r="T30" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -3532,17 +3543,17 @@
       <c r="X30" s="23"/>
     </row>
     <row r="31" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="19" t="s">
+      <c r="A31" s="20" t="s">
         <v>164</v>
       </c>
-      <c r="B31" s="19" t="s">
+      <c r="B31" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="C31" s="21" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D31" s="19" t="s">
+      <c r="C31" s="22" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D31" s="20" t="s">
         <v>102</v>
       </c>
       <c r="E31" s="23" t="s">
@@ -3551,15 +3562,15 @@
       <c r="F31" s="23" t="s">
         <v>165</v>
       </c>
-      <c r="G31" s="19" t="s">
+      <c r="G31" s="20" t="s">
         <v>166</v>
       </c>
-      <c r="H31" s="19" t="s">
+      <c r="H31" s="20" t="s">
         <v>167</v>
       </c>
-      <c r="I31" s="19"/>
-      <c r="J31" s="19"/>
-      <c r="K31" s="19"/>
+      <c r="I31" s="20"/>
+      <c r="J31" s="20"/>
+      <c r="K31" s="20"/>
       <c r="L31" s="23"/>
       <c r="M31" s="23" t="s">
         <v>168</v>
@@ -3572,7 +3583,7 @@
       <c r="Q31" s="23"/>
       <c r="R31" s="23"/>
       <c r="S31" s="23"/>
-      <c r="T31" s="21" t="b">
+      <c r="T31" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -3582,17 +3593,17 @@
       <c r="X31" s="23"/>
     </row>
     <row r="32" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="19" t="s">
+      <c r="A32" s="20" t="s">
         <v>169</v>
       </c>
-      <c r="B32" s="19" t="s">
+      <c r="B32" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="C32" s="21" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D32" s="19" t="s">
+      <c r="C32" s="22" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D32" s="20" t="s">
         <v>102</v>
       </c>
       <c r="E32" s="23" t="s">
@@ -3601,15 +3612,15 @@
       <c r="F32" s="23" t="s">
         <v>170</v>
       </c>
-      <c r="G32" s="19" t="s">
+      <c r="G32" s="20" t="s">
         <v>171</v>
       </c>
-      <c r="H32" s="19" t="s">
+      <c r="H32" s="20" t="s">
         <v>172</v>
       </c>
-      <c r="I32" s="19"/>
-      <c r="J32" s="19"/>
-      <c r="K32" s="19"/>
+      <c r="I32" s="20"/>
+      <c r="J32" s="20"/>
+      <c r="K32" s="20"/>
       <c r="L32" s="23"/>
       <c r="M32" s="23" t="s">
         <v>173</v>
@@ -3622,7 +3633,7 @@
       <c r="Q32" s="23"/>
       <c r="R32" s="23"/>
       <c r="S32" s="23"/>
-      <c r="T32" s="21" t="b">
+      <c r="T32" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -3632,17 +3643,17 @@
       <c r="X32" s="23"/>
     </row>
     <row r="33" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="19" t="s">
+      <c r="A33" s="20" t="s">
         <v>175</v>
       </c>
-      <c r="B33" s="19" t="s">
+      <c r="B33" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="C33" s="21" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D33" s="19" t="s">
+      <c r="C33" s="22" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D33" s="20" t="s">
         <v>102</v>
       </c>
       <c r="E33" s="23" t="s">
@@ -3651,17 +3662,17 @@
       <c r="F33" s="23" t="s">
         <v>176</v>
       </c>
-      <c r="G33" s="19" t="s">
+      <c r="G33" s="20" t="s">
         <v>177</v>
       </c>
-      <c r="H33" s="19" t="s">
+      <c r="H33" s="20" t="s">
         <v>178</v>
       </c>
-      <c r="I33" s="19"/>
-      <c r="J33" s="19"/>
-      <c r="K33" s="19"/>
+      <c r="I33" s="20"/>
+      <c r="J33" s="20"/>
+      <c r="K33" s="20"/>
       <c r="L33" s="23"/>
-      <c r="M33" s="19" t="s">
+      <c r="M33" s="20" t="s">
         <v>179</v>
       </c>
       <c r="N33" s="23"/>
@@ -3670,7 +3681,7 @@
       <c r="Q33" s="23"/>
       <c r="R33" s="23"/>
       <c r="S33" s="23"/>
-      <c r="T33" s="21" t="b">
+      <c r="T33" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -3680,17 +3691,17 @@
       <c r="X33" s="23"/>
     </row>
     <row r="34" customFormat="false" ht="85.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="19" t="s">
+      <c r="A34" s="20" t="s">
         <v>180</v>
       </c>
       <c r="B34" s="29" t="s">
         <v>69</v>
       </c>
-      <c r="C34" s="21" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D34" s="19" t="s">
+      <c r="C34" s="22" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D34" s="20" t="s">
         <v>102</v>
       </c>
       <c r="E34" s="23" t="s">
@@ -3699,21 +3710,21 @@
       <c r="F34" s="23" t="s">
         <v>181</v>
       </c>
-      <c r="G34" s="19" t="s">
+      <c r="G34" s="20" t="s">
         <v>182</v>
       </c>
-      <c r="H34" s="19" t="s">
+      <c r="H34" s="20" t="s">
         <v>183</v>
       </c>
-      <c r="I34" s="19" t="s">
+      <c r="I34" s="20" t="s">
         <v>184</v>
       </c>
-      <c r="J34" s="19" t="s">
+      <c r="J34" s="20" t="s">
         <v>185</v>
       </c>
-      <c r="K34" s="19"/>
+      <c r="K34" s="20"/>
       <c r="L34" s="23"/>
-      <c r="M34" s="19" t="s">
+      <c r="M34" s="20" t="s">
         <v>179</v>
       </c>
       <c r="N34" s="23"/>
@@ -3722,7 +3733,7 @@
       <c r="Q34" s="23"/>
       <c r="R34" s="23"/>
       <c r="S34" s="23"/>
-      <c r="T34" s="21" t="b">
+      <c r="T34" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -3732,17 +3743,17 @@
       <c r="X34" s="23"/>
     </row>
     <row r="35" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="19" t="s">
+      <c r="A35" s="20" t="s">
         <v>186</v>
       </c>
-      <c r="B35" s="19" t="s">
+      <c r="B35" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="C35" s="21" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D35" s="19" t="s">
+      <c r="C35" s="22" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D35" s="20" t="s">
         <v>102</v>
       </c>
       <c r="E35" s="23" t="s">
@@ -3751,17 +3762,17 @@
       <c r="F35" s="23" t="s">
         <v>187</v>
       </c>
-      <c r="G35" s="19" t="s">
+      <c r="G35" s="20" t="s">
         <v>188</v>
       </c>
-      <c r="H35" s="19" t="s">
+      <c r="H35" s="20" t="s">
         <v>189</v>
       </c>
-      <c r="I35" s="19"/>
-      <c r="J35" s="19"/>
-      <c r="K35" s="19"/>
+      <c r="I35" s="20"/>
+      <c r="J35" s="20"/>
+      <c r="K35" s="20"/>
       <c r="L35" s="23"/>
-      <c r="M35" s="19" t="s">
+      <c r="M35" s="20" t="s">
         <v>190</v>
       </c>
       <c r="N35" s="23"/>
@@ -3770,7 +3781,7 @@
       <c r="Q35" s="23"/>
       <c r="R35" s="23"/>
       <c r="S35" s="23"/>
-      <c r="T35" s="21" t="b">
+      <c r="T35" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -3780,17 +3791,17 @@
       <c r="X35" s="23"/>
     </row>
     <row r="36" customFormat="false" ht="85.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="19" t="s">
+      <c r="A36" s="20" t="s">
         <v>191</v>
       </c>
       <c r="B36" s="29" t="s">
         <v>69</v>
       </c>
-      <c r="C36" s="21" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D36" s="19" t="s">
+      <c r="C36" s="22" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D36" s="20" t="s">
         <v>102</v>
       </c>
       <c r="E36" s="23" t="s">
@@ -3799,16 +3810,16 @@
       <c r="F36" s="23" t="s">
         <v>192</v>
       </c>
-      <c r="G36" s="19" t="s">
+      <c r="G36" s="20" t="s">
         <v>193</v>
       </c>
-      <c r="H36" s="19" t="s">
+      <c r="H36" s="20" t="s">
         <v>194</v>
       </c>
-      <c r="I36" s="19" t="s">
+      <c r="I36" s="20" t="s">
         <v>195</v>
       </c>
-      <c r="J36" s="19" t="s">
+      <c r="J36" s="20" t="s">
         <v>196</v>
       </c>
       <c r="K36" s="30"/>
@@ -3820,7 +3831,7 @@
       <c r="Q36" s="31"/>
       <c r="R36" s="23"/>
       <c r="S36" s="23"/>
-      <c r="T36" s="21" t="b">
+      <c r="T36" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -3833,14 +3844,14 @@
       <c r="A37" s="28" t="s">
         <v>197</v>
       </c>
-      <c r="B37" s="19" t="s">
+      <c r="B37" s="20" t="s">
         <v>153</v>
       </c>
-      <c r="C37" s="21" t="b">
+      <c r="C37" s="22" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="D37" s="19" t="s">
+      <c r="D37" s="20" t="s">
         <v>102</v>
       </c>
       <c r="E37" s="23" t="s">
@@ -3849,15 +3860,15 @@
       <c r="F37" s="23" t="s">
         <v>198</v>
       </c>
-      <c r="G37" s="19" t="s">
+      <c r="G37" s="20" t="s">
         <v>199</v>
       </c>
-      <c r="H37" s="19" t="s">
+      <c r="H37" s="20" t="s">
         <v>200</v>
       </c>
-      <c r="I37" s="19"/>
-      <c r="J37" s="19"/>
-      <c r="K37" s="19"/>
+      <c r="I37" s="20"/>
+      <c r="J37" s="20"/>
+      <c r="K37" s="20"/>
       <c r="L37" s="23"/>
       <c r="M37" s="24"/>
       <c r="N37" s="24"/>
@@ -3868,7 +3879,7 @@
       <c r="Q37" s="23"/>
       <c r="R37" s="23"/>
       <c r="S37" s="23"/>
-      <c r="T37" s="21" t="b">
+      <c r="T37" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -3881,14 +3892,14 @@
       <c r="A38" s="28" t="s">
         <v>201</v>
       </c>
-      <c r="B38" s="19" t="s">
+      <c r="B38" s="20" t="s">
         <v>153</v>
       </c>
-      <c r="C38" s="21" t="b">
+      <c r="C38" s="22" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="D38" s="19" t="s">
+      <c r="D38" s="20" t="s">
         <v>102</v>
       </c>
       <c r="E38" s="23" t="s">
@@ -3897,15 +3908,15 @@
       <c r="F38" s="23" t="s">
         <v>202</v>
       </c>
-      <c r="G38" s="19" t="s">
+      <c r="G38" s="20" t="s">
         <v>203</v>
       </c>
-      <c r="H38" s="19" t="s">
+      <c r="H38" s="20" t="s">
         <v>204</v>
       </c>
-      <c r="I38" s="19"/>
-      <c r="J38" s="19"/>
-      <c r="K38" s="19"/>
+      <c r="I38" s="20"/>
+      <c r="J38" s="20"/>
+      <c r="K38" s="20"/>
       <c r="L38" s="23"/>
       <c r="M38" s="24"/>
       <c r="N38" s="24"/>
@@ -3916,7 +3927,7 @@
       <c r="Q38" s="23"/>
       <c r="R38" s="23"/>
       <c r="S38" s="23"/>
-      <c r="T38" s="21" t="b">
+      <c r="T38" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -3925,18 +3936,18 @@
       <c r="W38" s="23"/>
       <c r="X38" s="23"/>
     </row>
-    <row r="39" customFormat="false" ht="64.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" s="6" customFormat="true" ht="64.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="28" t="s">
         <v>205</v>
       </c>
-      <c r="B39" s="19" t="s">
+      <c r="B39" s="20" t="s">
         <v>153</v>
       </c>
-      <c r="C39" s="21" t="b">
+      <c r="C39" s="22" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="D39" s="19" t="s">
+      <c r="D39" s="20" t="s">
         <v>102</v>
       </c>
       <c r="E39" s="23" t="s">
@@ -3945,15 +3956,15 @@
       <c r="F39" s="23" t="s">
         <v>206</v>
       </c>
-      <c r="G39" s="19" t="s">
+      <c r="G39" s="20" t="s">
         <v>207</v>
       </c>
-      <c r="H39" s="19" t="s">
+      <c r="H39" s="20" t="s">
         <v>208</v>
       </c>
-      <c r="I39" s="19"/>
-      <c r="J39" s="19"/>
-      <c r="K39" s="19"/>
+      <c r="I39" s="20"/>
+      <c r="J39" s="20"/>
+      <c r="K39" s="20"/>
       <c r="L39" s="23"/>
       <c r="M39" s="24"/>
       <c r="N39" s="24"/>
@@ -3964,7 +3975,7 @@
       <c r="Q39" s="23"/>
       <c r="R39" s="23"/>
       <c r="S39" s="23"/>
-      <c r="T39" s="21" t="b">
+      <c r="T39" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -3977,14 +3988,14 @@
       <c r="A40" s="28" t="s">
         <v>209</v>
       </c>
-      <c r="B40" s="19" t="s">
+      <c r="B40" s="20" t="s">
         <v>153</v>
       </c>
-      <c r="C40" s="21" t="b">
+      <c r="C40" s="22" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="D40" s="19" t="s">
+      <c r="D40" s="20" t="s">
         <v>102</v>
       </c>
       <c r="E40" s="23" t="s">
@@ -3993,15 +4004,15 @@
       <c r="F40" s="23" t="s">
         <v>210</v>
       </c>
-      <c r="G40" s="19" t="s">
+      <c r="G40" s="20" t="s">
         <v>211</v>
       </c>
-      <c r="H40" s="19" t="s">
+      <c r="H40" s="20" t="s">
         <v>212</v>
       </c>
-      <c r="I40" s="19"/>
-      <c r="J40" s="19"/>
-      <c r="K40" s="19"/>
+      <c r="I40" s="20"/>
+      <c r="J40" s="20"/>
+      <c r="K40" s="20"/>
       <c r="L40" s="23"/>
       <c r="M40" s="24"/>
       <c r="N40" s="24"/>
@@ -4012,7 +4023,7 @@
       <c r="Q40" s="23"/>
       <c r="R40" s="23"/>
       <c r="S40" s="23"/>
-      <c r="T40" s="21" t="b">
+      <c r="T40" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -4021,7 +4032,7 @@
       <c r="W40" s="23"/>
       <c r="X40" s="23"/>
     </row>
-    <row r="41" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="33" t="s">
         <v>213</v>
       </c>
@@ -4779,7 +4790,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:H1048576"/>
   <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="49" width="21.3"/>
@@ -4817,23 +4828,23 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="51" t="s">
         <v>228</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="51" t="s">
         <v>270</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="51" t="s">
         <v>271</v>
       </c>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
+      <c r="E2" s="51"/>
+      <c r="F2" s="51"/>
+      <c r="G2" s="51"/>
+      <c r="H2" s="51"/>
     </row>
     <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
@@ -5667,6 +5678,7 @@
         <v>366</v>
       </c>
     </row>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -5699,37 +5711,37 @@
   </cols>
   <sheetData>
     <row r="1" s="50" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="51" t="s">
+      <c r="A1" s="52" t="s">
         <v>367</v>
       </c>
-      <c r="B1" s="51" t="s">
+      <c r="B1" s="52" t="s">
         <v>368</v>
       </c>
-      <c r="C1" s="51" t="s">
+      <c r="C1" s="52" t="s">
         <v>369</v>
       </c>
-      <c r="D1" s="51" t="s">
+      <c r="D1" s="52" t="s">
         <v>370</v>
       </c>
-      <c r="E1" s="51" t="s">
+      <c r="E1" s="52" t="s">
         <v>371</v>
       </c>
-      <c r="F1" s="51" t="s">
+      <c r="F1" s="52" t="s">
         <v>372</v>
       </c>
-      <c r="G1" s="51" t="s">
+      <c r="G1" s="52" t="s">
         <v>373</v>
       </c>
-      <c r="H1" s="51" t="s">
+      <c r="H1" s="52" t="s">
         <v>374</v>
       </c>
-      <c r="I1" s="51" t="s">
+      <c r="I1" s="52" t="s">
         <v>375</v>
       </c>
-      <c r="J1" s="51" t="s">
+      <c r="J1" s="52" t="s">
         <v>376</v>
       </c>
-      <c r="K1" s="51" t="s">
+      <c r="K1" s="52" t="s">
         <v>377</v>
       </c>
       <c r="L1" s="50" t="s">
@@ -5784,36 +5796,36 @@
       <c r="G1" s="39"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="52" t="s">
+      <c r="A2" s="53" t="s">
         <v>102</v>
       </c>
       <c r="B2" s="44" t="s">
         <v>379</v>
       </c>
-      <c r="C2" s="52" t="s">
+      <c r="C2" s="53" t="s">
         <v>380</v>
       </c>
-      <c r="D2" s="52" t="s">
+      <c r="D2" s="53" t="s">
         <v>381</v>
       </c>
-      <c r="E2" s="52"/>
-      <c r="F2" s="52"/>
+      <c r="E2" s="53"/>
+      <c r="F2" s="53"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="53" t="s">
         <v>102</v>
       </c>
       <c r="B3" s="44" t="s">
         <v>382</v>
       </c>
-      <c r="C3" s="52" t="s">
+      <c r="C3" s="53" t="s">
         <v>383</v>
       </c>
-      <c r="D3" s="52" t="s">
+      <c r="D3" s="53" t="s">
         <v>384</v>
       </c>
-      <c r="E3" s="52"/>
-      <c r="F3" s="52"/>
+      <c r="E3" s="53"/>
+      <c r="F3" s="53"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Refactor: Update conditionals to use hidden_value instead of default_value
- Changed the terminology from `default_value` to `hidden_value` in the conditionals logic, affecting the checkConditionals function, validation logic, and related documentation.
</commit_message>
<xml_diff>
--- a/example/demo_generator/references/Household_Travel_Generate_Survey.xlsx
+++ b/example/demo_generator/references/Household_Travel_Generate_Survey.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Widgets" sheetId="1" state="visible" r:id="rId3"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="681" uniqueCount="385">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="682" uniqueCount="386">
   <si>
     <t xml:space="preserve">questionName</t>
   </si>
@@ -753,6 +753,9 @@
   </si>
   <si>
     <t xml:space="preserve">parentheses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hidden_value</t>
   </si>
   <si>
     <t xml:space="preserve">hasHouseholdSize1Conditional</t>
@@ -4156,7 +4159,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="39" width="27.43"/>
@@ -4165,6 +4168,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="40" width="20.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="39" width="19.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="39" width="12.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="14.09"/>
   </cols>
   <sheetData>
     <row r="1" s="43" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4186,17 +4190,20 @@
       <c r="F1" s="41" t="s">
         <v>222</v>
       </c>
+      <c r="G1" s="41" t="s">
+        <v>223</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="44" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B2" s="44"/>
       <c r="C2" s="44" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="D2" s="45" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E2" s="44" t="n">
         <v>1</v>
@@ -4209,10 +4216,10 @@
       </c>
       <c r="B3" s="44"/>
       <c r="C3" s="44" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="D3" s="45" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E3" s="44" t="n">
         <v>2</v>
@@ -4225,13 +4232,13 @@
       </c>
       <c r="B4" s="44"/>
       <c r="C4" s="44" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="D4" s="45" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E4" s="44" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="F4" s="44"/>
     </row>
@@ -4240,13 +4247,13 @@
         <v>163</v>
       </c>
       <c r="B5" s="44" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C5" s="44" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="D5" s="45" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E5" s="44" t="n">
         <v>1</v>
@@ -4255,14 +4262,14 @@
     </row>
     <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="44" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B6" s="44"/>
       <c r="C6" s="44" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D6" s="45" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E6" s="44" t="n">
         <v>3</v>
@@ -4271,16 +4278,16 @@
     </row>
     <row r="7" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="44" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B7" s="44" t="s">
+        <v>233</v>
+      </c>
+      <c r="C7" s="44" t="s">
         <v>232</v>
       </c>
-      <c r="C7" s="44" t="s">
-        <v>231</v>
-      </c>
       <c r="D7" s="45" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E7" s="44" t="n">
         <v>5</v>
@@ -4289,14 +4296,14 @@
     </row>
     <row r="8" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="44" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B8" s="44"/>
       <c r="C8" s="44" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D8" s="45" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E8" s="44" t="n">
         <v>4</v>
@@ -4305,16 +4312,16 @@
     </row>
     <row r="9" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="44" t="s">
+        <v>235</v>
+      </c>
+      <c r="B9" s="44" t="s">
+        <v>233</v>
+      </c>
+      <c r="C9" s="44" t="s">
+        <v>232</v>
+      </c>
+      <c r="D9" s="45" t="s">
         <v>234</v>
-      </c>
-      <c r="B9" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="C9" s="44" t="s">
-        <v>231</v>
-      </c>
-      <c r="D9" s="45" t="s">
-        <v>233</v>
       </c>
       <c r="E9" s="44" t="n">
         <v>13</v>
@@ -4323,14 +4330,14 @@
     </row>
     <row r="10" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="44" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B10" s="44"/>
       <c r="C10" s="44" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D10" s="45" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E10" s="44" t="n">
         <v>5</v>
@@ -4343,10 +4350,10 @@
       </c>
       <c r="B11" s="44"/>
       <c r="C11" s="44" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D11" s="45" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E11" s="44" t="n">
         <v>5</v>
@@ -4359,10 +4366,10 @@
       </c>
       <c r="B12" s="44"/>
       <c r="C12" s="44" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D12" s="45" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E12" s="44" t="n">
         <v>6</v>
@@ -4371,14 +4378,14 @@
     </row>
     <row r="13" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="44" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B13" s="44"/>
       <c r="C13" s="44" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D13" s="45" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E13" s="44" t="n">
         <v>11</v>
@@ -4391,10 +4398,10 @@
       </c>
       <c r="B14" s="44"/>
       <c r="C14" s="44" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D14" s="45" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E14" s="44" t="n">
         <v>14</v>
@@ -4407,10 +4414,10 @@
       </c>
       <c r="B15" s="44"/>
       <c r="C15" s="44" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D15" s="45" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E15" s="44" t="n">
         <v>15</v>
@@ -4423,26 +4430,26 @@
       </c>
       <c r="B16" s="44"/>
       <c r="C16" s="44" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D16" s="45" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="E16" s="44" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="F16" s="44"/>
     </row>
     <row r="17" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="44" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B17" s="44"/>
       <c r="C17" s="44" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D17" s="45" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E17" s="44" t="n">
         <v>15</v>
@@ -4455,10 +4462,10 @@
       </c>
       <c r="B18" s="44"/>
       <c r="C18" s="44" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D18" s="45" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E18" s="44" t="n">
         <v>16</v>
@@ -4467,14 +4474,14 @@
     </row>
     <row r="19" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="44" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B19" s="44"/>
       <c r="C19" s="44" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D19" s="45" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E19" s="44" t="n">
         <v>40</v>
@@ -4487,13 +4494,13 @@
       </c>
       <c r="B20" s="44"/>
       <c r="C20" s="44" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D20" s="45" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E20" s="44" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="F20" s="44"/>
     </row>
@@ -4502,13 +4509,13 @@
         <v>168</v>
       </c>
       <c r="C21" s="39" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="D21" s="45" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E21" s="40" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4516,16 +4523,16 @@
         <v>168</v>
       </c>
       <c r="B22" s="39" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C22" s="39" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="D22" s="45" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E22" s="40" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4533,16 +4540,16 @@
         <v>168</v>
       </c>
       <c r="B23" s="39" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C23" s="39" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="D23" s="45" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E23" s="40" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4550,13 +4557,13 @@
         <v>173</v>
       </c>
       <c r="C24" s="39" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="D24" s="45" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E24" s="40" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4564,16 +4571,16 @@
         <v>173</v>
       </c>
       <c r="B25" s="39" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C25" s="39" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="D25" s="45" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E25" s="40" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4581,16 +4588,16 @@
         <v>173</v>
       </c>
       <c r="B26" s="39" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C26" s="39" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="D26" s="45" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E26" s="40" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4598,13 +4605,13 @@
         <v>179</v>
       </c>
       <c r="C27" s="39" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="D27" s="45" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E27" s="39" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4612,16 +4619,16 @@
         <v>179</v>
       </c>
       <c r="B28" s="39" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C28" s="39" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="D28" s="45" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E28" s="39" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4629,16 +4636,16 @@
         <v>179</v>
       </c>
       <c r="B29" s="39" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C29" s="39" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="D29" s="45" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E29" s="39" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
   </sheetData>
@@ -4675,25 +4682,25 @@
         <v>3</v>
       </c>
       <c r="B1" s="47" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C1" s="46" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D1" s="46" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E1" s="46" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="F1" s="46" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="H1" s="46" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4701,13 +4708,13 @@
         <v>26</v>
       </c>
       <c r="B2" s="44" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C2" s="44" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D2" s="44" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E2" s="48" t="b">
         <f aca="false">TRUE()</f>
@@ -4727,13 +4734,13 @@
         <v>102</v>
       </c>
       <c r="B3" s="44" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C3" s="44" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D3" s="44" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="E3" s="48" t="b">
         <f aca="false">TRUE()</f>
@@ -4753,13 +4760,13 @@
         <v>215</v>
       </c>
       <c r="B4" s="44" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C4" s="44" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D4" s="44" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="E4" s="48" t="b">
         <f aca="false">FALSE()</f>
@@ -4804,7 +4811,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="50" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B1" s="50" t="s">
         <v>221</v>
@@ -4822,24 +4829,24 @@
         <v>9</v>
       </c>
       <c r="G1" s="50" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="H1" s="50" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B2" s="51" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C2" s="51" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D2" s="51" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="E2" s="51"/>
       <c r="F2" s="51"/>
@@ -4848,16 +4855,16 @@
     </row>
     <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
@@ -4872,10 +4879,10 @@
         <v>136</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
@@ -4884,16 +4891,16 @@
     </row>
     <row r="5" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>136</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
@@ -4902,16 +4909,16 @@
     </row>
     <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
@@ -4920,16 +4927,16 @@
     </row>
     <row r="7" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
@@ -4946,7 +4953,7 @@
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
       <c r="G8" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="H8" s="1"/>
     </row>
@@ -4960,7 +4967,7 @@
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
       <c r="G9" s="1" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="H9" s="1"/>
     </row>
@@ -4988,7 +4995,7 @@
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
       <c r="G11" s="1" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="H11" s="1"/>
     </row>
@@ -5002,7 +5009,7 @@
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
       <c r="G12" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="H12" s="1"/>
     </row>
@@ -5016,7 +5023,7 @@
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
       <c r="G13" s="1" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="H13" s="1"/>
     </row>
@@ -5030,7 +5037,7 @@
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
       <c r="G14" s="1" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="H14" s="1"/>
     </row>
@@ -5039,13 +5046,13 @@
         <v>116</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
@@ -5057,13 +5064,13 @@
         <v>116</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
@@ -5080,7 +5087,7 @@
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
       <c r="G17" s="1" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="H17" s="1"/>
     </row>
@@ -5089,13 +5096,13 @@
         <v>125</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
@@ -5107,13 +5114,13 @@
         <v>125</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="E19" s="1"/>
       <c r="F19" s="1"/>
@@ -5130,7 +5137,7 @@
       <c r="E20" s="1"/>
       <c r="F20" s="1"/>
       <c r="G20" s="1" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="H20" s="1"/>
     </row>
@@ -5139,19 +5146,19 @@
         <v>132</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E21" s="1"/>
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
       <c r="H21" s="1" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5159,19 +5166,19 @@
         <v>132</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="E22" s="1"/>
       <c r="F22" s="1"/>
       <c r="G22" s="1"/>
       <c r="H22" s="1" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5179,19 +5186,19 @@
         <v>132</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="E23" s="1"/>
       <c r="F23" s="1"/>
       <c r="G23" s="1"/>
       <c r="H23" s="1" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5199,13 +5206,13 @@
         <v>132</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E24" s="1"/>
       <c r="F24" s="1"/>
@@ -5217,19 +5224,19 @@
         <v>132</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E25" s="1"/>
       <c r="F25" s="1"/>
       <c r="G25" s="1"/>
       <c r="H25" s="1" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5251,13 +5258,13 @@
         <v>137</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
@@ -5269,13 +5276,13 @@
         <v>137</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="E28" s="1"/>
       <c r="F28" s="1"/>
@@ -5287,13 +5294,13 @@
         <v>137</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="E29" s="1"/>
       <c r="F29" s="1"/>
@@ -5305,13 +5312,13 @@
         <v>137</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="E30" s="1"/>
       <c r="F30" s="1"/>
@@ -5323,13 +5330,13 @@
         <v>137</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="E31" s="1"/>
       <c r="F31" s="1"/>
@@ -5341,19 +5348,19 @@
         <v>137</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="E32" s="1"/>
       <c r="F32" s="1"/>
       <c r="G32" s="1"/>
       <c r="H32" s="1" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5361,13 +5368,13 @@
         <v>137</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="E33" s="1"/>
       <c r="F33" s="1"/>
@@ -5379,13 +5386,13 @@
         <v>137</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="E34" s="1"/>
       <c r="F34" s="1"/>
@@ -5397,13 +5404,13 @@
         <v>137</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="E35" s="1"/>
       <c r="F35" s="1"/>
@@ -5415,13 +5422,13 @@
         <v>137</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E36" s="1"/>
       <c r="F36" s="1"/>
@@ -5433,13 +5440,13 @@
         <v>137</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="E37" s="1"/>
       <c r="F37" s="1"/>
@@ -5454,10 +5461,10 @@
         <v>136</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="E38" s="1"/>
       <c r="F38" s="1"/>
@@ -5469,13 +5476,13 @@
         <v>137</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="E39" s="1"/>
       <c r="F39" s="1"/>
@@ -5492,7 +5499,7 @@
       <c r="E40" s="1"/>
       <c r="F40" s="1"/>
       <c r="G40" s="1" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="H40" s="1"/>
     </row>
@@ -5501,13 +5508,13 @@
         <v>158</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="E41" s="1"/>
       <c r="F41" s="1"/>
@@ -5519,13 +5526,13 @@
         <v>158</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="E42" s="1"/>
       <c r="F42" s="1"/>
@@ -5542,7 +5549,7 @@
       <c r="E43" s="1"/>
       <c r="F43" s="1"/>
       <c r="G43" s="1" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="H43" s="1"/>
     </row>
@@ -5551,13 +5558,13 @@
         <v>165</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="E44" s="1"/>
       <c r="F44" s="1"/>
@@ -5569,13 +5576,13 @@
         <v>165</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E45" s="1"/>
       <c r="F45" s="1"/>
@@ -5587,13 +5594,13 @@
         <v>165</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="E46" s="1"/>
       <c r="F46" s="1"/>
@@ -5605,13 +5612,13 @@
         <v>165</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="E47" s="1"/>
       <c r="F47" s="1"/>
@@ -5623,13 +5630,13 @@
         <v>165</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="E48" s="1"/>
       <c r="F48" s="1"/>
@@ -5641,13 +5648,13 @@
         <v>174</v>
       </c>
       <c r="B49" s="49" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C49" s="49" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="D49" s="49" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5655,13 +5662,13 @@
         <v>174</v>
       </c>
       <c r="B50" s="49" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C50" s="49" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="D50" s="49" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5669,13 +5676,13 @@
         <v>174</v>
       </c>
       <c r="B51" s="49" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C51" s="49" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="D51" s="49" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -5712,40 +5719,40 @@
   <sheetData>
     <row r="1" s="50" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="52" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="B1" s="52" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C1" s="52" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="D1" s="52" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="E1" s="52" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="F1" s="52" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="G1" s="52" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="H1" s="52" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="I1" s="52" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="J1" s="52" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="K1" s="52" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="L1" s="50" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
     </row>
   </sheetData>
@@ -5800,13 +5807,13 @@
         <v>102</v>
       </c>
       <c r="B2" s="44" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="C2" s="53" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="D2" s="53" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="E2" s="53"/>
       <c r="F2" s="53"/>
@@ -5816,13 +5823,13 @@
         <v>102</v>
       </c>
       <c r="B3" s="44" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="C3" s="53" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="D3" s="53" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="E3" s="53"/>
       <c r="F3" s="53"/>

</xml_diff>

<commit_message>
Feature: Add suffixLabel support to InputString component
Fix: #1241
- Introduced a new optional suffixLabel property in the InputString component, allowing for additional context next to the input field (e.g., units like %, days, hours).
</commit_message>
<xml_diff>
--- a/example/demo_generator/references/Household_Travel_Generate_Survey.xlsx
+++ b/example/demo_generator/references/Household_Travel_Generate_Survey.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Widgets" sheetId="1" state="visible" r:id="rId3"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="683" uniqueCount="386">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="682" uniqueCount="385">
   <si>
     <t xml:space="preserve">questionName</t>
   </si>
@@ -753,9 +753,6 @@
   </si>
   <si>
     <t xml:space="preserve">parentheses</t>
-  </si>
-  <si>
-    <t xml:space="preserve">value_when_hidden</t>
   </si>
   <si>
     <t xml:space="preserve">hasHouseholdSize1Conditional</t>
@@ -1248,13 +1245,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="General"/>
     <numFmt numFmtId="166" formatCode="@"/>
-    <numFmt numFmtId="167" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1296,6 +1292,12 @@
     <font>
       <sz val="10"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <name val="Calibri"/>
       <family val="0"/>
       <charset val="1"/>
@@ -1527,6 +1529,10 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1535,15 +1541,7 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1551,23 +1549,15 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1575,7 +1565,11 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1583,7 +1577,11 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1591,7 +1589,7 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1599,15 +1597,19 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1615,15 +1617,19 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1635,11 +1641,11 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1651,11 +1657,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1671,15 +1677,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1691,15 +1693,15 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2576,7 +2578,7 @@
       </c>
       <c r="X10" s="7"/>
     </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
         <v>64</v>
       </c>
@@ -2652,7 +2654,7 @@
       <c r="J12" s="7"/>
       <c r="K12" s="7"/>
       <c r="L12" s="7"/>
-      <c r="M12" s="10"/>
+      <c r="M12" s="11"/>
       <c r="N12" s="7"/>
       <c r="O12" s="7"/>
       <c r="P12" s="7"/>
@@ -2866,7 +2868,7 @@
       <c r="W16" s="7"/>
       <c r="X16" s="7"/>
     </row>
-    <row r="17" s="11" customFormat="true" ht="76.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="17" s="12" customFormat="true" ht="76.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
         <v>92</v>
       </c>
@@ -2916,33 +2918,33 @@
       <c r="X17" s="7"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="12" t="s">
+      <c r="A18" s="13" t="s">
         <v>97</v>
       </c>
-      <c r="B18" s="12" t="s">
+      <c r="B18" s="13" t="s">
         <v>98</v>
       </c>
-      <c r="C18" s="13" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D18" s="14" t="s">
+      <c r="C18" s="14" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D18" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E18" s="7"/>
-      <c r="F18" s="15" t="str">
+      <c r="F18" s="16" t="str">
         <f aca="false">REPLACE(A18, FIND("_", A18), 1, ".")</f>
         <v>home.save</v>
       </c>
-      <c r="G18" s="12" t="s">
+      <c r="G18" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="H18" s="12" t="s">
+      <c r="H18" s="13" t="s">
         <v>100</v>
       </c>
-      <c r="I18" s="12"/>
-      <c r="J18" s="12"/>
-      <c r="K18" s="12"/>
+      <c r="I18" s="13"/>
+      <c r="J18" s="13"/>
+      <c r="K18" s="13"/>
       <c r="L18" s="7"/>
       <c r="M18" s="7"/>
       <c r="N18" s="7"/>
@@ -2951,7 +2953,7 @@
       <c r="Q18" s="7"/>
       <c r="R18" s="7"/>
       <c r="S18" s="7"/>
-      <c r="T18" s="16" t="b">
+      <c r="T18" s="17" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2961,1129 +2963,1129 @@
       <c r="X18" s="7"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="17" t="s">
+      <c r="A19" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="B19" s="18" t="s">
+      <c r="B19" s="19" t="s">
         <v>69</v>
       </c>
-      <c r="C19" s="19" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D19" s="20" t="s">
+      <c r="C19" s="20" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D19" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E19" s="21"/>
-      <c r="F19" s="21"/>
-      <c r="G19" s="17"/>
-      <c r="H19" s="17"/>
-      <c r="I19" s="17"/>
-      <c r="J19" s="17"/>
-      <c r="K19" s="17"/>
-      <c r="L19" s="21"/>
-      <c r="M19" s="21"/>
-      <c r="N19" s="21"/>
-      <c r="O19" s="21"/>
-      <c r="P19" s="21"/>
-      <c r="Q19" s="21"/>
-      <c r="R19" s="21"/>
-      <c r="S19" s="21"/>
-      <c r="T19" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U19" s="21"/>
-      <c r="V19" s="21"/>
-      <c r="W19" s="21"/>
-      <c r="X19" s="21"/>
+      <c r="E19" s="22"/>
+      <c r="F19" s="22"/>
+      <c r="G19" s="18"/>
+      <c r="H19" s="18"/>
+      <c r="I19" s="18"/>
+      <c r="J19" s="18"/>
+      <c r="K19" s="18"/>
+      <c r="L19" s="22"/>
+      <c r="M19" s="22"/>
+      <c r="N19" s="22"/>
+      <c r="O19" s="22"/>
+      <c r="P19" s="22"/>
+      <c r="Q19" s="22"/>
+      <c r="R19" s="22"/>
+      <c r="S19" s="22"/>
+      <c r="T19" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U19" s="22"/>
+      <c r="V19" s="22"/>
+      <c r="W19" s="22"/>
+      <c r="X19" s="22"/>
     </row>
     <row r="20" customFormat="false" ht="144" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="20" t="s">
+      <c r="A20" s="21" t="s">
         <v>103</v>
       </c>
-      <c r="B20" s="20" t="s">
+      <c r="B20" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="C20" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D20" s="20" t="s">
+      <c r="C20" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D20" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E20" s="23" t="s">
+      <c r="E20" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F20" s="23" t="s">
+      <c r="F20" s="24" t="s">
         <v>104</v>
       </c>
-      <c r="G20" s="20" t="s">
+      <c r="G20" s="21" t="s">
         <v>105</v>
       </c>
-      <c r="H20" s="20" t="s">
+      <c r="H20" s="21" t="s">
         <v>106</v>
       </c>
-      <c r="I20" s="20"/>
-      <c r="J20" s="20"/>
-      <c r="K20" s="20"/>
-      <c r="L20" s="23"/>
-      <c r="M20" s="23" t="s">
+      <c r="I20" s="21"/>
+      <c r="J20" s="21"/>
+      <c r="K20" s="21"/>
+      <c r="L20" s="24"/>
+      <c r="M20" s="24" t="s">
         <v>95</v>
       </c>
-      <c r="N20" s="24"/>
-      <c r="O20" s="23"/>
-      <c r="P20" s="23"/>
-      <c r="Q20" s="23"/>
-      <c r="R20" s="23"/>
-      <c r="S20" s="23"/>
-      <c r="T20" s="20" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U20" s="23"/>
-      <c r="V20" s="23"/>
-      <c r="W20" s="23"/>
-      <c r="X20" s="23"/>
+      <c r="N20" s="25"/>
+      <c r="O20" s="24"/>
+      <c r="P20" s="24"/>
+      <c r="Q20" s="24"/>
+      <c r="R20" s="24"/>
+      <c r="S20" s="24"/>
+      <c r="T20" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U20" s="24"/>
+      <c r="V20" s="24"/>
+      <c r="W20" s="24"/>
+      <c r="X20" s="24"/>
     </row>
     <row r="21" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="20" t="s">
+      <c r="A21" s="21" t="s">
         <v>107</v>
       </c>
-      <c r="B21" s="20" t="s">
+      <c r="B21" s="21" t="s">
         <v>108</v>
       </c>
-      <c r="C21" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D21" s="20" t="s">
+      <c r="C21" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D21" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E21" s="23" t="s">
+      <c r="E21" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F21" s="23" t="s">
+      <c r="F21" s="24" t="s">
         <v>109</v>
       </c>
-      <c r="G21" s="20" t="s">
+      <c r="G21" s="21" t="s">
         <v>110</v>
       </c>
-      <c r="H21" s="20" t="s">
+      <c r="H21" s="21" t="s">
         <v>111</v>
       </c>
-      <c r="I21" s="20" t="s">
+      <c r="I21" s="21" t="s">
         <v>112</v>
       </c>
-      <c r="J21" s="20" t="s">
+      <c r="J21" s="21" t="s">
         <v>113</v>
       </c>
-      <c r="K21" s="20"/>
-      <c r="L21" s="23"/>
-      <c r="M21" s="23"/>
-      <c r="N21" s="23" t="s">
+      <c r="K21" s="21"/>
+      <c r="L21" s="24"/>
+      <c r="M21" s="24"/>
+      <c r="N21" s="24" t="s">
         <v>114</v>
       </c>
-      <c r="O21" s="23"/>
-      <c r="P21" s="23"/>
-      <c r="Q21" s="23"/>
-      <c r="R21" s="23"/>
-      <c r="S21" s="23"/>
-      <c r="T21" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U21" s="23"/>
-      <c r="V21" s="23"/>
-      <c r="W21" s="23"/>
-      <c r="X21" s="23"/>
+      <c r="O21" s="24"/>
+      <c r="P21" s="24"/>
+      <c r="Q21" s="24"/>
+      <c r="R21" s="24"/>
+      <c r="S21" s="24"/>
+      <c r="T21" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U21" s="24"/>
+      <c r="V21" s="24"/>
+      <c r="W21" s="24"/>
+      <c r="X21" s="24"/>
     </row>
     <row r="22" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="20" t="s">
+      <c r="A22" s="21" t="s">
         <v>115</v>
       </c>
-      <c r="B22" s="20" t="s">
+      <c r="B22" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="C22" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D22" s="20" t="s">
+      <c r="C22" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D22" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E22" s="23" t="s">
+      <c r="E22" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F22" s="23" t="s">
+      <c r="F22" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="G22" s="20" t="s">
+      <c r="G22" s="21" t="s">
         <v>117</v>
       </c>
-      <c r="H22" s="20" t="s">
+      <c r="H22" s="21" t="s">
         <v>118</v>
       </c>
-      <c r="I22" s="20"/>
-      <c r="J22" s="20"/>
-      <c r="K22" s="20"/>
-      <c r="L22" s="23"/>
-      <c r="M22" s="23" t="s">
+      <c r="I22" s="21"/>
+      <c r="J22" s="21"/>
+      <c r="K22" s="21"/>
+      <c r="L22" s="24"/>
+      <c r="M22" s="24" t="s">
         <v>119</v>
       </c>
-      <c r="N22" s="23"/>
-      <c r="O22" s="23" t="s">
+      <c r="N22" s="24"/>
+      <c r="O22" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="P22" s="23"/>
-      <c r="Q22" s="23"/>
-      <c r="R22" s="23"/>
-      <c r="S22" s="23"/>
-      <c r="T22" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U22" s="23"/>
-      <c r="V22" s="23"/>
-      <c r="W22" s="23"/>
-      <c r="X22" s="23"/>
+      <c r="P22" s="24"/>
+      <c r="Q22" s="24"/>
+      <c r="R22" s="24"/>
+      <c r="S22" s="24"/>
+      <c r="T22" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U22" s="24"/>
+      <c r="V22" s="24"/>
+      <c r="W22" s="24"/>
+      <c r="X22" s="24"/>
     </row>
     <row r="23" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="20" t="s">
+      <c r="A23" s="21" t="s">
         <v>120</v>
       </c>
-      <c r="B23" s="20" t="s">
+      <c r="B23" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="C23" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D23" s="20" t="s">
+      <c r="C23" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D23" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E23" s="23" t="s">
+      <c r="E23" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F23" s="23" t="s">
+      <c r="F23" s="24" t="s">
         <v>121</v>
       </c>
-      <c r="G23" s="20" t="s">
+      <c r="G23" s="21" t="s">
         <v>122</v>
       </c>
-      <c r="H23" s="20" t="s">
+      <c r="H23" s="21" t="s">
         <v>123</v>
       </c>
-      <c r="I23" s="20"/>
-      <c r="J23" s="20"/>
-      <c r="K23" s="20"/>
-      <c r="L23" s="23"/>
-      <c r="M23" s="23" t="s">
+      <c r="I23" s="21"/>
+      <c r="J23" s="21"/>
+      <c r="K23" s="21"/>
+      <c r="L23" s="24"/>
+      <c r="M23" s="24" t="s">
         <v>124</v>
       </c>
-      <c r="N23" s="23"/>
-      <c r="O23" s="23" t="s">
+      <c r="N23" s="24"/>
+      <c r="O23" s="24" t="s">
         <v>125</v>
       </c>
-      <c r="P23" s="23"/>
-      <c r="Q23" s="23"/>
-      <c r="R23" s="23"/>
-      <c r="S23" s="23"/>
-      <c r="T23" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U23" s="23"/>
-      <c r="V23" s="23"/>
-      <c r="W23" s="23"/>
-      <c r="X23" s="23"/>
+      <c r="P23" s="24"/>
+      <c r="Q23" s="24"/>
+      <c r="R23" s="24"/>
+      <c r="S23" s="24"/>
+      <c r="T23" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U23" s="24"/>
+      <c r="V23" s="24"/>
+      <c r="W23" s="24"/>
+      <c r="X23" s="24"/>
     </row>
     <row r="24" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="20" t="s">
+      <c r="A24" s="21" t="s">
         <v>126</v>
       </c>
-      <c r="B24" s="20" t="s">
+      <c r="B24" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="C24" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D24" s="20" t="s">
+      <c r="C24" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D24" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E24" s="23" t="s">
+      <c r="E24" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F24" s="23" t="s">
+      <c r="F24" s="24" t="s">
         <v>127</v>
       </c>
-      <c r="G24" s="20" t="s">
+      <c r="G24" s="21" t="s">
         <v>128</v>
       </c>
-      <c r="H24" s="20" t="s">
+      <c r="H24" s="21" t="s">
         <v>129</v>
       </c>
-      <c r="I24" s="20"/>
-      <c r="J24" s="20"/>
-      <c r="K24" s="20"/>
-      <c r="L24" s="23"/>
-      <c r="M24" s="23" t="s">
+      <c r="I24" s="21"/>
+      <c r="J24" s="21"/>
+      <c r="K24" s="21"/>
+      <c r="L24" s="24"/>
+      <c r="M24" s="24" t="s">
         <v>130</v>
       </c>
-      <c r="N24" s="23"/>
-      <c r="O24" s="23" t="s">
+      <c r="N24" s="24"/>
+      <c r="O24" s="24" t="s">
         <v>125</v>
       </c>
-      <c r="P24" s="24"/>
-      <c r="Q24" s="23"/>
-      <c r="R24" s="23"/>
-      <c r="S24" s="23"/>
-      <c r="T24" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U24" s="23"/>
-      <c r="V24" s="23"/>
-      <c r="W24" s="23"/>
-      <c r="X24" s="23"/>
+      <c r="P24" s="25"/>
+      <c r="Q24" s="24"/>
+      <c r="R24" s="24"/>
+      <c r="S24" s="24"/>
+      <c r="T24" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U24" s="24"/>
+      <c r="V24" s="24"/>
+      <c r="W24" s="24"/>
+      <c r="X24" s="24"/>
     </row>
     <row r="25" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="20" t="s">
+      <c r="A25" s="21" t="s">
         <v>131</v>
       </c>
-      <c r="B25" s="20" t="s">
+      <c r="B25" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="C25" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D25" s="20" t="s">
+      <c r="C25" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D25" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E25" s="23" t="s">
+      <c r="E25" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F25" s="23" t="s">
+      <c r="F25" s="24" t="s">
         <v>132</v>
       </c>
-      <c r="G25" s="20"/>
-      <c r="H25" s="20"/>
-      <c r="I25" s="20"/>
-      <c r="J25" s="20"/>
-      <c r="K25" s="25" t="s">
+      <c r="G25" s="21"/>
+      <c r="H25" s="21"/>
+      <c r="I25" s="21"/>
+      <c r="J25" s="21"/>
+      <c r="K25" s="26" t="s">
         <v>133</v>
       </c>
-      <c r="L25" s="23"/>
-      <c r="M25" s="26" t="s">
+      <c r="L25" s="24"/>
+      <c r="M25" s="27" t="s">
         <v>134</v>
       </c>
-      <c r="N25" s="23"/>
-      <c r="O25" s="23" t="s">
+      <c r="N25" s="24"/>
+      <c r="O25" s="24" t="s">
         <v>132</v>
       </c>
-      <c r="P25" s="23"/>
-      <c r="Q25" s="23"/>
-      <c r="R25" s="23"/>
-      <c r="S25" s="23"/>
-      <c r="T25" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U25" s="23" t="s">
+      <c r="P25" s="24"/>
+      <c r="Q25" s="24"/>
+      <c r="R25" s="24"/>
+      <c r="S25" s="24"/>
+      <c r="T25" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U25" s="24" t="s">
         <v>135</v>
       </c>
-      <c r="V25" s="23" t="s">
+      <c r="V25" s="24" t="s">
         <v>136</v>
       </c>
-      <c r="W25" s="23"/>
-      <c r="X25" s="23"/>
+      <c r="W25" s="24"/>
+      <c r="X25" s="24"/>
     </row>
     <row r="26" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="20" t="s">
+      <c r="A26" s="21" t="s">
         <v>137</v>
       </c>
-      <c r="B26" s="20" t="s">
+      <c r="B26" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="C26" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D26" s="20" t="s">
+      <c r="C26" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D26" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E26" s="23" t="s">
+      <c r="E26" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F26" s="27" t="s">
+      <c r="F26" s="28" t="s">
         <v>138</v>
       </c>
-      <c r="G26" s="20" t="s">
+      <c r="G26" s="21" t="s">
         <v>139</v>
       </c>
-      <c r="H26" s="20" t="s">
+      <c r="H26" s="21" t="s">
         <v>140</v>
       </c>
-      <c r="I26" s="20"/>
-      <c r="J26" s="20"/>
-      <c r="K26" s="20"/>
-      <c r="L26" s="23"/>
-      <c r="M26" s="23" t="s">
+      <c r="I26" s="21"/>
+      <c r="J26" s="21"/>
+      <c r="K26" s="21"/>
+      <c r="L26" s="24"/>
+      <c r="M26" s="24" t="s">
         <v>141</v>
       </c>
-      <c r="N26" s="23"/>
-      <c r="O26" s="23" t="s">
+      <c r="N26" s="24"/>
+      <c r="O26" s="24" t="s">
         <v>137</v>
       </c>
-      <c r="P26" s="23"/>
-      <c r="Q26" s="23"/>
-      <c r="R26" s="23"/>
-      <c r="S26" s="23"/>
-      <c r="T26" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U26" s="23"/>
-      <c r="V26" s="23"/>
-      <c r="W26" s="23"/>
-      <c r="X26" s="23"/>
+      <c r="P26" s="24"/>
+      <c r="Q26" s="24"/>
+      <c r="R26" s="24"/>
+      <c r="S26" s="24"/>
+      <c r="T26" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U26" s="24"/>
+      <c r="V26" s="24"/>
+      <c r="W26" s="24"/>
+      <c r="X26" s="24"/>
     </row>
     <row r="27" customFormat="false" ht="62.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="20" t="s">
+      <c r="A27" s="21" t="s">
         <v>142</v>
       </c>
-      <c r="B27" s="20" t="s">
+      <c r="B27" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="C27" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D27" s="20" t="s">
+      <c r="C27" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D27" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E27" s="23" t="s">
+      <c r="E27" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F27" s="23" t="s">
+      <c r="F27" s="24" t="s">
         <v>143</v>
       </c>
-      <c r="G27" s="20" t="s">
+      <c r="G27" s="21" t="s">
         <v>144</v>
       </c>
-      <c r="H27" s="20" t="s">
+      <c r="H27" s="21" t="s">
         <v>145</v>
       </c>
-      <c r="I27" s="20"/>
-      <c r="J27" s="20"/>
-      <c r="K27" s="20"/>
-      <c r="L27" s="23"/>
-      <c r="M27" s="23" t="s">
+      <c r="I27" s="21"/>
+      <c r="J27" s="21"/>
+      <c r="K27" s="21"/>
+      <c r="L27" s="24"/>
+      <c r="M27" s="24" t="s">
         <v>130</v>
       </c>
-      <c r="N27" s="23"/>
-      <c r="O27" s="23" t="s">
+      <c r="N27" s="24"/>
+      <c r="O27" s="24" t="s">
         <v>146</v>
       </c>
-      <c r="P27" s="23"/>
-      <c r="Q27" s="23"/>
-      <c r="R27" s="23"/>
-      <c r="S27" s="23"/>
-      <c r="T27" s="20" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U27" s="23"/>
-      <c r="V27" s="23"/>
-      <c r="W27" s="23"/>
-      <c r="X27" s="23"/>
+      <c r="P27" s="24"/>
+      <c r="Q27" s="24"/>
+      <c r="R27" s="24"/>
+      <c r="S27" s="24"/>
+      <c r="T27" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U27" s="24"/>
+      <c r="V27" s="24"/>
+      <c r="W27" s="24"/>
+      <c r="X27" s="24"/>
     </row>
     <row r="28" customFormat="false" ht="52.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="20" t="s">
+      <c r="A28" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="B28" s="20" t="s">
+      <c r="B28" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="C28" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D28" s="20" t="s">
+      <c r="C28" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D28" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E28" s="23" t="s">
+      <c r="E28" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F28" s="23" t="s">
+      <c r="F28" s="24" t="s">
         <v>148</v>
       </c>
-      <c r="G28" s="20" t="s">
+      <c r="G28" s="21" t="s">
         <v>149</v>
       </c>
-      <c r="H28" s="20" t="s">
+      <c r="H28" s="21" t="s">
         <v>150</v>
       </c>
-      <c r="I28" s="20"/>
-      <c r="J28" s="20"/>
-      <c r="K28" s="20"/>
-      <c r="L28" s="23"/>
-      <c r="M28" s="23" t="s">
+      <c r="I28" s="21"/>
+      <c r="J28" s="21"/>
+      <c r="K28" s="21"/>
+      <c r="L28" s="24"/>
+      <c r="M28" s="24" t="s">
         <v>151</v>
       </c>
-      <c r="N28" s="23"/>
-      <c r="O28" s="23" t="s">
+      <c r="N28" s="24"/>
+      <c r="O28" s="24" t="s">
         <v>146</v>
       </c>
-      <c r="P28" s="23"/>
-      <c r="Q28" s="23"/>
-      <c r="R28" s="23"/>
-      <c r="S28" s="23"/>
-      <c r="T28" s="20" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U28" s="23"/>
-      <c r="V28" s="23"/>
-      <c r="W28" s="23"/>
-      <c r="X28" s="23"/>
+      <c r="P28" s="24"/>
+      <c r="Q28" s="24"/>
+      <c r="R28" s="24"/>
+      <c r="S28" s="24"/>
+      <c r="T28" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U28" s="24"/>
+      <c r="V28" s="24"/>
+      <c r="W28" s="24"/>
+      <c r="X28" s="24"/>
     </row>
     <row r="29" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="28" t="s">
+      <c r="A29" s="29" t="s">
         <v>152</v>
       </c>
-      <c r="B29" s="20" t="s">
+      <c r="B29" s="21" t="s">
         <v>153</v>
       </c>
-      <c r="C29" s="22" t="b">
+      <c r="C29" s="23" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="D29" s="20" t="s">
+      <c r="D29" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E29" s="23" t="s">
+      <c r="E29" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F29" s="23" t="s">
+      <c r="F29" s="24" t="s">
         <v>154</v>
       </c>
-      <c r="G29" s="20" t="s">
+      <c r="G29" s="21" t="s">
         <v>155</v>
       </c>
-      <c r="H29" s="20" t="s">
+      <c r="H29" s="21" t="s">
         <v>156</v>
       </c>
-      <c r="I29" s="20"/>
-      <c r="J29" s="20"/>
-      <c r="K29" s="20"/>
-      <c r="L29" s="23"/>
-      <c r="M29" s="23" t="s">
+      <c r="I29" s="21"/>
+      <c r="J29" s="21"/>
+      <c r="K29" s="21"/>
+      <c r="L29" s="24"/>
+      <c r="M29" s="24" t="s">
         <v>157</v>
       </c>
-      <c r="N29" s="24"/>
-      <c r="O29" s="23" t="s">
+      <c r="N29" s="25"/>
+      <c r="O29" s="24" t="s">
         <v>158</v>
       </c>
-      <c r="P29" s="23"/>
-      <c r="Q29" s="23"/>
-      <c r="R29" s="23"/>
-      <c r="S29" s="23"/>
-      <c r="T29" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U29" s="23"/>
-      <c r="V29" s="23"/>
-      <c r="W29" s="23"/>
-      <c r="X29" s="23"/>
+      <c r="P29" s="24"/>
+      <c r="Q29" s="24"/>
+      <c r="R29" s="24"/>
+      <c r="S29" s="24"/>
+      <c r="T29" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U29" s="24"/>
+      <c r="V29" s="24"/>
+      <c r="W29" s="24"/>
+      <c r="X29" s="24"/>
     </row>
     <row r="30" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="20" t="s">
+      <c r="A30" s="21" t="s">
         <v>159</v>
       </c>
-      <c r="B30" s="20" t="s">
+      <c r="B30" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="C30" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D30" s="20" t="s">
+      <c r="C30" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D30" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E30" s="23" t="s">
+      <c r="E30" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F30" s="23" t="s">
+      <c r="F30" s="24" t="s">
         <v>160</v>
       </c>
-      <c r="G30" s="20" t="s">
+      <c r="G30" s="21" t="s">
         <v>161</v>
       </c>
-      <c r="H30" s="20" t="s">
+      <c r="H30" s="21" t="s">
         <v>162</v>
       </c>
-      <c r="I30" s="20"/>
-      <c r="J30" s="20"/>
-      <c r="K30" s="20"/>
-      <c r="L30" s="23"/>
-      <c r="M30" s="23" t="s">
+      <c r="I30" s="21"/>
+      <c r="J30" s="21"/>
+      <c r="K30" s="21"/>
+      <c r="L30" s="24"/>
+      <c r="M30" s="24" t="s">
         <v>163</v>
       </c>
-      <c r="N30" s="23"/>
-      <c r="O30" s="23" t="s">
+      <c r="N30" s="24"/>
+      <c r="O30" s="24" t="s">
         <v>96</v>
       </c>
-      <c r="P30" s="23"/>
-      <c r="Q30" s="23"/>
-      <c r="R30" s="23"/>
-      <c r="S30" s="23"/>
-      <c r="T30" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U30" s="23"/>
-      <c r="V30" s="23"/>
-      <c r="W30" s="23"/>
-      <c r="X30" s="23"/>
+      <c r="P30" s="24"/>
+      <c r="Q30" s="24"/>
+      <c r="R30" s="24"/>
+      <c r="S30" s="24"/>
+      <c r="T30" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U30" s="24"/>
+      <c r="V30" s="24"/>
+      <c r="W30" s="24"/>
+      <c r="X30" s="24"/>
     </row>
     <row r="31" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="20" t="s">
+      <c r="A31" s="21" t="s">
         <v>164</v>
       </c>
-      <c r="B31" s="20" t="s">
+      <c r="B31" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="C31" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D31" s="20" t="s">
+      <c r="C31" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D31" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E31" s="23" t="s">
+      <c r="E31" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F31" s="23" t="s">
+      <c r="F31" s="24" t="s">
         <v>165</v>
       </c>
-      <c r="G31" s="20" t="s">
+      <c r="G31" s="21" t="s">
         <v>166</v>
       </c>
-      <c r="H31" s="20" t="s">
+      <c r="H31" s="21" t="s">
         <v>167</v>
       </c>
-      <c r="I31" s="20"/>
-      <c r="J31" s="20"/>
-      <c r="K31" s="20"/>
-      <c r="L31" s="23"/>
-      <c r="M31" s="23" t="s">
+      <c r="I31" s="21"/>
+      <c r="J31" s="21"/>
+      <c r="K31" s="21"/>
+      <c r="L31" s="24"/>
+      <c r="M31" s="24" t="s">
         <v>168</v>
       </c>
-      <c r="N31" s="23"/>
-      <c r="O31" s="23" t="s">
+      <c r="N31" s="24"/>
+      <c r="O31" s="24" t="s">
         <v>165</v>
       </c>
-      <c r="P31" s="23"/>
-      <c r="Q31" s="23"/>
-      <c r="R31" s="23"/>
-      <c r="S31" s="23"/>
-      <c r="T31" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U31" s="23"/>
-      <c r="V31" s="23"/>
-      <c r="W31" s="23"/>
-      <c r="X31" s="23"/>
+      <c r="P31" s="24"/>
+      <c r="Q31" s="24"/>
+      <c r="R31" s="24"/>
+      <c r="S31" s="24"/>
+      <c r="T31" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U31" s="24"/>
+      <c r="V31" s="24"/>
+      <c r="W31" s="24"/>
+      <c r="X31" s="24"/>
     </row>
     <row r="32" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="20" t="s">
+      <c r="A32" s="21" t="s">
         <v>169</v>
       </c>
-      <c r="B32" s="20" t="s">
+      <c r="B32" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="C32" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D32" s="20" t="s">
+      <c r="C32" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D32" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E32" s="23" t="s">
+      <c r="E32" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F32" s="23" t="s">
+      <c r="F32" s="24" t="s">
         <v>170</v>
       </c>
-      <c r="G32" s="20" t="s">
+      <c r="G32" s="21" t="s">
         <v>171</v>
       </c>
-      <c r="H32" s="20" t="s">
+      <c r="H32" s="21" t="s">
         <v>172</v>
       </c>
-      <c r="I32" s="20"/>
-      <c r="J32" s="20"/>
-      <c r="K32" s="20"/>
-      <c r="L32" s="23"/>
-      <c r="M32" s="23" t="s">
+      <c r="I32" s="21"/>
+      <c r="J32" s="21"/>
+      <c r="K32" s="21"/>
+      <c r="L32" s="24"/>
+      <c r="M32" s="24" t="s">
         <v>173</v>
       </c>
-      <c r="N32" s="23"/>
-      <c r="O32" s="23" t="s">
+      <c r="N32" s="24"/>
+      <c r="O32" s="24" t="s">
         <v>174</v>
       </c>
-      <c r="P32" s="23"/>
-      <c r="Q32" s="23"/>
-      <c r="R32" s="23"/>
-      <c r="S32" s="23"/>
-      <c r="T32" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U32" s="23"/>
-      <c r="V32" s="23"/>
-      <c r="W32" s="23"/>
-      <c r="X32" s="23"/>
+      <c r="P32" s="24"/>
+      <c r="Q32" s="24"/>
+      <c r="R32" s="24"/>
+      <c r="S32" s="24"/>
+      <c r="T32" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U32" s="24"/>
+      <c r="V32" s="24"/>
+      <c r="W32" s="24"/>
+      <c r="X32" s="24"/>
     </row>
     <row r="33" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="20" t="s">
+      <c r="A33" s="21" t="s">
         <v>175</v>
       </c>
-      <c r="B33" s="20" t="s">
+      <c r="B33" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="C33" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D33" s="20" t="s">
+      <c r="C33" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D33" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E33" s="23" t="s">
+      <c r="E33" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F33" s="23" t="s">
+      <c r="F33" s="24" t="s">
         <v>176</v>
       </c>
-      <c r="G33" s="20" t="s">
+      <c r="G33" s="21" t="s">
         <v>177</v>
       </c>
-      <c r="H33" s="20" t="s">
+      <c r="H33" s="21" t="s">
         <v>178</v>
       </c>
-      <c r="I33" s="20"/>
-      <c r="J33" s="20"/>
-      <c r="K33" s="20"/>
-      <c r="L33" s="23"/>
-      <c r="M33" s="20" t="s">
+      <c r="I33" s="21"/>
+      <c r="J33" s="21"/>
+      <c r="K33" s="21"/>
+      <c r="L33" s="24"/>
+      <c r="M33" s="21" t="s">
         <v>179</v>
       </c>
-      <c r="N33" s="23"/>
-      <c r="O33" s="23"/>
-      <c r="P33" s="23"/>
-      <c r="Q33" s="23"/>
-      <c r="R33" s="23"/>
-      <c r="S33" s="23"/>
-      <c r="T33" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U33" s="23"/>
-      <c r="V33" s="23"/>
-      <c r="W33" s="23"/>
-      <c r="X33" s="23"/>
+      <c r="N33" s="24"/>
+      <c r="O33" s="24"/>
+      <c r="P33" s="24"/>
+      <c r="Q33" s="24"/>
+      <c r="R33" s="24"/>
+      <c r="S33" s="24"/>
+      <c r="T33" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U33" s="24"/>
+      <c r="V33" s="24"/>
+      <c r="W33" s="24"/>
+      <c r="X33" s="24"/>
     </row>
     <row r="34" customFormat="false" ht="85.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="20" t="s">
+      <c r="A34" s="21" t="s">
         <v>180</v>
       </c>
-      <c r="B34" s="29" t="s">
+      <c r="B34" s="30" t="s">
         <v>69</v>
       </c>
-      <c r="C34" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D34" s="20" t="s">
+      <c r="C34" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D34" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E34" s="23" t="s">
+      <c r="E34" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F34" s="23" t="s">
+      <c r="F34" s="24" t="s">
         <v>181</v>
       </c>
-      <c r="G34" s="20" t="s">
+      <c r="G34" s="21" t="s">
         <v>182</v>
       </c>
-      <c r="H34" s="20" t="s">
+      <c r="H34" s="21" t="s">
         <v>183</v>
       </c>
-      <c r="I34" s="20" t="s">
+      <c r="I34" s="21" t="s">
         <v>184</v>
       </c>
-      <c r="J34" s="20" t="s">
+      <c r="J34" s="21" t="s">
         <v>185</v>
       </c>
-      <c r="K34" s="20"/>
-      <c r="L34" s="23"/>
-      <c r="M34" s="20" t="s">
+      <c r="K34" s="21"/>
+      <c r="L34" s="24"/>
+      <c r="M34" s="21" t="s">
         <v>179</v>
       </c>
-      <c r="N34" s="23"/>
-      <c r="O34" s="23"/>
-      <c r="P34" s="23"/>
-      <c r="Q34" s="23"/>
-      <c r="R34" s="23"/>
-      <c r="S34" s="23"/>
-      <c r="T34" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U34" s="23"/>
-      <c r="V34" s="23"/>
-      <c r="W34" s="23"/>
-      <c r="X34" s="23"/>
+      <c r="N34" s="24"/>
+      <c r="O34" s="24"/>
+      <c r="P34" s="24"/>
+      <c r="Q34" s="24"/>
+      <c r="R34" s="24"/>
+      <c r="S34" s="24"/>
+      <c r="T34" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U34" s="24"/>
+      <c r="V34" s="24"/>
+      <c r="W34" s="24"/>
+      <c r="X34" s="24"/>
     </row>
     <row r="35" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="20" t="s">
+      <c r="A35" s="21" t="s">
         <v>186</v>
       </c>
-      <c r="B35" s="20" t="s">
+      <c r="B35" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="C35" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D35" s="20" t="s">
+      <c r="C35" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D35" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E35" s="23" t="s">
+      <c r="E35" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F35" s="23" t="s">
+      <c r="F35" s="24" t="s">
         <v>187</v>
       </c>
-      <c r="G35" s="20" t="s">
+      <c r="G35" s="21" t="s">
         <v>188</v>
       </c>
-      <c r="H35" s="20" t="s">
+      <c r="H35" s="21" t="s">
         <v>189</v>
       </c>
-      <c r="I35" s="20"/>
-      <c r="J35" s="20"/>
-      <c r="K35" s="20"/>
-      <c r="L35" s="23"/>
-      <c r="M35" s="20" t="s">
+      <c r="I35" s="21"/>
+      <c r="J35" s="21"/>
+      <c r="K35" s="21"/>
+      <c r="L35" s="24"/>
+      <c r="M35" s="21" t="s">
         <v>190</v>
       </c>
-      <c r="N35" s="23"/>
-      <c r="O35" s="23"/>
-      <c r="P35" s="23"/>
-      <c r="Q35" s="23"/>
-      <c r="R35" s="23"/>
-      <c r="S35" s="23"/>
-      <c r="T35" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U35" s="23"/>
-      <c r="V35" s="23"/>
-      <c r="W35" s="23"/>
-      <c r="X35" s="23"/>
+      <c r="N35" s="24"/>
+      <c r="O35" s="24"/>
+      <c r="P35" s="24"/>
+      <c r="Q35" s="24"/>
+      <c r="R35" s="24"/>
+      <c r="S35" s="24"/>
+      <c r="T35" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U35" s="24"/>
+      <c r="V35" s="24"/>
+      <c r="W35" s="24"/>
+      <c r="X35" s="24"/>
     </row>
     <row r="36" customFormat="false" ht="85.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="20" t="s">
+      <c r="A36" s="21" t="s">
         <v>191</v>
       </c>
-      <c r="B36" s="29" t="s">
+      <c r="B36" s="30" t="s">
         <v>69</v>
       </c>
-      <c r="C36" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D36" s="20" t="s">
+      <c r="C36" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D36" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E36" s="23" t="s">
+      <c r="E36" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F36" s="23" t="s">
+      <c r="F36" s="24" t="s">
         <v>192</v>
       </c>
-      <c r="G36" s="20" t="s">
+      <c r="G36" s="21" t="s">
         <v>193</v>
       </c>
-      <c r="H36" s="20" t="s">
+      <c r="H36" s="21" t="s">
         <v>194</v>
       </c>
-      <c r="I36" s="20" t="s">
+      <c r="I36" s="21" t="s">
         <v>195</v>
       </c>
-      <c r="J36" s="20" t="s">
+      <c r="J36" s="21" t="s">
         <v>196</v>
       </c>
-      <c r="K36" s="30"/>
-      <c r="L36" s="31"/>
-      <c r="M36" s="30"/>
-      <c r="N36" s="31"/>
-      <c r="O36" s="31"/>
-      <c r="P36" s="31"/>
-      <c r="Q36" s="31"/>
-      <c r="R36" s="23"/>
-      <c r="S36" s="23"/>
-      <c r="T36" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U36" s="23"/>
-      <c r="V36" s="23"/>
-      <c r="W36" s="23"/>
-      <c r="X36" s="23"/>
+      <c r="K36" s="31"/>
+      <c r="L36" s="32"/>
+      <c r="M36" s="31"/>
+      <c r="N36" s="32"/>
+      <c r="O36" s="32"/>
+      <c r="P36" s="32"/>
+      <c r="Q36" s="32"/>
+      <c r="R36" s="24"/>
+      <c r="S36" s="24"/>
+      <c r="T36" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U36" s="24"/>
+      <c r="V36" s="24"/>
+      <c r="W36" s="24"/>
+      <c r="X36" s="24"/>
     </row>
     <row r="37" customFormat="false" ht="86.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="28" t="s">
+      <c r="A37" s="29" t="s">
         <v>197</v>
       </c>
-      <c r="B37" s="20" t="s">
+      <c r="B37" s="21" t="s">
         <v>153</v>
       </c>
-      <c r="C37" s="22" t="b">
+      <c r="C37" s="23" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="D37" s="20" t="s">
+      <c r="D37" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E37" s="23" t="s">
+      <c r="E37" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F37" s="23" t="s">
+      <c r="F37" s="24" t="s">
         <v>198</v>
       </c>
-      <c r="G37" s="20" t="s">
+      <c r="G37" s="21" t="s">
         <v>199</v>
       </c>
-      <c r="H37" s="20" t="s">
+      <c r="H37" s="21" t="s">
         <v>200</v>
       </c>
-      <c r="I37" s="20"/>
-      <c r="J37" s="20"/>
-      <c r="K37" s="20"/>
-      <c r="L37" s="23"/>
-      <c r="M37" s="24"/>
-      <c r="N37" s="24"/>
-      <c r="O37" s="32" t="s">
+      <c r="I37" s="21"/>
+      <c r="J37" s="21"/>
+      <c r="K37" s="21"/>
+      <c r="L37" s="24"/>
+      <c r="M37" s="25"/>
+      <c r="N37" s="25"/>
+      <c r="O37" s="33" t="s">
         <v>146</v>
       </c>
-      <c r="P37" s="23"/>
-      <c r="Q37" s="23"/>
-      <c r="R37" s="23"/>
-      <c r="S37" s="23"/>
-      <c r="T37" s="20" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U37" s="23"/>
-      <c r="V37" s="23"/>
-      <c r="W37" s="23"/>
-      <c r="X37" s="23"/>
+      <c r="P37" s="24"/>
+      <c r="Q37" s="24"/>
+      <c r="R37" s="24"/>
+      <c r="S37" s="24"/>
+      <c r="T37" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U37" s="24"/>
+      <c r="V37" s="24"/>
+      <c r="W37" s="24"/>
+      <c r="X37" s="24"/>
     </row>
     <row r="38" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="28" t="s">
+      <c r="A38" s="29" t="s">
         <v>201</v>
       </c>
-      <c r="B38" s="20" t="s">
+      <c r="B38" s="21" t="s">
         <v>153</v>
       </c>
-      <c r="C38" s="22" t="b">
+      <c r="C38" s="23" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="D38" s="20" t="s">
+      <c r="D38" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E38" s="23" t="s">
+      <c r="E38" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F38" s="23" t="s">
+      <c r="F38" s="24" t="s">
         <v>202</v>
       </c>
-      <c r="G38" s="20" t="s">
+      <c r="G38" s="21" t="s">
         <v>203</v>
       </c>
-      <c r="H38" s="20" t="s">
+      <c r="H38" s="21" t="s">
         <v>204</v>
       </c>
-      <c r="I38" s="20"/>
-      <c r="J38" s="20"/>
-      <c r="K38" s="20"/>
-      <c r="L38" s="23"/>
-      <c r="M38" s="24"/>
-      <c r="N38" s="24"/>
-      <c r="O38" s="32" t="s">
+      <c r="I38" s="21"/>
+      <c r="J38" s="21"/>
+      <c r="K38" s="21"/>
+      <c r="L38" s="24"/>
+      <c r="M38" s="25"/>
+      <c r="N38" s="25"/>
+      <c r="O38" s="33" t="s">
         <v>146</v>
       </c>
-      <c r="P38" s="23"/>
-      <c r="Q38" s="23"/>
-      <c r="R38" s="23"/>
-      <c r="S38" s="23"/>
-      <c r="T38" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U38" s="23"/>
-      <c r="V38" s="23"/>
-      <c r="W38" s="23"/>
-      <c r="X38" s="23"/>
+      <c r="P38" s="24"/>
+      <c r="Q38" s="24"/>
+      <c r="R38" s="24"/>
+      <c r="S38" s="24"/>
+      <c r="T38" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U38" s="24"/>
+      <c r="V38" s="24"/>
+      <c r="W38" s="24"/>
+      <c r="X38" s="24"/>
     </row>
     <row r="39" s="6" customFormat="true" ht="64.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="28" t="s">
+      <c r="A39" s="29" t="s">
         <v>205</v>
       </c>
-      <c r="B39" s="20" t="s">
+      <c r="B39" s="21" t="s">
         <v>153</v>
       </c>
-      <c r="C39" s="22" t="b">
+      <c r="C39" s="23" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="D39" s="20" t="s">
+      <c r="D39" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E39" s="23" t="s">
+      <c r="E39" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F39" s="23" t="s">
+      <c r="F39" s="24" t="s">
         <v>206</v>
       </c>
-      <c r="G39" s="20" t="s">
+      <c r="G39" s="21" t="s">
         <v>207</v>
       </c>
-      <c r="H39" s="20" t="s">
+      <c r="H39" s="21" t="s">
         <v>208</v>
       </c>
-      <c r="I39" s="20"/>
-      <c r="J39" s="20"/>
-      <c r="K39" s="20"/>
-      <c r="L39" s="23"/>
-      <c r="M39" s="24"/>
-      <c r="N39" s="24"/>
-      <c r="O39" s="32" t="s">
+      <c r="I39" s="21"/>
+      <c r="J39" s="21"/>
+      <c r="K39" s="21"/>
+      <c r="L39" s="24"/>
+      <c r="M39" s="25"/>
+      <c r="N39" s="25"/>
+      <c r="O39" s="33" t="s">
         <v>146</v>
       </c>
-      <c r="P39" s="23"/>
-      <c r="Q39" s="23"/>
-      <c r="R39" s="23"/>
-      <c r="S39" s="23"/>
-      <c r="T39" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U39" s="23"/>
-      <c r="V39" s="23"/>
-      <c r="W39" s="23"/>
-      <c r="X39" s="23"/>
+      <c r="P39" s="24"/>
+      <c r="Q39" s="24"/>
+      <c r="R39" s="24"/>
+      <c r="S39" s="24"/>
+      <c r="T39" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U39" s="24"/>
+      <c r="V39" s="24"/>
+      <c r="W39" s="24"/>
+      <c r="X39" s="24"/>
     </row>
     <row r="40" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="28" t="s">
+      <c r="A40" s="29" t="s">
         <v>209</v>
       </c>
-      <c r="B40" s="20" t="s">
+      <c r="B40" s="21" t="s">
         <v>153</v>
       </c>
-      <c r="C40" s="22" t="b">
+      <c r="C40" s="23" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="D40" s="20" t="s">
+      <c r="D40" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E40" s="23" t="s">
+      <c r="E40" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F40" s="23" t="s">
+      <c r="F40" s="24" t="s">
         <v>210</v>
       </c>
-      <c r="G40" s="20" t="s">
+      <c r="G40" s="21" t="s">
         <v>211</v>
       </c>
-      <c r="H40" s="20" t="s">
+      <c r="H40" s="21" t="s">
         <v>212</v>
       </c>
-      <c r="I40" s="20"/>
-      <c r="J40" s="20"/>
-      <c r="K40" s="20"/>
-      <c r="L40" s="23"/>
-      <c r="M40" s="24"/>
-      <c r="N40" s="24"/>
-      <c r="O40" s="32" t="s">
+      <c r="I40" s="21"/>
+      <c r="J40" s="21"/>
+      <c r="K40" s="21"/>
+      <c r="L40" s="24"/>
+      <c r="M40" s="25"/>
+      <c r="N40" s="25"/>
+      <c r="O40" s="33" t="s">
         <v>146</v>
       </c>
-      <c r="P40" s="23"/>
-      <c r="Q40" s="23"/>
-      <c r="R40" s="23"/>
-      <c r="S40" s="23"/>
-      <c r="T40" s="22" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U40" s="23"/>
-      <c r="V40" s="23"/>
-      <c r="W40" s="23"/>
-      <c r="X40" s="23"/>
+      <c r="P40" s="24"/>
+      <c r="Q40" s="24"/>
+      <c r="R40" s="24"/>
+      <c r="S40" s="24"/>
+      <c r="T40" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U40" s="24"/>
+      <c r="V40" s="24"/>
+      <c r="W40" s="24"/>
+      <c r="X40" s="24"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="33" t="s">
+      <c r="A41" s="34" t="s">
         <v>213</v>
       </c>
-      <c r="B41" s="33" t="s">
+      <c r="B41" s="34" t="s">
         <v>98</v>
       </c>
-      <c r="C41" s="34" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D41" s="33" t="s">
+      <c r="C41" s="35" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D41" s="34" t="s">
         <v>102</v>
       </c>
-      <c r="E41" s="35"/>
-      <c r="F41" s="35" t="str">
+      <c r="E41" s="36"/>
+      <c r="F41" s="36" t="str">
         <f aca="false">REPLACE(A41, FIND("_", A41), 1, ".")</f>
         <v>household.save</v>
       </c>
-      <c r="G41" s="33" t="s">
+      <c r="G41" s="34" t="s">
         <v>99</v>
       </c>
-      <c r="H41" s="33" t="s">
+      <c r="H41" s="34" t="s">
         <v>100</v>
       </c>
-      <c r="I41" s="33"/>
-      <c r="J41" s="33"/>
-      <c r="K41" s="33"/>
-      <c r="L41" s="35"/>
-      <c r="M41" s="35"/>
-      <c r="N41" s="35"/>
-      <c r="O41" s="35"/>
-      <c r="P41" s="35"/>
-      <c r="Q41" s="35"/>
-      <c r="R41" s="35"/>
-      <c r="S41" s="35"/>
-      <c r="T41" s="34" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U41" s="35"/>
-      <c r="V41" s="35"/>
-      <c r="W41" s="35"/>
-      <c r="X41" s="35"/>
+      <c r="I41" s="34"/>
+      <c r="J41" s="34"/>
+      <c r="K41" s="34"/>
+      <c r="L41" s="36"/>
+      <c r="M41" s="36"/>
+      <c r="N41" s="36"/>
+      <c r="O41" s="36"/>
+      <c r="P41" s="36"/>
+      <c r="Q41" s="36"/>
+      <c r="R41" s="36"/>
+      <c r="S41" s="36"/>
+      <c r="T41" s="35" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U41" s="36"/>
+      <c r="V41" s="36"/>
+      <c r="W41" s="36"/>
+      <c r="X41" s="36"/>
     </row>
     <row r="42" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
@@ -4092,7 +4094,7 @@
       <c r="B42" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C42" s="36" t="b">
+      <c r="C42" s="37" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -4108,9 +4110,9 @@
       <c r="H42" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="L42" s="37"/>
-      <c r="M42" s="38"/>
-      <c r="T42" s="36" t="b">
+      <c r="L42" s="38"/>
+      <c r="M42" s="39"/>
+      <c r="T42" s="37" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -4164,496 +4166,491 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="39" width="27.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="39" width="15.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="39" width="31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="40" width="20.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="39" width="19.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="39" width="12.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="39" width="18.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="40" width="27.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="40" width="15.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="40" width="31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="41" width="20.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="40" width="19.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="40" width="12.14"/>
   </cols>
   <sheetData>
-    <row r="1" s="43" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="41" t="s">
+    <row r="1" s="44" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="42" t="s">
         <v>218</v>
       </c>
-      <c r="B1" s="41" t="s">
+      <c r="B1" s="42" t="s">
         <v>219</v>
       </c>
-      <c r="C1" s="41" t="s">
+      <c r="C1" s="42" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="42" t="s">
+      <c r="D1" s="43" t="s">
         <v>220</v>
       </c>
-      <c r="E1" s="41" t="s">
+      <c r="E1" s="42" t="s">
         <v>221</v>
       </c>
-      <c r="F1" s="41" t="s">
+      <c r="F1" s="42" t="s">
         <v>222</v>
       </c>
-      <c r="G1" s="41" t="s">
+    </row>
+    <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="45" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="44" t="s">
+      <c r="B2" s="45"/>
+      <c r="C2" s="45" t="s">
         <v>224</v>
       </c>
-      <c r="B2" s="44"/>
-      <c r="C2" s="44" t="s">
+      <c r="D2" s="46" t="s">
         <v>225</v>
       </c>
-      <c r="D2" s="45" t="s">
+      <c r="E2" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="45"/>
+    </row>
+    <row r="3" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="45" t="s">
+        <v>95</v>
+      </c>
+      <c r="B3" s="45"/>
+      <c r="C3" s="45" t="s">
+        <v>224</v>
+      </c>
+      <c r="D3" s="46" t="s">
         <v>226</v>
       </c>
-      <c r="E2" s="44" t="n">
-        <v>1</v>
-      </c>
-      <c r="F2" s="44"/>
-    </row>
-    <row r="3" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="44" t="s">
-        <v>95</v>
-      </c>
-      <c r="B3" s="44"/>
-      <c r="C3" s="44" t="s">
+      <c r="E3" s="45" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" s="45"/>
+    </row>
+    <row r="4" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="45" t="s">
+        <v>163</v>
+      </c>
+      <c r="B4" s="45"/>
+      <c r="C4" s="45" t="s">
+        <v>227</v>
+      </c>
+      <c r="D4" s="46" t="s">
         <v>225</v>
       </c>
-      <c r="D3" s="45" t="s">
-        <v>227</v>
-      </c>
-      <c r="E3" s="44" t="n">
-        <v>2</v>
-      </c>
-      <c r="F3" s="44"/>
-    </row>
-    <row r="4" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="44" t="s">
+      <c r="E4" s="45" t="s">
+        <v>228</v>
+      </c>
+      <c r="F4" s="45"/>
+    </row>
+    <row r="5" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="45" t="s">
         <v>163</v>
       </c>
-      <c r="B4" s="44"/>
-      <c r="C4" s="44" t="s">
+      <c r="B5" s="45" t="s">
+        <v>229</v>
+      </c>
+      <c r="C5" s="45" t="s">
+        <v>224</v>
+      </c>
+      <c r="D5" s="46" t="s">
+        <v>225</v>
+      </c>
+      <c r="E5" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="45"/>
+    </row>
+    <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="45" t="s">
+        <v>230</v>
+      </c>
+      <c r="B6" s="45"/>
+      <c r="C6" s="45" t="s">
+        <v>231</v>
+      </c>
+      <c r="D6" s="46" t="s">
+        <v>226</v>
+      </c>
+      <c r="E6" s="45" t="n">
+        <v>3</v>
+      </c>
+      <c r="F6" s="45"/>
+    </row>
+    <row r="7" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="45" t="s">
+        <v>230</v>
+      </c>
+      <c r="B7" s="45" t="s">
+        <v>232</v>
+      </c>
+      <c r="C7" s="45" t="s">
+        <v>231</v>
+      </c>
+      <c r="D7" s="46" t="s">
+        <v>233</v>
+      </c>
+      <c r="E7" s="45" t="n">
+        <v>5</v>
+      </c>
+      <c r="F7" s="45"/>
+    </row>
+    <row r="8" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="45" t="s">
+        <v>234</v>
+      </c>
+      <c r="B8" s="45"/>
+      <c r="C8" s="45" t="s">
+        <v>231</v>
+      </c>
+      <c r="D8" s="46" t="s">
+        <v>226</v>
+      </c>
+      <c r="E8" s="45" t="n">
+        <v>4</v>
+      </c>
+      <c r="F8" s="45"/>
+    </row>
+    <row r="9" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="45" t="s">
+        <v>234</v>
+      </c>
+      <c r="B9" s="45" t="s">
+        <v>232</v>
+      </c>
+      <c r="C9" s="45" t="s">
+        <v>231</v>
+      </c>
+      <c r="D9" s="46" t="s">
+        <v>233</v>
+      </c>
+      <c r="E9" s="45" t="n">
+        <v>13</v>
+      </c>
+      <c r="F9" s="45"/>
+    </row>
+    <row r="10" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="45" t="s">
+        <v>235</v>
+      </c>
+      <c r="B10" s="45"/>
+      <c r="C10" s="45" t="s">
+        <v>231</v>
+      </c>
+      <c r="D10" s="46" t="s">
+        <v>233</v>
+      </c>
+      <c r="E10" s="45" t="n">
+        <v>5</v>
+      </c>
+      <c r="F10" s="45"/>
+    </row>
+    <row r="11" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="45" t="s">
+        <v>119</v>
+      </c>
+      <c r="B11" s="45"/>
+      <c r="C11" s="45" t="s">
+        <v>231</v>
+      </c>
+      <c r="D11" s="46" t="s">
+        <v>226</v>
+      </c>
+      <c r="E11" s="45" t="n">
+        <v>5</v>
+      </c>
+      <c r="F11" s="45"/>
+    </row>
+    <row r="12" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="45" t="s">
+        <v>157</v>
+      </c>
+      <c r="B12" s="45"/>
+      <c r="C12" s="45" t="s">
+        <v>231</v>
+      </c>
+      <c r="D12" s="46" t="s">
+        <v>226</v>
+      </c>
+      <c r="E12" s="45" t="n">
+        <v>6</v>
+      </c>
+      <c r="F12" s="45"/>
+    </row>
+    <row r="13" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="45" t="s">
+        <v>236</v>
+      </c>
+      <c r="B13" s="45"/>
+      <c r="C13" s="45" t="s">
+        <v>231</v>
+      </c>
+      <c r="D13" s="46" t="s">
+        <v>226</v>
+      </c>
+      <c r="E13" s="45" t="n">
+        <v>11</v>
+      </c>
+      <c r="F13" s="45"/>
+    </row>
+    <row r="14" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="45" t="s">
+        <v>124</v>
+      </c>
+      <c r="B14" s="45"/>
+      <c r="C14" s="45" t="s">
+        <v>231</v>
+      </c>
+      <c r="D14" s="46" t="s">
+        <v>226</v>
+      </c>
+      <c r="E14" s="45" t="n">
+        <v>14</v>
+      </c>
+      <c r="F14" s="45"/>
+    </row>
+    <row r="15" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="45" t="s">
+        <v>134</v>
+      </c>
+      <c r="B15" s="45"/>
+      <c r="C15" s="45" t="s">
+        <v>231</v>
+      </c>
+      <c r="D15" s="46" t="s">
+        <v>233</v>
+      </c>
+      <c r="E15" s="45" t="n">
+        <v>15</v>
+      </c>
+      <c r="F15" s="45"/>
+    </row>
+    <row r="16" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="45" t="s">
+        <v>134</v>
+      </c>
+      <c r="B16" s="45" t="s">
+        <v>232</v>
+      </c>
+      <c r="C16" s="45" t="s">
+        <v>231</v>
+      </c>
+      <c r="D16" s="46" t="s">
+        <v>237</v>
+      </c>
+      <c r="E16" s="45" t="s">
+        <v>238</v>
+      </c>
+      <c r="F16" s="45"/>
+    </row>
+    <row r="17" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="45" t="s">
+        <v>239</v>
+      </c>
+      <c r="B17" s="45"/>
+      <c r="C17" s="45" t="s">
+        <v>231</v>
+      </c>
+      <c r="D17" s="46" t="s">
+        <v>226</v>
+      </c>
+      <c r="E17" s="45" t="n">
+        <v>15</v>
+      </c>
+      <c r="F17" s="45"/>
+    </row>
+    <row r="18" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="45" t="s">
+        <v>130</v>
+      </c>
+      <c r="B18" s="45"/>
+      <c r="C18" s="45" t="s">
+        <v>231</v>
+      </c>
+      <c r="D18" s="46" t="s">
+        <v>226</v>
+      </c>
+      <c r="E18" s="45" t="n">
+        <v>16</v>
+      </c>
+      <c r="F18" s="45"/>
+    </row>
+    <row r="19" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="45" t="s">
+        <v>240</v>
+      </c>
+      <c r="B19" s="45"/>
+      <c r="C19" s="45" t="s">
+        <v>231</v>
+      </c>
+      <c r="D19" s="46" t="s">
+        <v>226</v>
+      </c>
+      <c r="E19" s="45" t="n">
+        <v>40</v>
+      </c>
+      <c r="F19" s="45"/>
+    </row>
+    <row r="20" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="45" t="s">
+        <v>151</v>
+      </c>
+      <c r="B20" s="45"/>
+      <c r="C20" s="45" t="s">
+        <v>241</v>
+      </c>
+      <c r="D20" s="46" t="s">
+        <v>225</v>
+      </c>
+      <c r="E20" s="45" t="s">
         <v>228</v>
       </c>
-      <c r="D4" s="45" t="s">
-        <v>226</v>
-      </c>
-      <c r="E4" s="44" t="s">
+      <c r="F20" s="45"/>
+    </row>
+    <row r="21" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="40" t="s">
+        <v>168</v>
+      </c>
+      <c r="C21" s="40" t="s">
+        <v>242</v>
+      </c>
+      <c r="D21" s="46" t="s">
+        <v>225</v>
+      </c>
+      <c r="E21" s="41" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="40" t="s">
+        <v>168</v>
+      </c>
+      <c r="B22" s="40" t="s">
         <v>229</v>
       </c>
-      <c r="F4" s="44"/>
-    </row>
-    <row r="5" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="44" t="s">
-        <v>163</v>
-      </c>
-      <c r="B5" s="44" t="s">
-        <v>230</v>
-      </c>
-      <c r="C5" s="44" t="s">
+      <c r="C22" s="40" t="s">
+        <v>242</v>
+      </c>
+      <c r="D22" s="46" t="s">
         <v>225</v>
       </c>
-      <c r="D5" s="45" t="s">
-        <v>226</v>
-      </c>
-      <c r="E5" s="44" t="n">
-        <v>1</v>
-      </c>
-      <c r="F5" s="44"/>
-    </row>
-    <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="44" t="s">
-        <v>231</v>
-      </c>
-      <c r="B6" s="44"/>
-      <c r="C6" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="D6" s="45" t="s">
-        <v>227</v>
-      </c>
-      <c r="E6" s="44" t="n">
-        <v>3</v>
-      </c>
-      <c r="F6" s="44"/>
-    </row>
-    <row r="7" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="44" t="s">
-        <v>231</v>
-      </c>
-      <c r="B7" s="44" t="s">
-        <v>233</v>
-      </c>
-      <c r="C7" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="D7" s="45" t="s">
-        <v>234</v>
-      </c>
-      <c r="E7" s="44" t="n">
-        <v>5</v>
-      </c>
-      <c r="F7" s="44"/>
-    </row>
-    <row r="8" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="44" t="s">
-        <v>235</v>
-      </c>
-      <c r="B8" s="44"/>
-      <c r="C8" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="D8" s="45" t="s">
-        <v>227</v>
-      </c>
-      <c r="E8" s="44" t="n">
-        <v>4</v>
-      </c>
-      <c r="F8" s="44"/>
-    </row>
-    <row r="9" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="44" t="s">
-        <v>235</v>
-      </c>
-      <c r="B9" s="44" t="s">
-        <v>233</v>
-      </c>
-      <c r="C9" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="D9" s="45" t="s">
-        <v>234</v>
-      </c>
-      <c r="E9" s="44" t="n">
-        <v>13</v>
-      </c>
-      <c r="F9" s="44"/>
-      <c r="G9" s="46"/>
-    </row>
-    <row r="10" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="44" t="s">
-        <v>236</v>
-      </c>
-      <c r="B10" s="44"/>
-      <c r="C10" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="D10" s="45" t="s">
-        <v>234</v>
-      </c>
-      <c r="E10" s="44" t="n">
-        <v>5</v>
-      </c>
-      <c r="F10" s="44"/>
-    </row>
-    <row r="11" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="44" t="s">
-        <v>119</v>
-      </c>
-      <c r="B11" s="44"/>
-      <c r="C11" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="D11" s="45" t="s">
-        <v>227</v>
-      </c>
-      <c r="E11" s="44" t="n">
-        <v>5</v>
-      </c>
-      <c r="F11" s="44"/>
-    </row>
-    <row r="12" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="44" t="s">
-        <v>157</v>
-      </c>
-      <c r="B12" s="44"/>
-      <c r="C12" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="D12" s="45" t="s">
-        <v>227</v>
-      </c>
-      <c r="E12" s="44" t="n">
-        <v>6</v>
-      </c>
-      <c r="F12" s="44"/>
-    </row>
-    <row r="13" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="44" t="s">
-        <v>237</v>
-      </c>
-      <c r="B13" s="44"/>
-      <c r="C13" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="D13" s="45" t="s">
-        <v>227</v>
-      </c>
-      <c r="E13" s="44" t="n">
-        <v>11</v>
-      </c>
-      <c r="F13" s="44"/>
-    </row>
-    <row r="14" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="44" t="s">
-        <v>124</v>
-      </c>
-      <c r="B14" s="44"/>
-      <c r="C14" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="D14" s="45" t="s">
-        <v>227</v>
-      </c>
-      <c r="E14" s="44" t="n">
-        <v>14</v>
-      </c>
-      <c r="F14" s="44"/>
-    </row>
-    <row r="15" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="44" t="s">
-        <v>134</v>
-      </c>
-      <c r="B15" s="44"/>
-      <c r="C15" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="D15" s="45" t="s">
-        <v>234</v>
-      </c>
-      <c r="E15" s="44" t="n">
-        <v>15</v>
-      </c>
-      <c r="F15" s="44"/>
-    </row>
-    <row r="16" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="44" t="s">
-        <v>134</v>
-      </c>
-      <c r="B16" s="44" t="s">
-        <v>233</v>
-      </c>
-      <c r="C16" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="D16" s="45" t="s">
-        <v>238</v>
-      </c>
-      <c r="E16" s="44" t="s">
-        <v>239</v>
-      </c>
-      <c r="F16" s="44"/>
-    </row>
-    <row r="17" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="44" t="s">
-        <v>240</v>
-      </c>
-      <c r="B17" s="44"/>
-      <c r="C17" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="D17" s="45" t="s">
-        <v>227</v>
-      </c>
-      <c r="E17" s="44" t="n">
-        <v>15</v>
-      </c>
-      <c r="F17" s="44"/>
-    </row>
-    <row r="18" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="44" t="s">
-        <v>130</v>
-      </c>
-      <c r="B18" s="44"/>
-      <c r="C18" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="D18" s="45" t="s">
-        <v>227</v>
-      </c>
-      <c r="E18" s="44" t="n">
-        <v>16</v>
-      </c>
-      <c r="F18" s="44"/>
-    </row>
-    <row r="19" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="44" t="s">
-        <v>241</v>
-      </c>
-      <c r="B19" s="44"/>
-      <c r="C19" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="D19" s="45" t="s">
-        <v>227</v>
-      </c>
-      <c r="E19" s="44" t="n">
-        <v>40</v>
-      </c>
-      <c r="F19" s="44"/>
-    </row>
-    <row r="20" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="44" t="s">
-        <v>151</v>
-      </c>
-      <c r="B20" s="44"/>
-      <c r="C20" s="44" t="s">
+      <c r="E22" s="41" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="40" t="s">
+        <v>168</v>
+      </c>
+      <c r="B23" s="40" t="s">
+        <v>229</v>
+      </c>
+      <c r="C23" s="40" t="s">
         <v>242</v>
       </c>
-      <c r="D20" s="45" t="s">
-        <v>226</v>
-      </c>
-      <c r="E20" s="44" t="s">
+      <c r="D23" s="46" t="s">
+        <v>225</v>
+      </c>
+      <c r="E23" s="41" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="40" t="s">
+        <v>173</v>
+      </c>
+      <c r="C24" s="40" t="s">
+        <v>242</v>
+      </c>
+      <c r="D24" s="46" t="s">
+        <v>225</v>
+      </c>
+      <c r="E24" s="41" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="40" t="s">
+        <v>173</v>
+      </c>
+      <c r="B25" s="40" t="s">
         <v>229</v>
       </c>
-      <c r="F20" s="44"/>
-    </row>
-    <row r="21" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="39" t="s">
-        <v>168</v>
-      </c>
-      <c r="C21" s="39" t="s">
-        <v>243</v>
-      </c>
-      <c r="D21" s="45" t="s">
-        <v>226</v>
-      </c>
-      <c r="E21" s="40" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="39" t="s">
-        <v>168</v>
-      </c>
-      <c r="B22" s="39" t="s">
-        <v>230</v>
-      </c>
-      <c r="C22" s="39" t="s">
-        <v>243</v>
-      </c>
-      <c r="D22" s="45" t="s">
-        <v>226</v>
-      </c>
-      <c r="E22" s="40" t="s">
+      <c r="C25" s="40" t="s">
+        <v>242</v>
+      </c>
+      <c r="D25" s="46" t="s">
+        <v>225</v>
+      </c>
+      <c r="E25" s="41" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="40" t="s">
+        <v>173</v>
+      </c>
+      <c r="B26" s="40" t="s">
+        <v>229</v>
+      </c>
+      <c r="C26" s="40" t="s">
+        <v>242</v>
+      </c>
+      <c r="D26" s="46" t="s">
+        <v>225</v>
+      </c>
+      <c r="E26" s="41" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="39" t="s">
-        <v>168</v>
-      </c>
-      <c r="B23" s="39" t="s">
-        <v>230</v>
-      </c>
-      <c r="C23" s="39" t="s">
-        <v>243</v>
-      </c>
-      <c r="D23" s="45" t="s">
-        <v>226</v>
-      </c>
-      <c r="E23" s="40" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="39" t="s">
-        <v>173</v>
-      </c>
-      <c r="C24" s="39" t="s">
-        <v>243</v>
-      </c>
-      <c r="D24" s="45" t="s">
-        <v>226</v>
-      </c>
-      <c r="E24" s="40" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="39" t="s">
-        <v>173</v>
-      </c>
-      <c r="B25" s="39" t="s">
-        <v>230</v>
-      </c>
-      <c r="C25" s="39" t="s">
-        <v>243</v>
-      </c>
-      <c r="D25" s="45" t="s">
-        <v>226</v>
-      </c>
-      <c r="E25" s="40" t="s">
+    <row r="27" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="40" t="s">
+        <v>179</v>
+      </c>
+      <c r="C27" s="40" t="s">
         <v>248</v>
       </c>
-    </row>
-    <row r="26" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="39" t="s">
-        <v>173</v>
-      </c>
-      <c r="B26" s="39" t="s">
-        <v>230</v>
-      </c>
-      <c r="C26" s="39" t="s">
-        <v>243</v>
-      </c>
-      <c r="D26" s="45" t="s">
-        <v>226</v>
-      </c>
-      <c r="E26" s="40" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="39" t="s">
+      <c r="D27" s="46" t="s">
+        <v>225</v>
+      </c>
+      <c r="E27" s="40" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="40" t="s">
         <v>179</v>
       </c>
-      <c r="C27" s="39" t="s">
-        <v>249</v>
-      </c>
-      <c r="D27" s="45" t="s">
-        <v>226</v>
-      </c>
-      <c r="E27" s="39" t="s">
+      <c r="B28" s="40" t="s">
+        <v>229</v>
+      </c>
+      <c r="C28" s="40" t="s">
+        <v>248</v>
+      </c>
+      <c r="D28" s="46" t="s">
+        <v>225</v>
+      </c>
+      <c r="E28" s="40" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="39" t="s">
+    <row r="29" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="40" t="s">
         <v>179</v>
       </c>
-      <c r="B28" s="39" t="s">
-        <v>230</v>
-      </c>
-      <c r="C28" s="39" t="s">
-        <v>249</v>
-      </c>
-      <c r="D28" s="45" t="s">
-        <v>226</v>
-      </c>
-      <c r="E28" s="39" t="s">
+      <c r="B29" s="40" t="s">
+        <v>229</v>
+      </c>
+      <c r="C29" s="40" t="s">
+        <v>248</v>
+      </c>
+      <c r="D29" s="46" t="s">
+        <v>225</v>
+      </c>
+      <c r="E29" s="40" t="s">
         <v>251</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="39" t="s">
-        <v>179</v>
-      </c>
-      <c r="B29" s="39" t="s">
-        <v>230</v>
-      </c>
-      <c r="C29" s="39" t="s">
-        <v>249</v>
-      </c>
-      <c r="D29" s="45" t="s">
-        <v>226</v>
-      </c>
-      <c r="E29" s="39" t="s">
-        <v>252</v>
       </c>
     </row>
   </sheetData>
@@ -4675,14 +4672,14 @@
   <dimension ref="A1:H4"/>
   <sheetFormatPr defaultColWidth="10.69921875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="44" width="10.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="44" width="12.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="44" width="13.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="44" width="12.57"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="6" min="5" style="44" width="10.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="44" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="44" width="15.43"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="9" style="44" width="10.7"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="45" width="10.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="45" width="12.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="45" width="13.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="45" width="12.57"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="6" min="5" style="45" width="10.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="45" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="45" width="15.43"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="9" style="45" width="10.7"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4690,39 +4687,39 @@
         <v>3</v>
       </c>
       <c r="B1" s="48" t="s">
+        <v>252</v>
+      </c>
+      <c r="C1" s="47" t="s">
         <v>253</v>
       </c>
-      <c r="C1" s="47" t="s">
+      <c r="D1" s="47" t="s">
         <v>254</v>
       </c>
-      <c r="D1" s="47" t="s">
+      <c r="E1" s="47" t="s">
         <v>255</v>
       </c>
-      <c r="E1" s="47" t="s">
+      <c r="F1" s="47" t="s">
         <v>256</v>
       </c>
-      <c r="F1" s="47" t="s">
+      <c r="G1" s="6" t="s">
         <v>257</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="H1" s="47" t="s">
         <v>258</v>
       </c>
-      <c r="H1" s="47" t="s">
+    </row>
+    <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="45" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" s="45" t="s">
         <v>259</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="44" t="s">
-        <v>26</v>
-      </c>
-      <c r="B2" s="44" t="s">
+      <c r="C2" s="45" t="s">
         <v>260</v>
       </c>
-      <c r="C2" s="44" t="s">
+      <c r="D2" s="45" t="s">
         <v>261</v>
-      </c>
-      <c r="D2" s="44" t="s">
-        <v>262</v>
       </c>
       <c r="E2" s="49" t="b">
         <f aca="false">TRUE()</f>
@@ -4738,17 +4735,17 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="44" t="s">
+      <c r="A3" s="45" t="s">
         <v>102</v>
       </c>
-      <c r="B3" s="44" t="s">
+      <c r="B3" s="45" t="s">
+        <v>262</v>
+      </c>
+      <c r="C3" s="45" t="s">
         <v>263</v>
       </c>
-      <c r="C3" s="44" t="s">
+      <c r="D3" s="45" t="s">
         <v>264</v>
-      </c>
-      <c r="D3" s="44" t="s">
-        <v>265</v>
       </c>
       <c r="E3" s="49" t="b">
         <f aca="false">TRUE()</f>
@@ -4764,17 +4761,17 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="44" t="s">
+      <c r="A4" s="45" t="s">
         <v>215</v>
       </c>
-      <c r="B4" s="44" t="s">
+      <c r="B4" s="45" t="s">
+        <v>265</v>
+      </c>
+      <c r="C4" s="45" t="s">
         <v>266</v>
       </c>
-      <c r="C4" s="44" t="s">
+      <c r="D4" s="45" t="s">
         <v>267</v>
-      </c>
-      <c r="D4" s="44" t="s">
-        <v>268</v>
       </c>
       <c r="E4" s="49" t="b">
         <f aca="false">FALSE()</f>
@@ -4819,7 +4816,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="51" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B1" s="51" t="s">
         <v>221</v>
@@ -4837,7 +4834,7 @@
         <v>9</v>
       </c>
       <c r="G1" s="51" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="H1" s="51" t="s">
         <v>12</v>
@@ -4845,16 +4842,16 @@
     </row>
     <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B2" s="52" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C2" s="52" t="s">
+        <v>270</v>
+      </c>
+      <c r="D2" s="52" t="s">
         <v>271</v>
-      </c>
-      <c r="D2" s="52" t="s">
-        <v>272</v>
       </c>
       <c r="E2" s="52"/>
       <c r="F2" s="52"/>
@@ -4863,16 +4860,16 @@
     </row>
     <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>273</v>
-      </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>274</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>275</v>
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
@@ -4887,10 +4884,10 @@
         <v>136</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>276</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>277</v>
       </c>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
@@ -4899,16 +4896,16 @@
     </row>
     <row r="5" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>136</v>
       </c>
       <c r="C5" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>279</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>280</v>
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
@@ -4917,16 +4914,16 @@
     </row>
     <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>281</v>
-      </c>
-      <c r="C6" s="1" t="s">
+      <c r="D6" s="1" t="s">
         <v>282</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>283</v>
       </c>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
@@ -4935,16 +4932,16 @@
     </row>
     <row r="7" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>284</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>284</v>
-      </c>
-      <c r="C7" s="1" t="s">
+      <c r="D7" s="1" t="s">
         <v>285</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>286</v>
       </c>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
@@ -4961,7 +4958,7 @@
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
       <c r="G8" s="1" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="H8" s="1"/>
     </row>
@@ -4975,7 +4972,7 @@
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
       <c r="G9" s="1" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="H9" s="1"/>
     </row>
@@ -5003,7 +5000,7 @@
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
       <c r="G11" s="1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="H11" s="1"/>
     </row>
@@ -5017,7 +5014,7 @@
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
       <c r="G12" s="1" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="H12" s="1"/>
     </row>
@@ -5031,7 +5028,7 @@
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
       <c r="G13" s="1" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="H13" s="1"/>
     </row>
@@ -5045,7 +5042,7 @@
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
       <c r="G14" s="1" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="H14" s="1"/>
     </row>
@@ -5054,13 +5051,13 @@
         <v>116</v>
       </c>
       <c r="B15" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>287</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="D15" s="1" t="s">
         <v>288</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>289</v>
       </c>
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
@@ -5072,13 +5069,13 @@
         <v>116</v>
       </c>
       <c r="B16" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="C16" s="1" t="s">
         <v>290</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="D16" s="1" t="s">
         <v>291</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>292</v>
       </c>
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
@@ -5095,7 +5092,7 @@
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
       <c r="G17" s="1" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="H17" s="1"/>
     </row>
@@ -5104,13 +5101,13 @@
         <v>125</v>
       </c>
       <c r="B18" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="C18" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="D18" s="1" t="s">
         <v>294</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>295</v>
       </c>
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
@@ -5122,13 +5119,13 @@
         <v>125</v>
       </c>
       <c r="B19" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="C19" s="1" t="s">
         <v>296</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="D19" s="1" t="s">
         <v>297</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>298</v>
       </c>
       <c r="E19" s="1"/>
       <c r="F19" s="1"/>
@@ -5145,7 +5142,7 @@
       <c r="E20" s="1"/>
       <c r="F20" s="1"/>
       <c r="G20" s="1" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="H20" s="1"/>
     </row>
@@ -5154,19 +5151,19 @@
         <v>132</v>
       </c>
       <c r="B21" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="C21" s="1" t="s">
         <v>299</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="D21" s="1" t="s">
         <v>300</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>301</v>
       </c>
       <c r="E21" s="1"/>
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
       <c r="H21" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5174,19 +5171,19 @@
         <v>132</v>
       </c>
       <c r="B22" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="C22" s="1" t="s">
         <v>302</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="D22" s="1" t="s">
         <v>303</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>304</v>
       </c>
       <c r="E22" s="1"/>
       <c r="F22" s="1"/>
       <c r="G22" s="1"/>
       <c r="H22" s="1" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5194,19 +5191,19 @@
         <v>132</v>
       </c>
       <c r="B23" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="C23" s="1" t="s">
         <v>305</v>
       </c>
-      <c r="C23" s="1" t="s">
+      <c r="D23" s="1" t="s">
         <v>306</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>307</v>
       </c>
       <c r="E23" s="1"/>
       <c r="F23" s="1"/>
       <c r="G23" s="1"/>
       <c r="H23" s="1" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5214,13 +5211,13 @@
         <v>132</v>
       </c>
       <c r="B24" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="C24" s="1" t="s">
         <v>308</v>
       </c>
-      <c r="C24" s="1" t="s">
+      <c r="D24" s="1" t="s">
         <v>309</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>310</v>
       </c>
       <c r="E24" s="1"/>
       <c r="F24" s="1"/>
@@ -5232,19 +5229,19 @@
         <v>132</v>
       </c>
       <c r="B25" s="1" t="s">
+        <v>310</v>
+      </c>
+      <c r="C25" s="1" t="s">
         <v>311</v>
       </c>
-      <c r="C25" s="1" t="s">
+      <c r="D25" s="1" t="s">
         <v>312</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>313</v>
       </c>
       <c r="E25" s="1"/>
       <c r="F25" s="1"/>
       <c r="G25" s="1"/>
       <c r="H25" s="1" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5266,13 +5263,13 @@
         <v>137</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C27" s="1" t="s">
+        <v>313</v>
+      </c>
+      <c r="D27" s="1" t="s">
         <v>314</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>315</v>
       </c>
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
@@ -5284,13 +5281,13 @@
         <v>137</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C28" s="1" t="s">
+        <v>315</v>
+      </c>
+      <c r="D28" s="1" t="s">
         <v>316</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>317</v>
       </c>
       <c r="E28" s="1"/>
       <c r="F28" s="1"/>
@@ -5302,13 +5299,13 @@
         <v>137</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C29" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="D29" s="1" t="s">
         <v>318</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>319</v>
       </c>
       <c r="E29" s="1"/>
       <c r="F29" s="1"/>
@@ -5320,13 +5317,13 @@
         <v>137</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C30" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="D30" s="1" t="s">
         <v>320</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>321</v>
       </c>
       <c r="E30" s="1"/>
       <c r="F30" s="1"/>
@@ -5338,13 +5335,13 @@
         <v>137</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C31" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="D31" s="1" t="s">
         <v>322</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>323</v>
       </c>
       <c r="E31" s="1"/>
       <c r="F31" s="1"/>
@@ -5356,19 +5353,19 @@
         <v>137</v>
       </c>
       <c r="B32" s="1" t="s">
+        <v>323</v>
+      </c>
+      <c r="C32" s="1" t="s">
         <v>324</v>
       </c>
-      <c r="C32" s="1" t="s">
+      <c r="D32" s="1" t="s">
         <v>325</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>326</v>
       </c>
       <c r="E32" s="1"/>
       <c r="F32" s="1"/>
       <c r="G32" s="1"/>
       <c r="H32" s="1" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5376,13 +5373,13 @@
         <v>137</v>
       </c>
       <c r="B33" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="C33" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="C33" s="1" t="s">
+      <c r="D33" s="1" t="s">
         <v>328</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>329</v>
       </c>
       <c r="E33" s="1"/>
       <c r="F33" s="1"/>
@@ -5394,13 +5391,13 @@
         <v>137</v>
       </c>
       <c r="B34" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="C34" s="1" t="s">
         <v>330</v>
       </c>
-      <c r="C34" s="1" t="s">
+      <c r="D34" s="1" t="s">
         <v>331</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>332</v>
       </c>
       <c r="E34" s="1"/>
       <c r="F34" s="1"/>
@@ -5412,13 +5409,13 @@
         <v>137</v>
       </c>
       <c r="B35" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="C35" s="1" t="s">
         <v>333</v>
       </c>
-      <c r="C35" s="1" t="s">
+      <c r="D35" s="1" t="s">
         <v>334</v>
-      </c>
-      <c r="D35" s="1" t="s">
-        <v>335</v>
       </c>
       <c r="E35" s="1"/>
       <c r="F35" s="1"/>
@@ -5430,13 +5427,13 @@
         <v>137</v>
       </c>
       <c r="B36" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="C36" s="1" t="s">
         <v>336</v>
       </c>
-      <c r="C36" s="1" t="s">
+      <c r="D36" s="1" t="s">
         <v>337</v>
-      </c>
-      <c r="D36" s="1" t="s">
-        <v>338</v>
       </c>
       <c r="E36" s="1"/>
       <c r="F36" s="1"/>
@@ -5448,13 +5445,13 @@
         <v>137</v>
       </c>
       <c r="B37" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="C37" s="1" t="s">
         <v>339</v>
       </c>
-      <c r="C37" s="1" t="s">
+      <c r="D37" s="1" t="s">
         <v>340</v>
-      </c>
-      <c r="D37" s="1" t="s">
-        <v>341</v>
       </c>
       <c r="E37" s="1"/>
       <c r="F37" s="1"/>
@@ -5469,10 +5466,10 @@
         <v>136</v>
       </c>
       <c r="C38" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="D38" s="1" t="s">
         <v>279</v>
-      </c>
-      <c r="D38" s="1" t="s">
-        <v>280</v>
       </c>
       <c r="E38" s="1"/>
       <c r="F38" s="1"/>
@@ -5484,13 +5481,13 @@
         <v>137</v>
       </c>
       <c r="B39" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="C39" s="1" t="s">
         <v>342</v>
       </c>
-      <c r="C39" s="1" t="s">
+      <c r="D39" s="1" t="s">
         <v>343</v>
-      </c>
-      <c r="D39" s="1" t="s">
-        <v>344</v>
       </c>
       <c r="E39" s="1"/>
       <c r="F39" s="1"/>
@@ -5507,7 +5504,7 @@
       <c r="E40" s="1"/>
       <c r="F40" s="1"/>
       <c r="G40" s="1" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="H40" s="1"/>
     </row>
@@ -5516,13 +5513,13 @@
         <v>158</v>
       </c>
       <c r="B41" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="C41" s="1" t="s">
         <v>345</v>
       </c>
-      <c r="C41" s="1" t="s">
+      <c r="D41" s="1" t="s">
         <v>346</v>
-      </c>
-      <c r="D41" s="1" t="s">
-        <v>347</v>
       </c>
       <c r="E41" s="1"/>
       <c r="F41" s="1"/>
@@ -5534,13 +5531,13 @@
         <v>158</v>
       </c>
       <c r="B42" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="C42" s="1" t="s">
         <v>348</v>
       </c>
-      <c r="C42" s="1" t="s">
+      <c r="D42" s="1" t="s">
         <v>349</v>
-      </c>
-      <c r="D42" s="1" t="s">
-        <v>350</v>
       </c>
       <c r="E42" s="1"/>
       <c r="F42" s="1"/>
@@ -5557,7 +5554,7 @@
       <c r="E43" s="1"/>
       <c r="F43" s="1"/>
       <c r="G43" s="1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="H43" s="1"/>
     </row>
@@ -5566,13 +5563,13 @@
         <v>165</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C44" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="D44" s="1" t="s">
         <v>351</v>
-      </c>
-      <c r="D44" s="1" t="s">
-        <v>352</v>
       </c>
       <c r="E44" s="1"/>
       <c r="F44" s="1"/>
@@ -5584,13 +5581,13 @@
         <v>165</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C45" s="1" t="s">
+        <v>352</v>
+      </c>
+      <c r="D45" s="1" t="s">
         <v>353</v>
-      </c>
-      <c r="D45" s="1" t="s">
-        <v>354</v>
       </c>
       <c r="E45" s="1"/>
       <c r="F45" s="1"/>
@@ -5602,13 +5599,13 @@
         <v>165</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C46" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="D46" s="1" t="s">
         <v>355</v>
-      </c>
-      <c r="D46" s="1" t="s">
-        <v>356</v>
       </c>
       <c r="E46" s="1"/>
       <c r="F46" s="1"/>
@@ -5620,13 +5617,13 @@
         <v>165</v>
       </c>
       <c r="B47" s="1" t="s">
+        <v>356</v>
+      </c>
+      <c r="C47" s="1" t="s">
         <v>357</v>
       </c>
-      <c r="C47" s="1" t="s">
+      <c r="D47" s="1" t="s">
         <v>358</v>
-      </c>
-      <c r="D47" s="1" t="s">
-        <v>359</v>
       </c>
       <c r="E47" s="1"/>
       <c r="F47" s="1"/>
@@ -5638,13 +5635,13 @@
         <v>165</v>
       </c>
       <c r="B48" s="1" t="s">
+        <v>359</v>
+      </c>
+      <c r="C48" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="C48" s="1" t="s">
+      <c r="D48" s="1" t="s">
         <v>361</v>
-      </c>
-      <c r="D48" s="1" t="s">
-        <v>362</v>
       </c>
       <c r="E48" s="1"/>
       <c r="F48" s="1"/>
@@ -5656,13 +5653,13 @@
         <v>174</v>
       </c>
       <c r="B49" s="50" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C49" s="50" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D49" s="50" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5670,13 +5667,13 @@
         <v>174</v>
       </c>
       <c r="B50" s="50" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C50" s="50" t="s">
+        <v>363</v>
+      </c>
+      <c r="D50" s="50" t="s">
         <v>364</v>
-      </c>
-      <c r="D50" s="50" t="s">
-        <v>365</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5684,13 +5681,13 @@
         <v>174</v>
       </c>
       <c r="B51" s="50" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C51" s="50" t="s">
+        <v>365</v>
+      </c>
+      <c r="D51" s="50" t="s">
         <v>366</v>
-      </c>
-      <c r="D51" s="50" t="s">
-        <v>367</v>
       </c>
     </row>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -5713,54 +5710,54 @@
   <dimension ref="A1:L1"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="39" width="18.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="39" width="17.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="39" width="13.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="39" width="12.72"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="39" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="39" width="13.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="39" width="14.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="39" width="11.28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="39" width="13.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="39" width="14.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="40" width="18.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="40" width="17.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="40" width="13.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="40" width="12.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="40" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="40" width="13.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="40" width="14.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="40" width="11.28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="40" width="13.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="40" width="14.43"/>
   </cols>
   <sheetData>
     <row r="1" s="51" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="53" t="s">
+        <v>367</v>
+      </c>
+      <c r="B1" s="53" t="s">
         <v>368</v>
       </c>
-      <c r="B1" s="53" t="s">
+      <c r="C1" s="53" t="s">
         <v>369</v>
       </c>
-      <c r="C1" s="53" t="s">
+      <c r="D1" s="53" t="s">
         <v>370</v>
       </c>
-      <c r="D1" s="53" t="s">
+      <c r="E1" s="53" t="s">
         <v>371</v>
       </c>
-      <c r="E1" s="53" t="s">
+      <c r="F1" s="53" t="s">
         <v>372</v>
       </c>
-      <c r="F1" s="53" t="s">
+      <c r="G1" s="53" t="s">
         <v>373</v>
       </c>
-      <c r="G1" s="53" t="s">
+      <c r="H1" s="53" t="s">
         <v>374</v>
       </c>
-      <c r="H1" s="53" t="s">
+      <c r="I1" s="53" t="s">
         <v>375</v>
       </c>
-      <c r="I1" s="53" t="s">
+      <c r="J1" s="53" t="s">
         <v>376</v>
       </c>
-      <c r="J1" s="53" t="s">
+      <c r="K1" s="53" t="s">
         <v>377</v>
       </c>
-      <c r="K1" s="53" t="s">
+      <c r="L1" s="51" t="s">
         <v>378</v>
-      </c>
-      <c r="L1" s="51" t="s">
-        <v>379</v>
       </c>
     </row>
   </sheetData>
@@ -5782,11 +5779,11 @@
   <dimension ref="A1:G3"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="39" width="10.34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="39" width="32.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="39" width="43.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="39" width="46.08"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="39" width="28.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="40" width="10.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="40" width="32.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="40" width="43.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="40" width="46.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="40" width="28.55"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5808,20 +5805,20 @@
       <c r="F1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="39"/>
+      <c r="G1" s="40"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="54" t="s">
         <v>102</v>
       </c>
-      <c r="B2" s="44" t="s">
+      <c r="B2" s="45" t="s">
+        <v>379</v>
+      </c>
+      <c r="C2" s="54" t="s">
         <v>380</v>
       </c>
-      <c r="C2" s="54" t="s">
+      <c r="D2" s="54" t="s">
         <v>381</v>
-      </c>
-      <c r="D2" s="54" t="s">
-        <v>382</v>
       </c>
       <c r="E2" s="54"/>
       <c r="F2" s="54"/>
@@ -5830,14 +5827,14 @@
       <c r="A3" s="54" t="s">
         <v>102</v>
       </c>
-      <c r="B3" s="44" t="s">
+      <c r="B3" s="45" t="s">
+        <v>382</v>
+      </c>
+      <c r="C3" s="54" t="s">
         <v>383</v>
       </c>
-      <c r="C3" s="54" t="s">
+      <c r="D3" s="54" t="s">
         <v>384</v>
-      </c>
-      <c r="D3" s="54" t="s">
-        <v>385</v>
       </c>
       <c r="E3" s="54"/>
       <c r="F3" s="54"/>

</xml_diff>

<commit_message>
generator: use the questionName instead of path as label key
fixes #1530

Rename the `path` parameter in the translation functions to `label_key`
which represents more that the data is.

Pass the excel sheet name as well as the headers containing the
namespace and key of the translations.

The `Widgets` sheet uses the 'questionName' and 'section' respectively
as key and namespace. The `Labels` sheet is updated to use the
`namespace` and `key` header keys.
</commit_message>
<xml_diff>
--- a/example/demo_generator/references/Household_Travel_Generate_Survey.xlsx
+++ b/example/demo_generator/references/Household_Travel_Generate_Survey.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Widgets" sheetId="1" state="visible" r:id="rId3"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="684" uniqueCount="387">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="684" uniqueCount="389">
   <si>
     <t xml:space="preserve">questionName</t>
   </si>
@@ -1227,6 +1227,12 @@
   </si>
   <si>
     <t xml:space="preserve">input_color</t>
+  </si>
+  <si>
+    <t xml:space="preserve">namespace</t>
+  </si>
+  <si>
+    <t xml:space="preserve">key</t>
   </si>
   <si>
     <t xml:space="preserve">personSchoolTypeYoungChild</t>
@@ -1251,10 +1257,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="General"/>
-    <numFmt numFmtId="166" formatCode="@"/>
+    <numFmt numFmtId="165" formatCode="@"/>
   </numFmts>
   <fonts count="20">
     <font>
@@ -1494,7 +1499,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="48">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1527,10 +1532,6 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1551,19 +1552,11 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1575,19 +1568,11 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1635,15 +1620,7 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1659,7 +1636,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1667,7 +1644,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1679,7 +1656,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1691,11 +1668,7 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2068,7 +2041,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:X42"/>
-  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="19.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.86"/>
@@ -2169,14 +2142,14 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="26.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
         <v>24</v>
       </c>
       <c r="B2" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C2" s="8" t="b">
+      <c r="C2" s="7" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2198,13 +2171,13 @@
       <c r="K2" s="7"/>
       <c r="L2" s="7"/>
       <c r="M2" s="7"/>
-      <c r="N2" s="9"/>
+      <c r="N2" s="8"/>
       <c r="O2" s="7"/>
       <c r="P2" s="7"/>
       <c r="Q2" s="7"/>
       <c r="R2" s="7"/>
       <c r="S2" s="7"/>
-      <c r="T2" s="8" t="b">
+      <c r="T2" s="7" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2213,14 +2186,14 @@
       <c r="W2" s="7"/>
       <c r="X2" s="7"/>
     </row>
-    <row r="3" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="51.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
         <v>29</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="C3" s="8" t="b">
+      <c r="C3" s="7" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2240,8 +2213,8 @@
       <c r="I3" s="7"/>
       <c r="J3" s="7"/>
       <c r="K3" s="7"/>
-      <c r="M3" s="9"/>
-      <c r="N3" s="9"/>
+      <c r="M3" s="8"/>
+      <c r="N3" s="8"/>
       <c r="O3" s="7" t="s">
         <v>33</v>
       </c>
@@ -2249,7 +2222,7 @@
       <c r="Q3" s="7"/>
       <c r="R3" s="7"/>
       <c r="S3" s="7"/>
-      <c r="T3" s="8" t="b">
+      <c r="T3" s="7" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2258,14 +2231,14 @@
       <c r="W3" s="7"/>
       <c r="X3" s="7"/>
     </row>
-    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="26.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
         <v>34</v>
       </c>
       <c r="B4" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="C4" s="8" t="b">
+      <c r="C4" s="7" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2286,7 +2259,7 @@
       <c r="J4" s="7"/>
       <c r="K4" s="7"/>
       <c r="L4" s="7"/>
-      <c r="M4" s="9"/>
+      <c r="M4" s="8"/>
       <c r="N4" s="7"/>
       <c r="O4" s="7" t="s">
         <v>38</v>
@@ -2295,7 +2268,7 @@
       <c r="Q4" s="7"/>
       <c r="R4" s="7"/>
       <c r="S4" s="7"/>
-      <c r="T4" s="8" t="b">
+      <c r="T4" s="7" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2311,7 +2284,7 @@
       <c r="B5" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C5" s="8" t="b">
+      <c r="C5" s="7" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2332,7 +2305,7 @@
       <c r="J5" s="7"/>
       <c r="K5" s="7"/>
       <c r="L5" s="7"/>
-      <c r="M5" s="9"/>
+      <c r="M5" s="8"/>
       <c r="N5" s="7" t="s">
         <v>42</v>
       </c>
@@ -2341,7 +2314,7 @@
       <c r="Q5" s="7"/>
       <c r="R5" s="7"/>
       <c r="S5" s="7"/>
-      <c r="T5" s="8" t="b">
+      <c r="T5" s="7" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2350,14 +2323,14 @@
       <c r="W5" s="7"/>
       <c r="X5" s="7"/>
     </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="26.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
         <v>43</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C6" s="8" t="b">
+      <c r="C6" s="7" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2380,7 +2353,7 @@
       <c r="L6" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="M6" s="9"/>
+      <c r="M6" s="8"/>
       <c r="N6" s="7" t="s">
         <v>47</v>
       </c>
@@ -2389,7 +2362,7 @@
       <c r="Q6" s="7"/>
       <c r="R6" s="7"/>
       <c r="S6" s="7"/>
-      <c r="T6" s="8" t="b">
+      <c r="T6" s="7" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2405,7 +2378,7 @@
       <c r="B7" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="8" t="b">
+      <c r="C7" s="7" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2434,7 +2407,7 @@
       <c r="Q7" s="7"/>
       <c r="R7" s="7"/>
       <c r="S7" s="7"/>
-      <c r="T7" s="8" t="b">
+      <c r="T7" s="7" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2450,7 +2423,7 @@
       <c r="B8" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C8" s="8" t="b">
+      <c r="C8" s="7" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2481,7 +2454,7 @@
       <c r="Q8" s="7"/>
       <c r="R8" s="7"/>
       <c r="S8" s="7"/>
-      <c r="T8" s="8" t="b">
+      <c r="T8" s="7" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2490,14 +2463,14 @@
       <c r="W8" s="7"/>
       <c r="X8" s="7"/>
     </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="26.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
         <v>55</v>
       </c>
       <c r="B9" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="8" t="b">
+      <c r="C9" s="7" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2528,7 +2501,7 @@
       <c r="Q9" s="7"/>
       <c r="R9" s="7"/>
       <c r="S9" s="7"/>
-      <c r="T9" s="8" t="b">
+      <c r="T9" s="7" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2539,14 +2512,14 @@
       </c>
       <c r="X9" s="7"/>
     </row>
-    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="26.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
         <v>59</v>
       </c>
       <c r="B10" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C10" s="8" t="b">
+      <c r="C10" s="7" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2577,7 +2550,7 @@
       <c r="Q10" s="7"/>
       <c r="R10" s="7"/>
       <c r="S10" s="7"/>
-      <c r="T10" s="8" t="b">
+      <c r="T10" s="7" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2588,14 +2561,14 @@
       </c>
       <c r="X10" s="7"/>
     </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="26.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
         <v>64</v>
       </c>
       <c r="B11" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C11" s="8" t="b">
+      <c r="C11" s="7" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2626,7 +2599,7 @@
       <c r="Q11" s="7"/>
       <c r="R11" s="7"/>
       <c r="S11" s="7"/>
-      <c r="T11" s="8" t="b">
+      <c r="T11" s="7" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2636,13 +2609,13 @@
       <c r="X11" s="7"/>
     </row>
     <row r="12" customFormat="false" ht="117.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="10" t="s">
+      <c r="A12" s="9" t="s">
         <v>68</v>
       </c>
       <c r="B12" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="C12" s="8" t="b">
+      <c r="C12" s="7" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2664,7 +2637,7 @@
       <c r="J12" s="7"/>
       <c r="K12" s="7"/>
       <c r="L12" s="7"/>
-      <c r="M12" s="11"/>
+      <c r="M12" s="10"/>
       <c r="N12" s="7"/>
       <c r="O12" s="7"/>
       <c r="P12" s="7"/>
@@ -2687,7 +2660,7 @@
       <c r="B13" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="C13" s="8" t="b">
+      <c r="C13" s="7" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2722,7 +2695,7 @@
       <c r="Q13" s="7"/>
       <c r="R13" s="7"/>
       <c r="S13" s="7"/>
-      <c r="T13" s="8" t="b">
+      <c r="T13" s="7" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2738,7 +2711,7 @@
       <c r="B14" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="C14" s="8" t="b">
+      <c r="C14" s="7" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2773,7 +2746,7 @@
       <c r="Q14" s="7"/>
       <c r="R14" s="7"/>
       <c r="S14" s="7"/>
-      <c r="T14" s="8" t="b">
+      <c r="T14" s="7" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2789,7 +2762,7 @@
       <c r="B15" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="C15" s="8" t="b">
+      <c r="C15" s="7" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2822,7 +2795,7 @@
       <c r="Q15" s="7"/>
       <c r="R15" s="7"/>
       <c r="S15" s="7"/>
-      <c r="T15" s="8" t="b">
+      <c r="T15" s="7" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2831,14 +2804,14 @@
       <c r="W15" s="7"/>
       <c r="X15" s="7"/>
     </row>
-    <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="39.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
         <v>89</v>
       </c>
       <c r="B16" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="C16" s="8" t="b">
+      <c r="C16" s="7" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2862,14 +2835,14 @@
         <v>82</v>
       </c>
       <c r="L16" s="7"/>
-      <c r="M16" s="9"/>
-      <c r="N16" s="9"/>
+      <c r="M16" s="8"/>
+      <c r="N16" s="8"/>
       <c r="O16" s="7"/>
       <c r="P16" s="7"/>
       <c r="Q16" s="7"/>
       <c r="R16" s="7"/>
       <c r="S16" s="7"/>
-      <c r="T16" s="8" t="b">
+      <c r="T16" s="7" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2878,14 +2851,14 @@
       <c r="W16" s="7"/>
       <c r="X16" s="7"/>
     </row>
-    <row r="17" s="12" customFormat="true" ht="76.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="17" s="11" customFormat="true" ht="76.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
         <v>92</v>
       </c>
       <c r="B17" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="C17" s="8" t="b">
+      <c r="C17" s="7" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2918,7 +2891,7 @@
       <c r="Q17" s="7"/>
       <c r="R17" s="7"/>
       <c r="S17" s="7"/>
-      <c r="T17" s="8" t="b">
+      <c r="T17" s="7" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2928,33 +2901,33 @@
       <c r="X17" s="7"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="13" t="s">
+      <c r="A18" s="12" t="s">
         <v>97</v>
       </c>
-      <c r="B18" s="13" t="s">
+      <c r="B18" s="12" t="s">
         <v>98</v>
       </c>
-      <c r="C18" s="14" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D18" s="15" t="s">
+      <c r="C18" s="12" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D18" s="13" t="s">
         <v>26</v>
       </c>
       <c r="E18" s="7"/>
-      <c r="F18" s="16" t="str">
+      <c r="F18" s="14" t="str">
         <f aca="false">REPLACE(A18, FIND("_", A18), 1, ".")</f>
         <v>home.save</v>
       </c>
-      <c r="G18" s="13" t="s">
+      <c r="G18" s="12" t="s">
         <v>99</v>
       </c>
-      <c r="H18" s="13" t="s">
+      <c r="H18" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="I18" s="13"/>
-      <c r="J18" s="13"/>
-      <c r="K18" s="13"/>
+      <c r="I18" s="12"/>
+      <c r="J18" s="12"/>
+      <c r="K18" s="12"/>
       <c r="L18" s="7"/>
       <c r="M18" s="7"/>
       <c r="N18" s="7"/>
@@ -2963,7 +2936,7 @@
       <c r="Q18" s="7"/>
       <c r="R18" s="7"/>
       <c r="S18" s="7"/>
-      <c r="T18" s="17" t="b">
+      <c r="T18" s="13" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2973,1138 +2946,1138 @@
       <c r="X18" s="7"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="18" t="s">
+      <c r="A19" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="B19" s="19" t="s">
+      <c r="B19" s="16" t="s">
         <v>69</v>
       </c>
-      <c r="C19" s="20" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D19" s="21" t="s">
+      <c r="C19" s="15" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D19" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="E19" s="22"/>
-      <c r="F19" s="22"/>
-      <c r="G19" s="18"/>
-      <c r="H19" s="18"/>
-      <c r="I19" s="18"/>
-      <c r="J19" s="18"/>
-      <c r="K19" s="18"/>
-      <c r="L19" s="22"/>
-      <c r="M19" s="22"/>
-      <c r="N19" s="22"/>
-      <c r="O19" s="22"/>
-      <c r="P19" s="22"/>
-      <c r="Q19" s="22"/>
-      <c r="R19" s="22"/>
-      <c r="S19" s="22"/>
-      <c r="T19" s="23" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U19" s="22"/>
-      <c r="V19" s="22"/>
-      <c r="W19" s="22"/>
-      <c r="X19" s="22"/>
+      <c r="E19" s="18"/>
+      <c r="F19" s="18"/>
+      <c r="G19" s="15"/>
+      <c r="H19" s="15"/>
+      <c r="I19" s="15"/>
+      <c r="J19" s="15"/>
+      <c r="K19" s="15"/>
+      <c r="L19" s="18"/>
+      <c r="M19" s="18"/>
+      <c r="N19" s="18"/>
+      <c r="O19" s="18"/>
+      <c r="P19" s="18"/>
+      <c r="Q19" s="18"/>
+      <c r="R19" s="18"/>
+      <c r="S19" s="18"/>
+      <c r="T19" s="17" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U19" s="18"/>
+      <c r="V19" s="18"/>
+      <c r="W19" s="18"/>
+      <c r="X19" s="18"/>
     </row>
     <row r="20" customFormat="false" ht="144" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="21" t="s">
+      <c r="A20" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="B20" s="21" t="s">
+      <c r="B20" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="C20" s="23" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D20" s="21" t="s">
+      <c r="C20" s="17" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D20" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="E20" s="24" t="s">
+      <c r="E20" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="F20" s="24" t="s">
+      <c r="F20" s="19" t="s">
         <v>104</v>
       </c>
-      <c r="G20" s="21" t="s">
+      <c r="G20" s="17" t="s">
         <v>105</v>
       </c>
-      <c r="H20" s="21" t="s">
+      <c r="H20" s="17" t="s">
         <v>106</v>
       </c>
-      <c r="I20" s="21"/>
-      <c r="J20" s="21"/>
-      <c r="K20" s="21"/>
-      <c r="L20" s="24"/>
-      <c r="M20" s="24" t="s">
+      <c r="I20" s="17"/>
+      <c r="J20" s="17"/>
+      <c r="K20" s="17"/>
+      <c r="L20" s="19"/>
+      <c r="M20" s="19" t="s">
         <v>95</v>
       </c>
-      <c r="N20" s="25"/>
-      <c r="O20" s="24"/>
-      <c r="P20" s="24"/>
-      <c r="Q20" s="24"/>
-      <c r="R20" s="24"/>
-      <c r="S20" s="24"/>
-      <c r="T20" s="21" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U20" s="24"/>
-      <c r="V20" s="24"/>
-      <c r="W20" s="24"/>
-      <c r="X20" s="24"/>
+      <c r="N20" s="20"/>
+      <c r="O20" s="19"/>
+      <c r="P20" s="19"/>
+      <c r="Q20" s="19"/>
+      <c r="R20" s="19"/>
+      <c r="S20" s="19"/>
+      <c r="T20" s="17" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U20" s="19"/>
+      <c r="V20" s="19"/>
+      <c r="W20" s="19"/>
+      <c r="X20" s="19"/>
     </row>
     <row r="21" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="21" t="s">
+      <c r="A21" s="17" t="s">
         <v>107</v>
       </c>
-      <c r="B21" s="21" t="s">
+      <c r="B21" s="17" t="s">
         <v>108</v>
       </c>
-      <c r="C21" s="23" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D21" s="21" t="s">
+      <c r="C21" s="17" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D21" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="E21" s="24" t="s">
+      <c r="E21" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="F21" s="24" t="s">
+      <c r="F21" s="19" t="s">
         <v>109</v>
       </c>
-      <c r="G21" s="21" t="s">
+      <c r="G21" s="17" t="s">
         <v>110</v>
       </c>
-      <c r="H21" s="21" t="s">
+      <c r="H21" s="17" t="s">
         <v>111</v>
       </c>
-      <c r="I21" s="21" t="s">
+      <c r="I21" s="17" t="s">
         <v>112</v>
       </c>
-      <c r="J21" s="21" t="s">
+      <c r="J21" s="17" t="s">
         <v>113</v>
       </c>
-      <c r="K21" s="21"/>
-      <c r="L21" s="24"/>
-      <c r="M21" s="24"/>
-      <c r="N21" s="24" t="s">
+      <c r="K21" s="17"/>
+      <c r="L21" s="19"/>
+      <c r="M21" s="19"/>
+      <c r="N21" s="19" t="s">
         <v>114</v>
       </c>
-      <c r="O21" s="24"/>
-      <c r="P21" s="24"/>
-      <c r="Q21" s="24"/>
-      <c r="R21" s="24"/>
-      <c r="S21" s="24"/>
-      <c r="T21" s="23" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U21" s="24"/>
-      <c r="V21" s="24"/>
-      <c r="W21" s="24"/>
-      <c r="X21" s="24"/>
-    </row>
-    <row r="22" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="21" t="s">
+      <c r="O21" s="19"/>
+      <c r="P21" s="19"/>
+      <c r="Q21" s="19"/>
+      <c r="R21" s="19"/>
+      <c r="S21" s="19"/>
+      <c r="T21" s="17" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U21" s="19"/>
+      <c r="V21" s="19"/>
+      <c r="W21" s="19"/>
+      <c r="X21" s="19"/>
+    </row>
+    <row r="22" customFormat="false" ht="33.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="B22" s="21" t="s">
+      <c r="B22" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="C22" s="23" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D22" s="21" t="s">
+      <c r="C22" s="17" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D22" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="E22" s="24" t="s">
+      <c r="E22" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="F22" s="24" t="s">
+      <c r="F22" s="19" t="s">
         <v>116</v>
       </c>
-      <c r="G22" s="21" t="s">
+      <c r="G22" s="17" t="s">
         <v>117</v>
       </c>
-      <c r="H22" s="21" t="s">
+      <c r="H22" s="17" t="s">
         <v>118</v>
       </c>
-      <c r="I22" s="21"/>
-      <c r="J22" s="21"/>
-      <c r="K22" s="21"/>
-      <c r="L22" s="24"/>
-      <c r="M22" s="24" t="s">
+      <c r="I22" s="17"/>
+      <c r="J22" s="17"/>
+      <c r="K22" s="17"/>
+      <c r="L22" s="19"/>
+      <c r="M22" s="19" t="s">
         <v>119</v>
       </c>
-      <c r="N22" s="24"/>
-      <c r="O22" s="24" t="s">
+      <c r="N22" s="19"/>
+      <c r="O22" s="19" t="s">
         <v>116</v>
       </c>
-      <c r="P22" s="24"/>
-      <c r="Q22" s="24"/>
-      <c r="R22" s="24"/>
-      <c r="S22" s="24"/>
-      <c r="T22" s="23" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U22" s="24"/>
-      <c r="V22" s="24"/>
-      <c r="W22" s="24"/>
-      <c r="X22" s="24"/>
-    </row>
-    <row r="23" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="21" t="s">
+      <c r="P22" s="19"/>
+      <c r="Q22" s="19"/>
+      <c r="R22" s="19"/>
+      <c r="S22" s="19"/>
+      <c r="T22" s="17" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U22" s="19"/>
+      <c r="V22" s="19"/>
+      <c r="W22" s="19"/>
+      <c r="X22" s="19"/>
+    </row>
+    <row r="23" customFormat="false" ht="33.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="17" t="s">
         <v>120</v>
       </c>
-      <c r="B23" s="21" t="s">
+      <c r="B23" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="C23" s="23" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D23" s="21" t="s">
+      <c r="C23" s="17" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D23" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="E23" s="24" t="s">
+      <c r="E23" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="F23" s="24" t="s">
+      <c r="F23" s="19" t="s">
         <v>121</v>
       </c>
-      <c r="G23" s="21" t="s">
+      <c r="G23" s="17" t="s">
         <v>122</v>
       </c>
-      <c r="H23" s="21" t="s">
+      <c r="H23" s="17" t="s">
         <v>123</v>
       </c>
-      <c r="I23" s="21"/>
-      <c r="J23" s="21"/>
-      <c r="K23" s="21"/>
-      <c r="L23" s="24"/>
-      <c r="M23" s="24" t="s">
+      <c r="I23" s="17"/>
+      <c r="J23" s="17"/>
+      <c r="K23" s="17"/>
+      <c r="L23" s="19"/>
+      <c r="M23" s="19" t="s">
         <v>124</v>
       </c>
-      <c r="N23" s="24"/>
-      <c r="O23" s="24" t="s">
+      <c r="N23" s="19"/>
+      <c r="O23" s="19" t="s">
         <v>125</v>
       </c>
-      <c r="P23" s="24"/>
-      <c r="Q23" s="24"/>
-      <c r="R23" s="24"/>
-      <c r="S23" s="24"/>
-      <c r="T23" s="23" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U23" s="24"/>
-      <c r="V23" s="24"/>
-      <c r="W23" s="24"/>
-      <c r="X23" s="24"/>
+      <c r="P23" s="19"/>
+      <c r="Q23" s="19"/>
+      <c r="R23" s="19"/>
+      <c r="S23" s="19"/>
+      <c r="T23" s="17" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U23" s="19"/>
+      <c r="V23" s="19"/>
+      <c r="W23" s="19"/>
+      <c r="X23" s="19"/>
     </row>
     <row r="24" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="21" t="s">
+      <c r="A24" s="17" t="s">
         <v>126</v>
       </c>
-      <c r="B24" s="21" t="s">
+      <c r="B24" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="C24" s="23" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D24" s="21" t="s">
+      <c r="C24" s="17" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D24" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="E24" s="24" t="s">
+      <c r="E24" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="F24" s="24" t="s">
+      <c r="F24" s="19" t="s">
         <v>127</v>
       </c>
-      <c r="G24" s="21" t="s">
+      <c r="G24" s="17" t="s">
         <v>128</v>
       </c>
-      <c r="H24" s="21" t="s">
+      <c r="H24" s="17" t="s">
         <v>129</v>
       </c>
-      <c r="I24" s="21"/>
-      <c r="J24" s="21"/>
-      <c r="K24" s="21"/>
-      <c r="L24" s="24"/>
-      <c r="M24" s="24" t="s">
+      <c r="I24" s="17"/>
+      <c r="J24" s="17"/>
+      <c r="K24" s="17"/>
+      <c r="L24" s="19"/>
+      <c r="M24" s="19" t="s">
         <v>130</v>
       </c>
-      <c r="N24" s="24"/>
-      <c r="O24" s="24" t="s">
+      <c r="N24" s="19"/>
+      <c r="O24" s="19" t="s">
         <v>125</v>
       </c>
-      <c r="P24" s="25"/>
-      <c r="Q24" s="24"/>
-      <c r="R24" s="24"/>
-      <c r="S24" s="24"/>
-      <c r="T24" s="23" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U24" s="24"/>
-      <c r="V24" s="24"/>
-      <c r="W24" s="24"/>
-      <c r="X24" s="24"/>
+      <c r="P24" s="20"/>
+      <c r="Q24" s="19"/>
+      <c r="R24" s="19"/>
+      <c r="S24" s="19"/>
+      <c r="T24" s="17" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U24" s="19"/>
+      <c r="V24" s="19"/>
+      <c r="W24" s="19"/>
+      <c r="X24" s="19"/>
     </row>
     <row r="25" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="21" t="s">
+      <c r="A25" s="17" t="s">
         <v>131</v>
       </c>
-      <c r="B25" s="21" t="s">
+      <c r="B25" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="C25" s="23" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D25" s="21" t="s">
+      <c r="C25" s="17" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D25" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="E25" s="24" t="s">
+      <c r="E25" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="F25" s="24" t="s">
+      <c r="F25" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="G25" s="21"/>
-      <c r="H25" s="21"/>
-      <c r="I25" s="21"/>
-      <c r="J25" s="21"/>
-      <c r="K25" s="26" t="s">
+      <c r="G25" s="17"/>
+      <c r="H25" s="17"/>
+      <c r="I25" s="17"/>
+      <c r="J25" s="17"/>
+      <c r="K25" s="21" t="s">
         <v>133</v>
       </c>
-      <c r="L25" s="24"/>
-      <c r="M25" s="27" t="s">
+      <c r="L25" s="19"/>
+      <c r="M25" s="22" t="s">
         <v>134</v>
       </c>
-      <c r="N25" s="24"/>
-      <c r="O25" s="24" t="s">
+      <c r="N25" s="19"/>
+      <c r="O25" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="P25" s="24"/>
-      <c r="Q25" s="24"/>
-      <c r="R25" s="24"/>
-      <c r="S25" s="24"/>
-      <c r="T25" s="23" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U25" s="24" t="s">
+      <c r="P25" s="19"/>
+      <c r="Q25" s="19"/>
+      <c r="R25" s="19"/>
+      <c r="S25" s="19"/>
+      <c r="T25" s="17" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U25" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="V25" s="24" t="s">
+      <c r="V25" s="19" t="s">
         <v>136</v>
       </c>
-      <c r="W25" s="24"/>
-      <c r="X25" s="24"/>
+      <c r="W25" s="19"/>
+      <c r="X25" s="19"/>
     </row>
     <row r="26" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="21" t="s">
+      <c r="A26" s="17" t="s">
         <v>137</v>
       </c>
-      <c r="B26" s="21" t="s">
+      <c r="B26" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="C26" s="23" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D26" s="21" t="s">
+      <c r="C26" s="17" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D26" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="E26" s="24" t="s">
+      <c r="E26" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="F26" s="28" t="s">
+      <c r="F26" s="23" t="s">
         <v>138</v>
       </c>
-      <c r="G26" s="21" t="s">
+      <c r="G26" s="17" t="s">
         <v>139</v>
       </c>
-      <c r="H26" s="21" t="s">
+      <c r="H26" s="17" t="s">
         <v>140</v>
       </c>
-      <c r="I26" s="21"/>
-      <c r="J26" s="21"/>
-      <c r="K26" s="21"/>
-      <c r="L26" s="24"/>
-      <c r="M26" s="24" t="s">
+      <c r="I26" s="17"/>
+      <c r="J26" s="17"/>
+      <c r="K26" s="17"/>
+      <c r="L26" s="19"/>
+      <c r="M26" s="19" t="s">
         <v>141</v>
       </c>
-      <c r="N26" s="24"/>
-      <c r="O26" s="24" t="s">
+      <c r="N26" s="19"/>
+      <c r="O26" s="19" t="s">
         <v>137</v>
       </c>
-      <c r="P26" s="24"/>
-      <c r="Q26" s="24"/>
-      <c r="R26" s="24"/>
-      <c r="S26" s="24"/>
-      <c r="T26" s="23" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U26" s="24"/>
-      <c r="V26" s="24"/>
-      <c r="W26" s="24"/>
-      <c r="X26" s="24"/>
+      <c r="P26" s="19"/>
+      <c r="Q26" s="19"/>
+      <c r="R26" s="19"/>
+      <c r="S26" s="19"/>
+      <c r="T26" s="17" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U26" s="19"/>
+      <c r="V26" s="19"/>
+      <c r="W26" s="19"/>
+      <c r="X26" s="19"/>
     </row>
     <row r="27" customFormat="false" ht="62.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="21" t="s">
+      <c r="A27" s="17" t="s">
         <v>142</v>
       </c>
-      <c r="B27" s="21" t="s">
+      <c r="B27" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="C27" s="23" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D27" s="21" t="s">
+      <c r="C27" s="17" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D27" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="E27" s="24" t="s">
+      <c r="E27" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="F27" s="24" t="s">
+      <c r="F27" s="19" t="s">
         <v>143</v>
       </c>
-      <c r="G27" s="21" t="s">
+      <c r="G27" s="17" t="s">
         <v>144</v>
       </c>
-      <c r="H27" s="21" t="s">
+      <c r="H27" s="17" t="s">
         <v>145</v>
       </c>
-      <c r="I27" s="21"/>
-      <c r="J27" s="21"/>
-      <c r="K27" s="21"/>
-      <c r="L27" s="24"/>
-      <c r="M27" s="24" t="s">
+      <c r="I27" s="17"/>
+      <c r="J27" s="17"/>
+      <c r="K27" s="17"/>
+      <c r="L27" s="19"/>
+      <c r="M27" s="19" t="s">
         <v>130</v>
       </c>
-      <c r="N27" s="24"/>
-      <c r="O27" s="24" t="s">
+      <c r="N27" s="19"/>
+      <c r="O27" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="P27" s="24"/>
-      <c r="Q27" s="24"/>
-      <c r="R27" s="24"/>
-      <c r="S27" s="24"/>
-      <c r="T27" s="23" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U27" s="24"/>
-      <c r="V27" s="24"/>
-      <c r="W27" s="24"/>
-      <c r="X27" s="24"/>
+      <c r="P27" s="19"/>
+      <c r="Q27" s="19"/>
+      <c r="R27" s="19"/>
+      <c r="S27" s="19"/>
+      <c r="T27" s="17" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U27" s="19"/>
+      <c r="V27" s="19"/>
+      <c r="W27" s="19"/>
+      <c r="X27" s="19"/>
     </row>
     <row r="28" customFormat="false" ht="52.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="21" t="s">
+      <c r="A28" s="17" t="s">
         <v>147</v>
       </c>
-      <c r="B28" s="21" t="s">
+      <c r="B28" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="C28" s="23" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D28" s="21" t="s">
+      <c r="C28" s="17" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D28" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="E28" s="24" t="s">
+      <c r="E28" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="F28" s="24" t="s">
+      <c r="F28" s="19" t="s">
         <v>148</v>
       </c>
-      <c r="G28" s="21" t="s">
+      <c r="G28" s="17" t="s">
         <v>149</v>
       </c>
-      <c r="H28" s="21" t="s">
+      <c r="H28" s="17" t="s">
         <v>150</v>
       </c>
-      <c r="I28" s="21"/>
-      <c r="J28" s="21"/>
-      <c r="K28" s="21"/>
-      <c r="L28" s="24"/>
-      <c r="M28" s="24" t="s">
+      <c r="I28" s="17"/>
+      <c r="J28" s="17"/>
+      <c r="K28" s="17"/>
+      <c r="L28" s="19"/>
+      <c r="M28" s="19" t="s">
         <v>151</v>
       </c>
-      <c r="N28" s="24"/>
-      <c r="O28" s="24" t="s">
+      <c r="N28" s="19"/>
+      <c r="O28" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="P28" s="24"/>
-      <c r="Q28" s="24"/>
-      <c r="R28" s="24"/>
-      <c r="S28" s="24"/>
-      <c r="T28" s="23" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U28" s="24"/>
-      <c r="V28" s="24"/>
-      <c r="W28" s="24"/>
-      <c r="X28" s="24"/>
-    </row>
-    <row r="29" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="29" t="s">
+      <c r="P28" s="19"/>
+      <c r="Q28" s="19"/>
+      <c r="R28" s="19"/>
+      <c r="S28" s="19"/>
+      <c r="T28" s="17" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U28" s="19"/>
+      <c r="V28" s="19"/>
+      <c r="W28" s="19"/>
+      <c r="X28" s="19"/>
+    </row>
+    <row r="29" customFormat="false" ht="33.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="24" t="s">
         <v>152</v>
       </c>
-      <c r="B29" s="21" t="s">
+      <c r="B29" s="17" t="s">
         <v>153</v>
       </c>
-      <c r="C29" s="23" t="b">
+      <c r="C29" s="17" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="D29" s="21" t="s">
+      <c r="D29" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="E29" s="24" t="s">
+      <c r="E29" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="F29" s="24" t="s">
+      <c r="F29" s="19" t="s">
         <v>154</v>
       </c>
-      <c r="G29" s="21" t="s">
+      <c r="G29" s="17" t="s">
         <v>155</v>
       </c>
-      <c r="H29" s="21" t="s">
+      <c r="H29" s="17" t="s">
         <v>156</v>
       </c>
-      <c r="I29" s="21"/>
-      <c r="J29" s="21"/>
-      <c r="K29" s="21"/>
-      <c r="L29" s="24"/>
-      <c r="M29" s="24" t="s">
+      <c r="I29" s="17"/>
+      <c r="J29" s="17"/>
+      <c r="K29" s="17"/>
+      <c r="L29" s="19"/>
+      <c r="M29" s="19" t="s">
         <v>157</v>
       </c>
-      <c r="N29" s="25"/>
-      <c r="O29" s="24" t="s">
+      <c r="N29" s="20"/>
+      <c r="O29" s="19" t="s">
         <v>158</v>
       </c>
-      <c r="P29" s="24"/>
-      <c r="Q29" s="24"/>
-      <c r="R29" s="24"/>
-      <c r="S29" s="24"/>
-      <c r="T29" s="23" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U29" s="24"/>
-      <c r="V29" s="24"/>
-      <c r="W29" s="24"/>
-      <c r="X29" s="24"/>
-    </row>
-    <row r="30" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="21" t="s">
+      <c r="P29" s="19"/>
+      <c r="Q29" s="19"/>
+      <c r="R29" s="19"/>
+      <c r="S29" s="19"/>
+      <c r="T29" s="17" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U29" s="19"/>
+      <c r="V29" s="19"/>
+      <c r="W29" s="19"/>
+      <c r="X29" s="19"/>
+    </row>
+    <row r="30" customFormat="false" ht="33.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="17" t="s">
         <v>159</v>
       </c>
-      <c r="B30" s="21" t="s">
+      <c r="B30" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="C30" s="23" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D30" s="21" t="s">
+      <c r="C30" s="17" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D30" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="E30" s="24" t="s">
+      <c r="E30" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="F30" s="24" t="s">
+      <c r="F30" s="19" t="s">
         <v>160</v>
       </c>
-      <c r="G30" s="21" t="s">
+      <c r="G30" s="17" t="s">
         <v>161</v>
       </c>
-      <c r="H30" s="21" t="s">
+      <c r="H30" s="17" t="s">
         <v>162</v>
       </c>
-      <c r="I30" s="21"/>
-      <c r="J30" s="21"/>
-      <c r="K30" s="21"/>
-      <c r="L30" s="24"/>
-      <c r="M30" s="24" t="s">
+      <c r="I30" s="17"/>
+      <c r="J30" s="17"/>
+      <c r="K30" s="17"/>
+      <c r="L30" s="19"/>
+      <c r="M30" s="19" t="s">
         <v>163</v>
       </c>
-      <c r="N30" s="24"/>
-      <c r="O30" s="24" t="s">
+      <c r="N30" s="19"/>
+      <c r="O30" s="19" t="s">
         <v>96</v>
       </c>
-      <c r="P30" s="24"/>
-      <c r="Q30" s="24"/>
-      <c r="R30" s="24"/>
-      <c r="S30" s="24"/>
-      <c r="T30" s="23" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U30" s="24"/>
-      <c r="V30" s="24"/>
-      <c r="W30" s="24"/>
-      <c r="X30" s="24"/>
+      <c r="P30" s="19"/>
+      <c r="Q30" s="19"/>
+      <c r="R30" s="19"/>
+      <c r="S30" s="19"/>
+      <c r="T30" s="17" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U30" s="19"/>
+      <c r="V30" s="19"/>
+      <c r="W30" s="19"/>
+      <c r="X30" s="19"/>
     </row>
     <row r="31" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="21" t="s">
+      <c r="A31" s="17" t="s">
         <v>164</v>
       </c>
-      <c r="B31" s="21" t="s">
+      <c r="B31" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="C31" s="23" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D31" s="21" t="s">
+      <c r="C31" s="17" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D31" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="E31" s="24" t="s">
+      <c r="E31" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="F31" s="24" t="s">
+      <c r="F31" s="19" t="s">
         <v>165</v>
       </c>
-      <c r="G31" s="21" t="s">
+      <c r="G31" s="17" t="s">
         <v>166</v>
       </c>
-      <c r="H31" s="21" t="s">
+      <c r="H31" s="17" t="s">
         <v>167</v>
       </c>
-      <c r="I31" s="21"/>
-      <c r="J31" s="21"/>
-      <c r="K31" s="21"/>
-      <c r="L31" s="24"/>
-      <c r="M31" s="24" t="s">
+      <c r="I31" s="17"/>
+      <c r="J31" s="17"/>
+      <c r="K31" s="17"/>
+      <c r="L31" s="19"/>
+      <c r="M31" s="19" t="s">
         <v>168</v>
       </c>
-      <c r="N31" s="24"/>
-      <c r="O31" s="24" t="s">
+      <c r="N31" s="19"/>
+      <c r="O31" s="19" t="s">
         <v>165</v>
       </c>
-      <c r="P31" s="24"/>
-      <c r="Q31" s="24"/>
-      <c r="R31" s="24"/>
-      <c r="S31" s="24"/>
-      <c r="T31" s="23" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U31" s="24"/>
-      <c r="V31" s="24"/>
-      <c r="W31" s="24"/>
-      <c r="X31" s="24"/>
+      <c r="P31" s="19"/>
+      <c r="Q31" s="19"/>
+      <c r="R31" s="19"/>
+      <c r="S31" s="19"/>
+      <c r="T31" s="17" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U31" s="19"/>
+      <c r="V31" s="19"/>
+      <c r="W31" s="19"/>
+      <c r="X31" s="19"/>
     </row>
     <row r="32" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="21" t="s">
+      <c r="A32" s="17" t="s">
         <v>169</v>
       </c>
-      <c r="B32" s="21" t="s">
+      <c r="B32" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="C32" s="23" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D32" s="21" t="s">
+      <c r="C32" s="17" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D32" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="E32" s="24" t="s">
+      <c r="E32" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="F32" s="24" t="s">
+      <c r="F32" s="19" t="s">
         <v>170</v>
       </c>
-      <c r="G32" s="21" t="s">
+      <c r="G32" s="17" t="s">
         <v>171</v>
       </c>
-      <c r="H32" s="21" t="s">
+      <c r="H32" s="17" t="s">
         <v>172</v>
       </c>
-      <c r="I32" s="21"/>
-      <c r="J32" s="21"/>
-      <c r="K32" s="21"/>
-      <c r="L32" s="24"/>
-      <c r="M32" s="24" t="s">
+      <c r="I32" s="17"/>
+      <c r="J32" s="17"/>
+      <c r="K32" s="17"/>
+      <c r="L32" s="19"/>
+      <c r="M32" s="19" t="s">
         <v>173</v>
       </c>
-      <c r="N32" s="24"/>
-      <c r="O32" s="24" t="s">
+      <c r="N32" s="19"/>
+      <c r="O32" s="19" t="s">
         <v>174</v>
       </c>
-      <c r="P32" s="24"/>
-      <c r="Q32" s="24"/>
-      <c r="R32" s="24"/>
-      <c r="S32" s="24"/>
-      <c r="T32" s="23" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U32" s="24"/>
-      <c r="V32" s="24"/>
-      <c r="W32" s="24"/>
-      <c r="X32" s="24"/>
+      <c r="P32" s="19"/>
+      <c r="Q32" s="19"/>
+      <c r="R32" s="19"/>
+      <c r="S32" s="19"/>
+      <c r="T32" s="17" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U32" s="19"/>
+      <c r="V32" s="19"/>
+      <c r="W32" s="19"/>
+      <c r="X32" s="19"/>
     </row>
     <row r="33" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="21" t="s">
+      <c r="A33" s="17" t="s">
         <v>175</v>
       </c>
-      <c r="B33" s="21" t="s">
+      <c r="B33" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="C33" s="23" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D33" s="21" t="s">
+      <c r="C33" s="17" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D33" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="E33" s="24" t="s">
+      <c r="E33" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="F33" s="24" t="s">
+      <c r="F33" s="19" t="s">
         <v>176</v>
       </c>
-      <c r="G33" s="21" t="s">
+      <c r="G33" s="17" t="s">
         <v>177</v>
       </c>
-      <c r="H33" s="21" t="s">
+      <c r="H33" s="17" t="s">
         <v>178</v>
       </c>
-      <c r="I33" s="21"/>
-      <c r="J33" s="21"/>
-      <c r="K33" s="21"/>
-      <c r="L33" s="24"/>
-      <c r="M33" s="21" t="s">
+      <c r="I33" s="17"/>
+      <c r="J33" s="17"/>
+      <c r="K33" s="17"/>
+      <c r="L33" s="19"/>
+      <c r="M33" s="17" t="s">
         <v>179</v>
       </c>
-      <c r="N33" s="24"/>
-      <c r="O33" s="24"/>
-      <c r="P33" s="24"/>
-      <c r="Q33" s="24"/>
-      <c r="R33" s="24"/>
-      <c r="S33" s="24"/>
-      <c r="T33" s="23" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U33" s="24"/>
-      <c r="V33" s="24"/>
-      <c r="W33" s="24"/>
-      <c r="X33" s="24"/>
-    </row>
-    <row r="34" customFormat="false" ht="85.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="21" t="s">
+      <c r="N33" s="19"/>
+      <c r="O33" s="19"/>
+      <c r="P33" s="19"/>
+      <c r="Q33" s="19"/>
+      <c r="R33" s="19"/>
+      <c r="S33" s="19"/>
+      <c r="T33" s="17" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U33" s="19"/>
+      <c r="V33" s="19"/>
+      <c r="W33" s="19"/>
+      <c r="X33" s="19"/>
+    </row>
+    <row r="34" customFormat="false" ht="87.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="17" t="s">
         <v>180</v>
       </c>
-      <c r="B34" s="30" t="s">
+      <c r="B34" s="25" t="s">
         <v>69</v>
       </c>
-      <c r="C34" s="23" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D34" s="21" t="s">
+      <c r="C34" s="17" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D34" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="E34" s="24" t="s">
+      <c r="E34" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="F34" s="24" t="s">
+      <c r="F34" s="19" t="s">
         <v>181</v>
       </c>
-      <c r="G34" s="21" t="s">
+      <c r="G34" s="17" t="s">
         <v>182</v>
       </c>
-      <c r="H34" s="21" t="s">
+      <c r="H34" s="17" t="s">
         <v>183</v>
       </c>
-      <c r="I34" s="21" t="s">
+      <c r="I34" s="17" t="s">
         <v>184</v>
       </c>
-      <c r="J34" s="21" t="s">
+      <c r="J34" s="17" t="s">
         <v>185</v>
       </c>
-      <c r="K34" s="21"/>
-      <c r="L34" s="24"/>
-      <c r="M34" s="21" t="s">
+      <c r="K34" s="17"/>
+      <c r="L34" s="19"/>
+      <c r="M34" s="17" t="s">
         <v>179</v>
       </c>
-      <c r="N34" s="24"/>
-      <c r="O34" s="24"/>
-      <c r="P34" s="24"/>
-      <c r="Q34" s="24"/>
-      <c r="R34" s="24"/>
-      <c r="S34" s="24"/>
-      <c r="T34" s="23" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U34" s="24"/>
-      <c r="V34" s="24"/>
-      <c r="W34" s="24"/>
-      <c r="X34" s="24"/>
+      <c r="N34" s="19"/>
+      <c r="O34" s="19"/>
+      <c r="P34" s="19"/>
+      <c r="Q34" s="19"/>
+      <c r="R34" s="19"/>
+      <c r="S34" s="19"/>
+      <c r="T34" s="17" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U34" s="19"/>
+      <c r="V34" s="19"/>
+      <c r="W34" s="19"/>
+      <c r="X34" s="19"/>
     </row>
     <row r="35" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="21" t="s">
+      <c r="A35" s="17" t="s">
         <v>186</v>
       </c>
-      <c r="B35" s="21" t="s">
+      <c r="B35" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="C35" s="23" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D35" s="21" t="s">
+      <c r="C35" s="17" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D35" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="E35" s="24" t="s">
+      <c r="E35" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="F35" s="24" t="s">
+      <c r="F35" s="19" t="s">
         <v>187</v>
       </c>
-      <c r="G35" s="21" t="s">
+      <c r="G35" s="17" t="s">
         <v>188</v>
       </c>
-      <c r="H35" s="21" t="s">
+      <c r="H35" s="17" t="s">
         <v>189</v>
       </c>
-      <c r="I35" s="21"/>
-      <c r="J35" s="21"/>
-      <c r="K35" s="21"/>
-      <c r="L35" s="24"/>
-      <c r="M35" s="21" t="s">
+      <c r="I35" s="17"/>
+      <c r="J35" s="17"/>
+      <c r="K35" s="17"/>
+      <c r="L35" s="19"/>
+      <c r="M35" s="17" t="s">
         <v>190</v>
       </c>
-      <c r="N35" s="24"/>
-      <c r="O35" s="24"/>
-      <c r="P35" s="24"/>
-      <c r="Q35" s="24"/>
-      <c r="R35" s="24"/>
-      <c r="S35" s="24"/>
-      <c r="T35" s="23" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U35" s="24"/>
-      <c r="V35" s="24"/>
-      <c r="W35" s="24"/>
-      <c r="X35" s="24"/>
-    </row>
-    <row r="36" customFormat="false" ht="85.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="21" t="s">
+      <c r="N35" s="19"/>
+      <c r="O35" s="19"/>
+      <c r="P35" s="19"/>
+      <c r="Q35" s="19"/>
+      <c r="R35" s="19"/>
+      <c r="S35" s="19"/>
+      <c r="T35" s="17" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U35" s="19"/>
+      <c r="V35" s="19"/>
+      <c r="W35" s="19"/>
+      <c r="X35" s="19"/>
+    </row>
+    <row r="36" customFormat="false" ht="87.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="17" t="s">
         <v>191</v>
       </c>
-      <c r="B36" s="30" t="s">
+      <c r="B36" s="25" t="s">
         <v>69</v>
       </c>
-      <c r="C36" s="23" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D36" s="21" t="s">
+      <c r="C36" s="17" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D36" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="E36" s="24" t="s">
+      <c r="E36" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="F36" s="24" t="s">
+      <c r="F36" s="19" t="s">
         <v>192</v>
       </c>
-      <c r="G36" s="21" t="s">
+      <c r="G36" s="17" t="s">
         <v>193</v>
       </c>
-      <c r="H36" s="21" t="s">
+      <c r="H36" s="17" t="s">
         <v>194</v>
       </c>
-      <c r="I36" s="21" t="s">
+      <c r="I36" s="17" t="s">
         <v>195</v>
       </c>
-      <c r="J36" s="21" t="s">
+      <c r="J36" s="17" t="s">
         <v>196</v>
       </c>
-      <c r="K36" s="31"/>
-      <c r="L36" s="32"/>
-      <c r="M36" s="31"/>
-      <c r="N36" s="32"/>
-      <c r="O36" s="32"/>
-      <c r="P36" s="32"/>
-      <c r="Q36" s="32"/>
-      <c r="R36" s="24"/>
-      <c r="S36" s="24"/>
-      <c r="T36" s="23" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U36" s="24"/>
-      <c r="V36" s="24"/>
-      <c r="W36" s="24"/>
-      <c r="X36" s="24"/>
+      <c r="K36" s="26"/>
+      <c r="L36" s="27"/>
+      <c r="M36" s="26"/>
+      <c r="N36" s="27"/>
+      <c r="O36" s="27"/>
+      <c r="P36" s="27"/>
+      <c r="Q36" s="27"/>
+      <c r="R36" s="19"/>
+      <c r="S36" s="19"/>
+      <c r="T36" s="17" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U36" s="19"/>
+      <c r="V36" s="19"/>
+      <c r="W36" s="19"/>
+      <c r="X36" s="19"/>
     </row>
     <row r="37" customFormat="false" ht="86.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="29" t="s">
+      <c r="A37" s="24" t="s">
         <v>197</v>
       </c>
-      <c r="B37" s="21" t="s">
+      <c r="B37" s="17" t="s">
         <v>153</v>
       </c>
-      <c r="C37" s="23" t="b">
+      <c r="C37" s="17" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="D37" s="21" t="s">
+      <c r="D37" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="E37" s="24" t="s">
+      <c r="E37" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="F37" s="24" t="s">
+      <c r="F37" s="19" t="s">
         <v>198</v>
       </c>
-      <c r="G37" s="21" t="s">
+      <c r="G37" s="17" t="s">
         <v>199</v>
       </c>
-      <c r="H37" s="21" t="s">
+      <c r="H37" s="17" t="s">
         <v>200</v>
       </c>
-      <c r="I37" s="21"/>
-      <c r="J37" s="21"/>
-      <c r="K37" s="21"/>
-      <c r="L37" s="24"/>
-      <c r="M37" s="25"/>
-      <c r="N37" s="25"/>
-      <c r="O37" s="33" t="s">
+      <c r="I37" s="17"/>
+      <c r="J37" s="17"/>
+      <c r="K37" s="17"/>
+      <c r="L37" s="19"/>
+      <c r="M37" s="20"/>
+      <c r="N37" s="20"/>
+      <c r="O37" s="28" t="s">
         <v>146</v>
       </c>
-      <c r="P37" s="24"/>
-      <c r="Q37" s="24"/>
-      <c r="R37" s="24"/>
-      <c r="S37" s="24"/>
-      <c r="T37" s="23" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U37" s="24"/>
-      <c r="V37" s="24"/>
-      <c r="W37" s="24"/>
-      <c r="X37" s="24"/>
+      <c r="P37" s="19"/>
+      <c r="Q37" s="19"/>
+      <c r="R37" s="19"/>
+      <c r="S37" s="19"/>
+      <c r="T37" s="17" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U37" s="19"/>
+      <c r="V37" s="19"/>
+      <c r="W37" s="19"/>
+      <c r="X37" s="19"/>
     </row>
     <row r="38" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="29" t="s">
+      <c r="A38" s="24" t="s">
         <v>201</v>
       </c>
-      <c r="B38" s="21" t="s">
+      <c r="B38" s="17" t="s">
         <v>153</v>
       </c>
-      <c r="C38" s="23" t="b">
+      <c r="C38" s="17" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="D38" s="21" t="s">
+      <c r="D38" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="E38" s="24" t="s">
+      <c r="E38" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="F38" s="24" t="s">
+      <c r="F38" s="19" t="s">
         <v>202</v>
       </c>
-      <c r="G38" s="21" t="s">
+      <c r="G38" s="17" t="s">
         <v>203</v>
       </c>
-      <c r="H38" s="21" t="s">
+      <c r="H38" s="17" t="s">
         <v>204</v>
       </c>
-      <c r="I38" s="21"/>
-      <c r="J38" s="21"/>
-      <c r="K38" s="21"/>
-      <c r="L38" s="24"/>
-      <c r="M38" s="25"/>
-      <c r="N38" s="25"/>
-      <c r="O38" s="33" t="s">
+      <c r="I38" s="17"/>
+      <c r="J38" s="17"/>
+      <c r="K38" s="17"/>
+      <c r="L38" s="19"/>
+      <c r="M38" s="20"/>
+      <c r="N38" s="20"/>
+      <c r="O38" s="28" t="s">
         <v>146</v>
       </c>
-      <c r="P38" s="24"/>
-      <c r="Q38" s="24"/>
-      <c r="R38" s="24"/>
-      <c r="S38" s="24"/>
-      <c r="T38" s="23" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U38" s="24"/>
-      <c r="V38" s="24"/>
-      <c r="W38" s="24"/>
-      <c r="X38" s="24"/>
-    </row>
-    <row r="39" s="6" customFormat="true" ht="64.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="29" t="s">
+      <c r="P38" s="19"/>
+      <c r="Q38" s="19"/>
+      <c r="R38" s="19"/>
+      <c r="S38" s="19"/>
+      <c r="T38" s="17" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U38" s="19"/>
+      <c r="V38" s="19"/>
+      <c r="W38" s="19"/>
+      <c r="X38" s="19"/>
+    </row>
+    <row r="39" s="6" customFormat="true" ht="55.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="24" t="s">
         <v>205</v>
       </c>
-      <c r="B39" s="21" t="s">
+      <c r="B39" s="17" t="s">
         <v>153</v>
       </c>
-      <c r="C39" s="23" t="b">
+      <c r="C39" s="17" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="D39" s="21" t="s">
+      <c r="D39" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="E39" s="24" t="s">
+      <c r="E39" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="F39" s="24" t="s">
+      <c r="F39" s="19" t="s">
         <v>206</v>
       </c>
-      <c r="G39" s="21" t="s">
+      <c r="G39" s="17" t="s">
         <v>207</v>
       </c>
-      <c r="H39" s="21" t="s">
+      <c r="H39" s="17" t="s">
         <v>208</v>
       </c>
-      <c r="I39" s="21"/>
-      <c r="J39" s="21"/>
-      <c r="K39" s="21"/>
-      <c r="L39" s="24"/>
-      <c r="M39" s="25"/>
-      <c r="N39" s="25"/>
-      <c r="O39" s="33" t="s">
+      <c r="I39" s="17"/>
+      <c r="J39" s="17"/>
+      <c r="K39" s="17"/>
+      <c r="L39" s="19"/>
+      <c r="M39" s="20"/>
+      <c r="N39" s="20"/>
+      <c r="O39" s="28" t="s">
         <v>146</v>
       </c>
-      <c r="P39" s="24"/>
-      <c r="Q39" s="24"/>
-      <c r="R39" s="24"/>
-      <c r="S39" s="24"/>
-      <c r="T39" s="23" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U39" s="24"/>
-      <c r="V39" s="24"/>
-      <c r="W39" s="24"/>
-      <c r="X39" s="24"/>
+      <c r="P39" s="19"/>
+      <c r="Q39" s="19"/>
+      <c r="R39" s="19"/>
+      <c r="S39" s="19"/>
+      <c r="T39" s="17" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U39" s="19"/>
+      <c r="V39" s="19"/>
+      <c r="W39" s="19"/>
+      <c r="X39" s="19"/>
     </row>
     <row r="40" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="29" t="s">
+      <c r="A40" s="24" t="s">
         <v>209</v>
       </c>
-      <c r="B40" s="21" t="s">
+      <c r="B40" s="17" t="s">
         <v>153</v>
       </c>
-      <c r="C40" s="23" t="b">
+      <c r="C40" s="17" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="D40" s="21" t="s">
+      <c r="D40" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="E40" s="24" t="s">
+      <c r="E40" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="F40" s="24" t="s">
+      <c r="F40" s="19" t="s">
         <v>210</v>
       </c>
-      <c r="G40" s="21" t="s">
+      <c r="G40" s="17" t="s">
         <v>211</v>
       </c>
-      <c r="H40" s="21" t="s">
+      <c r="H40" s="17" t="s">
         <v>212</v>
       </c>
-      <c r="I40" s="21"/>
-      <c r="J40" s="21"/>
-      <c r="K40" s="21"/>
-      <c r="L40" s="24"/>
-      <c r="M40" s="25"/>
-      <c r="N40" s="25"/>
-      <c r="O40" s="33" t="s">
+      <c r="I40" s="17"/>
+      <c r="J40" s="17"/>
+      <c r="K40" s="17"/>
+      <c r="L40" s="19"/>
+      <c r="M40" s="20"/>
+      <c r="N40" s="20"/>
+      <c r="O40" s="28" t="s">
         <v>146</v>
       </c>
-      <c r="P40" s="24"/>
-      <c r="Q40" s="24"/>
-      <c r="R40" s="24"/>
-      <c r="S40" s="24"/>
-      <c r="T40" s="23" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U40" s="24"/>
-      <c r="V40" s="24"/>
-      <c r="W40" s="24"/>
-      <c r="X40" s="24"/>
+      <c r="P40" s="19"/>
+      <c r="Q40" s="19"/>
+      <c r="R40" s="19"/>
+      <c r="S40" s="19"/>
+      <c r="T40" s="17" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U40" s="19"/>
+      <c r="V40" s="19"/>
+      <c r="W40" s="19"/>
+      <c r="X40" s="19"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="34" t="s">
+      <c r="A41" s="29" t="s">
         <v>213</v>
       </c>
-      <c r="B41" s="34" t="s">
+      <c r="B41" s="29" t="s">
         <v>98</v>
       </c>
-      <c r="C41" s="35" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D41" s="34" t="s">
+      <c r="C41" s="29" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D41" s="29" t="s">
         <v>102</v>
       </c>
-      <c r="E41" s="36"/>
-      <c r="F41" s="36" t="str">
+      <c r="E41" s="30"/>
+      <c r="F41" s="30" t="str">
         <f aca="false">REPLACE(A41, FIND("_", A41), 1, ".")</f>
         <v>household.save</v>
       </c>
-      <c r="G41" s="34" t="s">
+      <c r="G41" s="29" t="s">
         <v>99</v>
       </c>
-      <c r="H41" s="34" t="s">
+      <c r="H41" s="29" t="s">
         <v>100</v>
       </c>
-      <c r="I41" s="34"/>
-      <c r="J41" s="34"/>
-      <c r="K41" s="34"/>
-      <c r="L41" s="36"/>
-      <c r="M41" s="36"/>
-      <c r="N41" s="36"/>
-      <c r="O41" s="36"/>
-      <c r="P41" s="36"/>
-      <c r="Q41" s="36"/>
-      <c r="R41" s="36"/>
-      <c r="S41" s="36"/>
-      <c r="T41" s="35" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U41" s="36"/>
-      <c r="V41" s="36"/>
-      <c r="W41" s="36"/>
-      <c r="X41" s="36"/>
-    </row>
-    <row r="42" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I41" s="29"/>
+      <c r="J41" s="29"/>
+      <c r="K41" s="29"/>
+      <c r="L41" s="30"/>
+      <c r="M41" s="30"/>
+      <c r="N41" s="30"/>
+      <c r="O41" s="30"/>
+      <c r="P41" s="30"/>
+      <c r="Q41" s="30"/>
+      <c r="R41" s="30"/>
+      <c r="S41" s="30"/>
+      <c r="T41" s="29" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U41" s="30"/>
+      <c r="V41" s="30"/>
+      <c r="W41" s="30"/>
+      <c r="X41" s="30"/>
+    </row>
+    <row r="42" customFormat="false" ht="116.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
         <v>214</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C42" s="37" t="b">
+      <c r="C42" s="1" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -4120,9 +4093,9 @@
       <c r="H42" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="L42" s="38"/>
-      <c r="M42" s="39"/>
-      <c r="T42" s="37" t="b">
+      <c r="L42" s="31"/>
+      <c r="M42" s="32"/>
+      <c r="T42" s="1" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -4177,489 +4150,489 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F29"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="40" width="27.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="40" width="15.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="40" width="31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="41" width="20.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="40" width="19.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="40" width="12.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="33" width="27.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="33" width="15.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="33" width="31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="34" width="20.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="33" width="19.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="33" width="12.14"/>
   </cols>
   <sheetData>
-    <row r="1" s="44" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="42" t="s">
+    <row r="1" s="37" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="35" t="s">
         <v>218</v>
       </c>
-      <c r="B1" s="42" t="s">
+      <c r="B1" s="35" t="s">
         <v>219</v>
       </c>
-      <c r="C1" s="42" t="s">
+      <c r="C1" s="35" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="43" t="s">
+      <c r="D1" s="36" t="s">
         <v>220</v>
       </c>
-      <c r="E1" s="42" t="s">
+      <c r="E1" s="35" t="s">
         <v>221</v>
       </c>
-      <c r="F1" s="42" t="s">
+      <c r="F1" s="35" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="45" t="s">
+    <row r="2" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="38" t="s">
         <v>223</v>
       </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45" t="s">
+      <c r="B2" s="38"/>
+      <c r="C2" s="38" t="s">
         <v>224</v>
       </c>
-      <c r="D2" s="46" t="s">
+      <c r="D2" s="39" t="s">
         <v>225</v>
       </c>
-      <c r="E2" s="45" t="n">
-        <v>1</v>
-      </c>
-      <c r="F2" s="45"/>
-    </row>
-    <row r="3" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="45" t="s">
+      <c r="E2" s="38" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="38"/>
+    </row>
+    <row r="3" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="38" t="s">
         <v>95</v>
       </c>
-      <c r="B3" s="45"/>
-      <c r="C3" s="45" t="s">
+      <c r="B3" s="38"/>
+      <c r="C3" s="38" t="s">
         <v>224</v>
       </c>
-      <c r="D3" s="46" t="s">
+      <c r="D3" s="39" t="s">
         <v>226</v>
       </c>
-      <c r="E3" s="45" t="n">
+      <c r="E3" s="38" t="n">
         <v>2</v>
       </c>
-      <c r="F3" s="45"/>
-    </row>
-    <row r="4" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="45" t="s">
+      <c r="F3" s="38"/>
+    </row>
+    <row r="4" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="38" t="s">
         <v>163</v>
       </c>
-      <c r="B4" s="45"/>
-      <c r="C4" s="45" t="s">
+      <c r="B4" s="38"/>
+      <c r="C4" s="38" t="s">
         <v>227</v>
       </c>
-      <c r="D4" s="46" t="s">
+      <c r="D4" s="39" t="s">
         <v>225</v>
       </c>
-      <c r="E4" s="45" t="s">
+      <c r="E4" s="38" t="s">
         <v>228</v>
       </c>
-      <c r="F4" s="45"/>
-    </row>
-    <row r="5" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="45" t="s">
+      <c r="F4" s="38"/>
+    </row>
+    <row r="5" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="38" t="s">
         <v>163</v>
       </c>
-      <c r="B5" s="45" t="s">
+      <c r="B5" s="38" t="s">
         <v>229</v>
       </c>
-      <c r="C5" s="45" t="s">
+      <c r="C5" s="38" t="s">
         <v>224</v>
       </c>
-      <c r="D5" s="46" t="s">
+      <c r="D5" s="39" t="s">
         <v>225</v>
       </c>
-      <c r="E5" s="45" t="n">
-        <v>1</v>
-      </c>
-      <c r="F5" s="45"/>
-    </row>
-    <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="45" t="s">
+      <c r="E5" s="38" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="38"/>
+    </row>
+    <row r="6" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="38" t="s">
         <v>230</v>
       </c>
-      <c r="B6" s="45"/>
-      <c r="C6" s="45" t="s">
+      <c r="B6" s="38"/>
+      <c r="C6" s="38" t="s">
         <v>231</v>
       </c>
-      <c r="D6" s="46" t="s">
+      <c r="D6" s="39" t="s">
         <v>226</v>
       </c>
-      <c r="E6" s="45" t="n">
+      <c r="E6" s="38" t="n">
         <v>3</v>
       </c>
-      <c r="F6" s="45"/>
-    </row>
-    <row r="7" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="45" t="s">
+      <c r="F6" s="38"/>
+    </row>
+    <row r="7" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="38" t="s">
         <v>230</v>
       </c>
-      <c r="B7" s="45" t="s">
+      <c r="B7" s="38" t="s">
         <v>232</v>
       </c>
-      <c r="C7" s="45" t="s">
+      <c r="C7" s="38" t="s">
         <v>231</v>
       </c>
-      <c r="D7" s="46" t="s">
+      <c r="D7" s="39" t="s">
         <v>233</v>
       </c>
-      <c r="E7" s="45" t="n">
+      <c r="E7" s="38" t="n">
         <v>5</v>
       </c>
-      <c r="F7" s="45"/>
-    </row>
-    <row r="8" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="45" t="s">
+      <c r="F7" s="38"/>
+    </row>
+    <row r="8" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="38" t="s">
         <v>234</v>
       </c>
-      <c r="B8" s="45"/>
-      <c r="C8" s="45" t="s">
+      <c r="B8" s="38"/>
+      <c r="C8" s="38" t="s">
         <v>231</v>
       </c>
-      <c r="D8" s="46" t="s">
+      <c r="D8" s="39" t="s">
         <v>226</v>
       </c>
-      <c r="E8" s="45" t="n">
+      <c r="E8" s="38" t="n">
         <v>4</v>
       </c>
-      <c r="F8" s="45"/>
-    </row>
-    <row r="9" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="45" t="s">
+      <c r="F8" s="38"/>
+    </row>
+    <row r="9" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="38" t="s">
         <v>234</v>
       </c>
-      <c r="B9" s="45" t="s">
+      <c r="B9" s="38" t="s">
         <v>232</v>
       </c>
-      <c r="C9" s="45" t="s">
+      <c r="C9" s="38" t="s">
         <v>231</v>
       </c>
-      <c r="D9" s="46" t="s">
+      <c r="D9" s="39" t="s">
         <v>233</v>
       </c>
-      <c r="E9" s="45" t="n">
+      <c r="E9" s="38" t="n">
         <v>13</v>
       </c>
-      <c r="F9" s="45"/>
-    </row>
-    <row r="10" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="45" t="s">
+      <c r="F9" s="38"/>
+    </row>
+    <row r="10" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="38" t="s">
         <v>235</v>
       </c>
-      <c r="B10" s="45"/>
-      <c r="C10" s="45" t="s">
+      <c r="B10" s="38"/>
+      <c r="C10" s="38" t="s">
         <v>231</v>
       </c>
-      <c r="D10" s="46" t="s">
+      <c r="D10" s="39" t="s">
         <v>233</v>
       </c>
-      <c r="E10" s="45" t="n">
+      <c r="E10" s="38" t="n">
         <v>5</v>
       </c>
-      <c r="F10" s="45"/>
-    </row>
-    <row r="11" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="45" t="s">
+      <c r="F10" s="38"/>
+    </row>
+    <row r="11" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="38" t="s">
         <v>119</v>
       </c>
-      <c r="B11" s="45"/>
-      <c r="C11" s="45" t="s">
+      <c r="B11" s="38"/>
+      <c r="C11" s="38" t="s">
         <v>231</v>
       </c>
-      <c r="D11" s="46" t="s">
+      <c r="D11" s="39" t="s">
         <v>226</v>
       </c>
-      <c r="E11" s="45" t="n">
+      <c r="E11" s="38" t="n">
         <v>5</v>
       </c>
-      <c r="F11" s="45"/>
-    </row>
-    <row r="12" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="45" t="s">
+      <c r="F11" s="38"/>
+    </row>
+    <row r="12" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="38" t="s">
         <v>157</v>
       </c>
-      <c r="B12" s="45"/>
-      <c r="C12" s="45" t="s">
+      <c r="B12" s="38"/>
+      <c r="C12" s="38" t="s">
         <v>231</v>
       </c>
-      <c r="D12" s="46" t="s">
+      <c r="D12" s="39" t="s">
         <v>226</v>
       </c>
-      <c r="E12" s="45" t="n">
+      <c r="E12" s="38" t="n">
         <v>6</v>
       </c>
-      <c r="F12" s="45"/>
-    </row>
-    <row r="13" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="45" t="s">
+      <c r="F12" s="38"/>
+    </row>
+    <row r="13" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="38" t="s">
         <v>236</v>
       </c>
-      <c r="B13" s="45"/>
-      <c r="C13" s="45" t="s">
+      <c r="B13" s="38"/>
+      <c r="C13" s="38" t="s">
         <v>231</v>
       </c>
-      <c r="D13" s="46" t="s">
+      <c r="D13" s="39" t="s">
         <v>226</v>
       </c>
-      <c r="E13" s="45" t="n">
+      <c r="E13" s="38" t="n">
         <v>11</v>
       </c>
-      <c r="F13" s="45"/>
-    </row>
-    <row r="14" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="45" t="s">
+      <c r="F13" s="38"/>
+    </row>
+    <row r="14" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="38" t="s">
         <v>124</v>
       </c>
-      <c r="B14" s="45"/>
-      <c r="C14" s="45" t="s">
+      <c r="B14" s="38"/>
+      <c r="C14" s="38" t="s">
         <v>231</v>
       </c>
-      <c r="D14" s="46" t="s">
+      <c r="D14" s="39" t="s">
         <v>226</v>
       </c>
-      <c r="E14" s="45" t="n">
+      <c r="E14" s="38" t="n">
         <v>14</v>
       </c>
-      <c r="F14" s="45"/>
-    </row>
-    <row r="15" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="45" t="s">
+      <c r="F14" s="38"/>
+    </row>
+    <row r="15" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="38" t="s">
         <v>134</v>
       </c>
-      <c r="B15" s="45"/>
-      <c r="C15" s="45" t="s">
+      <c r="B15" s="38"/>
+      <c r="C15" s="38" t="s">
         <v>231</v>
       </c>
-      <c r="D15" s="46" t="s">
+      <c r="D15" s="39" t="s">
         <v>233</v>
       </c>
-      <c r="E15" s="45" t="n">
+      <c r="E15" s="38" t="n">
         <v>15</v>
       </c>
-      <c r="F15" s="45"/>
-    </row>
-    <row r="16" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="45" t="s">
+      <c r="F15" s="38"/>
+    </row>
+    <row r="16" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="38" t="s">
         <v>134</v>
       </c>
-      <c r="B16" s="45" t="s">
+      <c r="B16" s="38" t="s">
         <v>232</v>
       </c>
-      <c r="C16" s="45" t="s">
+      <c r="C16" s="38" t="s">
         <v>231</v>
       </c>
-      <c r="D16" s="46" t="s">
+      <c r="D16" s="39" t="s">
         <v>237</v>
       </c>
-      <c r="E16" s="45" t="s">
+      <c r="E16" s="38" t="s">
         <v>238</v>
       </c>
-      <c r="F16" s="45"/>
-    </row>
-    <row r="17" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="45" t="s">
+      <c r="F16" s="38"/>
+    </row>
+    <row r="17" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="38" t="s">
         <v>239</v>
       </c>
-      <c r="B17" s="45"/>
-      <c r="C17" s="45" t="s">
+      <c r="B17" s="38"/>
+      <c r="C17" s="38" t="s">
         <v>231</v>
       </c>
-      <c r="D17" s="46" t="s">
+      <c r="D17" s="39" t="s">
         <v>226</v>
       </c>
-      <c r="E17" s="45" t="n">
+      <c r="E17" s="38" t="n">
         <v>15</v>
       </c>
-      <c r="F17" s="45"/>
-    </row>
-    <row r="18" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="45" t="s">
+      <c r="F17" s="38"/>
+    </row>
+    <row r="18" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="38" t="s">
         <v>130</v>
       </c>
-      <c r="B18" s="45"/>
-      <c r="C18" s="45" t="s">
+      <c r="B18" s="38"/>
+      <c r="C18" s="38" t="s">
         <v>231</v>
       </c>
-      <c r="D18" s="46" t="s">
+      <c r="D18" s="39" t="s">
         <v>226</v>
       </c>
-      <c r="E18" s="45" t="n">
+      <c r="E18" s="38" t="n">
         <v>16</v>
       </c>
-      <c r="F18" s="45"/>
-    </row>
-    <row r="19" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="45" t="s">
+      <c r="F18" s="38"/>
+    </row>
+    <row r="19" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="38" t="s">
         <v>240</v>
       </c>
-      <c r="B19" s="45"/>
-      <c r="C19" s="45" t="s">
+      <c r="B19" s="38"/>
+      <c r="C19" s="38" t="s">
         <v>231</v>
       </c>
-      <c r="D19" s="46" t="s">
+      <c r="D19" s="39" t="s">
         <v>226</v>
       </c>
-      <c r="E19" s="45" t="n">
+      <c r="E19" s="38" t="n">
         <v>40</v>
       </c>
-      <c r="F19" s="45"/>
-    </row>
-    <row r="20" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="45" t="s">
+      <c r="F19" s="38"/>
+    </row>
+    <row r="20" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="38" t="s">
         <v>151</v>
       </c>
-      <c r="B20" s="45"/>
-      <c r="C20" s="45" t="s">
+      <c r="B20" s="38"/>
+      <c r="C20" s="38" t="s">
         <v>241</v>
       </c>
-      <c r="D20" s="46" t="s">
+      <c r="D20" s="39" t="s">
         <v>225</v>
       </c>
-      <c r="E20" s="45" t="s">
+      <c r="E20" s="38" t="s">
         <v>228</v>
       </c>
-      <c r="F20" s="45"/>
-    </row>
-    <row r="21" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="40" t="s">
+      <c r="F20" s="38"/>
+    </row>
+    <row r="21" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="33" t="s">
         <v>168</v>
       </c>
-      <c r="C21" s="40" t="s">
+      <c r="C21" s="33" t="s">
         <v>242</v>
       </c>
-      <c r="D21" s="46" t="s">
+      <c r="D21" s="39" t="s">
         <v>225</v>
       </c>
-      <c r="E21" s="41" t="s">
+      <c r="E21" s="34" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="40" t="s">
+    <row r="22" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="33" t="s">
         <v>168</v>
       </c>
-      <c r="B22" s="40" t="s">
+      <c r="B22" s="33" t="s">
         <v>229</v>
       </c>
-      <c r="C22" s="40" t="s">
+      <c r="C22" s="33" t="s">
         <v>242</v>
       </c>
-      <c r="D22" s="46" t="s">
+      <c r="D22" s="39" t="s">
         <v>225</v>
       </c>
-      <c r="E22" s="41" t="s">
+      <c r="E22" s="34" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="40" t="s">
+    <row r="23" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="33" t="s">
         <v>168</v>
       </c>
-      <c r="B23" s="40" t="s">
+      <c r="B23" s="33" t="s">
         <v>229</v>
       </c>
-      <c r="C23" s="40" t="s">
+      <c r="C23" s="33" t="s">
         <v>242</v>
       </c>
-      <c r="D23" s="46" t="s">
+      <c r="D23" s="39" t="s">
         <v>225</v>
       </c>
-      <c r="E23" s="41" t="s">
+      <c r="E23" s="34" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="40" t="s">
+    <row r="24" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="33" t="s">
         <v>173</v>
       </c>
-      <c r="C24" s="40" t="s">
+      <c r="C24" s="33" t="s">
         <v>242</v>
       </c>
-      <c r="D24" s="46" t="s">
+      <c r="D24" s="39" t="s">
         <v>225</v>
       </c>
-      <c r="E24" s="41" t="s">
+      <c r="E24" s="34" t="s">
         <v>246</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="40" t="s">
+    <row r="25" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="33" t="s">
         <v>173</v>
       </c>
-      <c r="B25" s="40" t="s">
+      <c r="B25" s="33" t="s">
         <v>229</v>
       </c>
-      <c r="C25" s="40" t="s">
+      <c r="C25" s="33" t="s">
         <v>242</v>
       </c>
-      <c r="D25" s="46" t="s">
+      <c r="D25" s="39" t="s">
         <v>225</v>
       </c>
-      <c r="E25" s="41" t="s">
+      <c r="E25" s="34" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="40" t="s">
+    <row r="26" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="33" t="s">
         <v>173</v>
       </c>
-      <c r="B26" s="40" t="s">
+      <c r="B26" s="33" t="s">
         <v>229</v>
       </c>
-      <c r="C26" s="40" t="s">
+      <c r="C26" s="33" t="s">
         <v>242</v>
       </c>
-      <c r="D26" s="46" t="s">
+      <c r="D26" s="39" t="s">
         <v>225</v>
       </c>
-      <c r="E26" s="41" t="s">
+      <c r="E26" s="34" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="40" t="s">
+    <row r="27" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="33" t="s">
         <v>179</v>
       </c>
-      <c r="C27" s="40" t="s">
+      <c r="C27" s="33" t="s">
         <v>248</v>
       </c>
-      <c r="D27" s="46" t="s">
+      <c r="D27" s="39" t="s">
         <v>225</v>
       </c>
-      <c r="E27" s="40" t="s">
+      <c r="E27" s="33" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="40" t="s">
+    <row r="28" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="33" t="s">
         <v>179</v>
       </c>
-      <c r="B28" s="40" t="s">
+      <c r="B28" s="33" t="s">
         <v>229</v>
       </c>
-      <c r="C28" s="40" t="s">
+      <c r="C28" s="33" t="s">
         <v>248</v>
       </c>
-      <c r="D28" s="46" t="s">
+      <c r="D28" s="39" t="s">
         <v>225</v>
       </c>
-      <c r="E28" s="40" t="s">
+      <c r="E28" s="33" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="40" t="s">
+    <row r="29" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="33" t="s">
         <v>179</v>
       </c>
-      <c r="B29" s="40" t="s">
+      <c r="B29" s="33" t="s">
         <v>229</v>
       </c>
-      <c r="C29" s="40" t="s">
+      <c r="C29" s="33" t="s">
         <v>248</v>
       </c>
-      <c r="D29" s="46" t="s">
+      <c r="D29" s="39" t="s">
         <v>225</v>
       </c>
-      <c r="E29" s="40" t="s">
+      <c r="E29" s="33" t="s">
         <v>251</v>
       </c>
     </row>
@@ -4680,127 +4653,126 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:J4"/>
-  <sheetFormatPr defaultColWidth="10.69921875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.69921875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="45" width="10.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="45" width="12.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="45" width="13.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="45" width="12.57"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="6" min="5" style="45" width="10.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="45" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="45" width="15.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="45" width="15.68"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="45" width="21.93"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="11" style="45" width="10.7"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="38" width="10.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="38" width="12.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="38" width="13.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="38" width="12.57"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="6" min="5" style="38" width="10.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="38" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="38" width="15.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="38" width="15.68"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="38" width="21.93"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="11" style="38" width="10.7"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="47" t="s">
+      <c r="A1" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="48" t="s">
+      <c r="B1" s="41" t="s">
         <v>252</v>
       </c>
-      <c r="C1" s="47" t="s">
+      <c r="C1" s="40" t="s">
         <v>253</v>
       </c>
-      <c r="D1" s="47" t="s">
+      <c r="D1" s="40" t="s">
         <v>254</v>
       </c>
-      <c r="E1" s="47" t="s">
+      <c r="E1" s="40" t="s">
         <v>255</v>
       </c>
-      <c r="F1" s="47" t="s">
+      <c r="F1" s="40" t="s">
         <v>256</v>
       </c>
-      <c r="G1" s="47" t="s">
+      <c r="G1" s="40" t="s">
         <v>257</v>
       </c>
-      <c r="H1" s="47" t="s">
+      <c r="H1" s="40" t="s">
         <v>258</v>
       </c>
-      <c r="I1" s="47" t="s">
+      <c r="I1" s="40" t="s">
         <v>259</v>
       </c>
-      <c r="J1" s="47" t="s">
+      <c r="J1" s="40" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="45" t="s">
+    <row r="2" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="45" t="s">
+      <c r="B2" s="38" t="s">
         <v>261</v>
       </c>
-      <c r="C2" s="45" t="s">
+      <c r="C2" s="38" t="s">
         <v>262</v>
       </c>
-      <c r="D2" s="45" t="s">
+      <c r="D2" s="38" t="s">
         <v>263</v>
       </c>
-      <c r="E2" s="49" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="F2" s="49" t="b">
+      <c r="E2" s="42" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="F2" s="42" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="G2" s="49" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="45" t="s">
+      <c r="G2" s="42" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="38" t="s">
         <v>102</v>
       </c>
-      <c r="B3" s="45" t="s">
+      <c r="B3" s="38" t="s">
         <v>264</v>
       </c>
-      <c r="C3" s="45" t="s">
+      <c r="C3" s="38" t="s">
         <v>265</v>
       </c>
-      <c r="D3" s="45" t="s">
+      <c r="D3" s="38" t="s">
         <v>266</v>
       </c>
-      <c r="E3" s="49" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="F3" s="49" t="b">
+      <c r="E3" s="42" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="F3" s="42" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="G3" s="49" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="I3" s="50"/>
-    </row>
-    <row r="4" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="45" t="s">
+      <c r="G3" s="42" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="38" t="s">
         <v>215</v>
       </c>
-      <c r="B4" s="45" t="s">
+      <c r="B4" s="38" t="s">
         <v>267</v>
       </c>
-      <c r="C4" s="45" t="s">
+      <c r="C4" s="38" t="s">
         <v>268</v>
       </c>
-      <c r="D4" s="45" t="s">
+      <c r="D4" s="38" t="s">
         <v>269</v>
       </c>
-      <c r="E4" s="49" t="b">
+      <c r="E4" s="42" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="F4" s="49" t="b">
+      <c r="F4" s="42" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="G4" s="49" t="b">
+      <c r="G4" s="42" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -4822,62 +4794,62 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H1048576"/>
-  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="51" width="21.3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="51" width="15.72"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="51" width="23.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="51" width="19.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="51" width="21.08"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="51" width="24.29"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="9" style="51" width="9.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="43" width="21.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="43" width="15.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="43" width="23.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="43" width="19.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="43" width="21.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="43" width="24.29"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="9" style="43" width="9.14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="52" t="s">
+      <c r="A1" s="44" t="s">
         <v>270</v>
       </c>
-      <c r="B1" s="52" t="s">
+      <c r="B1" s="44" t="s">
         <v>221</v>
       </c>
-      <c r="C1" s="52" t="s">
+      <c r="C1" s="44" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="52" t="s">
+      <c r="D1" s="44" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="52" t="s">
+      <c r="E1" s="44" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="52" t="s">
+      <c r="F1" s="44" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="52" t="s">
+      <c r="G1" s="44" t="s">
         <v>271</v>
       </c>
-      <c r="H1" s="52" t="s">
+      <c r="H1" s="44" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="B2" s="53" t="s">
+      <c r="B2" s="45" t="s">
         <v>228</v>
       </c>
-      <c r="C2" s="53" t="s">
+      <c r="C2" s="45" t="s">
         <v>272</v>
       </c>
-      <c r="D2" s="53" t="s">
+      <c r="D2" s="45" t="s">
         <v>273</v>
       </c>
-      <c r="E2" s="53"/>
-      <c r="F2" s="53"/>
-      <c r="G2" s="53"/>
-      <c r="H2" s="53"/>
-    </row>
-    <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
+    </row>
+    <row r="3" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
         <v>274</v>
       </c>
@@ -4895,7 +4867,7 @@
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
     </row>
-    <row r="4" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
         <v>136</v>
       </c>
@@ -4913,7 +4885,7 @@
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
     </row>
-    <row r="5" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
         <v>279</v>
       </c>
@@ -4931,7 +4903,7 @@
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
     </row>
-    <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
         <v>282</v>
       </c>
@@ -4949,7 +4921,7 @@
       <c r="G6" s="1"/>
       <c r="H6" s="1"/>
     </row>
-    <row r="7" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
         <v>285</v>
       </c>
@@ -4967,7 +4939,7 @@
       <c r="G7" s="1"/>
       <c r="H7" s="1"/>
     </row>
-    <row r="8" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
         <v>33</v>
       </c>
@@ -4981,7 +4953,7 @@
       </c>
       <c r="H8" s="1"/>
     </row>
-    <row r="9" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
         <v>33</v>
       </c>
@@ -4995,7 +4967,7 @@
       </c>
       <c r="H9" s="1"/>
     </row>
-    <row r="10" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
         <v>146</v>
       </c>
@@ -5009,7 +4981,7 @@
       </c>
       <c r="H10" s="1"/>
     </row>
-    <row r="11" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
         <v>146</v>
       </c>
@@ -5023,7 +4995,7 @@
       </c>
       <c r="H11" s="1"/>
     </row>
-    <row r="12" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
         <v>96</v>
       </c>
@@ -5037,7 +5009,7 @@
       </c>
       <c r="H12" s="1"/>
     </row>
-    <row r="13" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
         <v>96</v>
       </c>
@@ -5051,7 +5023,7 @@
       </c>
       <c r="H13" s="1"/>
     </row>
-    <row r="14" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
         <v>96</v>
       </c>
@@ -5065,7 +5037,7 @@
       </c>
       <c r="H14" s="1"/>
     </row>
-    <row r="15" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
         <v>116</v>
       </c>
@@ -5083,7 +5055,7 @@
       <c r="G15" s="1"/>
       <c r="H15" s="1"/>
     </row>
-    <row r="16" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
         <v>116</v>
       </c>
@@ -5101,7 +5073,7 @@
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
     </row>
-    <row r="17" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
         <v>116</v>
       </c>
@@ -5115,7 +5087,7 @@
       </c>
       <c r="H17" s="1"/>
     </row>
-    <row r="18" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
         <v>125</v>
       </c>
@@ -5133,7 +5105,7 @@
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
     </row>
-    <row r="19" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
         <v>125</v>
       </c>
@@ -5151,7 +5123,7 @@
       <c r="G19" s="1"/>
       <c r="H19" s="1"/>
     </row>
-    <row r="20" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
         <v>125</v>
       </c>
@@ -5165,7 +5137,7 @@
       </c>
       <c r="H20" s="1"/>
     </row>
-    <row r="21" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
         <v>132</v>
       </c>
@@ -5185,7 +5157,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
         <v>132</v>
       </c>
@@ -5205,7 +5177,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
         <v>132</v>
       </c>
@@ -5225,7 +5197,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
         <v>132</v>
       </c>
@@ -5243,7 +5215,7 @@
       <c r="G24" s="1"/>
       <c r="H24" s="1"/>
     </row>
-    <row r="25" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
         <v>132</v>
       </c>
@@ -5263,7 +5235,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
         <v>132</v>
       </c>
@@ -5277,7 +5249,7 @@
       </c>
       <c r="H26" s="1"/>
     </row>
-    <row r="27" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
         <v>137</v>
       </c>
@@ -5295,7 +5267,7 @@
       <c r="G27" s="1"/>
       <c r="H27" s="1"/>
     </row>
-    <row r="28" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
         <v>137</v>
       </c>
@@ -5313,7 +5285,7 @@
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
     </row>
-    <row r="29" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
         <v>137</v>
       </c>
@@ -5331,7 +5303,7 @@
       <c r="G29" s="1"/>
       <c r="H29" s="1"/>
     </row>
-    <row r="30" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
         <v>137</v>
       </c>
@@ -5349,7 +5321,7 @@
       <c r="G30" s="1"/>
       <c r="H30" s="1"/>
     </row>
-    <row r="31" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
         <v>137</v>
       </c>
@@ -5367,7 +5339,7 @@
       <c r="G31" s="1"/>
       <c r="H31" s="1"/>
     </row>
-    <row r="32" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
         <v>137</v>
       </c>
@@ -5387,7 +5359,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
         <v>137</v>
       </c>
@@ -5405,7 +5377,7 @@
       <c r="G33" s="1"/>
       <c r="H33" s="1"/>
     </row>
-    <row r="34" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
         <v>137</v>
       </c>
@@ -5423,7 +5395,7 @@
       <c r="G34" s="1"/>
       <c r="H34" s="1"/>
     </row>
-    <row r="35" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
         <v>137</v>
       </c>
@@ -5441,7 +5413,7 @@
       <c r="G35" s="1"/>
       <c r="H35" s="1"/>
     </row>
-    <row r="36" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
         <v>137</v>
       </c>
@@ -5459,7 +5431,7 @@
       <c r="G36" s="1"/>
       <c r="H36" s="1"/>
     </row>
-    <row r="37" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
         <v>137</v>
       </c>
@@ -5477,7 +5449,7 @@
       <c r="G37" s="1"/>
       <c r="H37" s="1"/>
     </row>
-    <row r="38" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
         <v>137</v>
       </c>
@@ -5495,7 +5467,7 @@
       <c r="G38" s="1"/>
       <c r="H38" s="1"/>
     </row>
-    <row r="39" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
         <v>137</v>
       </c>
@@ -5513,7 +5485,7 @@
       <c r="G39" s="1"/>
       <c r="H39" s="1"/>
     </row>
-    <row r="40" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
         <v>158</v>
       </c>
@@ -5527,7 +5499,7 @@
       </c>
       <c r="H40" s="1"/>
     </row>
-    <row r="41" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
         <v>158</v>
       </c>
@@ -5545,7 +5517,7 @@
       <c r="G41" s="1"/>
       <c r="H41" s="1"/>
     </row>
-    <row r="42" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
         <v>158</v>
       </c>
@@ -5563,7 +5535,7 @@
       <c r="G42" s="1"/>
       <c r="H42" s="1"/>
     </row>
-    <row r="43" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
         <v>158</v>
       </c>
@@ -5577,7 +5549,7 @@
       </c>
       <c r="H43" s="1"/>
     </row>
-    <row r="44" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
         <v>165</v>
       </c>
@@ -5595,7 +5567,7 @@
       <c r="G44" s="1"/>
       <c r="H44" s="1"/>
     </row>
-    <row r="45" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
         <v>165</v>
       </c>
@@ -5613,7 +5585,7 @@
       <c r="G45" s="1"/>
       <c r="H45" s="1"/>
     </row>
-    <row r="46" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="73.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
         <v>165</v>
       </c>
@@ -5631,7 +5603,7 @@
       <c r="G46" s="1"/>
       <c r="H46" s="1"/>
     </row>
-    <row r="47" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
         <v>165</v>
       </c>
@@ -5649,7 +5621,7 @@
       <c r="G47" s="1"/>
       <c r="H47" s="1"/>
     </row>
-    <row r="48" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
         <v>165</v>
       </c>
@@ -5667,45 +5639,45 @@
       <c r="G48" s="1"/>
       <c r="H48" s="1"/>
     </row>
-    <row r="49" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="51" t="s">
+    <row r="49" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="43" t="s">
         <v>174</v>
       </c>
-      <c r="B49" s="51" t="s">
+      <c r="B49" s="43" t="s">
         <v>249</v>
       </c>
-      <c r="C49" s="51" t="s">
+      <c r="C49" s="43" t="s">
         <v>364</v>
       </c>
-      <c r="D49" s="51" t="s">
+      <c r="D49" s="43" t="s">
         <v>353</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="51" t="s">
+    <row r="50" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="43" t="s">
         <v>174</v>
       </c>
-      <c r="B50" s="51" t="s">
+      <c r="B50" s="43" t="s">
         <v>250</v>
       </c>
-      <c r="C50" s="51" t="s">
+      <c r="C50" s="43" t="s">
         <v>365</v>
       </c>
-      <c r="D50" s="51" t="s">
+      <c r="D50" s="43" t="s">
         <v>366</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="51" t="s">
+    <row r="51" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="43" t="s">
         <v>174</v>
       </c>
-      <c r="B51" s="51" t="s">
+      <c r="B51" s="43" t="s">
         <v>361</v>
       </c>
-      <c r="C51" s="51" t="s">
+      <c r="C51" s="43" t="s">
         <v>367</v>
       </c>
-      <c r="D51" s="51" t="s">
+      <c r="D51" s="43" t="s">
         <v>368</v>
       </c>
     </row>
@@ -5727,55 +5699,55 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L1"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="40" width="18.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="40" width="17.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="40" width="13.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="40" width="12.72"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="40" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="40" width="13.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="40" width="14.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="40" width="11.28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="40" width="13.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="40" width="14.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="33" width="18.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="33" width="17.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="33" width="13.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="33" width="12.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="33" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="33" width="13.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="33" width="14.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="33" width="11.28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="33" width="13.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="33" width="14.43"/>
   </cols>
   <sheetData>
-    <row r="1" s="52" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="54" t="s">
+    <row r="1" s="44" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="46" t="s">
         <v>369</v>
       </c>
-      <c r="B1" s="54" t="s">
+      <c r="B1" s="46" t="s">
         <v>370</v>
       </c>
-      <c r="C1" s="54" t="s">
+      <c r="C1" s="46" t="s">
         <v>371</v>
       </c>
-      <c r="D1" s="54" t="s">
+      <c r="D1" s="46" t="s">
         <v>372</v>
       </c>
-      <c r="E1" s="54" t="s">
+      <c r="E1" s="46" t="s">
         <v>373</v>
       </c>
-      <c r="F1" s="54" t="s">
+      <c r="F1" s="46" t="s">
         <v>374</v>
       </c>
-      <c r="G1" s="54" t="s">
+      <c r="G1" s="46" t="s">
         <v>375</v>
       </c>
-      <c r="H1" s="54" t="s">
+      <c r="H1" s="46" t="s">
         <v>376</v>
       </c>
-      <c r="I1" s="54" t="s">
+      <c r="I1" s="46" t="s">
         <v>377</v>
       </c>
-      <c r="J1" s="54" t="s">
+      <c r="J1" s="46" t="s">
         <v>378</v>
       </c>
-      <c r="K1" s="54" t="s">
+      <c r="K1" s="46" t="s">
         <v>379</v>
       </c>
-      <c r="L1" s="52" t="s">
+      <c r="L1" s="44" t="s">
         <v>380</v>
       </c>
     </row>
@@ -5796,21 +5768,21 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G3"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="40" width="10.34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="40" width="32.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="40" width="43.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="40" width="46.08"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="40" width="28.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="33" width="10.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="33" width="32.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="33" width="43.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="33" width="46.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="33" width="28.55"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>3</v>
+        <v>381</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>5</v>
+        <v>382</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>6</v>
@@ -5824,39 +5796,39 @@
       <c r="F1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="40"/>
+      <c r="G1" s="33"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="55" t="s">
+      <c r="A2" s="47" t="s">
         <v>102</v>
       </c>
-      <c r="B2" s="45" t="s">
-        <v>381</v>
-      </c>
-      <c r="C2" s="55" t="s">
-        <v>382</v>
-      </c>
-      <c r="D2" s="55" t="s">
+      <c r="B2" s="38" t="s">
         <v>383</v>
       </c>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
+      <c r="C2" s="47" t="s">
+        <v>384</v>
+      </c>
+      <c r="D2" s="47" t="s">
+        <v>385</v>
+      </c>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="55" t="s">
+      <c r="A3" s="47" t="s">
         <v>102</v>
       </c>
-      <c r="B3" s="45" t="s">
-        <v>384</v>
-      </c>
-      <c r="C3" s="55" t="s">
-        <v>385</v>
-      </c>
-      <c r="D3" s="55" t="s">
+      <c r="B3" s="38" t="s">
         <v>386</v>
       </c>
-      <c r="E3" s="55"/>
-      <c r="F3" s="55"/>
+      <c r="C3" s="47" t="s">
+        <v>387</v>
+      </c>
+      <c r="D3" s="47" t="s">
+        <v>388</v>
+      </c>
+      <c r="E3" s="47"/>
+      <c r="F3" s="47"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Generator: Add section configuration generation with custom conditionals
Fixes: #997
- Updated SectionConfig to support WidgetConditional for enableConditional and completionConditional properties.
- Add the new columns in the demo-generator Excel file.
</commit_message>
<xml_diff>
--- a/example/demo_generator/references/Household_Travel_Generate_Survey.xlsx
+++ b/example/demo_generator/references/Household_Travel_Generate_Survey.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Widgets" sheetId="1" state="visible" r:id="rId3"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="682" uniqueCount="385">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="684" uniqueCount="387">
   <si>
     <t xml:space="preserve">questionName</t>
   </si>
@@ -861,6 +861,12 @@
   </si>
   <si>
     <t xml:space="preserve">parent_section</t>
+  </si>
+  <si>
+    <t xml:space="preserve">enable_conditional</t>
+  </si>
+  <si>
+    <t xml:space="preserve">completion_conditional</t>
   </si>
   <si>
     <t xml:space="preserve">h_</t>
@@ -1488,7 +1494,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="56">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1686,6 +1692,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2578,7 +2588,7 @@
       </c>
       <c r="X10" s="7"/>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
         <v>64</v>
       </c>
@@ -2712,7 +2722,7 @@
       <c r="Q13" s="7"/>
       <c r="R13" s="7"/>
       <c r="S13" s="7"/>
-      <c r="T13" s="7" t="b">
+      <c r="T13" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2763,7 +2773,7 @@
       <c r="Q14" s="7"/>
       <c r="R14" s="7"/>
       <c r="S14" s="7"/>
-      <c r="T14" s="7" t="b">
+      <c r="T14" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2812,7 +2822,7 @@
       <c r="Q15" s="7"/>
       <c r="R15" s="7"/>
       <c r="S15" s="7"/>
-      <c r="T15" s="7" t="b">
+      <c r="T15" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2908,7 +2918,7 @@
       <c r="Q17" s="7"/>
       <c r="R17" s="7"/>
       <c r="S17" s="7"/>
-      <c r="T17" s="7" t="b">
+      <c r="T17" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -3039,7 +3049,7 @@
       <c r="Q20" s="24"/>
       <c r="R20" s="24"/>
       <c r="S20" s="24"/>
-      <c r="T20" s="23" t="b">
+      <c r="T20" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -4669,7 +4679,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr defaultColWidth="10.69921875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="45" width="10.7"/>
@@ -4679,7 +4689,9 @@
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="6" min="5" style="45" width="10.7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="45" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="45" width="15.43"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="9" style="45" width="10.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="45" width="15.68"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="45" width="21.93"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="11" style="45" width="10.7"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4701,25 +4713,31 @@
       <c r="F1" s="47" t="s">
         <v>256</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="47" t="s">
         <v>257</v>
       </c>
       <c r="H1" s="47" t="s">
         <v>258</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1" s="47" t="s">
+        <v>259</v>
+      </c>
+      <c r="J1" s="47" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="45" t="s">
         <v>26</v>
       </c>
       <c r="B2" s="45" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="C2" s="45" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="D2" s="45" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="E2" s="49" t="b">
         <f aca="false">TRUE()</f>
@@ -4734,18 +4752,18 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="45" t="s">
         <v>102</v>
       </c>
       <c r="B3" s="45" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="C3" s="45" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="D3" s="45" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="E3" s="49" t="b">
         <f aca="false">TRUE()</f>
@@ -4759,19 +4777,20 @@
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
+      <c r="I3" s="50"/>
     </row>
     <row r="4" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="45" t="s">
         <v>215</v>
       </c>
       <c r="B4" s="45" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="C4" s="45" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="D4" s="45" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="E4" s="49" t="b">
         <f aca="false">FALSE()</f>
@@ -4805,38 +4824,38 @@
   <dimension ref="A1:H1048576"/>
   <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="50" width="21.3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="50" width="15.72"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="50" width="23.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="50" width="19.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="50" width="21.08"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="50" width="24.29"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="9" style="50" width="9.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="51" width="21.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="51" width="15.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="51" width="23.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="51" width="19.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="51" width="21.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="51" width="24.29"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="9" style="51" width="9.14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="51" t="s">
-        <v>268</v>
-      </c>
-      <c r="B1" s="51" t="s">
+      <c r="A1" s="52" t="s">
+        <v>270</v>
+      </c>
+      <c r="B1" s="52" t="s">
         <v>221</v>
       </c>
-      <c r="C1" s="51" t="s">
+      <c r="C1" s="52" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="51" t="s">
+      <c r="D1" s="52" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="51" t="s">
+      <c r="E1" s="52" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="51" t="s">
+      <c r="F1" s="52" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="51" t="s">
-        <v>269</v>
-      </c>
-      <c r="H1" s="51" t="s">
+      <c r="G1" s="52" t="s">
+        <v>271</v>
+      </c>
+      <c r="H1" s="52" t="s">
         <v>12</v>
       </c>
     </row>
@@ -4844,32 +4863,32 @@
       <c r="A2" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="B2" s="52" t="s">
+      <c r="B2" s="53" t="s">
         <v>228</v>
       </c>
-      <c r="C2" s="52" t="s">
-        <v>270</v>
-      </c>
-      <c r="D2" s="52" t="s">
-        <v>271</v>
-      </c>
-      <c r="E2" s="52"/>
-      <c r="F2" s="52"/>
-      <c r="G2" s="52"/>
-      <c r="H2" s="52"/>
+      <c r="C2" s="53" t="s">
+        <v>272</v>
+      </c>
+      <c r="D2" s="53" t="s">
+        <v>273</v>
+      </c>
+      <c r="E2" s="53"/>
+      <c r="F2" s="53"/>
+      <c r="G2" s="53"/>
+      <c r="H2" s="53"/>
     </row>
     <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
@@ -4884,10 +4903,10 @@
         <v>136</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
@@ -4896,16 +4915,16 @@
     </row>
     <row r="5" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>136</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
@@ -4914,16 +4933,16 @@
     </row>
     <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
@@ -4932,16 +4951,16 @@
     </row>
     <row r="7" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
@@ -4972,7 +4991,7 @@
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
       <c r="G9" s="1" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="H9" s="1"/>
     </row>
@@ -5000,7 +5019,7 @@
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
       <c r="G11" s="1" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="H11" s="1"/>
     </row>
@@ -5028,7 +5047,7 @@
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
       <c r="G13" s="1" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="H13" s="1"/>
     </row>
@@ -5042,7 +5061,7 @@
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
       <c r="G14" s="1" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="H14" s="1"/>
     </row>
@@ -5051,13 +5070,13 @@
         <v>116</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
@@ -5069,13 +5088,13 @@
         <v>116</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
@@ -5092,7 +5111,7 @@
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
       <c r="G17" s="1" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="H17" s="1"/>
     </row>
@@ -5101,13 +5120,13 @@
         <v>125</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
@@ -5119,13 +5138,13 @@
         <v>125</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="E19" s="1"/>
       <c r="F19" s="1"/>
@@ -5142,7 +5161,7 @@
       <c r="E20" s="1"/>
       <c r="F20" s="1"/>
       <c r="G20" s="1" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="H20" s="1"/>
     </row>
@@ -5151,13 +5170,13 @@
         <v>132</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="E21" s="1"/>
       <c r="F21" s="1"/>
@@ -5171,13 +5190,13 @@
         <v>132</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="E22" s="1"/>
       <c r="F22" s="1"/>
@@ -5191,13 +5210,13 @@
         <v>132</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E23" s="1"/>
       <c r="F23" s="1"/>
@@ -5211,13 +5230,13 @@
         <v>132</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="E24" s="1"/>
       <c r="F24" s="1"/>
@@ -5229,13 +5248,13 @@
         <v>132</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="E25" s="1"/>
       <c r="F25" s="1"/>
@@ -5266,10 +5285,10 @@
         <v>243</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
@@ -5284,10 +5303,10 @@
         <v>244</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="E28" s="1"/>
       <c r="F28" s="1"/>
@@ -5302,10 +5321,10 @@
         <v>245</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="E29" s="1"/>
       <c r="F29" s="1"/>
@@ -5320,10 +5339,10 @@
         <v>246</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="E30" s="1"/>
       <c r="F30" s="1"/>
@@ -5338,10 +5357,10 @@
         <v>247</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="E31" s="1"/>
       <c r="F31" s="1"/>
@@ -5353,13 +5372,13 @@
         <v>137</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="E32" s="1"/>
       <c r="F32" s="1"/>
@@ -5373,13 +5392,13 @@
         <v>137</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="E33" s="1"/>
       <c r="F33" s="1"/>
@@ -5391,13 +5410,13 @@
         <v>137</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="E34" s="1"/>
       <c r="F34" s="1"/>
@@ -5409,13 +5428,13 @@
         <v>137</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="E35" s="1"/>
       <c r="F35" s="1"/>
@@ -5427,13 +5446,13 @@
         <v>137</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="E36" s="1"/>
       <c r="F36" s="1"/>
@@ -5445,13 +5464,13 @@
         <v>137</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="E37" s="1"/>
       <c r="F37" s="1"/>
@@ -5466,10 +5485,10 @@
         <v>136</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="E38" s="1"/>
       <c r="F38" s="1"/>
@@ -5481,13 +5500,13 @@
         <v>137</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="E39" s="1"/>
       <c r="F39" s="1"/>
@@ -5504,7 +5523,7 @@
       <c r="E40" s="1"/>
       <c r="F40" s="1"/>
       <c r="G40" s="1" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="H40" s="1"/>
     </row>
@@ -5513,13 +5532,13 @@
         <v>158</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="E41" s="1"/>
       <c r="F41" s="1"/>
@@ -5531,13 +5550,13 @@
         <v>158</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="E42" s="1"/>
       <c r="F42" s="1"/>
@@ -5554,7 +5573,7 @@
       <c r="E43" s="1"/>
       <c r="F43" s="1"/>
       <c r="G43" s="1" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="H43" s="1"/>
     </row>
@@ -5566,10 +5585,10 @@
         <v>249</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="E44" s="1"/>
       <c r="F44" s="1"/>
@@ -5584,10 +5603,10 @@
         <v>250</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="E45" s="1"/>
       <c r="F45" s="1"/>
@@ -5602,10 +5621,10 @@
         <v>251</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="E46" s="1"/>
       <c r="F46" s="1"/>
@@ -5617,13 +5636,13 @@
         <v>165</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="E47" s="1"/>
       <c r="F47" s="1"/>
@@ -5635,13 +5654,13 @@
         <v>165</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="E48" s="1"/>
       <c r="F48" s="1"/>
@@ -5649,45 +5668,45 @@
       <c r="H48" s="1"/>
     </row>
     <row r="49" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="50" t="s">
+      <c r="A49" s="51" t="s">
         <v>174</v>
       </c>
-      <c r="B49" s="50" t="s">
+      <c r="B49" s="51" t="s">
         <v>249</v>
       </c>
-      <c r="C49" s="50" t="s">
-        <v>362</v>
-      </c>
-      <c r="D49" s="50" t="s">
-        <v>351</v>
+      <c r="C49" s="51" t="s">
+        <v>364</v>
+      </c>
+      <c r="D49" s="51" t="s">
+        <v>353</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="50" t="s">
+      <c r="A50" s="51" t="s">
         <v>174</v>
       </c>
-      <c r="B50" s="50" t="s">
+      <c r="B50" s="51" t="s">
         <v>250</v>
       </c>
-      <c r="C50" s="50" t="s">
-        <v>363</v>
-      </c>
-      <c r="D50" s="50" t="s">
-        <v>364</v>
+      <c r="C50" s="51" t="s">
+        <v>365</v>
+      </c>
+      <c r="D50" s="51" t="s">
+        <v>366</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="50" t="s">
+      <c r="A51" s="51" t="s">
         <v>174</v>
       </c>
-      <c r="B51" s="50" t="s">
-        <v>359</v>
-      </c>
-      <c r="C51" s="50" t="s">
-        <v>365</v>
-      </c>
-      <c r="D51" s="50" t="s">
-        <v>366</v>
+      <c r="B51" s="51" t="s">
+        <v>361</v>
+      </c>
+      <c r="C51" s="51" t="s">
+        <v>367</v>
+      </c>
+      <c r="D51" s="51" t="s">
+        <v>368</v>
       </c>
     </row>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -5722,42 +5741,42 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="40" width="14.43"/>
   </cols>
   <sheetData>
-    <row r="1" s="51" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="53" t="s">
-        <v>367</v>
-      </c>
-      <c r="B1" s="53" t="s">
-        <v>368</v>
-      </c>
-      <c r="C1" s="53" t="s">
+    <row r="1" s="52" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="54" t="s">
         <v>369</v>
       </c>
-      <c r="D1" s="53" t="s">
+      <c r="B1" s="54" t="s">
         <v>370</v>
       </c>
-      <c r="E1" s="53" t="s">
+      <c r="C1" s="54" t="s">
         <v>371</v>
       </c>
-      <c r="F1" s="53" t="s">
+      <c r="D1" s="54" t="s">
         <v>372</v>
       </c>
-      <c r="G1" s="53" t="s">
+      <c r="E1" s="54" t="s">
         <v>373</v>
       </c>
-      <c r="H1" s="53" t="s">
+      <c r="F1" s="54" t="s">
         <v>374</v>
       </c>
-      <c r="I1" s="53" t="s">
+      <c r="G1" s="54" t="s">
         <v>375</v>
       </c>
-      <c r="J1" s="53" t="s">
+      <c r="H1" s="54" t="s">
         <v>376</v>
       </c>
-      <c r="K1" s="53" t="s">
+      <c r="I1" s="54" t="s">
         <v>377</v>
       </c>
-      <c r="L1" s="51" t="s">
+      <c r="J1" s="54" t="s">
         <v>378</v>
+      </c>
+      <c r="K1" s="54" t="s">
+        <v>379</v>
+      </c>
+      <c r="L1" s="52" t="s">
+        <v>380</v>
       </c>
     </row>
   </sheetData>
@@ -5808,36 +5827,36 @@
       <c r="G1" s="40"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="54" t="s">
+      <c r="A2" s="55" t="s">
         <v>102</v>
       </c>
       <c r="B2" s="45" t="s">
-        <v>379</v>
-      </c>
-      <c r="C2" s="54" t="s">
-        <v>380</v>
-      </c>
-      <c r="D2" s="54" t="s">
         <v>381</v>
       </c>
-      <c r="E2" s="54"/>
-      <c r="F2" s="54"/>
+      <c r="C2" s="55" t="s">
+        <v>382</v>
+      </c>
+      <c r="D2" s="55" t="s">
+        <v>383</v>
+      </c>
+      <c r="E2" s="55"/>
+      <c r="F2" s="55"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="54" t="s">
+      <c r="A3" s="55" t="s">
         <v>102</v>
       </c>
       <c r="B3" s="45" t="s">
-        <v>382</v>
-      </c>
-      <c r="C3" s="54" t="s">
-        <v>383</v>
-      </c>
-      <c r="D3" s="54" t="s">
         <v>384</v>
       </c>
-      <c r="E3" s="54"/>
-      <c r="F3" s="54"/>
+      <c r="C3" s="55" t="s">
+        <v>385</v>
+      </c>
+      <c r="D3" s="55" t="s">
+        <v>386</v>
+      </c>
+      <c r="E3" s="55"/>
+      <c r="F3" s="55"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Generator: Copy Excel to CSV for improved version control
Fix: #1580
- Added functionality to copy each sheet of the Generator Excel file to a separate CSV file, facilitating easier review of changes in git diffs.
- Updated `generatorConfigs.yaml` to enable this feature with `copy_excel_to_csv: true`.
- Introduced a new script `excel_to_csv_generator.py` to handle the conversion process.
</commit_message>
<xml_diff>
--- a/example/demo_generator/references/Household_Travel_Generate_Survey.xlsx
+++ b/example/demo_generator/references/Household_Travel_Generate_Survey.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Widgets" sheetId="1" state="visible" r:id="rId3"/>
@@ -1257,9 +1257,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="@"/>
+    <numFmt numFmtId="165" formatCode="General"/>
+    <numFmt numFmtId="166" formatCode="@"/>
   </numFmts>
   <fonts count="20">
     <font>
@@ -1499,7 +1500,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="55">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1532,6 +1533,10 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1552,11 +1557,19 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1568,11 +1581,19 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1620,7 +1641,15 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1636,7 +1665,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1644,7 +1673,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1656,7 +1685,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1668,7 +1697,7 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2041,7 +2070,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:X42"/>
-  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="19.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.86"/>
@@ -2142,14 +2171,14 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="26.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
         <v>24</v>
       </c>
       <c r="B2" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C2" s="7" t="b">
+      <c r="C2" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2171,13 +2200,13 @@
       <c r="K2" s="7"/>
       <c r="L2" s="7"/>
       <c r="M2" s="7"/>
-      <c r="N2" s="8"/>
+      <c r="N2" s="9"/>
       <c r="O2" s="7"/>
       <c r="P2" s="7"/>
       <c r="Q2" s="7"/>
       <c r="R2" s="7"/>
       <c r="S2" s="7"/>
-      <c r="T2" s="7" t="b">
+      <c r="T2" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2186,14 +2215,14 @@
       <c r="W2" s="7"/>
       <c r="X2" s="7"/>
     </row>
-    <row r="3" customFormat="false" ht="51.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
         <v>29</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="C3" s="7" t="b">
+      <c r="C3" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2213,8 +2242,8 @@
       <c r="I3" s="7"/>
       <c r="J3" s="7"/>
       <c r="K3" s="7"/>
-      <c r="M3" s="8"/>
-      <c r="N3" s="8"/>
+      <c r="M3" s="9"/>
+      <c r="N3" s="9"/>
       <c r="O3" s="7" t="s">
         <v>33</v>
       </c>
@@ -2222,7 +2251,7 @@
       <c r="Q3" s="7"/>
       <c r="R3" s="7"/>
       <c r="S3" s="7"/>
-      <c r="T3" s="7" t="b">
+      <c r="T3" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2231,14 +2260,14 @@
       <c r="W3" s="7"/>
       <c r="X3" s="7"/>
     </row>
-    <row r="4" customFormat="false" ht="26.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
         <v>34</v>
       </c>
       <c r="B4" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="C4" s="7" t="b">
+      <c r="C4" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2259,7 +2288,7 @@
       <c r="J4" s="7"/>
       <c r="K4" s="7"/>
       <c r="L4" s="7"/>
-      <c r="M4" s="8"/>
+      <c r="M4" s="9"/>
       <c r="N4" s="7"/>
       <c r="O4" s="7" t="s">
         <v>38</v>
@@ -2268,7 +2297,7 @@
       <c r="Q4" s="7"/>
       <c r="R4" s="7"/>
       <c r="S4" s="7"/>
-      <c r="T4" s="7" t="b">
+      <c r="T4" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2284,7 +2313,7 @@
       <c r="B5" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C5" s="7" t="b">
+      <c r="C5" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2305,7 +2334,7 @@
       <c r="J5" s="7"/>
       <c r="K5" s="7"/>
       <c r="L5" s="7"/>
-      <c r="M5" s="8"/>
+      <c r="M5" s="9"/>
       <c r="N5" s="7" t="s">
         <v>42</v>
       </c>
@@ -2314,7 +2343,7 @@
       <c r="Q5" s="7"/>
       <c r="R5" s="7"/>
       <c r="S5" s="7"/>
-      <c r="T5" s="7" t="b">
+      <c r="T5" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2323,14 +2352,14 @@
       <c r="W5" s="7"/>
       <c r="X5" s="7"/>
     </row>
-    <row r="6" customFormat="false" ht="26.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
         <v>43</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C6" s="7" t="b">
+      <c r="C6" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2353,7 +2382,7 @@
       <c r="L6" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="M6" s="8"/>
+      <c r="M6" s="9"/>
       <c r="N6" s="7" t="s">
         <v>47</v>
       </c>
@@ -2362,7 +2391,7 @@
       <c r="Q6" s="7"/>
       <c r="R6" s="7"/>
       <c r="S6" s="7"/>
-      <c r="T6" s="7" t="b">
+      <c r="T6" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2378,7 +2407,7 @@
       <c r="B7" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="7" t="b">
+      <c r="C7" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2407,7 +2436,7 @@
       <c r="Q7" s="7"/>
       <c r="R7" s="7"/>
       <c r="S7" s="7"/>
-      <c r="T7" s="7" t="b">
+      <c r="T7" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2423,7 +2452,7 @@
       <c r="B8" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C8" s="7" t="b">
+      <c r="C8" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2454,7 +2483,7 @@
       <c r="Q8" s="7"/>
       <c r="R8" s="7"/>
       <c r="S8" s="7"/>
-      <c r="T8" s="7" t="b">
+      <c r="T8" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2463,14 +2492,14 @@
       <c r="W8" s="7"/>
       <c r="X8" s="7"/>
     </row>
-    <row r="9" customFormat="false" ht="26.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
         <v>55</v>
       </c>
       <c r="B9" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="7" t="b">
+      <c r="C9" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2501,7 +2530,7 @@
       <c r="Q9" s="7"/>
       <c r="R9" s="7"/>
       <c r="S9" s="7"/>
-      <c r="T9" s="7" t="b">
+      <c r="T9" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2512,14 +2541,14 @@
       </c>
       <c r="X9" s="7"/>
     </row>
-    <row r="10" customFormat="false" ht="26.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
         <v>59</v>
       </c>
       <c r="B10" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C10" s="7" t="b">
+      <c r="C10" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2550,7 +2579,7 @@
       <c r="Q10" s="7"/>
       <c r="R10" s="7"/>
       <c r="S10" s="7"/>
-      <c r="T10" s="7" t="b">
+      <c r="T10" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2561,14 +2590,14 @@
       </c>
       <c r="X10" s="7"/>
     </row>
-    <row r="11" customFormat="false" ht="26.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
         <v>64</v>
       </c>
       <c r="B11" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C11" s="7" t="b">
+      <c r="C11" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2599,7 +2628,7 @@
       <c r="Q11" s="7"/>
       <c r="R11" s="7"/>
       <c r="S11" s="7"/>
-      <c r="T11" s="7" t="b">
+      <c r="T11" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2609,13 +2638,13 @@
       <c r="X11" s="7"/>
     </row>
     <row r="12" customFormat="false" ht="117.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="9" t="s">
+      <c r="A12" s="10" t="s">
         <v>68</v>
       </c>
       <c r="B12" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="C12" s="7" t="b">
+      <c r="C12" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2637,14 +2666,14 @@
       <c r="J12" s="7"/>
       <c r="K12" s="7"/>
       <c r="L12" s="7"/>
-      <c r="M12" s="10"/>
+      <c r="M12" s="11"/>
       <c r="N12" s="7"/>
       <c r="O12" s="7"/>
       <c r="P12" s="7"/>
       <c r="Q12" s="7"/>
       <c r="R12" s="7"/>
       <c r="S12" s="7"/>
-      <c r="T12" s="7" t="b">
+      <c r="T12" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2660,7 +2689,7 @@
       <c r="B13" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="C13" s="7" t="b">
+      <c r="C13" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2695,7 +2724,7 @@
       <c r="Q13" s="7"/>
       <c r="R13" s="7"/>
       <c r="S13" s="7"/>
-      <c r="T13" s="7" t="b">
+      <c r="T13" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2711,7 +2740,7 @@
       <c r="B14" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="C14" s="7" t="b">
+      <c r="C14" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2746,7 +2775,7 @@
       <c r="Q14" s="7"/>
       <c r="R14" s="7"/>
       <c r="S14" s="7"/>
-      <c r="T14" s="7" t="b">
+      <c r="T14" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2762,7 +2791,7 @@
       <c r="B15" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="C15" s="7" t="b">
+      <c r="C15" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2795,7 +2824,7 @@
       <c r="Q15" s="7"/>
       <c r="R15" s="7"/>
       <c r="S15" s="7"/>
-      <c r="T15" s="7" t="b">
+      <c r="T15" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2804,14 +2833,14 @@
       <c r="W15" s="7"/>
       <c r="X15" s="7"/>
     </row>
-    <row r="16" customFormat="false" ht="39.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
         <v>89</v>
       </c>
       <c r="B16" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="C16" s="7" t="b">
+      <c r="C16" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2835,14 +2864,14 @@
         <v>82</v>
       </c>
       <c r="L16" s="7"/>
-      <c r="M16" s="8"/>
-      <c r="N16" s="8"/>
+      <c r="M16" s="9"/>
+      <c r="N16" s="9"/>
       <c r="O16" s="7"/>
       <c r="P16" s="7"/>
       <c r="Q16" s="7"/>
       <c r="R16" s="7"/>
       <c r="S16" s="7"/>
-      <c r="T16" s="7" t="b">
+      <c r="T16" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2851,14 +2880,14 @@
       <c r="W16" s="7"/>
       <c r="X16" s="7"/>
     </row>
-    <row r="17" s="11" customFormat="true" ht="76.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="17" s="12" customFormat="true" ht="76.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
         <v>92</v>
       </c>
       <c r="B17" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="C17" s="7" t="b">
+      <c r="C17" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2891,7 +2920,7 @@
       <c r="Q17" s="7"/>
       <c r="R17" s="7"/>
       <c r="S17" s="7"/>
-      <c r="T17" s="7" t="b">
+      <c r="T17" s="8" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2901,33 +2930,33 @@
       <c r="X17" s="7"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="12" t="s">
+      <c r="A18" s="13" t="s">
         <v>97</v>
       </c>
-      <c r="B18" s="12" t="s">
+      <c r="B18" s="13" t="s">
         <v>98</v>
       </c>
-      <c r="C18" s="12" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D18" s="13" t="s">
+      <c r="C18" s="14" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D18" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E18" s="7"/>
-      <c r="F18" s="14" t="str">
+      <c r="F18" s="16" t="str">
         <f aca="false">REPLACE(A18, FIND("_", A18), 1, ".")</f>
         <v>home.save</v>
       </c>
-      <c r="G18" s="12" t="s">
+      <c r="G18" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="H18" s="12" t="s">
+      <c r="H18" s="13" t="s">
         <v>100</v>
       </c>
-      <c r="I18" s="12"/>
-      <c r="J18" s="12"/>
-      <c r="K18" s="12"/>
+      <c r="I18" s="13"/>
+      <c r="J18" s="13"/>
+      <c r="K18" s="13"/>
       <c r="L18" s="7"/>
       <c r="M18" s="7"/>
       <c r="N18" s="7"/>
@@ -2936,7 +2965,7 @@
       <c r="Q18" s="7"/>
       <c r="R18" s="7"/>
       <c r="S18" s="7"/>
-      <c r="T18" s="13" t="b">
+      <c r="T18" s="17" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -2946,1138 +2975,1138 @@
       <c r="X18" s="7"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="15" t="s">
+      <c r="A19" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="B19" s="16" t="s">
+      <c r="B19" s="19" t="s">
         <v>69</v>
       </c>
-      <c r="C19" s="15" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D19" s="17" t="s">
+      <c r="C19" s="20" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D19" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E19" s="18"/>
-      <c r="F19" s="18"/>
-      <c r="G19" s="15"/>
-      <c r="H19" s="15"/>
-      <c r="I19" s="15"/>
-      <c r="J19" s="15"/>
-      <c r="K19" s="15"/>
-      <c r="L19" s="18"/>
-      <c r="M19" s="18"/>
-      <c r="N19" s="18"/>
-      <c r="O19" s="18"/>
-      <c r="P19" s="18"/>
-      <c r="Q19" s="18"/>
-      <c r="R19" s="18"/>
-      <c r="S19" s="18"/>
-      <c r="T19" s="17" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U19" s="18"/>
-      <c r="V19" s="18"/>
-      <c r="W19" s="18"/>
-      <c r="X19" s="18"/>
+      <c r="E19" s="22"/>
+      <c r="F19" s="22"/>
+      <c r="G19" s="18"/>
+      <c r="H19" s="18"/>
+      <c r="I19" s="18"/>
+      <c r="J19" s="18"/>
+      <c r="K19" s="18"/>
+      <c r="L19" s="22"/>
+      <c r="M19" s="22"/>
+      <c r="N19" s="22"/>
+      <c r="O19" s="22"/>
+      <c r="P19" s="22"/>
+      <c r="Q19" s="22"/>
+      <c r="R19" s="22"/>
+      <c r="S19" s="22"/>
+      <c r="T19" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U19" s="22"/>
+      <c r="V19" s="22"/>
+      <c r="W19" s="22"/>
+      <c r="X19" s="22"/>
     </row>
     <row r="20" customFormat="false" ht="144" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="17" t="s">
+      <c r="A20" s="21" t="s">
         <v>103</v>
       </c>
-      <c r="B20" s="17" t="s">
+      <c r="B20" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="C20" s="17" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D20" s="17" t="s">
+      <c r="C20" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D20" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E20" s="19" t="s">
+      <c r="E20" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F20" s="19" t="s">
+      <c r="F20" s="24" t="s">
         <v>104</v>
       </c>
-      <c r="G20" s="17" t="s">
+      <c r="G20" s="21" t="s">
         <v>105</v>
       </c>
-      <c r="H20" s="17" t="s">
+      <c r="H20" s="21" t="s">
         <v>106</v>
       </c>
-      <c r="I20" s="17"/>
-      <c r="J20" s="17"/>
-      <c r="K20" s="17"/>
-      <c r="L20" s="19"/>
-      <c r="M20" s="19" t="s">
+      <c r="I20" s="21"/>
+      <c r="J20" s="21"/>
+      <c r="K20" s="21"/>
+      <c r="L20" s="24"/>
+      <c r="M20" s="24" t="s">
         <v>95</v>
       </c>
-      <c r="N20" s="20"/>
-      <c r="O20" s="19"/>
-      <c r="P20" s="19"/>
-      <c r="Q20" s="19"/>
-      <c r="R20" s="19"/>
-      <c r="S20" s="19"/>
-      <c r="T20" s="17" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U20" s="19"/>
-      <c r="V20" s="19"/>
-      <c r="W20" s="19"/>
-      <c r="X20" s="19"/>
+      <c r="N20" s="25"/>
+      <c r="O20" s="24"/>
+      <c r="P20" s="24"/>
+      <c r="Q20" s="24"/>
+      <c r="R20" s="24"/>
+      <c r="S20" s="24"/>
+      <c r="T20" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U20" s="24"/>
+      <c r="V20" s="24"/>
+      <c r="W20" s="24"/>
+      <c r="X20" s="24"/>
     </row>
     <row r="21" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="17" t="s">
+      <c r="A21" s="21" t="s">
         <v>107</v>
       </c>
-      <c r="B21" s="17" t="s">
+      <c r="B21" s="21" t="s">
         <v>108</v>
       </c>
-      <c r="C21" s="17" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D21" s="17" t="s">
+      <c r="C21" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D21" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E21" s="19" t="s">
+      <c r="E21" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F21" s="19" t="s">
+      <c r="F21" s="24" t="s">
         <v>109</v>
       </c>
-      <c r="G21" s="17" t="s">
+      <c r="G21" s="21" t="s">
         <v>110</v>
       </c>
-      <c r="H21" s="17" t="s">
+      <c r="H21" s="21" t="s">
         <v>111</v>
       </c>
-      <c r="I21" s="17" t="s">
+      <c r="I21" s="21" t="s">
         <v>112</v>
       </c>
-      <c r="J21" s="17" t="s">
+      <c r="J21" s="21" t="s">
         <v>113</v>
       </c>
-      <c r="K21" s="17"/>
-      <c r="L21" s="19"/>
-      <c r="M21" s="19"/>
-      <c r="N21" s="19" t="s">
+      <c r="K21" s="21"/>
+      <c r="L21" s="24"/>
+      <c r="M21" s="24"/>
+      <c r="N21" s="24" t="s">
         <v>114</v>
       </c>
-      <c r="O21" s="19"/>
-      <c r="P21" s="19"/>
-      <c r="Q21" s="19"/>
-      <c r="R21" s="19"/>
-      <c r="S21" s="19"/>
-      <c r="T21" s="17" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U21" s="19"/>
-      <c r="V21" s="19"/>
-      <c r="W21" s="19"/>
-      <c r="X21" s="19"/>
-    </row>
-    <row r="22" customFormat="false" ht="33.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="17" t="s">
+      <c r="O21" s="24"/>
+      <c r="P21" s="24"/>
+      <c r="Q21" s="24"/>
+      <c r="R21" s="24"/>
+      <c r="S21" s="24"/>
+      <c r="T21" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U21" s="24"/>
+      <c r="V21" s="24"/>
+      <c r="W21" s="24"/>
+      <c r="X21" s="24"/>
+    </row>
+    <row r="22" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="21" t="s">
         <v>115</v>
       </c>
-      <c r="B22" s="17" t="s">
+      <c r="B22" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="C22" s="17" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D22" s="17" t="s">
+      <c r="C22" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D22" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E22" s="19" t="s">
+      <c r="E22" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F22" s="19" t="s">
+      <c r="F22" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="G22" s="17" t="s">
+      <c r="G22" s="21" t="s">
         <v>117</v>
       </c>
-      <c r="H22" s="17" t="s">
+      <c r="H22" s="21" t="s">
         <v>118</v>
       </c>
-      <c r="I22" s="17"/>
-      <c r="J22" s="17"/>
-      <c r="K22" s="17"/>
-      <c r="L22" s="19"/>
-      <c r="M22" s="19" t="s">
+      <c r="I22" s="21"/>
+      <c r="J22" s="21"/>
+      <c r="K22" s="21"/>
+      <c r="L22" s="24"/>
+      <c r="M22" s="24" t="s">
         <v>119</v>
       </c>
-      <c r="N22" s="19"/>
-      <c r="O22" s="19" t="s">
+      <c r="N22" s="24"/>
+      <c r="O22" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="P22" s="19"/>
-      <c r="Q22" s="19"/>
-      <c r="R22" s="19"/>
-      <c r="S22" s="19"/>
-      <c r="T22" s="17" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U22" s="19"/>
-      <c r="V22" s="19"/>
-      <c r="W22" s="19"/>
-      <c r="X22" s="19"/>
-    </row>
-    <row r="23" customFormat="false" ht="33.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="17" t="s">
+      <c r="P22" s="24"/>
+      <c r="Q22" s="24"/>
+      <c r="R22" s="24"/>
+      <c r="S22" s="24"/>
+      <c r="T22" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U22" s="24"/>
+      <c r="V22" s="24"/>
+      <c r="W22" s="24"/>
+      <c r="X22" s="24"/>
+    </row>
+    <row r="23" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="21" t="s">
         <v>120</v>
       </c>
-      <c r="B23" s="17" t="s">
+      <c r="B23" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="C23" s="17" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D23" s="17" t="s">
+      <c r="C23" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D23" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E23" s="19" t="s">
+      <c r="E23" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F23" s="19" t="s">
+      <c r="F23" s="24" t="s">
         <v>121</v>
       </c>
-      <c r="G23" s="17" t="s">
+      <c r="G23" s="21" t="s">
         <v>122</v>
       </c>
-      <c r="H23" s="17" t="s">
+      <c r="H23" s="21" t="s">
         <v>123</v>
       </c>
-      <c r="I23" s="17"/>
-      <c r="J23" s="17"/>
-      <c r="K23" s="17"/>
-      <c r="L23" s="19"/>
-      <c r="M23" s="19" t="s">
+      <c r="I23" s="21"/>
+      <c r="J23" s="21"/>
+      <c r="K23" s="21"/>
+      <c r="L23" s="24"/>
+      <c r="M23" s="24" t="s">
         <v>124</v>
       </c>
-      <c r="N23" s="19"/>
-      <c r="O23" s="19" t="s">
+      <c r="N23" s="24"/>
+      <c r="O23" s="24" t="s">
         <v>125</v>
       </c>
-      <c r="P23" s="19"/>
-      <c r="Q23" s="19"/>
-      <c r="R23" s="19"/>
-      <c r="S23" s="19"/>
-      <c r="T23" s="17" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U23" s="19"/>
-      <c r="V23" s="19"/>
-      <c r="W23" s="19"/>
-      <c r="X23" s="19"/>
+      <c r="P23" s="24"/>
+      <c r="Q23" s="24"/>
+      <c r="R23" s="24"/>
+      <c r="S23" s="24"/>
+      <c r="T23" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U23" s="24"/>
+      <c r="V23" s="24"/>
+      <c r="W23" s="24"/>
+      <c r="X23" s="24"/>
     </row>
     <row r="24" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="17" t="s">
+      <c r="A24" s="21" t="s">
         <v>126</v>
       </c>
-      <c r="B24" s="17" t="s">
+      <c r="B24" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="C24" s="17" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D24" s="17" t="s">
+      <c r="C24" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D24" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E24" s="19" t="s">
+      <c r="E24" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F24" s="19" t="s">
+      <c r="F24" s="24" t="s">
         <v>127</v>
       </c>
-      <c r="G24" s="17" t="s">
+      <c r="G24" s="21" t="s">
         <v>128</v>
       </c>
-      <c r="H24" s="17" t="s">
+      <c r="H24" s="21" t="s">
         <v>129</v>
       </c>
-      <c r="I24" s="17"/>
-      <c r="J24" s="17"/>
-      <c r="K24" s="17"/>
-      <c r="L24" s="19"/>
-      <c r="M24" s="19" t="s">
+      <c r="I24" s="21"/>
+      <c r="J24" s="21"/>
+      <c r="K24" s="21"/>
+      <c r="L24" s="24"/>
+      <c r="M24" s="24" t="s">
         <v>130</v>
       </c>
-      <c r="N24" s="19"/>
-      <c r="O24" s="19" t="s">
+      <c r="N24" s="24"/>
+      <c r="O24" s="24" t="s">
         <v>125</v>
       </c>
-      <c r="P24" s="20"/>
-      <c r="Q24" s="19"/>
-      <c r="R24" s="19"/>
-      <c r="S24" s="19"/>
-      <c r="T24" s="17" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U24" s="19"/>
-      <c r="V24" s="19"/>
-      <c r="W24" s="19"/>
-      <c r="X24" s="19"/>
+      <c r="P24" s="25"/>
+      <c r="Q24" s="24"/>
+      <c r="R24" s="24"/>
+      <c r="S24" s="24"/>
+      <c r="T24" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U24" s="24"/>
+      <c r="V24" s="24"/>
+      <c r="W24" s="24"/>
+      <c r="X24" s="24"/>
     </row>
     <row r="25" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="17" t="s">
+      <c r="A25" s="21" t="s">
         <v>131</v>
       </c>
-      <c r="B25" s="17" t="s">
+      <c r="B25" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="C25" s="17" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D25" s="17" t="s">
+      <c r="C25" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D25" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E25" s="19" t="s">
+      <c r="E25" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F25" s="19" t="s">
+      <c r="F25" s="24" t="s">
         <v>132</v>
       </c>
-      <c r="G25" s="17"/>
-      <c r="H25" s="17"/>
-      <c r="I25" s="17"/>
-      <c r="J25" s="17"/>
-      <c r="K25" s="21" t="s">
+      <c r="G25" s="21"/>
+      <c r="H25" s="21"/>
+      <c r="I25" s="21"/>
+      <c r="J25" s="21"/>
+      <c r="K25" s="26" t="s">
         <v>133</v>
       </c>
-      <c r="L25" s="19"/>
-      <c r="M25" s="22" t="s">
+      <c r="L25" s="24"/>
+      <c r="M25" s="27" t="s">
         <v>134</v>
       </c>
-      <c r="N25" s="19"/>
-      <c r="O25" s="19" t="s">
+      <c r="N25" s="24"/>
+      <c r="O25" s="24" t="s">
         <v>132</v>
       </c>
-      <c r="P25" s="19"/>
-      <c r="Q25" s="19"/>
-      <c r="R25" s="19"/>
-      <c r="S25" s="19"/>
-      <c r="T25" s="17" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U25" s="19" t="s">
+      <c r="P25" s="24"/>
+      <c r="Q25" s="24"/>
+      <c r="R25" s="24"/>
+      <c r="S25" s="24"/>
+      <c r="T25" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U25" s="24" t="s">
         <v>135</v>
       </c>
-      <c r="V25" s="19" t="s">
+      <c r="V25" s="24" t="s">
         <v>136</v>
       </c>
-      <c r="W25" s="19"/>
-      <c r="X25" s="19"/>
+      <c r="W25" s="24"/>
+      <c r="X25" s="24"/>
     </row>
     <row r="26" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="17" t="s">
+      <c r="A26" s="21" t="s">
         <v>137</v>
       </c>
-      <c r="B26" s="17" t="s">
+      <c r="B26" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="C26" s="17" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D26" s="17" t="s">
+      <c r="C26" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D26" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E26" s="19" t="s">
+      <c r="E26" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F26" s="23" t="s">
+      <c r="F26" s="28" t="s">
         <v>138</v>
       </c>
-      <c r="G26" s="17" t="s">
+      <c r="G26" s="21" t="s">
         <v>139</v>
       </c>
-      <c r="H26" s="17" t="s">
+      <c r="H26" s="21" t="s">
         <v>140</v>
       </c>
-      <c r="I26" s="17"/>
-      <c r="J26" s="17"/>
-      <c r="K26" s="17"/>
-      <c r="L26" s="19"/>
-      <c r="M26" s="19" t="s">
+      <c r="I26" s="21"/>
+      <c r="J26" s="21"/>
+      <c r="K26" s="21"/>
+      <c r="L26" s="24"/>
+      <c r="M26" s="24" t="s">
         <v>141</v>
       </c>
-      <c r="N26" s="19"/>
-      <c r="O26" s="19" t="s">
+      <c r="N26" s="24"/>
+      <c r="O26" s="24" t="s">
         <v>137</v>
       </c>
-      <c r="P26" s="19"/>
-      <c r="Q26" s="19"/>
-      <c r="R26" s="19"/>
-      <c r="S26" s="19"/>
-      <c r="T26" s="17" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U26" s="19"/>
-      <c r="V26" s="19"/>
-      <c r="W26" s="19"/>
-      <c r="X26" s="19"/>
+      <c r="P26" s="24"/>
+      <c r="Q26" s="24"/>
+      <c r="R26" s="24"/>
+      <c r="S26" s="24"/>
+      <c r="T26" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U26" s="24"/>
+      <c r="V26" s="24"/>
+      <c r="W26" s="24"/>
+      <c r="X26" s="24"/>
     </row>
     <row r="27" customFormat="false" ht="62.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="17" t="s">
+      <c r="A27" s="21" t="s">
         <v>142</v>
       </c>
-      <c r="B27" s="17" t="s">
+      <c r="B27" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="C27" s="17" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D27" s="17" t="s">
+      <c r="C27" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D27" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E27" s="19" t="s">
+      <c r="E27" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F27" s="19" t="s">
+      <c r="F27" s="24" t="s">
         <v>143</v>
       </c>
-      <c r="G27" s="17" t="s">
+      <c r="G27" s="21" t="s">
         <v>144</v>
       </c>
-      <c r="H27" s="17" t="s">
+      <c r="H27" s="21" t="s">
         <v>145</v>
       </c>
-      <c r="I27" s="17"/>
-      <c r="J27" s="17"/>
-      <c r="K27" s="17"/>
-      <c r="L27" s="19"/>
-      <c r="M27" s="19" t="s">
+      <c r="I27" s="21"/>
+      <c r="J27" s="21"/>
+      <c r="K27" s="21"/>
+      <c r="L27" s="24"/>
+      <c r="M27" s="24" t="s">
         <v>130</v>
       </c>
-      <c r="N27" s="19"/>
-      <c r="O27" s="19" t="s">
+      <c r="N27" s="24"/>
+      <c r="O27" s="24" t="s">
         <v>146</v>
       </c>
-      <c r="P27" s="19"/>
-      <c r="Q27" s="19"/>
-      <c r="R27" s="19"/>
-      <c r="S27" s="19"/>
-      <c r="T27" s="17" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U27" s="19"/>
-      <c r="V27" s="19"/>
-      <c r="W27" s="19"/>
-      <c r="X27" s="19"/>
+      <c r="P27" s="24"/>
+      <c r="Q27" s="24"/>
+      <c r="R27" s="24"/>
+      <c r="S27" s="24"/>
+      <c r="T27" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U27" s="24"/>
+      <c r="V27" s="24"/>
+      <c r="W27" s="24"/>
+      <c r="X27" s="24"/>
     </row>
     <row r="28" customFormat="false" ht="52.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="17" t="s">
+      <c r="A28" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="B28" s="17" t="s">
+      <c r="B28" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="C28" s="17" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D28" s="17" t="s">
+      <c r="C28" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D28" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E28" s="19" t="s">
+      <c r="E28" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F28" s="19" t="s">
+      <c r="F28" s="24" t="s">
         <v>148</v>
       </c>
-      <c r="G28" s="17" t="s">
+      <c r="G28" s="21" t="s">
         <v>149</v>
       </c>
-      <c r="H28" s="17" t="s">
+      <c r="H28" s="21" t="s">
         <v>150</v>
       </c>
-      <c r="I28" s="17"/>
-      <c r="J28" s="17"/>
-      <c r="K28" s="17"/>
-      <c r="L28" s="19"/>
-      <c r="M28" s="19" t="s">
+      <c r="I28" s="21"/>
+      <c r="J28" s="21"/>
+      <c r="K28" s="21"/>
+      <c r="L28" s="24"/>
+      <c r="M28" s="24" t="s">
         <v>151</v>
       </c>
-      <c r="N28" s="19"/>
-      <c r="O28" s="19" t="s">
+      <c r="N28" s="24"/>
+      <c r="O28" s="24" t="s">
         <v>146</v>
       </c>
-      <c r="P28" s="19"/>
-      <c r="Q28" s="19"/>
-      <c r="R28" s="19"/>
-      <c r="S28" s="19"/>
-      <c r="T28" s="17" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U28" s="19"/>
-      <c r="V28" s="19"/>
-      <c r="W28" s="19"/>
-      <c r="X28" s="19"/>
-    </row>
-    <row r="29" customFormat="false" ht="33.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="24" t="s">
+      <c r="P28" s="24"/>
+      <c r="Q28" s="24"/>
+      <c r="R28" s="24"/>
+      <c r="S28" s="24"/>
+      <c r="T28" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U28" s="24"/>
+      <c r="V28" s="24"/>
+      <c r="W28" s="24"/>
+      <c r="X28" s="24"/>
+    </row>
+    <row r="29" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="29" t="s">
         <v>152</v>
       </c>
-      <c r="B29" s="17" t="s">
+      <c r="B29" s="21" t="s">
         <v>153</v>
       </c>
-      <c r="C29" s="17" t="b">
+      <c r="C29" s="23" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="D29" s="17" t="s">
+      <c r="D29" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E29" s="19" t="s">
+      <c r="E29" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F29" s="19" t="s">
+      <c r="F29" s="24" t="s">
         <v>154</v>
       </c>
-      <c r="G29" s="17" t="s">
+      <c r="G29" s="21" t="s">
         <v>155</v>
       </c>
-      <c r="H29" s="17" t="s">
+      <c r="H29" s="21" t="s">
         <v>156</v>
       </c>
-      <c r="I29" s="17"/>
-      <c r="J29" s="17"/>
-      <c r="K29" s="17"/>
-      <c r="L29" s="19"/>
-      <c r="M29" s="19" t="s">
+      <c r="I29" s="21"/>
+      <c r="J29" s="21"/>
+      <c r="K29" s="21"/>
+      <c r="L29" s="24"/>
+      <c r="M29" s="24" t="s">
         <v>157</v>
       </c>
-      <c r="N29" s="20"/>
-      <c r="O29" s="19" t="s">
+      <c r="N29" s="25"/>
+      <c r="O29" s="24" t="s">
         <v>158</v>
       </c>
-      <c r="P29" s="19"/>
-      <c r="Q29" s="19"/>
-      <c r="R29" s="19"/>
-      <c r="S29" s="19"/>
-      <c r="T29" s="17" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U29" s="19"/>
-      <c r="V29" s="19"/>
-      <c r="W29" s="19"/>
-      <c r="X29" s="19"/>
-    </row>
-    <row r="30" customFormat="false" ht="33.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="17" t="s">
+      <c r="P29" s="24"/>
+      <c r="Q29" s="24"/>
+      <c r="R29" s="24"/>
+      <c r="S29" s="24"/>
+      <c r="T29" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U29" s="24"/>
+      <c r="V29" s="24"/>
+      <c r="W29" s="24"/>
+      <c r="X29" s="24"/>
+    </row>
+    <row r="30" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="21" t="s">
         <v>159</v>
       </c>
-      <c r="B30" s="17" t="s">
+      <c r="B30" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="C30" s="17" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D30" s="17" t="s">
+      <c r="C30" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D30" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E30" s="19" t="s">
+      <c r="E30" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F30" s="19" t="s">
+      <c r="F30" s="24" t="s">
         <v>160</v>
       </c>
-      <c r="G30" s="17" t="s">
+      <c r="G30" s="21" t="s">
         <v>161</v>
       </c>
-      <c r="H30" s="17" t="s">
+      <c r="H30" s="21" t="s">
         <v>162</v>
       </c>
-      <c r="I30" s="17"/>
-      <c r="J30" s="17"/>
-      <c r="K30" s="17"/>
-      <c r="L30" s="19"/>
-      <c r="M30" s="19" t="s">
+      <c r="I30" s="21"/>
+      <c r="J30" s="21"/>
+      <c r="K30" s="21"/>
+      <c r="L30" s="24"/>
+      <c r="M30" s="24" t="s">
         <v>163</v>
       </c>
-      <c r="N30" s="19"/>
-      <c r="O30" s="19" t="s">
+      <c r="N30" s="24"/>
+      <c r="O30" s="24" t="s">
         <v>96</v>
       </c>
-      <c r="P30" s="19"/>
-      <c r="Q30" s="19"/>
-      <c r="R30" s="19"/>
-      <c r="S30" s="19"/>
-      <c r="T30" s="17" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U30" s="19"/>
-      <c r="V30" s="19"/>
-      <c r="W30" s="19"/>
-      <c r="X30" s="19"/>
+      <c r="P30" s="24"/>
+      <c r="Q30" s="24"/>
+      <c r="R30" s="24"/>
+      <c r="S30" s="24"/>
+      <c r="T30" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U30" s="24"/>
+      <c r="V30" s="24"/>
+      <c r="W30" s="24"/>
+      <c r="X30" s="24"/>
     </row>
     <row r="31" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="17" t="s">
+      <c r="A31" s="21" t="s">
         <v>164</v>
       </c>
-      <c r="B31" s="17" t="s">
+      <c r="B31" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="C31" s="17" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D31" s="17" t="s">
+      <c r="C31" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D31" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E31" s="19" t="s">
+      <c r="E31" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F31" s="19" t="s">
+      <c r="F31" s="24" t="s">
         <v>165</v>
       </c>
-      <c r="G31" s="17" t="s">
+      <c r="G31" s="21" t="s">
         <v>166</v>
       </c>
-      <c r="H31" s="17" t="s">
+      <c r="H31" s="21" t="s">
         <v>167</v>
       </c>
-      <c r="I31" s="17"/>
-      <c r="J31" s="17"/>
-      <c r="K31" s="17"/>
-      <c r="L31" s="19"/>
-      <c r="M31" s="19" t="s">
+      <c r="I31" s="21"/>
+      <c r="J31" s="21"/>
+      <c r="K31" s="21"/>
+      <c r="L31" s="24"/>
+      <c r="M31" s="24" t="s">
         <v>168</v>
       </c>
-      <c r="N31" s="19"/>
-      <c r="O31" s="19" t="s">
+      <c r="N31" s="24"/>
+      <c r="O31" s="24" t="s">
         <v>165</v>
       </c>
-      <c r="P31" s="19"/>
-      <c r="Q31" s="19"/>
-      <c r="R31" s="19"/>
-      <c r="S31" s="19"/>
-      <c r="T31" s="17" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U31" s="19"/>
-      <c r="V31" s="19"/>
-      <c r="W31" s="19"/>
-      <c r="X31" s="19"/>
+      <c r="P31" s="24"/>
+      <c r="Q31" s="24"/>
+      <c r="R31" s="24"/>
+      <c r="S31" s="24"/>
+      <c r="T31" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U31" s="24"/>
+      <c r="V31" s="24"/>
+      <c r="W31" s="24"/>
+      <c r="X31" s="24"/>
     </row>
     <row r="32" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="17" t="s">
+      <c r="A32" s="21" t="s">
         <v>169</v>
       </c>
-      <c r="B32" s="17" t="s">
+      <c r="B32" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="C32" s="17" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D32" s="17" t="s">
+      <c r="C32" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D32" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E32" s="19" t="s">
+      <c r="E32" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F32" s="19" t="s">
+      <c r="F32" s="24" t="s">
         <v>170</v>
       </c>
-      <c r="G32" s="17" t="s">
+      <c r="G32" s="21" t="s">
         <v>171</v>
       </c>
-      <c r="H32" s="17" t="s">
+      <c r="H32" s="21" t="s">
         <v>172</v>
       </c>
-      <c r="I32" s="17"/>
-      <c r="J32" s="17"/>
-      <c r="K32" s="17"/>
-      <c r="L32" s="19"/>
-      <c r="M32" s="19" t="s">
+      <c r="I32" s="21"/>
+      <c r="J32" s="21"/>
+      <c r="K32" s="21"/>
+      <c r="L32" s="24"/>
+      <c r="M32" s="24" t="s">
         <v>173</v>
       </c>
-      <c r="N32" s="19"/>
-      <c r="O32" s="19" t="s">
+      <c r="N32" s="24"/>
+      <c r="O32" s="24" t="s">
         <v>174</v>
       </c>
-      <c r="P32" s="19"/>
-      <c r="Q32" s="19"/>
-      <c r="R32" s="19"/>
-      <c r="S32" s="19"/>
-      <c r="T32" s="17" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U32" s="19"/>
-      <c r="V32" s="19"/>
-      <c r="W32" s="19"/>
-      <c r="X32" s="19"/>
+      <c r="P32" s="24"/>
+      <c r="Q32" s="24"/>
+      <c r="R32" s="24"/>
+      <c r="S32" s="24"/>
+      <c r="T32" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U32" s="24"/>
+      <c r="V32" s="24"/>
+      <c r="W32" s="24"/>
+      <c r="X32" s="24"/>
     </row>
     <row r="33" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="17" t="s">
+      <c r="A33" s="21" t="s">
         <v>175</v>
       </c>
-      <c r="B33" s="17" t="s">
+      <c r="B33" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="C33" s="17" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D33" s="17" t="s">
+      <c r="C33" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D33" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E33" s="19" t="s">
+      <c r="E33" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F33" s="19" t="s">
+      <c r="F33" s="24" t="s">
         <v>176</v>
       </c>
-      <c r="G33" s="17" t="s">
+      <c r="G33" s="21" t="s">
         <v>177</v>
       </c>
-      <c r="H33" s="17" t="s">
+      <c r="H33" s="21" t="s">
         <v>178</v>
       </c>
-      <c r="I33" s="17"/>
-      <c r="J33" s="17"/>
-      <c r="K33" s="17"/>
-      <c r="L33" s="19"/>
-      <c r="M33" s="17" t="s">
+      <c r="I33" s="21"/>
+      <c r="J33" s="21"/>
+      <c r="K33" s="21"/>
+      <c r="L33" s="24"/>
+      <c r="M33" s="21" t="s">
         <v>179</v>
       </c>
-      <c r="N33" s="19"/>
-      <c r="O33" s="19"/>
-      <c r="P33" s="19"/>
-      <c r="Q33" s="19"/>
-      <c r="R33" s="19"/>
-      <c r="S33" s="19"/>
-      <c r="T33" s="17" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U33" s="19"/>
-      <c r="V33" s="19"/>
-      <c r="W33" s="19"/>
-      <c r="X33" s="19"/>
-    </row>
-    <row r="34" customFormat="false" ht="87.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="17" t="s">
+      <c r="N33" s="24"/>
+      <c r="O33" s="24"/>
+      <c r="P33" s="24"/>
+      <c r="Q33" s="24"/>
+      <c r="R33" s="24"/>
+      <c r="S33" s="24"/>
+      <c r="T33" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U33" s="24"/>
+      <c r="V33" s="24"/>
+      <c r="W33" s="24"/>
+      <c r="X33" s="24"/>
+    </row>
+    <row r="34" customFormat="false" ht="85.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="21" t="s">
         <v>180</v>
       </c>
-      <c r="B34" s="25" t="s">
+      <c r="B34" s="30" t="s">
         <v>69</v>
       </c>
-      <c r="C34" s="17" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D34" s="17" t="s">
+      <c r="C34" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D34" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E34" s="19" t="s">
+      <c r="E34" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F34" s="19" t="s">
+      <c r="F34" s="24" t="s">
         <v>181</v>
       </c>
-      <c r="G34" s="17" t="s">
+      <c r="G34" s="21" t="s">
         <v>182</v>
       </c>
-      <c r="H34" s="17" t="s">
+      <c r="H34" s="21" t="s">
         <v>183</v>
       </c>
-      <c r="I34" s="17" t="s">
+      <c r="I34" s="21" t="s">
         <v>184</v>
       </c>
-      <c r="J34" s="17" t="s">
+      <c r="J34" s="21" t="s">
         <v>185</v>
       </c>
-      <c r="K34" s="17"/>
-      <c r="L34" s="19"/>
-      <c r="M34" s="17" t="s">
+      <c r="K34" s="21"/>
+      <c r="L34" s="24"/>
+      <c r="M34" s="21" t="s">
         <v>179</v>
       </c>
-      <c r="N34" s="19"/>
-      <c r="O34" s="19"/>
-      <c r="P34" s="19"/>
-      <c r="Q34" s="19"/>
-      <c r="R34" s="19"/>
-      <c r="S34" s="19"/>
-      <c r="T34" s="17" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U34" s="19"/>
-      <c r="V34" s="19"/>
-      <c r="W34" s="19"/>
-      <c r="X34" s="19"/>
+      <c r="N34" s="24"/>
+      <c r="O34" s="24"/>
+      <c r="P34" s="24"/>
+      <c r="Q34" s="24"/>
+      <c r="R34" s="24"/>
+      <c r="S34" s="24"/>
+      <c r="T34" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U34" s="24"/>
+      <c r="V34" s="24"/>
+      <c r="W34" s="24"/>
+      <c r="X34" s="24"/>
     </row>
     <row r="35" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="17" t="s">
+      <c r="A35" s="21" t="s">
         <v>186</v>
       </c>
-      <c r="B35" s="17" t="s">
+      <c r="B35" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="C35" s="17" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D35" s="17" t="s">
+      <c r="C35" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D35" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E35" s="19" t="s">
+      <c r="E35" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F35" s="19" t="s">
+      <c r="F35" s="24" t="s">
         <v>187</v>
       </c>
-      <c r="G35" s="17" t="s">
+      <c r="G35" s="21" t="s">
         <v>188</v>
       </c>
-      <c r="H35" s="17" t="s">
+      <c r="H35" s="21" t="s">
         <v>189</v>
       </c>
-      <c r="I35" s="17"/>
-      <c r="J35" s="17"/>
-      <c r="K35" s="17"/>
-      <c r="L35" s="19"/>
-      <c r="M35" s="17" t="s">
+      <c r="I35" s="21"/>
+      <c r="J35" s="21"/>
+      <c r="K35" s="21"/>
+      <c r="L35" s="24"/>
+      <c r="M35" s="21" t="s">
         <v>190</v>
       </c>
-      <c r="N35" s="19"/>
-      <c r="O35" s="19"/>
-      <c r="P35" s="19"/>
-      <c r="Q35" s="19"/>
-      <c r="R35" s="19"/>
-      <c r="S35" s="19"/>
-      <c r="T35" s="17" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U35" s="19"/>
-      <c r="V35" s="19"/>
-      <c r="W35" s="19"/>
-      <c r="X35" s="19"/>
-    </row>
-    <row r="36" customFormat="false" ht="87.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="17" t="s">
+      <c r="N35" s="24"/>
+      <c r="O35" s="24"/>
+      <c r="P35" s="24"/>
+      <c r="Q35" s="24"/>
+      <c r="R35" s="24"/>
+      <c r="S35" s="24"/>
+      <c r="T35" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U35" s="24"/>
+      <c r="V35" s="24"/>
+      <c r="W35" s="24"/>
+      <c r="X35" s="24"/>
+    </row>
+    <row r="36" customFormat="false" ht="85.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="21" t="s">
         <v>191</v>
       </c>
-      <c r="B36" s="25" t="s">
+      <c r="B36" s="30" t="s">
         <v>69</v>
       </c>
-      <c r="C36" s="17" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D36" s="17" t="s">
+      <c r="C36" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D36" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E36" s="19" t="s">
+      <c r="E36" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F36" s="19" t="s">
+      <c r="F36" s="24" t="s">
         <v>192</v>
       </c>
-      <c r="G36" s="17" t="s">
+      <c r="G36" s="21" t="s">
         <v>193</v>
       </c>
-      <c r="H36" s="17" t="s">
+      <c r="H36" s="21" t="s">
         <v>194</v>
       </c>
-      <c r="I36" s="17" t="s">
+      <c r="I36" s="21" t="s">
         <v>195</v>
       </c>
-      <c r="J36" s="17" t="s">
+      <c r="J36" s="21" t="s">
         <v>196</v>
       </c>
-      <c r="K36" s="26"/>
-      <c r="L36" s="27"/>
-      <c r="M36" s="26"/>
-      <c r="N36" s="27"/>
-      <c r="O36" s="27"/>
-      <c r="P36" s="27"/>
-      <c r="Q36" s="27"/>
-      <c r="R36" s="19"/>
-      <c r="S36" s="19"/>
-      <c r="T36" s="17" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U36" s="19"/>
-      <c r="V36" s="19"/>
-      <c r="W36" s="19"/>
-      <c r="X36" s="19"/>
+      <c r="K36" s="31"/>
+      <c r="L36" s="32"/>
+      <c r="M36" s="31"/>
+      <c r="N36" s="32"/>
+      <c r="O36" s="32"/>
+      <c r="P36" s="32"/>
+      <c r="Q36" s="32"/>
+      <c r="R36" s="24"/>
+      <c r="S36" s="24"/>
+      <c r="T36" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U36" s="24"/>
+      <c r="V36" s="24"/>
+      <c r="W36" s="24"/>
+      <c r="X36" s="24"/>
     </row>
     <row r="37" customFormat="false" ht="86.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="24" t="s">
+      <c r="A37" s="29" t="s">
         <v>197</v>
       </c>
-      <c r="B37" s="17" t="s">
+      <c r="B37" s="21" t="s">
         <v>153</v>
       </c>
-      <c r="C37" s="17" t="b">
+      <c r="C37" s="23" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="D37" s="17" t="s">
+      <c r="D37" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E37" s="19" t="s">
+      <c r="E37" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F37" s="19" t="s">
+      <c r="F37" s="24" t="s">
         <v>198</v>
       </c>
-      <c r="G37" s="17" t="s">
+      <c r="G37" s="21" t="s">
         <v>199</v>
       </c>
-      <c r="H37" s="17" t="s">
+      <c r="H37" s="21" t="s">
         <v>200</v>
       </c>
-      <c r="I37" s="17"/>
-      <c r="J37" s="17"/>
-      <c r="K37" s="17"/>
-      <c r="L37" s="19"/>
-      <c r="M37" s="20"/>
-      <c r="N37" s="20"/>
-      <c r="O37" s="28" t="s">
+      <c r="I37" s="21"/>
+      <c r="J37" s="21"/>
+      <c r="K37" s="21"/>
+      <c r="L37" s="24"/>
+      <c r="M37" s="25"/>
+      <c r="N37" s="25"/>
+      <c r="O37" s="33" t="s">
         <v>146</v>
       </c>
-      <c r="P37" s="19"/>
-      <c r="Q37" s="19"/>
-      <c r="R37" s="19"/>
-      <c r="S37" s="19"/>
-      <c r="T37" s="17" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U37" s="19"/>
-      <c r="V37" s="19"/>
-      <c r="W37" s="19"/>
-      <c r="X37" s="19"/>
+      <c r="P37" s="24"/>
+      <c r="Q37" s="24"/>
+      <c r="R37" s="24"/>
+      <c r="S37" s="24"/>
+      <c r="T37" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U37" s="24"/>
+      <c r="V37" s="24"/>
+      <c r="W37" s="24"/>
+      <c r="X37" s="24"/>
     </row>
     <row r="38" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="24" t="s">
+      <c r="A38" s="29" t="s">
         <v>201</v>
       </c>
-      <c r="B38" s="17" t="s">
+      <c r="B38" s="21" t="s">
         <v>153</v>
       </c>
-      <c r="C38" s="17" t="b">
+      <c r="C38" s="23" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="D38" s="17" t="s">
+      <c r="D38" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E38" s="19" t="s">
+      <c r="E38" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F38" s="19" t="s">
+      <c r="F38" s="24" t="s">
         <v>202</v>
       </c>
-      <c r="G38" s="17" t="s">
+      <c r="G38" s="21" t="s">
         <v>203</v>
       </c>
-      <c r="H38" s="17" t="s">
+      <c r="H38" s="21" t="s">
         <v>204</v>
       </c>
-      <c r="I38" s="17"/>
-      <c r="J38" s="17"/>
-      <c r="K38" s="17"/>
-      <c r="L38" s="19"/>
-      <c r="M38" s="20"/>
-      <c r="N38" s="20"/>
-      <c r="O38" s="28" t="s">
+      <c r="I38" s="21"/>
+      <c r="J38" s="21"/>
+      <c r="K38" s="21"/>
+      <c r="L38" s="24"/>
+      <c r="M38" s="25"/>
+      <c r="N38" s="25"/>
+      <c r="O38" s="33" t="s">
         <v>146</v>
       </c>
-      <c r="P38" s="19"/>
-      <c r="Q38" s="19"/>
-      <c r="R38" s="19"/>
-      <c r="S38" s="19"/>
-      <c r="T38" s="17" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U38" s="19"/>
-      <c r="V38" s="19"/>
-      <c r="W38" s="19"/>
-      <c r="X38" s="19"/>
-    </row>
-    <row r="39" s="6" customFormat="true" ht="55.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="24" t="s">
+      <c r="P38" s="24"/>
+      <c r="Q38" s="24"/>
+      <c r="R38" s="24"/>
+      <c r="S38" s="24"/>
+      <c r="T38" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U38" s="24"/>
+      <c r="V38" s="24"/>
+      <c r="W38" s="24"/>
+      <c r="X38" s="24"/>
+    </row>
+    <row r="39" s="6" customFormat="true" ht="64.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="29" t="s">
         <v>205</v>
       </c>
-      <c r="B39" s="17" t="s">
+      <c r="B39" s="21" t="s">
         <v>153</v>
       </c>
-      <c r="C39" s="17" t="b">
+      <c r="C39" s="23" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="D39" s="17" t="s">
+      <c r="D39" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E39" s="19" t="s">
+      <c r="E39" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F39" s="19" t="s">
+      <c r="F39" s="24" t="s">
         <v>206</v>
       </c>
-      <c r="G39" s="17" t="s">
+      <c r="G39" s="21" t="s">
         <v>207</v>
       </c>
-      <c r="H39" s="17" t="s">
+      <c r="H39" s="21" t="s">
         <v>208</v>
       </c>
-      <c r="I39" s="17"/>
-      <c r="J39" s="17"/>
-      <c r="K39" s="17"/>
-      <c r="L39" s="19"/>
-      <c r="M39" s="20"/>
-      <c r="N39" s="20"/>
-      <c r="O39" s="28" t="s">
+      <c r="I39" s="21"/>
+      <c r="J39" s="21"/>
+      <c r="K39" s="21"/>
+      <c r="L39" s="24"/>
+      <c r="M39" s="25"/>
+      <c r="N39" s="25"/>
+      <c r="O39" s="33" t="s">
         <v>146</v>
       </c>
-      <c r="P39" s="19"/>
-      <c r="Q39" s="19"/>
-      <c r="R39" s="19"/>
-      <c r="S39" s="19"/>
-      <c r="T39" s="17" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U39" s="19"/>
-      <c r="V39" s="19"/>
-      <c r="W39" s="19"/>
-      <c r="X39" s="19"/>
+      <c r="P39" s="24"/>
+      <c r="Q39" s="24"/>
+      <c r="R39" s="24"/>
+      <c r="S39" s="24"/>
+      <c r="T39" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U39" s="24"/>
+      <c r="V39" s="24"/>
+      <c r="W39" s="24"/>
+      <c r="X39" s="24"/>
     </row>
     <row r="40" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="24" t="s">
+      <c r="A40" s="29" t="s">
         <v>209</v>
       </c>
-      <c r="B40" s="17" t="s">
+      <c r="B40" s="21" t="s">
         <v>153</v>
       </c>
-      <c r="C40" s="17" t="b">
+      <c r="C40" s="23" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="D40" s="17" t="s">
+      <c r="D40" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E40" s="19" t="s">
+      <c r="E40" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F40" s="19" t="s">
+      <c r="F40" s="24" t="s">
         <v>210</v>
       </c>
-      <c r="G40" s="17" t="s">
+      <c r="G40" s="21" t="s">
         <v>211</v>
       </c>
-      <c r="H40" s="17" t="s">
+      <c r="H40" s="21" t="s">
         <v>212</v>
       </c>
-      <c r="I40" s="17"/>
-      <c r="J40" s="17"/>
-      <c r="K40" s="17"/>
-      <c r="L40" s="19"/>
-      <c r="M40" s="20"/>
-      <c r="N40" s="20"/>
-      <c r="O40" s="28" t="s">
+      <c r="I40" s="21"/>
+      <c r="J40" s="21"/>
+      <c r="K40" s="21"/>
+      <c r="L40" s="24"/>
+      <c r="M40" s="25"/>
+      <c r="N40" s="25"/>
+      <c r="O40" s="33" t="s">
         <v>146</v>
       </c>
-      <c r="P40" s="19"/>
-      <c r="Q40" s="19"/>
-      <c r="R40" s="19"/>
-      <c r="S40" s="19"/>
-      <c r="T40" s="17" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U40" s="19"/>
-      <c r="V40" s="19"/>
-      <c r="W40" s="19"/>
-      <c r="X40" s="19"/>
+      <c r="P40" s="24"/>
+      <c r="Q40" s="24"/>
+      <c r="R40" s="24"/>
+      <c r="S40" s="24"/>
+      <c r="T40" s="23" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U40" s="24"/>
+      <c r="V40" s="24"/>
+      <c r="W40" s="24"/>
+      <c r="X40" s="24"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="29" t="s">
+      <c r="A41" s="34" t="s">
         <v>213</v>
       </c>
-      <c r="B41" s="29" t="s">
+      <c r="B41" s="34" t="s">
         <v>98</v>
       </c>
-      <c r="C41" s="29" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D41" s="29" t="s">
+      <c r="C41" s="35" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D41" s="34" t="s">
         <v>102</v>
       </c>
-      <c r="E41" s="30"/>
-      <c r="F41" s="30" t="str">
+      <c r="E41" s="36"/>
+      <c r="F41" s="36" t="str">
         <f aca="false">REPLACE(A41, FIND("_", A41), 1, ".")</f>
         <v>household.save</v>
       </c>
-      <c r="G41" s="29" t="s">
+      <c r="G41" s="34" t="s">
         <v>99</v>
       </c>
-      <c r="H41" s="29" t="s">
+      <c r="H41" s="34" t="s">
         <v>100</v>
       </c>
-      <c r="I41" s="29"/>
-      <c r="J41" s="29"/>
-      <c r="K41" s="29"/>
-      <c r="L41" s="30"/>
-      <c r="M41" s="30"/>
-      <c r="N41" s="30"/>
-      <c r="O41" s="30"/>
-      <c r="P41" s="30"/>
-      <c r="Q41" s="30"/>
-      <c r="R41" s="30"/>
-      <c r="S41" s="30"/>
-      <c r="T41" s="29" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U41" s="30"/>
-      <c r="V41" s="30"/>
-      <c r="W41" s="30"/>
-      <c r="X41" s="30"/>
-    </row>
-    <row r="42" customFormat="false" ht="116.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I41" s="34"/>
+      <c r="J41" s="34"/>
+      <c r="K41" s="34"/>
+      <c r="L41" s="36"/>
+      <c r="M41" s="36"/>
+      <c r="N41" s="36"/>
+      <c r="O41" s="36"/>
+      <c r="P41" s="36"/>
+      <c r="Q41" s="36"/>
+      <c r="R41" s="36"/>
+      <c r="S41" s="36"/>
+      <c r="T41" s="35" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U41" s="36"/>
+      <c r="V41" s="36"/>
+      <c r="W41" s="36"/>
+      <c r="X41" s="36"/>
+    </row>
+    <row r="42" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
         <v>214</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C42" s="1" t="b">
+      <c r="C42" s="37" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -4093,9 +4122,9 @@
       <c r="H42" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="L42" s="31"/>
-      <c r="M42" s="32"/>
-      <c r="T42" s="1" t="b">
+      <c r="L42" s="38"/>
+      <c r="M42" s="39"/>
+      <c r="T42" s="37" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -4150,489 +4179,489 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F29"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="33" width="27.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="33" width="15.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="33" width="31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="34" width="20.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="33" width="19.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="33" width="12.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="40" width="27.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="40" width="15.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="40" width="31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="41" width="20.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="40" width="19.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="40" width="12.14"/>
   </cols>
   <sheetData>
-    <row r="1" s="37" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="35" t="s">
+    <row r="1" s="44" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="42" t="s">
         <v>218</v>
       </c>
-      <c r="B1" s="35" t="s">
+      <c r="B1" s="42" t="s">
         <v>219</v>
       </c>
-      <c r="C1" s="35" t="s">
+      <c r="C1" s="42" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="36" t="s">
+      <c r="D1" s="43" t="s">
         <v>220</v>
       </c>
-      <c r="E1" s="35" t="s">
+      <c r="E1" s="42" t="s">
         <v>221</v>
       </c>
-      <c r="F1" s="35" t="s">
+      <c r="F1" s="42" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="38" t="s">
+    <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="45" t="s">
         <v>223</v>
       </c>
-      <c r="B2" s="38"/>
-      <c r="C2" s="38" t="s">
+      <c r="B2" s="45"/>
+      <c r="C2" s="45" t="s">
         <v>224</v>
       </c>
-      <c r="D2" s="39" t="s">
+      <c r="D2" s="46" t="s">
         <v>225</v>
       </c>
-      <c r="E2" s="38" t="n">
-        <v>1</v>
-      </c>
-      <c r="F2" s="38"/>
-    </row>
-    <row r="3" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="38" t="s">
+      <c r="E2" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="45"/>
+    </row>
+    <row r="3" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="45" t="s">
         <v>95</v>
       </c>
-      <c r="B3" s="38"/>
-      <c r="C3" s="38" t="s">
+      <c r="B3" s="45"/>
+      <c r="C3" s="45" t="s">
         <v>224</v>
       </c>
-      <c r="D3" s="39" t="s">
+      <c r="D3" s="46" t="s">
         <v>226</v>
       </c>
-      <c r="E3" s="38" t="n">
+      <c r="E3" s="45" t="n">
         <v>2</v>
       </c>
-      <c r="F3" s="38"/>
-    </row>
-    <row r="4" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="38" t="s">
+      <c r="F3" s="45"/>
+    </row>
+    <row r="4" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="45" t="s">
         <v>163</v>
       </c>
-      <c r="B4" s="38"/>
-      <c r="C4" s="38" t="s">
+      <c r="B4" s="45"/>
+      <c r="C4" s="45" t="s">
         <v>227</v>
       </c>
-      <c r="D4" s="39" t="s">
+      <c r="D4" s="46" t="s">
         <v>225</v>
       </c>
-      <c r="E4" s="38" t="s">
+      <c r="E4" s="45" t="s">
         <v>228</v>
       </c>
-      <c r="F4" s="38"/>
-    </row>
-    <row r="5" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="38" t="s">
+      <c r="F4" s="45"/>
+    </row>
+    <row r="5" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="45" t="s">
         <v>163</v>
       </c>
-      <c r="B5" s="38" t="s">
+      <c r="B5" s="45" t="s">
         <v>229</v>
       </c>
-      <c r="C5" s="38" t="s">
+      <c r="C5" s="45" t="s">
         <v>224</v>
       </c>
-      <c r="D5" s="39" t="s">
+      <c r="D5" s="46" t="s">
         <v>225</v>
       </c>
-      <c r="E5" s="38" t="n">
-        <v>1</v>
-      </c>
-      <c r="F5" s="38"/>
-    </row>
-    <row r="6" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="38" t="s">
+      <c r="E5" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="45"/>
+    </row>
+    <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="45" t="s">
         <v>230</v>
       </c>
-      <c r="B6" s="38"/>
-      <c r="C6" s="38" t="s">
+      <c r="B6" s="45"/>
+      <c r="C6" s="45" t="s">
         <v>231</v>
       </c>
-      <c r="D6" s="39" t="s">
+      <c r="D6" s="46" t="s">
         <v>226</v>
       </c>
-      <c r="E6" s="38" t="n">
+      <c r="E6" s="45" t="n">
         <v>3</v>
       </c>
-      <c r="F6" s="38"/>
-    </row>
-    <row r="7" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="38" t="s">
+      <c r="F6" s="45"/>
+    </row>
+    <row r="7" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="45" t="s">
         <v>230</v>
       </c>
-      <c r="B7" s="38" t="s">
+      <c r="B7" s="45" t="s">
         <v>232</v>
       </c>
-      <c r="C7" s="38" t="s">
+      <c r="C7" s="45" t="s">
         <v>231</v>
       </c>
-      <c r="D7" s="39" t="s">
+      <c r="D7" s="46" t="s">
         <v>233</v>
       </c>
-      <c r="E7" s="38" t="n">
+      <c r="E7" s="45" t="n">
         <v>5</v>
       </c>
-      <c r="F7" s="38"/>
-    </row>
-    <row r="8" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="38" t="s">
+      <c r="F7" s="45"/>
+    </row>
+    <row r="8" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="45" t="s">
         <v>234</v>
       </c>
-      <c r="B8" s="38"/>
-      <c r="C8" s="38" t="s">
+      <c r="B8" s="45"/>
+      <c r="C8" s="45" t="s">
         <v>231</v>
       </c>
-      <c r="D8" s="39" t="s">
+      <c r="D8" s="46" t="s">
         <v>226</v>
       </c>
-      <c r="E8" s="38" t="n">
+      <c r="E8" s="45" t="n">
         <v>4</v>
       </c>
-      <c r="F8" s="38"/>
-    </row>
-    <row r="9" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="38" t="s">
+      <c r="F8" s="45"/>
+    </row>
+    <row r="9" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="45" t="s">
         <v>234</v>
       </c>
-      <c r="B9" s="38" t="s">
+      <c r="B9" s="45" t="s">
         <v>232</v>
       </c>
-      <c r="C9" s="38" t="s">
+      <c r="C9" s="45" t="s">
         <v>231</v>
       </c>
-      <c r="D9" s="39" t="s">
+      <c r="D9" s="46" t="s">
         <v>233</v>
       </c>
-      <c r="E9" s="38" t="n">
+      <c r="E9" s="45" t="n">
         <v>13</v>
       </c>
-      <c r="F9" s="38"/>
-    </row>
-    <row r="10" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="38" t="s">
+      <c r="F9" s="45"/>
+    </row>
+    <row r="10" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="45" t="s">
         <v>235</v>
       </c>
-      <c r="B10" s="38"/>
-      <c r="C10" s="38" t="s">
+      <c r="B10" s="45"/>
+      <c r="C10" s="45" t="s">
         <v>231</v>
       </c>
-      <c r="D10" s="39" t="s">
+      <c r="D10" s="46" t="s">
         <v>233</v>
       </c>
-      <c r="E10" s="38" t="n">
+      <c r="E10" s="45" t="n">
         <v>5</v>
       </c>
-      <c r="F10" s="38"/>
-    </row>
-    <row r="11" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="38" t="s">
+      <c r="F10" s="45"/>
+    </row>
+    <row r="11" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="45" t="s">
         <v>119</v>
       </c>
-      <c r="B11" s="38"/>
-      <c r="C11" s="38" t="s">
+      <c r="B11" s="45"/>
+      <c r="C11" s="45" t="s">
         <v>231</v>
       </c>
-      <c r="D11" s="39" t="s">
+      <c r="D11" s="46" t="s">
         <v>226</v>
       </c>
-      <c r="E11" s="38" t="n">
+      <c r="E11" s="45" t="n">
         <v>5</v>
       </c>
-      <c r="F11" s="38"/>
-    </row>
-    <row r="12" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="38" t="s">
+      <c r="F11" s="45"/>
+    </row>
+    <row r="12" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="45" t="s">
         <v>157</v>
       </c>
-      <c r="B12" s="38"/>
-      <c r="C12" s="38" t="s">
+      <c r="B12" s="45"/>
+      <c r="C12" s="45" t="s">
         <v>231</v>
       </c>
-      <c r="D12" s="39" t="s">
+      <c r="D12" s="46" t="s">
         <v>226</v>
       </c>
-      <c r="E12" s="38" t="n">
+      <c r="E12" s="45" t="n">
         <v>6</v>
       </c>
-      <c r="F12" s="38"/>
-    </row>
-    <row r="13" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="38" t="s">
+      <c r="F12" s="45"/>
+    </row>
+    <row r="13" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="45" t="s">
         <v>236</v>
       </c>
-      <c r="B13" s="38"/>
-      <c r="C13" s="38" t="s">
+      <c r="B13" s="45"/>
+      <c r="C13" s="45" t="s">
         <v>231</v>
       </c>
-      <c r="D13" s="39" t="s">
+      <c r="D13" s="46" t="s">
         <v>226</v>
       </c>
-      <c r="E13" s="38" t="n">
+      <c r="E13" s="45" t="n">
         <v>11</v>
       </c>
-      <c r="F13" s="38"/>
-    </row>
-    <row r="14" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="38" t="s">
+      <c r="F13" s="45"/>
+    </row>
+    <row r="14" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="45" t="s">
         <v>124</v>
       </c>
-      <c r="B14" s="38"/>
-      <c r="C14" s="38" t="s">
+      <c r="B14" s="45"/>
+      <c r="C14" s="45" t="s">
         <v>231</v>
       </c>
-      <c r="D14" s="39" t="s">
+      <c r="D14" s="46" t="s">
         <v>226</v>
       </c>
-      <c r="E14" s="38" t="n">
+      <c r="E14" s="45" t="n">
         <v>14</v>
       </c>
-      <c r="F14" s="38"/>
-    </row>
-    <row r="15" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="38" t="s">
+      <c r="F14" s="45"/>
+    </row>
+    <row r="15" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="45" t="s">
         <v>134</v>
       </c>
-      <c r="B15" s="38"/>
-      <c r="C15" s="38" t="s">
+      <c r="B15" s="45"/>
+      <c r="C15" s="45" t="s">
         <v>231</v>
       </c>
-      <c r="D15" s="39" t="s">
+      <c r="D15" s="46" t="s">
         <v>233</v>
       </c>
-      <c r="E15" s="38" t="n">
+      <c r="E15" s="45" t="n">
         <v>15</v>
       </c>
-      <c r="F15" s="38"/>
-    </row>
-    <row r="16" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="38" t="s">
+      <c r="F15" s="45"/>
+    </row>
+    <row r="16" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="45" t="s">
         <v>134</v>
       </c>
-      <c r="B16" s="38" t="s">
+      <c r="B16" s="45" t="s">
         <v>232</v>
       </c>
-      <c r="C16" s="38" t="s">
+      <c r="C16" s="45" t="s">
         <v>231</v>
       </c>
-      <c r="D16" s="39" t="s">
+      <c r="D16" s="46" t="s">
         <v>237</v>
       </c>
-      <c r="E16" s="38" t="s">
+      <c r="E16" s="45" t="s">
         <v>238</v>
       </c>
-      <c r="F16" s="38"/>
-    </row>
-    <row r="17" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="38" t="s">
+      <c r="F16" s="45"/>
+    </row>
+    <row r="17" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="45" t="s">
         <v>239</v>
       </c>
-      <c r="B17" s="38"/>
-      <c r="C17" s="38" t="s">
+      <c r="B17" s="45"/>
+      <c r="C17" s="45" t="s">
         <v>231</v>
       </c>
-      <c r="D17" s="39" t="s">
+      <c r="D17" s="46" t="s">
         <v>226</v>
       </c>
-      <c r="E17" s="38" t="n">
+      <c r="E17" s="45" t="n">
         <v>15</v>
       </c>
-      <c r="F17" s="38"/>
-    </row>
-    <row r="18" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="38" t="s">
+      <c r="F17" s="45"/>
+    </row>
+    <row r="18" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="45" t="s">
         <v>130</v>
       </c>
-      <c r="B18" s="38"/>
-      <c r="C18" s="38" t="s">
+      <c r="B18" s="45"/>
+      <c r="C18" s="45" t="s">
         <v>231</v>
       </c>
-      <c r="D18" s="39" t="s">
+      <c r="D18" s="46" t="s">
         <v>226</v>
       </c>
-      <c r="E18" s="38" t="n">
+      <c r="E18" s="45" t="n">
         <v>16</v>
       </c>
-      <c r="F18" s="38"/>
-    </row>
-    <row r="19" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="38" t="s">
+      <c r="F18" s="45"/>
+    </row>
+    <row r="19" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="45" t="s">
         <v>240</v>
       </c>
-      <c r="B19" s="38"/>
-      <c r="C19" s="38" t="s">
+      <c r="B19" s="45"/>
+      <c r="C19" s="45" t="s">
         <v>231</v>
       </c>
-      <c r="D19" s="39" t="s">
+      <c r="D19" s="46" t="s">
         <v>226</v>
       </c>
-      <c r="E19" s="38" t="n">
+      <c r="E19" s="45" t="n">
         <v>40</v>
       </c>
-      <c r="F19" s="38"/>
-    </row>
-    <row r="20" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="38" t="s">
+      <c r="F19" s="45"/>
+    </row>
+    <row r="20" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="45" t="s">
         <v>151</v>
       </c>
-      <c r="B20" s="38"/>
-      <c r="C20" s="38" t="s">
+      <c r="B20" s="45"/>
+      <c r="C20" s="45" t="s">
         <v>241</v>
       </c>
-      <c r="D20" s="39" t="s">
+      <c r="D20" s="46" t="s">
         <v>225</v>
       </c>
-      <c r="E20" s="38" t="s">
+      <c r="E20" s="45" t="s">
         <v>228</v>
       </c>
-      <c r="F20" s="38"/>
-    </row>
-    <row r="21" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="33" t="s">
+      <c r="F20" s="45"/>
+    </row>
+    <row r="21" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="40" t="s">
         <v>168</v>
       </c>
-      <c r="C21" s="33" t="s">
+      <c r="C21" s="40" t="s">
         <v>242</v>
       </c>
-      <c r="D21" s="39" t="s">
+      <c r="D21" s="46" t="s">
         <v>225</v>
       </c>
-      <c r="E21" s="34" t="s">
+      <c r="E21" s="41" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="33" t="s">
+    <row r="22" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="40" t="s">
         <v>168</v>
       </c>
-      <c r="B22" s="33" t="s">
+      <c r="B22" s="40" t="s">
         <v>229</v>
       </c>
-      <c r="C22" s="33" t="s">
+      <c r="C22" s="40" t="s">
         <v>242</v>
       </c>
-      <c r="D22" s="39" t="s">
+      <c r="D22" s="46" t="s">
         <v>225</v>
       </c>
-      <c r="E22" s="34" t="s">
+      <c r="E22" s="41" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="33" t="s">
+    <row r="23" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="40" t="s">
         <v>168</v>
       </c>
-      <c r="B23" s="33" t="s">
+      <c r="B23" s="40" t="s">
         <v>229</v>
       </c>
-      <c r="C23" s="33" t="s">
+      <c r="C23" s="40" t="s">
         <v>242</v>
       </c>
-      <c r="D23" s="39" t="s">
+      <c r="D23" s="46" t="s">
         <v>225</v>
       </c>
-      <c r="E23" s="34" t="s">
+      <c r="E23" s="41" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="33" t="s">
+    <row r="24" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="40" t="s">
         <v>173</v>
       </c>
-      <c r="C24" s="33" t="s">
+      <c r="C24" s="40" t="s">
         <v>242</v>
       </c>
-      <c r="D24" s="39" t="s">
+      <c r="D24" s="46" t="s">
         <v>225</v>
       </c>
-      <c r="E24" s="34" t="s">
+      <c r="E24" s="41" t="s">
         <v>246</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="33" t="s">
+    <row r="25" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="40" t="s">
         <v>173</v>
       </c>
-      <c r="B25" s="33" t="s">
+      <c r="B25" s="40" t="s">
         <v>229</v>
       </c>
-      <c r="C25" s="33" t="s">
+      <c r="C25" s="40" t="s">
         <v>242</v>
       </c>
-      <c r="D25" s="39" t="s">
+      <c r="D25" s="46" t="s">
         <v>225</v>
       </c>
-      <c r="E25" s="34" t="s">
+      <c r="E25" s="41" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="33" t="s">
+    <row r="26" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="40" t="s">
         <v>173</v>
       </c>
-      <c r="B26" s="33" t="s">
+      <c r="B26" s="40" t="s">
         <v>229</v>
       </c>
-      <c r="C26" s="33" t="s">
+      <c r="C26" s="40" t="s">
         <v>242</v>
       </c>
-      <c r="D26" s="39" t="s">
+      <c r="D26" s="46" t="s">
         <v>225</v>
       </c>
-      <c r="E26" s="34" t="s">
+      <c r="E26" s="41" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="33" t="s">
+    <row r="27" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="40" t="s">
         <v>179</v>
       </c>
-      <c r="C27" s="33" t="s">
+      <c r="C27" s="40" t="s">
         <v>248</v>
       </c>
-      <c r="D27" s="39" t="s">
+      <c r="D27" s="46" t="s">
         <v>225</v>
       </c>
-      <c r="E27" s="33" t="s">
+      <c r="E27" s="40" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="33" t="s">
+    <row r="28" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="40" t="s">
         <v>179</v>
       </c>
-      <c r="B28" s="33" t="s">
+      <c r="B28" s="40" t="s">
         <v>229</v>
       </c>
-      <c r="C28" s="33" t="s">
+      <c r="C28" s="40" t="s">
         <v>248</v>
       </c>
-      <c r="D28" s="39" t="s">
+      <c r="D28" s="46" t="s">
         <v>225</v>
       </c>
-      <c r="E28" s="33" t="s">
+      <c r="E28" s="40" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="33" t="s">
+    <row r="29" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="40" t="s">
         <v>179</v>
       </c>
-      <c r="B29" s="33" t="s">
+      <c r="B29" s="40" t="s">
         <v>229</v>
       </c>
-      <c r="C29" s="33" t="s">
+      <c r="C29" s="40" t="s">
         <v>248</v>
       </c>
-      <c r="D29" s="39" t="s">
+      <c r="D29" s="46" t="s">
         <v>225</v>
       </c>
-      <c r="E29" s="33" t="s">
+      <c r="E29" s="40" t="s">
         <v>251</v>
       </c>
     </row>
@@ -4653,126 +4682,126 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:J4"/>
-  <sheetFormatPr defaultColWidth="10.69921875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.69921875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="38" width="10.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="38" width="12.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="38" width="13.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="38" width="12.57"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="6" min="5" style="38" width="10.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="38" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="38" width="15.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="38" width="15.68"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="38" width="21.93"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="11" style="38" width="10.7"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="45" width="10.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="45" width="12.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="45" width="13.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="45" width="12.57"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="6" min="5" style="45" width="10.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="45" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="45" width="15.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="45" width="15.68"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="45" width="21.93"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="11" style="45" width="10.7"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="47" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="41" t="s">
+      <c r="B1" s="48" t="s">
         <v>252</v>
       </c>
-      <c r="C1" s="40" t="s">
+      <c r="C1" s="47" t="s">
         <v>253</v>
       </c>
-      <c r="D1" s="40" t="s">
+      <c r="D1" s="47" t="s">
         <v>254</v>
       </c>
-      <c r="E1" s="40" t="s">
+      <c r="E1" s="47" t="s">
         <v>255</v>
       </c>
-      <c r="F1" s="40" t="s">
+      <c r="F1" s="47" t="s">
         <v>256</v>
       </c>
-      <c r="G1" s="40" t="s">
+      <c r="G1" s="47" t="s">
         <v>257</v>
       </c>
-      <c r="H1" s="40" t="s">
+      <c r="H1" s="47" t="s">
         <v>258</v>
       </c>
-      <c r="I1" s="40" t="s">
+      <c r="I1" s="47" t="s">
         <v>259</v>
       </c>
-      <c r="J1" s="40" t="s">
+      <c r="J1" s="47" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="38" t="s">
+    <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="45" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="38" t="s">
+      <c r="B2" s="45" t="s">
         <v>261</v>
       </c>
-      <c r="C2" s="38" t="s">
+      <c r="C2" s="45" t="s">
         <v>262</v>
       </c>
-      <c r="D2" s="38" t="s">
+      <c r="D2" s="45" t="s">
         <v>263</v>
       </c>
-      <c r="E2" s="42" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="F2" s="42" t="b">
+      <c r="E2" s="49" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="F2" s="49" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="G2" s="42" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="38" t="s">
+      <c r="G2" s="49" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="45" t="s">
         <v>102</v>
       </c>
-      <c r="B3" s="38" t="s">
+      <c r="B3" s="45" t="s">
         <v>264</v>
       </c>
-      <c r="C3" s="38" t="s">
+      <c r="C3" s="45" t="s">
         <v>265</v>
       </c>
-      <c r="D3" s="38" t="s">
+      <c r="D3" s="45" t="s">
         <v>266</v>
       </c>
-      <c r="E3" s="42" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="F3" s="42" t="b">
+      <c r="E3" s="49" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="F3" s="49" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="G3" s="42" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="38" t="s">
+      <c r="G3" s="49" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="45" t="s">
         <v>215</v>
       </c>
-      <c r="B4" s="38" t="s">
+      <c r="B4" s="45" t="s">
         <v>267</v>
       </c>
-      <c r="C4" s="38" t="s">
+      <c r="C4" s="45" t="s">
         <v>268</v>
       </c>
-      <c r="D4" s="38" t="s">
+      <c r="D4" s="45" t="s">
         <v>269</v>
       </c>
-      <c r="E4" s="42" t="b">
+      <c r="E4" s="49" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="F4" s="42" t="b">
+      <c r="F4" s="49" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="G4" s="42" t="b">
+      <c r="G4" s="49" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -4793,63 +4822,63 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H1048576"/>
-  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:H51"/>
+  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="43" width="21.3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="43" width="15.72"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="43" width="23.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="43" width="19.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="43" width="21.08"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="43" width="24.29"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="9" style="43" width="9.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="50" width="21.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="50" width="15.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="50" width="23.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="50" width="19.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="50" width="21.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="50" width="24.29"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="9" style="50" width="9.14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="51" t="s">
         <v>270</v>
       </c>
-      <c r="B1" s="44" t="s">
+      <c r="B1" s="51" t="s">
         <v>221</v>
       </c>
-      <c r="C1" s="44" t="s">
+      <c r="C1" s="51" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="44" t="s">
+      <c r="D1" s="51" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="44" t="s">
+      <c r="E1" s="51" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="44" t="s">
+      <c r="F1" s="51" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="44" t="s">
+      <c r="G1" s="51" t="s">
         <v>271</v>
       </c>
-      <c r="H1" s="44" t="s">
+      <c r="H1" s="51" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="B2" s="45" t="s">
+      <c r="B2" s="52" t="s">
         <v>228</v>
       </c>
-      <c r="C2" s="45" t="s">
+      <c r="C2" s="52" t="s">
         <v>272</v>
       </c>
-      <c r="D2" s="45" t="s">
+      <c r="D2" s="52" t="s">
         <v>273</v>
       </c>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
-    </row>
-    <row r="3" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="52"/>
+      <c r="H2" s="52"/>
+    </row>
+    <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
         <v>274</v>
       </c>
@@ -4867,7 +4896,7 @@
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
     </row>
-    <row r="4" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
         <v>136</v>
       </c>
@@ -4885,7 +4914,7 @@
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
     </row>
-    <row r="5" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
         <v>279</v>
       </c>
@@ -4903,7 +4932,7 @@
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
     </row>
-    <row r="6" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
         <v>282</v>
       </c>
@@ -4921,7 +4950,7 @@
       <c r="G6" s="1"/>
       <c r="H6" s="1"/>
     </row>
-    <row r="7" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
         <v>285</v>
       </c>
@@ -4939,7 +4968,7 @@
       <c r="G7" s="1"/>
       <c r="H7" s="1"/>
     </row>
-    <row r="8" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
         <v>33</v>
       </c>
@@ -4953,7 +4982,7 @@
       </c>
       <c r="H8" s="1"/>
     </row>
-    <row r="9" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
         <v>33</v>
       </c>
@@ -4967,7 +4996,7 @@
       </c>
       <c r="H9" s="1"/>
     </row>
-    <row r="10" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
         <v>146</v>
       </c>
@@ -4981,7 +5010,7 @@
       </c>
       <c r="H10" s="1"/>
     </row>
-    <row r="11" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
         <v>146</v>
       </c>
@@ -4995,7 +5024,7 @@
       </c>
       <c r="H11" s="1"/>
     </row>
-    <row r="12" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
         <v>96</v>
       </c>
@@ -5009,7 +5038,7 @@
       </c>
       <c r="H12" s="1"/>
     </row>
-    <row r="13" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
         <v>96</v>
       </c>
@@ -5023,7 +5052,7 @@
       </c>
       <c r="H13" s="1"/>
     </row>
-    <row r="14" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
         <v>96</v>
       </c>
@@ -5037,7 +5066,7 @@
       </c>
       <c r="H14" s="1"/>
     </row>
-    <row r="15" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
         <v>116</v>
       </c>
@@ -5055,7 +5084,7 @@
       <c r="G15" s="1"/>
       <c r="H15" s="1"/>
     </row>
-    <row r="16" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
         <v>116</v>
       </c>
@@ -5073,7 +5102,7 @@
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
     </row>
-    <row r="17" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
         <v>116</v>
       </c>
@@ -5087,7 +5116,7 @@
       </c>
       <c r="H17" s="1"/>
     </row>
-    <row r="18" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
         <v>125</v>
       </c>
@@ -5105,7 +5134,7 @@
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
     </row>
-    <row r="19" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
         <v>125</v>
       </c>
@@ -5123,7 +5152,7 @@
       <c r="G19" s="1"/>
       <c r="H19" s="1"/>
     </row>
-    <row r="20" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
         <v>125</v>
       </c>
@@ -5137,7 +5166,7 @@
       </c>
       <c r="H20" s="1"/>
     </row>
-    <row r="21" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
         <v>132</v>
       </c>
@@ -5157,7 +5186,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
         <v>132</v>
       </c>
@@ -5177,7 +5206,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
         <v>132</v>
       </c>
@@ -5197,7 +5226,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
         <v>132</v>
       </c>
@@ -5215,7 +5244,7 @@
       <c r="G24" s="1"/>
       <c r="H24" s="1"/>
     </row>
-    <row r="25" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
         <v>132</v>
       </c>
@@ -5235,7 +5264,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
         <v>132</v>
       </c>
@@ -5249,7 +5278,7 @@
       </c>
       <c r="H26" s="1"/>
     </row>
-    <row r="27" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
         <v>137</v>
       </c>
@@ -5267,7 +5296,7 @@
       <c r="G27" s="1"/>
       <c r="H27" s="1"/>
     </row>
-    <row r="28" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
         <v>137</v>
       </c>
@@ -5285,7 +5314,7 @@
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
     </row>
-    <row r="29" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
         <v>137</v>
       </c>
@@ -5303,7 +5332,7 @@
       <c r="G29" s="1"/>
       <c r="H29" s="1"/>
     </row>
-    <row r="30" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
         <v>137</v>
       </c>
@@ -5321,7 +5350,7 @@
       <c r="G30" s="1"/>
       <c r="H30" s="1"/>
     </row>
-    <row r="31" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
         <v>137</v>
       </c>
@@ -5339,7 +5368,7 @@
       <c r="G31" s="1"/>
       <c r="H31" s="1"/>
     </row>
-    <row r="32" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
         <v>137</v>
       </c>
@@ -5359,7 +5388,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
         <v>137</v>
       </c>
@@ -5377,7 +5406,7 @@
       <c r="G33" s="1"/>
       <c r="H33" s="1"/>
     </row>
-    <row r="34" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
         <v>137</v>
       </c>
@@ -5395,7 +5424,7 @@
       <c r="G34" s="1"/>
       <c r="H34" s="1"/>
     </row>
-    <row r="35" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
         <v>137</v>
       </c>
@@ -5413,7 +5442,7 @@
       <c r="G35" s="1"/>
       <c r="H35" s="1"/>
     </row>
-    <row r="36" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
         <v>137</v>
       </c>
@@ -5431,7 +5460,7 @@
       <c r="G36" s="1"/>
       <c r="H36" s="1"/>
     </row>
-    <row r="37" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
         <v>137</v>
       </c>
@@ -5449,7 +5478,7 @@
       <c r="G37" s="1"/>
       <c r="H37" s="1"/>
     </row>
-    <row r="38" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
         <v>137</v>
       </c>
@@ -5467,7 +5496,7 @@
       <c r="G38" s="1"/>
       <c r="H38" s="1"/>
     </row>
-    <row r="39" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
         <v>137</v>
       </c>
@@ -5485,7 +5514,7 @@
       <c r="G39" s="1"/>
       <c r="H39" s="1"/>
     </row>
-    <row r="40" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
         <v>158</v>
       </c>
@@ -5499,7 +5528,7 @@
       </c>
       <c r="H40" s="1"/>
     </row>
-    <row r="41" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
         <v>158</v>
       </c>
@@ -5517,7 +5546,7 @@
       <c r="G41" s="1"/>
       <c r="H41" s="1"/>
     </row>
-    <row r="42" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
         <v>158</v>
       </c>
@@ -5535,7 +5564,7 @@
       <c r="G42" s="1"/>
       <c r="H42" s="1"/>
     </row>
-    <row r="43" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
         <v>158</v>
       </c>
@@ -5549,7 +5578,7 @@
       </c>
       <c r="H43" s="1"/>
     </row>
-    <row r="44" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
         <v>165</v>
       </c>
@@ -5567,7 +5596,7 @@
       <c r="G44" s="1"/>
       <c r="H44" s="1"/>
     </row>
-    <row r="45" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
         <v>165</v>
       </c>
@@ -5585,7 +5614,7 @@
       <c r="G45" s="1"/>
       <c r="H45" s="1"/>
     </row>
-    <row r="46" customFormat="false" ht="73.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
         <v>165</v>
       </c>
@@ -5603,7 +5632,7 @@
       <c r="G46" s="1"/>
       <c r="H46" s="1"/>
     </row>
-    <row r="47" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
         <v>165</v>
       </c>
@@ -5621,7 +5650,7 @@
       <c r="G47" s="1"/>
       <c r="H47" s="1"/>
     </row>
-    <row r="48" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
         <v>165</v>
       </c>
@@ -5639,49 +5668,48 @@
       <c r="G48" s="1"/>
       <c r="H48" s="1"/>
     </row>
-    <row r="49" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="43" t="s">
+    <row r="49" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="50" t="s">
         <v>174</v>
       </c>
-      <c r="B49" s="43" t="s">
+      <c r="B49" s="50" t="s">
         <v>249</v>
       </c>
-      <c r="C49" s="43" t="s">
+      <c r="C49" s="50" t="s">
         <v>364</v>
       </c>
-      <c r="D49" s="43" t="s">
+      <c r="D49" s="50" t="s">
         <v>353</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="43" t="s">
+    <row r="50" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="50" t="s">
         <v>174</v>
       </c>
-      <c r="B50" s="43" t="s">
+      <c r="B50" s="50" t="s">
         <v>250</v>
       </c>
-      <c r="C50" s="43" t="s">
+      <c r="C50" s="50" t="s">
         <v>365</v>
       </c>
-      <c r="D50" s="43" t="s">
+      <c r="D50" s="50" t="s">
         <v>366</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="43" t="s">
+    <row r="51" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="50" t="s">
         <v>174</v>
       </c>
-      <c r="B51" s="43" t="s">
+      <c r="B51" s="50" t="s">
         <v>361</v>
       </c>
-      <c r="C51" s="43" t="s">
+      <c r="C51" s="50" t="s">
         <v>367</v>
       </c>
-      <c r="D51" s="43" t="s">
+      <c r="D51" s="50" t="s">
         <v>368</v>
       </c>
     </row>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -5699,55 +5727,55 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L1"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="33" width="18.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="33" width="17.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="33" width="13.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="33" width="12.72"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="33" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="33" width="13.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="33" width="14.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="33" width="11.28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="33" width="13.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="33" width="14.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="40" width="18.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="40" width="17.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="40" width="13.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="40" width="12.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="40" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="40" width="13.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="40" width="14.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="40" width="11.28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="40" width="13.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="40" width="14.43"/>
   </cols>
   <sheetData>
-    <row r="1" s="44" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="46" t="s">
+    <row r="1" s="51" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="53" t="s">
         <v>369</v>
       </c>
-      <c r="B1" s="46" t="s">
+      <c r="B1" s="53" t="s">
         <v>370</v>
       </c>
-      <c r="C1" s="46" t="s">
+      <c r="C1" s="53" t="s">
         <v>371</v>
       </c>
-      <c r="D1" s="46" t="s">
+      <c r="D1" s="53" t="s">
         <v>372</v>
       </c>
-      <c r="E1" s="46" t="s">
+      <c r="E1" s="53" t="s">
         <v>373</v>
       </c>
-      <c r="F1" s="46" t="s">
+      <c r="F1" s="53" t="s">
         <v>374</v>
       </c>
-      <c r="G1" s="46" t="s">
+      <c r="G1" s="53" t="s">
         <v>375</v>
       </c>
-      <c r="H1" s="46" t="s">
+      <c r="H1" s="53" t="s">
         <v>376</v>
       </c>
-      <c r="I1" s="46" t="s">
+      <c r="I1" s="53" t="s">
         <v>377</v>
       </c>
-      <c r="J1" s="46" t="s">
+      <c r="J1" s="53" t="s">
         <v>378</v>
       </c>
-      <c r="K1" s="46" t="s">
+      <c r="K1" s="53" t="s">
         <v>379</v>
       </c>
-      <c r="L1" s="44" t="s">
+      <c r="L1" s="51" t="s">
         <v>380</v>
       </c>
     </row>
@@ -5768,13 +5796,13 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G3"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="33" width="10.34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="33" width="32.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="33" width="43.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="33" width="46.08"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="33" width="28.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="40" width="10.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="40" width="32.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="40" width="43.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="40" width="46.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="40" width="28.55"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5796,39 +5824,39 @@
       <c r="F1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="33"/>
+      <c r="G1" s="40"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="47" t="s">
+      <c r="A2" s="54" t="s">
         <v>102</v>
       </c>
-      <c r="B2" s="38" t="s">
+      <c r="B2" s="45" t="s">
         <v>383</v>
       </c>
-      <c r="C2" s="47" t="s">
+      <c r="C2" s="54" t="s">
         <v>384</v>
       </c>
-      <c r="D2" s="47" t="s">
+      <c r="D2" s="54" t="s">
         <v>385</v>
       </c>
-      <c r="E2" s="47"/>
-      <c r="F2" s="47"/>
+      <c r="E2" s="54"/>
+      <c r="F2" s="54"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="47" t="s">
+      <c r="A3" s="54" t="s">
         <v>102</v>
       </c>
-      <c r="B3" s="38" t="s">
+      <c r="B3" s="45" t="s">
         <v>386</v>
       </c>
-      <c r="C3" s="47" t="s">
+      <c r="C3" s="54" t="s">
         <v>387</v>
       </c>
-      <c r="D3" s="47" t="s">
+      <c r="D3" s="54" t="s">
         <v>388</v>
       </c>
-      <c r="E3" s="47"/>
-      <c r="F3" s="47"/>
+      <c r="E3" s="54"/>
+      <c r="F3" s="54"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>